<commit_message>
docs: requisitos adicionales documentados, avance 80,5 %
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -632,10 +632,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D4" t="n">
         <v>6</v>
@@ -644,10 +644,10 @@
         <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.8461538461538461</v>
       </c>
     </row>
     <row r="5">
@@ -657,10 +657,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -669,10 +669,10 @@
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.7333333333333333</v>
       </c>
     </row>
     <row r="6">
@@ -682,16 +682,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>0.7241379310344828</v>
+        <v>0.8048780487804879</v>
       </c>
     </row>
     <row r="8">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23.2</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="9">
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2.2</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="11">
@@ -733,7 +733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1220,6 +1220,206 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>RQF-19</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Gestión de Usuarios</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>routes/auth.js POST /signup y RegisterOwnerPage.jsx: registro del gimnasio y de la cuenta del propietario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>RQF-20</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>routes/config.js (GET/PUT /admin/config), ConfigPage.jsx y tabla config_gimnasio: planes, precios y recordatorios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RQF-21</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Gestión de Miembros</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Tabla plan_cobro (migración 004): tipo de plan, vigencia, valor total y pagado, método y estado de pago por miembro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>RQF-22</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cumplimiento</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>routes/auth.js DELETE /auth/account y EliminarCuentaPage.jsx: elimina cuenta y datos del gimnasio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RQF-23</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>routes/notificaciones.js GET /admin/notificaciones: avisos accionables en la campana del encabezado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>RQF-24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Check-in y Asistencia</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>routes/asistencia.js GET /api/asistencia: listado de check-ins con resumen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RQF-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Gestión de Miembros</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>routes/vista.js GET /api/vista/miembros-activos: vista de miembros activos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RQF-26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>App del miembro</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>routes/cliente.js PUT /api/cliente/me: el miembro edita su perfil desde la app.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1231,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1543,6 +1743,106 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RQNF-12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cumplimiento</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Rutas /legal/terminos, /legal/privacidad y /legal/datos (TerminosPage, PrivacidadPage, PoliticaDatosPage).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>RQNF-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Observabilidad</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>index.js: endpoints /api/healthz y /api/health.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>RQNF-14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Mantenibilidad</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>lib/errors.js, lib/asyncHandler.js y errorHandler central: respuestas de error consistentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RQNF-15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Implementado</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>index.js: CORS restringido por origen configurado.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(avance): actualiza la evidencia del CI tras fusionar main
El PR #5 agrego el check de nombre de rama y movio las lineas de
ci.yml citadas en RQNF-09 (EV-34). Las cifras no cambian.
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31FA15C-BEE1-4D18-A125-51497B3774A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3663D572-96CE-47BF-98D0-5A89291EE09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -745,7 +745,7 @@
     <t>Validación automática en integración continua (GitHub Actions) en cada pull request y en main.</t>
   </si>
   <si>
-    <t>.github/workflows/ci.yml corre en pull_request y en push a main (:3-6): backend npm ci + node --check (:27-29), frontend npm ci + build (:43-44); ejecución exitosa en main 54b19fa (pestaña Actions).</t>
+    <t>.github/workflows/ci.yml corre en pull_request y en push a main (:3-6): el job rama valida el nombre de la rama en cada PR (:13-26), backend npm ci + node --check (:42-44) y frontend npm ci + build (:58-59); ejecución exitosa en main 8acab31 (pestaña Actions).</t>
   </si>
   <si>
     <t>Observación: el CI todavía no corre pruebas ni mide cobertura.</t>
@@ -1069,10 +1069,10 @@
     <t>Configuración / ejecución</t>
   </si>
   <si>
-    <t>.github/workflows/ci.yml:3-6, :27-29, :43-44; https://github.com/Luis140721/Proyecto_Fitloyalty/actions (CI en main 54b19fa: success)</t>
-  </si>
-  <si>
-    <t>CI en cada PR y en main con instalación limpia, sintaxis y build.</t>
+    <t>.github/workflows/ci.yml:3-6, :13-26, :42-44, :58-59; https://github.com/Luis140721/Proyecto_Fitloyalty/actions (CI en main 8acab31: success)</t>
+  </si>
+  <si>
+    <t>CI en cada PR y en main: nombre de rama, instalación limpia, sintaxis y build.</t>
   </si>
 </sst>
 </file>
@@ -1499,7 +1499,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-66A4-45C5-852A-009F11104544}"/>
+              <c16:uniqueId val="{00000000-4F9B-4E09-ADF8-D06A1030C661}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1596,7 +1596,7 @@
               </c14:invertSolidFillFmt>
             </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-66A4-45C5-852A-009F11104544}"/>
+              <c16:uniqueId val="{00000001-4F9B-4E09-ADF8-D06A1030C661}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3826,7 +3826,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="39.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="52.8" x14ac:dyDescent="0.3">
       <c r="A13" s="24" t="s">
         <v>232</v>
       </c>

</xml_diff>

<commit_message>
docs(avance): RQF-26 apunta a su historia propia (HU-66)
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{071556A5-1659-4C9B-A408-7574E03B5E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F27D41B-F4D3-4AD4-B194-A1EC2C31F350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -620,7 +620,7 @@
     <t>PUT /api/cliente/me actualiza teléfono, correo y contacto de emergencia solo del miembro autenticado (cliente.js:171-225, requireClient en :112); pantalla editar_perfil_screen.dart y perfil_service.dart.</t>
   </si>
   <si>
-    <t>HU-58</t>
+    <t>HU-66</t>
   </si>
   <si>
     <t>EV-36</t>
@@ -1798,7 +1798,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9AFB-4C1A-8484-4925770688D2}"/>
+              <c16:uniqueId val="{00000000-16D0-4AF3-AFC5-2301F25F3C9A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1968,7 +1968,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2282-4F3F-8AB3-CB3FA28619EA}"/>
+              <c16:uniqueId val="{00000000-4401-4E9C-9AD6-1F871F89D66C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
docs(avance): retira RQF-23..25 y fusiona RQF-26 en RQF-15 en el Excel
Se quitan sus filas de RF y sus evidencias (las EV quedan EV-01..50, sin
referencias rotas); RQF-15 suma la evidencia de la edicion del perfil.
Formulas, resumen y graficos siguen en sus rangos (Resumen!G6:G8 y
J6:K8). Resultado: RF 63,6 % (14/22), RNF 60,0 % (9/15), global 62,2 %
(23/37); faltan 6,6 puntos para el 80 %.
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0763257D-39F7-4D98-A4C6-CF93004C605E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C26BE2-6673-44F3-8F95-488B0B4EF963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,8 +20,8 @@
     <sheet name="Evidencias" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Evidencias!$A$1:$G$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">RF!$A$1:$J$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Evidencias!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">RF!$A$1:$J$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">RNF!$A$1:$J$16</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="436">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -197,7 +197,7 @@
     <t>Observación: al editar no se vuelven a validar duplicados de documento o correo (criterio 2 de HU-09).</t>
   </si>
   <si>
-    <t>HU-07, HU-08, HU-09, HU-10</t>
+    <t>HU-07, HU-08, HU-09, HU-10, HU-65</t>
   </si>
   <si>
     <t>EV-05, EV-06</t>
@@ -236,7 +236,7 @@
     <t>—</t>
   </si>
   <si>
-    <t>HU-14, HU-32, HU-33</t>
+    <t>HU-14, HU-32, HU-33, HU-34</t>
   </si>
   <si>
     <t>EV-09, EV-10</t>
@@ -275,7 +275,7 @@
     <t>Gráfica de horas pico (la gráfica agrupa por día de la semana, dashboard.js:189) y actualización automática (el panel se carga una sola vez, DashboardPage.jsx:165-179).</t>
   </si>
   <si>
-    <t>HU-16, HU-41, HU-42, HU-43</t>
+    <t>HU-16, HU-34, HU-41, HU-42, HU-43</t>
   </si>
   <si>
     <t>EV-12</t>
@@ -296,7 +296,7 @@
     <t>Ejecución diaria del motor (el scheduler solo programa vencimientos, scheduler.js:46), los dos niveles Amarilla / Roja, registro en alerta_abandono (tabla sin uso) y pantalla para configurar el umbral (el dashboard usa 15 días fijos).</t>
   </si>
   <si>
-    <t>HU-17, HU-18, HU-44</t>
+    <t>HU-17, HU-18, HU-44, HU-64</t>
   </si>
   <si>
     <t>EV-13, EV-14</t>
@@ -431,19 +431,19 @@
     <t>App del miembro</t>
   </si>
   <si>
-    <t>POST /api/cliente/login con teléfono y contraseña bcrypt (cliente.js:51, :88) y JWT de 30 días (auth-helpers.js:145); rutas protegidas con requireClient (cliente.js:112); /qr, /membresia, /asistencia, /gamificacion y /retos (cliente.js:227, :259, :292, :340, :392); app Flutter: login_screen.dart, qr_tab.dart, plan_tab.dart, asistencia_screen.dart, gamificacion_screen.dart; token en FlutterSecureStorage (api_client.dart:41).</t>
-  </si>
-  <si>
-    <t>Ajuste de redacción: el PR #4 decía «rachas», que no se calculan (ver RQF-11); la app muestra hitos y retos de solo lectura. Sin pruebas automatizadas reales (widget_test.dart es una prueba mínima).</t>
-  </si>
-  <si>
-    <t>HU-57, HU-58</t>
-  </si>
-  <si>
-    <t>EV-22, EV-23</t>
-  </si>
-  <si>
-    <t>El sistema debe ofrecer una aplicación móvil para el miembro con inicio de sesión, código QR personal, estado de membresía, historial de asistencia, hitos y retos activos.</t>
+    <t>POST /api/cliente/login con teléfono y contraseña bcrypt (cliente.js:51, :88) y JWT de 30 días (auth-helpers.js:145); rutas protegidas con requireClient (cliente.js:112); /qr, /membresia, /asistencia, /gamificacion y /retos (cliente.js:227, :259, :292, :340, :392); edición del perfil con PUT /api/cliente/me, que valida el correo único (cliente.js:171-225); app Flutter: login_screen.dart, qr_tab.dart, plan_tab.dart, asistencia_screen.dart, gamificacion_screen.dart, editar_perfil_screen.dart; token en FlutterSecureStorage (api_client.dart:41).</t>
+  </si>
+  <si>
+    <t>Ajuste de redacción: el PR #4 decía «rachas», que no se calculan (ver RQF-11); la app muestra hitos y retos de solo lectura. Absorbe RQF-26 (edición del perfil), que el PR #4 contaba aparte. Sin pruebas automatizadas reales (widget_test.dart es una prueba mínima).</t>
+  </si>
+  <si>
+    <t>HU-57, HU-58, HU-66</t>
+  </si>
+  <si>
+    <t>EV-22, EV-23, EV-24</t>
+  </si>
+  <si>
+    <t>El sistema debe ofrecer una aplicación móvil para el miembro con inicio de sesión, código QR personal, estado de membresía, historial de asistencia, hitos y retos activos, y edición del perfil.</t>
   </si>
   <si>
     <t>RQF-16</t>
@@ -461,931 +461,835 @@
     <t>HU-56</t>
   </si>
   <si>
+    <t>EV-25</t>
+  </si>
+  <si>
+    <t>El sistema debe ofrecer una prueba gratuita de 14 días, mostrar su estado al administrador y bloquear las operaciones del gimnasio cuando la prueba vence.</t>
+  </si>
+  <si>
+    <t>RQF-17</t>
+  </si>
+  <si>
+    <t>POST /api/auth/forgot-password genera un código de 6 dígitos con vigencia de 15 minutos y lo envía (auth.js:304-340, email.js:289); POST /verify-reset-code (auth.js:360) y POST /reset-password con bcrypt (auth.js:399, :447); pantalla ForgotPasswordPage.jsx:121, :143, :161; límite de 3 solicitudes por minuto solo en forgot-password (index.js:68, :80).</t>
+  </si>
+  <si>
+    <t>Riesgo de seguridad: si el correo no sale (o con SHOW_DEV_CODE_IN_UI=true), la API devuelve el código en la respuesta (auth.js:337-346), así que cualquiera que sepa el correo de un usuario puede cambiarle la contraseña; además verify-reset-code y reset-password no tienen límite de intentos (ver RQNF-09).</t>
+  </si>
+  <si>
+    <t>HU-59</t>
+  </si>
+  <si>
+    <t>EV-26, EV-27</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir recuperar la contraseña del personal mediante un código enviado al correo electrónico.</t>
+  </si>
+  <si>
+    <t>RQF-18</t>
+  </si>
+  <si>
+    <t>GET /api/admin/dashboard/export arma un CSV RFC 4180 de miembros activos con su plan (dashboard.js:288-337, helpers :31-50); el panel lo descarga (DashboardPage.jsx:193-203).</t>
+  </si>
+  <si>
+    <t>HU-60</t>
+  </si>
+  <si>
+    <t>EV-28</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir exportar a CSV el listado de miembros activos con su membresía.</t>
+  </si>
+  <si>
+    <t>RQF-19</t>
+  </si>
+  <si>
+    <t>POST /api/auth/signup crea el gimnasio y la cuenta del administrador dueño en una transacción (auth.js:100-190, INSERT en :134 y COMMIT en :162); pantalla RegisterOwnerPage.jsx (ruta /register-owner, App.jsx:38).</t>
+  </si>
+  <si>
+    <t>EV-29</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir registrar un gimnasio junto con la cuenta de su propietario.</t>
+  </si>
+  <si>
+    <t>RQF-20</t>
+  </si>
+  <si>
+    <t>Configuración</t>
+  </si>
+  <si>
+    <t>GET y PUT /api/admin/config con precios por tipo de plan, recordatorio_cobro_activo y dias_recordatorio_default (config.js:20-30, :41, :77); pantalla ConfigPage.jsx:26, :44; los avisos de cobro lo usan (notificaciones.js:44-67).</t>
+  </si>
+  <si>
+    <t>Ajuste de redacción: el PR #4 decía «los planes»; no hay catálogo editable de planes, sino precios para tipos de plan fijos.</t>
+  </si>
+  <si>
+    <t>HU-61</t>
+  </si>
+  <si>
+    <t>EV-30</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir configurar por gimnasio el precio de cada tipo de plan y los recordatorios de cobro.</t>
+  </si>
+  <si>
+    <t>RQF-21</t>
+  </si>
+  <si>
+    <t>Esquema de alta con valor_total, valor_pagado, metodo_pago y estado_pago (miembros.js:88-95); inserción en plan_cobro (miembros.js:439-450, migración 004); edición del plan (miembros.js:754); validaciones en MiembrosPage.jsx:349-350.</t>
+  </si>
+  <si>
+    <t>Ajuste de redacción: se acotó al pago, porque el plan y su vigencia ya están en RQF-04.</t>
+  </si>
+  <si>
+    <t>HU-62</t>
+  </si>
+  <si>
+    <t>EV-31</t>
+  </si>
+  <si>
+    <t>El sistema debe registrar por miembro el valor total y pagado, el método y el estado del pago de su plan.</t>
+  </si>
+  <si>
+    <t>RQF-22</t>
+  </si>
+  <si>
+    <t>Cumplimiento</t>
+  </si>
+  <si>
+    <t>DELETE /api/auth/account (auth.js:480-561) borra en una transacción con safe(), que solo ignora el código 42P01 y no usa SAVEPOINT (auth.js:496-502). En PostgreSQL cualquier error, incluso el ignorado, aborta la transacción: con las migraciones falla en DELETE FROM auditoria (ninguna migración crea esa tabla) y con el esquema de ConsultasDB el INSERT en auditoria viola la llave foránea hacia el usuario borrado. En los dos casos el gimnasio queda intacto y la API responde 500. Probado en PostgreSQL 18 en el informe del verificador (70dd13c, sección 11.2.1).</t>
+  </si>
+  <si>
+    <t>Un SAVEPOINT por cada safe() (o quitar las tablas que no existen) y no insertar en auditoria filas que apunten al usuario y al gimnasio que se borran. Si se corrige y se prueba, puede volver a Implementado. El PR #4 y mi versión anterior lo daban por Implementado leyendo solo el código.</t>
+  </si>
+  <si>
+    <t>HU-63</t>
+  </si>
+  <si>
+    <t>EV-32, EV-33</t>
+  </si>
+  <si>
+    <t>El sistema debe permitir al propietario eliminar su cuenta y los datos asociados del gimnasio.</t>
+  </si>
+  <si>
+    <t>RQNF-01</t>
+  </si>
+  <si>
+    <t>Rendimiento</t>
+  </si>
+  <si>
+    <t>No hay medición registrada.</t>
+  </si>
+  <si>
+    <t>Medir y documentar (p. ej. 30 check-ins contra el entorno desplegado, tiempo de respuesta de POST /api/admin/checkin). Riesgo: si el QR no coincide directo, checkin.js:83-101 descifra en memoria los QR de todos los miembros del gimnasio.</t>
+  </si>
+  <si>
+    <t>EV-34</t>
+  </si>
+  <si>
+    <t>El sistema debe procesar y confirmar cada registro de check-in en un tiempo máximo de 2 segundos desde la lectura del dispositivo HID.</t>
+  </si>
+  <si>
+    <t>RQNF-02</t>
+  </si>
+  <si>
+    <t>Disponibilidad</t>
+  </si>
+  <si>
+    <t>Existen /api/healthz y /api/health (index.js:101, :103), pero no hay monitoreo ni reporte de disponibilidad.</t>
+  </si>
+  <si>
+    <t>Monitor externo sobre /api/healthz con reporte del período; el plan gratuito de Render suspende el servicio por inactividad (scheduler.js:9-10).</t>
+  </si>
+  <si>
+    <t>EV-35</t>
+  </si>
+  <si>
+    <t>El sistema debe garantizar una disponibilidad mínima del 99% durante el horario operativo del gimnasio (lunes a domingo, 5:00 a.m. – 10:00 p.m.).</t>
+  </si>
+  <si>
+    <t>RQNF-03</t>
+  </si>
+  <si>
+    <t>Seguridad</t>
+  </si>
+  <si>
+    <t>bcrypt.hash / compare en registro, login, restablecimiento e invitación (auth.js:145, :231, :447; staff.js:431) y para miembros (miembros.js:388, :625; cliente.js:88); API de producción por HTTPS (frontend/src/api.js:26) y frontend en Vercel con HTTPS.</t>
+  </si>
+  <si>
+    <t>Observación: la clave de cifrado del QR tiene un valor por defecto en el código (miembros.js:36, checkin.js:19).</t>
+  </si>
+  <si>
+    <t>EV-36</t>
+  </si>
+  <si>
+    <t>El sistema debe almacenar las contraseñas del personal utilizando cifrado hash (bcrypt o equivalente) y todas las comunicaciones deben realizarse bajo protocolo HTTPS.</t>
+  </si>
+  <si>
+    <t>RQNF-04</t>
+  </si>
+  <si>
+    <t>Usabilidad</t>
+  </si>
+  <si>
+    <t>Registro manual en 2 interacciones: escribir el documento y pulsar «Registrar» (CheckinPage.jsx:333, :341-347); el código QR se envía con Enter (CheckinPage.jsx:221-223).</t>
+  </si>
+  <si>
+    <t>Prueba de usabilidad documentada con personal sin formación técnica (p. ej. 3 personas, conteo de interacciones y tiempo).</t>
+  </si>
+  <si>
+    <t>HU-32</t>
+  </si>
+  <si>
+    <t>EV-37</t>
+  </si>
+  <si>
+    <t>La interfaz del módulo de check-in debe ser operable por personal sin formación técnica, con un flujo de no más de 2 interacciones para registrar una entrada de forma manual.</t>
+  </si>
+  <si>
+    <t>RQNF-05</t>
+  </si>
+  <si>
+    <t>Escalabilidad</t>
+  </si>
+  <si>
+    <t>Cada gimnasio nuevo se crea por registro, sin tocar código (auth.js:100, :134); casi todas las consultas filtran por el id_gimnasio del token (p. ej. miembros.js:358, checkin.js:76, dashboard.js:123, notificaciones.js:199; admin-contrato.js:92).</t>
+  </si>
+  <si>
+    <t>GET /api/vista/miembros-activos no filtra por gimnasio (vista.js:27-42) y rompe el aislamiento entre gimnasios. No hay prueba de carga que respalde «sin degradación del rendimiento».</t>
+  </si>
+  <si>
+    <t>EV-38, EV-39</t>
+  </si>
+  <si>
+    <t>La arquitectura SaaS debe soportar el registro de múltiples gimnasios (multitenancy) sin degradación del rendimiento, permitiendo incorporar nuevos establecimientos sin modificaciones en el código base.</t>
+  </si>
+  <si>
+    <t>RQNF-06</t>
+  </si>
+  <si>
+    <t>Compatibilidad</t>
+  </si>
+  <si>
+    <t>Aplicación web React / Vite servida por Vercel que solo requiere navegador (frontend/package.json, vercel.json); QA responsive a 375 px (Evidencias_Sustentacion/QA_Responsive_375px.md).</t>
+  </si>
+  <si>
+    <t>Prueba documentada en Chrome, Firefox y Edge (lista de verificación de las pantallas principales con capturas).</t>
+  </si>
+  <si>
+    <t>EV-40</t>
+  </si>
+  <si>
+    <t>El sistema debe funcionar correctamente en los navegadores Chrome, Firefox y Edge en sus dos últimas versiones mayores, sin requerir instalación de software adicional en el cliente.</t>
+  </si>
+  <si>
+    <t>RQNF-07</t>
+  </si>
+  <si>
+    <t>Mantenibilidad</t>
+  </si>
+  <si>
+    <t>Capas en backend/src (routes, lib, middleware, jobs, db) y diagrama de arquitectura en el documento (sección 8). Cobertura medida el 2026-10-16: 0 % en routes/checkin.js y routes/notificaciones.js, 1,48 % de líneas en todo el backend; 23 pruebas, 2 fallan.</t>
+  </si>
+  <si>
+    <t>Script «test» en backend/package.json, pruebas de check-in y alertas hasta ≥ 70 % y corregir las 2 pruebas que fallan.</t>
+  </si>
+  <si>
+    <t>EV-41, EV-42</t>
+  </si>
+  <si>
+    <t>El código fuente debe seguir una arquitectura en capas documentada, con una cobertura mínima de pruebas unitarias del 70% sobre los módulos de check-in y alertas de abandono.</t>
+  </si>
+  <si>
+    <t>RQNF-08</t>
+  </si>
+  <si>
+    <t>Portabilidad</t>
+  </si>
+  <si>
+    <t>backend/Dockerfile (node:24-alpine, multietapa), frontend/Dockerfile + nginx.conf y docker-compose.yml; despliegue en la nube en Render y Vercel (render.yaml, vercel.json).</t>
+  </si>
+  <si>
+    <t>Observación: no se verificó la construcción de la imagen (Docker Desktop apagado) y Render usa el entorno Node nativo, no el contenedor. Sugerencia: agregar docker build al CI.</t>
+  </si>
+  <si>
+    <t>EV-43</t>
+  </si>
+  <si>
+    <t>El sistema debe poder desplegarse en servicios de nube (AWS, Railway, Render o equivalentes) mediante contenedores Docker, sin dependencia de infraestructura física local.</t>
+  </si>
+  <si>
+    <t>RQNF-09</t>
+  </si>
+  <si>
+    <t>express-rate-limit: inicio de sesión 5 por minuto, recuperación de contraseña 3 por minuto y login de la app 10 por minuto (index.js:63-77, :79-80, :94); trust proxy para tomar la IP real detrás de Render (index.js:43).</t>
+  </si>
+  <si>
+    <t>verify-reset-code (auth.js:360) y reset-password (auth.js:399) no tienen límite: el código de 6 dígitos se puede probar sin límite durante sus 15 minutos de vida.</t>
+  </si>
+  <si>
+    <t>EV-44</t>
+  </si>
+  <si>
+    <t>El sistema debe limitar la tasa de intentos en los endpoints de inicio de sesión, recuperación de contraseña e inicio de sesión de la app del miembro.</t>
+  </si>
+  <si>
+    <t>RQNF-10</t>
+  </si>
+  <si>
+    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 008 en backend/migrations.</t>
+  </si>
+  <si>
+    <t>Una base creada solo con backend/migrations no tiene vista_miembros_activos ni auditoria, y reto tiene meta en lugar de meta_asistencias (002_esquema_inicial.sql:278-290); el esquema de producción salió de ConsultasDB/ y de cambios manuales. Probado en el informe del verificador (70dd13c, sección 11.2.1). Además hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica.</t>
+  </si>
+  <si>
+    <t>EV-45</t>
+  </si>
+  <si>
+    <t>El esquema de la base de datos debe evolucionar mediante migraciones versionadas aplicadas automáticamente al iniciar el servicio.</t>
+  </si>
+  <si>
+    <t>RQNF-11</t>
+  </si>
+  <si>
+    <t>.github/workflows/ci.yml corre en pull_request y en push a main (:3-6): el job rama valida el nombre de la rama en cada PR (:13-26), backend npm ci + node --check (:42-44) y frontend npm ci + build (:58-59); ejecución exitosa en main 8acab31 (pestaña Actions).</t>
+  </si>
+  <si>
+    <t>Observación: el CI todavía no corre pruebas ni mide cobertura.</t>
+  </si>
+  <si>
+    <t>EV-46</t>
+  </si>
+  <si>
+    <t>El repositorio debe ejecutar integración continua en cada pull request y en cada cambio de la rama principal: nombre de la rama, instalación limpia de dependencias, comprobación de sintaxis del backend y compilación del frontend.</t>
+  </si>
+  <si>
+    <t>RQNF-12</t>
+  </si>
+  <si>
+    <t>Rutas públicas /legal/terminos, /legal/privacidad y /legal/datos (App.jsx:43-45) con TerminosPage.jsx, PrivacidadPage.jsx y PoliticaDatosPage.jsx.</t>
+  </si>
+  <si>
+    <t>EV-47</t>
+  </si>
+  <si>
+    <t>El sistema debe publicar los términos de uso, la política de privacidad y la política de tratamiento de datos personales.</t>
+  </si>
+  <si>
+    <t>RQNF-13</t>
+  </si>
+  <si>
+    <t>Observabilidad</t>
+  </si>
+  <si>
+    <t>/api/healthz responde estado y uptime (index.js:101); /api/health comprueba la base de datos y responde 503 si no hay conexión (index.js:103-110).</t>
+  </si>
+  <si>
+    <t>EV-48</t>
+  </si>
+  <si>
+    <t>El sistema debe exponer un endpoint de verificación de salud para el monitoreo del servicio.</t>
+  </si>
+  <si>
+    <t>RQNF-14</t>
+  </si>
+  <si>
+    <t>Manejador central y 404 JSON (middleware/errorHandler.js:17, :24-49) registrados al final de la app (index.js:113-117); AppError con código y estado (lib/errors.js) y asyncHandler para rutas async (lib/asyncHandler.js).</t>
+  </si>
+  <si>
+    <t>EV-49</t>
+  </si>
+  <si>
+    <t>El sistema debe manejar los errores de forma centralizada, devolviendo respuestas consistentes.</t>
+  </si>
+  <si>
+    <t>RQNF-15</t>
+  </si>
+  <si>
+    <t>La configuración de CORS lee FRONTEND_URL (index.js:45-48), pero el callback devuelve permitido también para orígenes que no están en la lista (index.js:54), con credentials: true.</t>
+  </si>
+  <si>
+    <t>Rechazar los orígenes que no estén en FRONTEND_URL (cambiar index.js:54). El PR #4 lo marcaba Implementado.</t>
+  </si>
+  <si>
+    <t>EV-50</t>
+  </si>
+  <si>
+    <t>El sistema debe restringir las solicitudes entre orígenes (CORS) a los dominios configurados.</t>
+  </si>
+  <si>
+    <t>Acción propuesta</t>
+  </si>
+  <si>
+    <t>Responsable</t>
+  </si>
+  <si>
+    <t>Esfuerzo</t>
+  </si>
+  <si>
+    <t>Puntos que suma</t>
+  </si>
+  <si>
+    <t>Avance global acumulado</t>
+  </si>
+  <si>
+    <t>Rechazar en CORS los orígenes que no estén en FRONTEND_URL (index.js:54)</t>
+  </si>
+  <si>
+    <t>Santiago</t>
+  </si>
+  <si>
+    <t>Bajo</t>
+  </si>
+  <si>
+    <t>Un SAVEPOINT por cada safe() y no insertar en auditoria lo que se borra; probar la eliminación</t>
+  </si>
+  <si>
+    <t>Relanzar el error en sendWhatsAppText para que un envío fallido no quede como exitoso</t>
+  </si>
+  <si>
+    <t>No marcar el aviso como enviado si WhatsApp no está listo (reintentar) y llevar los días a Configuración</t>
+  </si>
+  <si>
+    <t>Límite de intentos en verify-reset-code y reset-password</t>
+  </si>
+  <si>
+    <t>Prueba de usabilidad del check-in manual con 3 personas sin formación técnica</t>
+  </si>
+  <si>
+    <t>Luis</t>
+  </si>
+  <si>
+    <t>Lista de verificación con capturas en Chrome, Firefox y Edge</t>
+  </si>
+  <si>
+    <t>Cierre de sesión por inactividad en el frontend y expiración real del JWT</t>
+  </si>
+  <si>
+    <t>Gráfica de horas pico y refresco automático del dashboard</t>
+  </si>
+  <si>
+    <t>Registrar el acceso bloqueado y mostrarlo en la campana del administrador</t>
+  </si>
+  <si>
+    <t>Cerrar la fuga de vista.js, exigir rol de personal en /api/asistencia y quitar scryptSync del recorrido del check-in</t>
+  </si>
+  <si>
+    <t>Medio</t>
+  </si>
+  <si>
+    <t>Con la búsqueda del QR ya corregida (paso anterior), medir el check-in con un volumen realista (unos 200 miembros)</t>
+  </si>
+  <si>
+    <t>Luis o Santiago</t>
+  </si>
+  <si>
+    <t>Editar y desactivar cuentas del personal</t>
+  </si>
+  <si>
+    <t>Congelar y descongelar membresías</t>
+  </si>
+  <si>
+    <t>Motor diario con Alerta Amarilla / Roja y umbrales editables</t>
+  </si>
+  <si>
+    <t>Script test, pruebas de check-in y alertas hasta ≥ 70 % de cobertura</t>
+  </si>
+  <si>
+    <t>Migración que cree vista_miembros_activos, auditoria y las columnas que usa el código</t>
+  </si>
+  <si>
+    <t>Cálculo de rachas, hitos y mensaje en el check-in</t>
+  </si>
+  <si>
+    <t>Monitor externo de disponibilidad con reporte (depende del plan de Render)</t>
+  </si>
+  <si>
+    <t>CRUD de retos, progreso automático y aviso al completar</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Módulo de campañas y plantillas</t>
+  </si>
+  <si>
+    <t>Orden de menor a mayor esfuerzo. «Avance global acumulado» suma los puntos de cada acción, en orden, sobre el avance actual y se pone verde al llegar a la meta. Lo decide Luis; las implementaciones las hace Santiago.</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Requisito</t>
+  </si>
+  <si>
+    <t>Ubicación (archivo:línea, endpoint o enlace)</t>
+  </si>
+  <si>
+    <t>Qué demuestra</t>
+  </si>
+  <si>
+    <t>Fecha de verificación</t>
+  </si>
+  <si>
+    <t>Verificado por</t>
+  </si>
+  <si>
+    <t>EV-01</t>
+  </si>
+  <si>
+    <t>backend/src/routes/staff.js:109, :198, :227, :329, :384</t>
+  </si>
+  <si>
+    <t>Invitar, listar y revocar personal; aceptar la invitación crea la cuenta.</t>
+  </si>
+  <si>
+    <t>2026-10-16</t>
+  </si>
+  <si>
+    <t>Agente ejecutor (Claude)</t>
+  </si>
+  <si>
+    <t>EV-02</t>
+  </si>
+  <si>
+    <t>backend/src/routes/staff.js:112; miembros.js:667; checkin.js:57; middleware/auth.js:29</t>
+  </si>
+  <si>
+    <t>Permisos distintos para Administrador y Recepcionista.</t>
+  </si>
+  <si>
+    <t>EV-03</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:200, :231, :295; frontend/src/context/AuthContext.jsx:95</t>
+  </si>
+  <si>
+    <t>Login con bcrypt + JWT y cierre de sesión manual.</t>
+  </si>
+  <si>
+    <t>EV-04</t>
+  </si>
+  <si>
+    <t>Código (hallazgo)</t>
+  </si>
+  <si>
+    <t>backend/src/lib/auth-helpers.js:102-113</t>
+  </si>
+  <si>
+    <t>generarToken no aplica JWT_EXPIRES_IN: el token del personal no expira.</t>
+  </si>
+  <si>
+    <t>EV-05</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:357-369, :371-379</t>
+  </si>
+  <si>
+    <t>Rechazo de documento / correo duplicado y QR único.</t>
+  </si>
+  <si>
+    <t>EV-06</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:607, :664-675; frontend/src/pages/MiembrosPage.jsx:627, :919, :442</t>
+  </si>
+  <si>
+    <t>Editar y desactivar (soft delete) desde la pantalla de miembros.</t>
+  </si>
+  <si>
+    <t>EV-07</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:185, :382, :276-284, :754</t>
+  </si>
+  <si>
+    <t>Fecha de vencimiento automática, estado vencido / por vencer y renovación.</t>
+  </si>
+  <si>
+    <t>EV-08</t>
+  </si>
+  <si>
+    <t>Esquema</t>
+  </si>
+  <si>
+    <t>backend/migrations/002_esquema_inicial.sql:217</t>
+  </si>
+  <si>
+    <t>congelacion_membresia existe pero no se usa (falta Congelada).</t>
+  </si>
+  <si>
+    <t>EV-09</t>
+  </si>
+  <si>
+    <t>frontend/src/pages/CheckinPage.jsx:66, :221-223, :329-331</t>
+  </si>
+  <si>
+    <t>Lectura HID tipo teclado (autoFocus + Enter) y por cámara.</t>
+  </si>
+  <si>
+    <t>EV-10</t>
+  </si>
+  <si>
+    <t>Código / esquema</t>
+  </si>
+  <si>
+    <t>backend/src/routes/checkin.js:54, :167-172; backend/migrations/002_esquema_inicial.sql:100</t>
+  </si>
+  <si>
+    <t>Inserción del ingreso con marca de tiempo automática.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/checkin.js:116-136; frontend/src/pages/CheckinPage.jsx:133-143</t>
+  </si>
+  <si>
+    <t>Bloqueo de membresía vencida; no hay aviso del intento al administrador.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/dashboard.js:123, :128, :146, :189, :204; frontend/src/pages/DashboardPage.jsx:165-179, :446-473</t>
+  </si>
+  <si>
+    <t>KPIs del día y próximos vencimientos; gráfica por día de semana; carga única.</t>
+  </si>
+  <si>
+    <t>EV-13</t>
+  </si>
+  <si>
+    <t>backend/src/routes/notificaciones.js:38, :66, :125-137; dashboard.js:161, :182; miembros.js:263</t>
+  </si>
+  <si>
+    <t>Lista de miembros en riesgo calculada al consultar, un solo umbral.</t>
+  </si>
+  <si>
+    <t>EV-14</t>
+  </si>
+  <si>
+    <t>backend/src/jobs/scheduler.js:46</t>
+  </si>
+  <si>
+    <t>El único cron programado es el de vencimientos (no hay motor de abandono).</t>
+  </si>
+  <si>
+    <t>frontend/src/components/MenuNotificaciones.jsx:86-90; MiembrosPage.jsx:796-802; backend/src/routes/notificaciones.js:188-224</t>
+  </si>
+  <si>
+    <t>Envío por WhatsApp y registro en envio_mensaje con fecha y estado.</t>
+  </si>
+  <si>
+    <t>backend/migrations/002_esquema_inicial.sql:171-202</t>
+  </si>
+  <si>
+    <t>Tablas de campañas y plantillas sin rutas ni pantalla.</t>
+  </si>
+  <si>
+    <t>Código / datos</t>
+  </si>
+  <si>
+    <t>backend/src/routes/cliente.js:340-381; ConsultasDB/Poblar_Tablas.sql:384-419</t>
+  </si>
+  <si>
+    <t>Hitos solo de lectura, cargados por SQL; no hay cálculo de rachas.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/cliente.js:392-418; ConsultasDB/Poblar_Tablas.sql:456-490</t>
+  </si>
+  <si>
+    <t>Retos solo de lectura, cargados por SQL; sin CRUD ni progreso automático.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/admin-contrato.js:76-160, :167, :195; backend/migrations/008_contrato_enviado.sql; frontend/src/pages/MiembrosPage.jsx:855-880</t>
+  </si>
+  <si>
+    <t>Envío del contrato por WhatsApp con registro de cada intento.</t>
+  </si>
+  <si>
+    <t>EV-20</t>
+  </si>
+  <si>
+    <t>backend/src/jobs/scheduler.js:46; backend/src/jobs/expiracion.js:43, :74, :94, :117, :151</t>
+  </si>
+  <si>
+    <t>Aviso diario automático de vencimiento, sin duplicados.</t>
+  </si>
+  <si>
+    <t>EV-21</t>
+  </si>
+  <si>
+    <t>backend/src/routes/jobs.js:27, :38; backend/migrations/006_gimnasio_dias_aviso.sql; 007_alerta_vencimiento_enviada.sql</t>
+  </si>
+  <si>
+    <t>Ejecución manual y vista previa; días de aviso y anti-duplicado en BD.</t>
+  </si>
+  <si>
+    <t>EV-22</t>
+  </si>
+  <si>
+    <t>backend/src/routes/cliente.js:51, :88, :112, :227, :259, :292, :340, :392; backend/src/lib/auth-helpers.js:145</t>
+  </si>
+  <si>
+    <t>API de la app: login del miembro y consultas protegidas.</t>
+  </si>
+  <si>
+    <t>EV-23</t>
+  </si>
+  <si>
+    <t>Código (Flutter)</t>
+  </si>
+  <si>
+    <t>fitloyalty_cliente/lib/cliente/screens/login_screen.dart, qr_tab.dart, plan_tab.dart, asistencia_screen.dart, gamificacion_screen.dart; services/api_client.dart:41</t>
+  </si>
+  <si>
+    <t>Pantallas de la app móvil y almacenamiento seguro del token.</t>
+  </si>
+  <si>
     <t>EV-24</t>
   </si>
   <si>
-    <t>El sistema debe ofrecer una prueba gratuita de 14 días, mostrar su estado al administrador y bloquear las operaciones del gimnasio cuando la prueba vence.</t>
-  </si>
-  <si>
-    <t>RQF-17</t>
-  </si>
-  <si>
-    <t>POST /api/auth/forgot-password genera un código de 6 dígitos con vigencia de 15 minutos y lo envía (auth.js:304-340, email.js:289); POST /verify-reset-code (auth.js:360) y POST /reset-password con bcrypt (auth.js:399, :447); pantalla ForgotPasswordPage.jsx:121, :143, :161; límite de 3 solicitudes por minuto solo en forgot-password (index.js:68, :80).</t>
-  </si>
-  <si>
-    <t>Riesgo de seguridad: si el correo no sale (o con SHOW_DEV_CODE_IN_UI=true), la API devuelve el código en la respuesta (auth.js:337-346), así que cualquiera que sepa el correo de un usuario puede cambiarle la contraseña; además verify-reset-code y reset-password no tienen límite de intentos (ver RQNF-09).</t>
-  </si>
-  <si>
-    <t>HU-59</t>
-  </si>
-  <si>
-    <t>EV-25, EV-26</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir recuperar la contraseña del personal mediante un código enviado al correo electrónico.</t>
-  </si>
-  <si>
-    <t>RQF-18</t>
-  </si>
-  <si>
-    <t>GET /api/admin/dashboard/export arma un CSV RFC 4180 de miembros activos con su plan (dashboard.js:288-337, helpers :31-50); el panel lo descarga (DashboardPage.jsx:193-203).</t>
-  </si>
-  <si>
-    <t>HU-60</t>
+    <t>backend/src/routes/cliente.js:171-225; fitloyalty_cliente/lib/cliente/screens/editar_perfil_screen.dart; services/perfil_service.dart</t>
+  </si>
+  <si>
+    <t>Edición del perfil desde la app (antes RQF-26).</t>
+  </si>
+  <si>
+    <t>Código / configuración</t>
+  </si>
+  <si>
+    <t>backend/src/lib/trial.js:17, :52-74; backend/src/routes/billing.js:19; backend/src/routes/auth.js:126-138; render.yaml; frontend/src/components/AdminLayout.jsx:155</t>
+  </si>
+  <si>
+    <t>Prueba de 14 días, estado visible y bloqueo 402 al vencer.</t>
+  </si>
+  <si>
+    <t>EV-26</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:304, :360, :399, :447; backend/src/lib/email.js:289; frontend/src/pages/ForgotPasswordPage.jsx:121, :143, :161</t>
+  </si>
+  <si>
+    <t>Recuperación de contraseña con código por correo.</t>
   </si>
   <si>
     <t>EV-27</t>
   </si>
   <si>
-    <t>El sistema debe permitir exportar a CSV el listado de miembros activos con su membresía.</t>
-  </si>
-  <si>
-    <t>RQF-19</t>
-  </si>
-  <si>
-    <t>POST /api/auth/signup crea el gimnasio y la cuenta del administrador dueño en una transacción (auth.js:100-190, INSERT en :134 y COMMIT en :162); pantalla RegisterOwnerPage.jsx (ruta /register-owner, App.jsx:38).</t>
-  </si>
-  <si>
-    <t>EV-28</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir registrar un gimnasio junto con la cuenta de su propietario.</t>
-  </si>
-  <si>
-    <t>RQF-20</t>
-  </si>
-  <si>
-    <t>Configuración</t>
-  </si>
-  <si>
-    <t>GET y PUT /api/admin/config con precios por tipo de plan, recordatorio_cobro_activo y dias_recordatorio_default (config.js:20-30, :41, :77); pantalla ConfigPage.jsx:26, :44; los avisos de cobro lo usan (notificaciones.js:44-67).</t>
-  </si>
-  <si>
-    <t>Ajuste de redacción: el PR #4 decía «los planes»; no hay catálogo editable de planes, sino precios para tipos de plan fijos.</t>
-  </si>
-  <si>
-    <t>HU-61</t>
-  </si>
-  <si>
-    <t>EV-29</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir configurar por gimnasio el precio de cada tipo de plan y los recordatorios de cobro.</t>
-  </si>
-  <si>
-    <t>RQF-21</t>
-  </si>
-  <si>
-    <t>Esquema de alta con valor_total, valor_pagado, metodo_pago y estado_pago (miembros.js:88-95); inserción en plan_cobro (miembros.js:439-450, migración 004); edición del plan (miembros.js:754); validaciones en MiembrosPage.jsx:349-350.</t>
-  </si>
-  <si>
-    <t>Ajuste de redacción: se acotó al pago, porque el plan y su vigencia ya están en RQF-04.</t>
-  </si>
-  <si>
-    <t>HU-62</t>
-  </si>
-  <si>
-    <t>EV-30</t>
-  </si>
-  <si>
-    <t>El sistema debe registrar por miembro el valor total y pagado, el método y el estado del pago de su plan.</t>
-  </si>
-  <si>
-    <t>RQF-22</t>
-  </si>
-  <si>
-    <t>Cumplimiento</t>
-  </si>
-  <si>
-    <t>DELETE /api/auth/account (auth.js:480-561) borra en una transacción con safe(), que solo ignora el código 42P01 y no usa SAVEPOINT (auth.js:496-502). En PostgreSQL cualquier error, incluso el ignorado, aborta la transacción: con las migraciones falla en DELETE FROM auditoria (ninguna migración crea esa tabla) y con el esquema de ConsultasDB el INSERT en auditoria viola la llave foránea hacia el usuario borrado. En los dos casos el gimnasio queda intacto y la API responde 500. Probado en PostgreSQL 18 en el informe del verificador (70dd13c, sección 11.2.1).</t>
-  </si>
-  <si>
-    <t>Un SAVEPOINT por cada safe() (o quitar las tablas que no existen) y no insertar en auditoria filas que apunten al usuario y al gimnasio que se borran. Si se corrige y se prueba, puede volver a Implementado. El PR #4 y mi versión anterior lo daban por Implementado leyendo solo el código.</t>
-  </si>
-  <si>
-    <t>HU-63</t>
-  </si>
-  <si>
-    <t>EV-31, EV-32</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir al propietario eliminar su cuenta y los datos asociados del gimnasio.</t>
-  </si>
-  <si>
-    <t>RQF-23</t>
-  </si>
-  <si>
-    <t>GET /api/admin/notificaciones arma avisos de membresías vencidas, por vencer y miembros en riesgo con el mensaje listo (notificaciones.js:73-180); la campana los muestra y permite contactar por WhatsApp (MenuNotificaciones.jsx:38, :86-90).</t>
-  </si>
-  <si>
-    <t>HU-64</t>
+    <t>backend/src/routes/auth.js:337-346</t>
+  </si>
+  <si>
+    <t>El código se devuelve en la respuesta si el correo no sale.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/dashboard.js:31-50, :288-337; frontend/src/pages/DashboardPage.jsx:193-203</t>
+  </si>
+  <si>
+    <t>Exportación CSV de miembros activos con su membresía.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:100-190; frontend/src/pages/RegisterOwnerPage.jsx; frontend/src/App.jsx:38</t>
+  </si>
+  <si>
+    <t>Registro del gimnasio y de su administrador.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/config.js:20-30, :41, :77; frontend/src/pages/ConfigPage.jsx:26, :44; backend/src/routes/notificaciones.js:44-67</t>
+  </si>
+  <si>
+    <t>Configuración de precios y recordatorios por gimnasio.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:88-95, :439-450, :754; backend/migrations/004_extender_miembro_cobros.sql:54; frontend/src/pages/MiembrosPage.jsx:207-208, :349-350</t>
+  </si>
+  <si>
+    <t>Registro del plan y del pago por miembro.</t>
+  </si>
+  <si>
+    <t>EV-32</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:480-561 (safe() en :496-502); frontend/src/pages/EliminarCuentaPage.jsx:22</t>
+  </si>
+  <si>
+    <t>Flujo de eliminación; safe() sin SAVEPOINT.</t>
   </si>
   <si>
     <t>EV-33</t>
   </si>
   <si>
-    <t>El sistema debe mostrar al administrador avisos accionables (vencimientos y riesgo de abandono) en un centro de notificaciones.</t>
-  </si>
-  <si>
-    <t>RQF-24</t>
-  </si>
-  <si>
-    <t>GET /api/asistencia devuelve los últimos 50 ingresos del gimnasio con total y entradas de hoy (asistencia.js:26-60); GET /api/admin/checkin alimenta la lista de ingresos de la pantalla de check-in (checkin.js:199-224, CheckinPage.jsx:46).</t>
-  </si>
-  <si>
-    <t>Observación: DashboardUsuario.jsx consume /api/asistencia pero no tiene ruta en App.jsx; /api/asistencia no exige rol de personal (asistencia.js:21).</t>
-  </si>
-  <si>
-    <t>HU-34</t>
-  </si>
-  <si>
-    <t>EV-34</t>
-  </si>
-  <si>
-    <t>El sistema debe listar los check-ins del gimnasio con un resumen de asistencia.</t>
-  </si>
-  <si>
-    <t>RQF-25</t>
-  </si>
-  <si>
-    <t>GET /api/vista/miembros-activos consulta vista_miembros_activos sin filtrar por id_gimnasio y solo con authenticate (vista.js:18, :27, :38): cualquier token, incluido el de un miembro de la app, ve nombre, documento, teléfono, correo y QR de todos los gimnasios. La vista solo se crea en ConsultasDB/Query_Inicial_Crear_Tablas.sql:473 (no en backend/migrations) y lee la tabla membresia, que el alta de miembros no llena (lib/planes.js:4-7). Ninguna pantalla llama a /api/vista.</t>
-  </si>
-  <si>
-    <t>Filtrar por req.user.gymId y exigir rol de personal (o retirar la ruta), crear la vista en una migración que lea plan_cobro, y una pantalla que la use.</t>
-  </si>
-  <si>
-    <t>HU-65</t>
-  </si>
-  <si>
-    <t>EV-35, EV-36</t>
-  </si>
-  <si>
-    <t>El sistema debe ofrecer una vista de los miembros activos del gimnasio.</t>
-  </si>
-  <si>
-    <t>RQF-26</t>
-  </si>
-  <si>
-    <t>PUT /api/cliente/me actualiza teléfono, correo y contacto de emergencia solo del miembro autenticado (cliente.js:171-225, requireClient en :112); pantalla editar_perfil_screen.dart y perfil_service.dart.</t>
-  </si>
-  <si>
-    <t>HU-66</t>
-  </si>
-  <si>
-    <t>EV-37</t>
-  </si>
-  <si>
-    <t>El sistema debe permitir al miembro editar sus datos de perfil desde la aplicación móvil.</t>
-  </si>
-  <si>
-    <t>RQNF-01</t>
-  </si>
-  <si>
-    <t>Rendimiento</t>
-  </si>
-  <si>
-    <t>No hay medición registrada.</t>
-  </si>
-  <si>
-    <t>Medir y documentar (p. ej. 30 check-ins contra el entorno desplegado, tiempo de respuesta de POST /api/admin/checkin). Riesgo: si el QR no coincide directo, checkin.js:83-101 descifra en memoria los QR de todos los miembros del gimnasio.</t>
+    <t>Prueba (verificador)</t>
+  </si>
+  <si>
+    <t>Informe del verificador, commit 70dd13c, docs/verificacion-requisitos.md §11.2.1</t>
+  </si>
+  <si>
+    <t>En PostgreSQL 18 la transacción aborta y el gimnasio no se borra (dos esquemas).</t>
+  </si>
+  <si>
+    <t>Sin medición</t>
+  </si>
+  <si>
+    <t>— (riesgo en backend/src/routes/checkin.js:83-101)</t>
+  </si>
+  <si>
+    <t>No hay evidencia de tiempos; posible lentitud con muchos miembros.</t>
+  </si>
+  <si>
+    <t>backend/src/index.js:101, :103</t>
+  </si>
+  <si>
+    <t>Endpoints de salud disponibles para monitoreo; sin reporte.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:145, :231, :447; staff.js:431; miembros.js:388, :625; cliente.js:88; frontend/src/api.js:26</t>
+  </si>
+  <si>
+    <t>bcrypt en todas las contraseñas y API por HTTPS.</t>
+  </si>
+  <si>
+    <t>frontend/src/pages/CheckinPage.jsx:221-223, :333, :341-347</t>
+  </si>
+  <si>
+    <t>Flujo manual de 2 interacciones (sin prueba con usuarios).</t>
   </si>
   <si>
     <t>EV-38</t>
   </si>
   <si>
-    <t>El sistema debe procesar y confirmar cada registro de check-in en un tiempo máximo de 2 segundos desde la lectura del dispositivo HID.</t>
-  </si>
-  <si>
-    <t>RQNF-02</t>
-  </si>
-  <si>
-    <t>Disponibilidad</t>
-  </si>
-  <si>
-    <t>Existen /api/healthz y /api/health (index.js:101, :103), pero no hay monitoreo ni reporte de disponibilidad.</t>
-  </si>
-  <si>
-    <t>Monitor externo sobre /api/healthz con reporte del período; el plan gratuito de Render suspende el servicio por inactividad (scheduler.js:9-10).</t>
+    <t>backend/src/routes/auth.js:100, :134; miembros.js:358; checkin.js:76; dashboard.js:123; notificaciones.js:199; admin-contrato.js:92</t>
+  </si>
+  <si>
+    <t>Alta de gimnasios sin código y aislamiento por id_gimnasio.</t>
   </si>
   <si>
     <t>EV-39</t>
   </si>
   <si>
-    <t>El sistema debe garantizar una disponibilidad mínima del 99% durante el horario operativo del gimnasio (lunes a domingo, 5:00 a.m. – 10:00 p.m.).</t>
-  </si>
-  <si>
-    <t>RQNF-03</t>
-  </si>
-  <si>
-    <t>Seguridad</t>
-  </si>
-  <si>
-    <t>bcrypt.hash / compare en registro, login, restablecimiento e invitación (auth.js:145, :231, :447; staff.js:431) y para miembros (miembros.js:388, :625; cliente.js:88); API de producción por HTTPS (frontend/src/api.js:26) y frontend en Vercel con HTTPS.</t>
-  </si>
-  <si>
-    <t>Observación: la clave de cifrado del QR tiene un valor por defecto en el código (miembros.js:36, checkin.js:19).</t>
-  </si>
-  <si>
-    <t>EV-40</t>
-  </si>
-  <si>
-    <t>El sistema debe almacenar las contraseñas del personal utilizando cifrado hash (bcrypt o equivalente) y todas las comunicaciones deben realizarse bajo protocolo HTTPS.</t>
-  </si>
-  <si>
-    <t>RQNF-04</t>
-  </si>
-  <si>
-    <t>Usabilidad</t>
-  </si>
-  <si>
-    <t>Registro manual en 2 interacciones: escribir el documento y pulsar «Registrar» (CheckinPage.jsx:333, :341-347); el código QR se envía con Enter (CheckinPage.jsx:221-223).</t>
-  </si>
-  <si>
-    <t>Prueba de usabilidad documentada con personal sin formación técnica (p. ej. 3 personas, conteo de interacciones y tiempo).</t>
-  </si>
-  <si>
-    <t>HU-32</t>
+    <t>backend/src/routes/vista.js:27-42</t>
+  </si>
+  <si>
+    <t>Única consulta sin filtro de gimnasio encontrada.</t>
+  </si>
+  <si>
+    <t>Documento</t>
+  </si>
+  <si>
+    <t>Evidencias_Sustentacion/QA_Responsive_375px.md; frontend/package.json; vercel.json</t>
+  </si>
+  <si>
+    <t>App web sin instalación; sin prueba en los 3 navegadores.</t>
   </si>
   <si>
     <t>EV-41</t>
   </si>
   <si>
-    <t>La interfaz del módulo de check-in debe ser operable por personal sin formación técnica, con un flujo de no más de 2 interacciones para registrar una entrada de forma manual.</t>
-  </si>
-  <si>
-    <t>RQNF-05</t>
-  </si>
-  <si>
-    <t>Escalabilidad</t>
-  </si>
-  <si>
-    <t>Cada gimnasio nuevo se crea por registro, sin tocar código (auth.js:100, :134); casi todas las consultas filtran por el id_gimnasio del token (p. ej. miembros.js:358, checkin.js:76, dashboard.js:123, notificaciones.js:199; admin-contrato.js:92).</t>
-  </si>
-  <si>
-    <t>GET /api/vista/miembros-activos no filtra por gimnasio (vista.js:27-42) y rompe el aislamiento entre gimnasios. No hay prueba de carga que respalde «sin degradación del rendimiento».</t>
-  </si>
-  <si>
-    <t>EV-42, EV-43</t>
-  </si>
-  <si>
-    <t>La arquitectura SaaS debe soportar el registro de múltiples gimnasios (multitenancy) sin degradación del rendimiento, permitiendo incorporar nuevos establecimientos sin modificaciones en el código base.</t>
-  </si>
-  <si>
-    <t>RQNF-06</t>
-  </si>
-  <si>
-    <t>Compatibilidad</t>
-  </si>
-  <si>
-    <t>Aplicación web React / Vite servida por Vercel que solo requiere navegador (frontend/package.json, vercel.json); QA responsive a 375 px (Evidencias_Sustentacion/QA_Responsive_375px.md).</t>
-  </si>
-  <si>
-    <t>Prueba documentada en Chrome, Firefox y Edge (lista de verificación de las pantallas principales con capturas).</t>
-  </si>
-  <si>
-    <t>EV-44</t>
-  </si>
-  <si>
-    <t>El sistema debe funcionar correctamente en los navegadores Chrome, Firefox y Edge en sus dos últimas versiones mayores, sin requerir instalación de software adicional en el cliente.</t>
-  </si>
-  <si>
-    <t>RQNF-07</t>
-  </si>
-  <si>
-    <t>Mantenibilidad</t>
-  </si>
-  <si>
-    <t>Capas en backend/src (routes, lib, middleware, jobs, db) y diagrama de arquitectura en el documento (sección 8). Cobertura medida el 2026-10-16: 0 % en routes/checkin.js y routes/notificaciones.js, 1,48 % de líneas en todo el backend; 23 pruebas, 2 fallan.</t>
-  </si>
-  <si>
-    <t>Script «test» en backend/package.json, pruebas de check-in y alertas hasta ≥ 70 % y corregir las 2 pruebas que fallan.</t>
-  </si>
-  <si>
-    <t>EV-45, EV-46</t>
-  </si>
-  <si>
-    <t>El código fuente debe seguir una arquitectura en capas documentada, con una cobertura mínima de pruebas unitarias del 70% sobre los módulos de check-in y alertas de abandono.</t>
-  </si>
-  <si>
-    <t>RQNF-08</t>
-  </si>
-  <si>
-    <t>Portabilidad</t>
-  </si>
-  <si>
-    <t>backend/Dockerfile (node:24-alpine, multietapa), frontend/Dockerfile + nginx.conf y docker-compose.yml; despliegue en la nube en Render y Vercel (render.yaml, vercel.json).</t>
-  </si>
-  <si>
-    <t>Observación: no se verificó la construcción de la imagen (Docker Desktop apagado) y Render usa el entorno Node nativo, no el contenedor. Sugerencia: agregar docker build al CI.</t>
-  </si>
-  <si>
-    <t>EV-47</t>
-  </si>
-  <si>
-    <t>El sistema debe poder desplegarse en servicios de nube (AWS, Railway, Render o equivalentes) mediante contenedores Docker, sin dependencia de infraestructura física local.</t>
-  </si>
-  <si>
-    <t>RQNF-09</t>
-  </si>
-  <si>
-    <t>express-rate-limit: inicio de sesión 5 por minuto, recuperación de contraseña 3 por minuto y login de la app 10 por minuto (index.js:63-77, :79-80, :94); trust proxy para tomar la IP real detrás de Render (index.js:43).</t>
-  </si>
-  <si>
-    <t>verify-reset-code (auth.js:360) y reset-password (auth.js:399) no tienen límite: el código de 6 dígitos se puede probar sin límite durante sus 15 minutos de vida.</t>
-  </si>
-  <si>
-    <t>EV-48</t>
-  </si>
-  <si>
-    <t>El sistema debe limitar la tasa de intentos en los endpoints de inicio de sesión, recuperación de contraseña e inicio de sesión de la app del miembro.</t>
-  </si>
-  <si>
-    <t>RQNF-10</t>
-  </si>
-  <si>
-    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 008 en backend/migrations.</t>
-  </si>
-  <si>
-    <t>Una base creada solo con backend/migrations no tiene vista_miembros_activos ni auditoria, y reto tiene meta en lugar de meta_asistencias (002_esquema_inicial.sql:278-290); el esquema de producción salió de ConsultasDB/ y de cambios manuales. Probado en el informe del verificador (70dd13c, sección 11.2.1). Además hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica.</t>
-  </si>
-  <si>
-    <t>EV-49</t>
-  </si>
-  <si>
-    <t>El esquema de la base de datos debe evolucionar mediante migraciones versionadas aplicadas automáticamente al iniciar el servicio.</t>
-  </si>
-  <si>
-    <t>RQNF-11</t>
-  </si>
-  <si>
-    <t>.github/workflows/ci.yml corre en pull_request y en push a main (:3-6): el job rama valida el nombre de la rama en cada PR (:13-26), backend npm ci + node --check (:42-44) y frontend npm ci + build (:58-59); ejecución exitosa en main 8acab31 (pestaña Actions).</t>
-  </si>
-  <si>
-    <t>Observación: el CI todavía no corre pruebas ni mide cobertura.</t>
-  </si>
-  <si>
-    <t>EV-50</t>
-  </si>
-  <si>
-    <t>El repositorio debe ejecutar integración continua en cada pull request y en cada cambio de la rama principal: nombre de la rama, instalación limpia de dependencias, comprobación de sintaxis del backend y compilación del frontend.</t>
-  </si>
-  <si>
-    <t>RQNF-12</t>
-  </si>
-  <si>
-    <t>Rutas públicas /legal/terminos, /legal/privacidad y /legal/datos (App.jsx:43-45) con TerminosPage.jsx, PrivacidadPage.jsx y PoliticaDatosPage.jsx.</t>
-  </si>
-  <si>
-    <t>EV-51</t>
-  </si>
-  <si>
-    <t>El sistema debe publicar los términos de uso, la política de privacidad y la política de tratamiento de datos personales.</t>
-  </si>
-  <si>
-    <t>RQNF-13</t>
-  </si>
-  <si>
-    <t>Observabilidad</t>
-  </si>
-  <si>
-    <t>/api/healthz responde estado y uptime (index.js:101); /api/health comprueba la base de datos y responde 503 si no hay conexión (index.js:103-110).</t>
-  </si>
-  <si>
-    <t>EV-52</t>
-  </si>
-  <si>
-    <t>El sistema debe exponer un endpoint de verificación de salud para el monitoreo del servicio.</t>
-  </si>
-  <si>
-    <t>RQNF-14</t>
-  </si>
-  <si>
-    <t>Manejador central y 404 JSON (middleware/errorHandler.js:17, :24-49) registrados al final de la app (index.js:113-117); AppError con código y estado (lib/errors.js) y asyncHandler para rutas async (lib/asyncHandler.js).</t>
-  </si>
-  <si>
-    <t>EV-53</t>
-  </si>
-  <si>
-    <t>El sistema debe manejar los errores de forma centralizada, devolviendo respuestas consistentes.</t>
-  </si>
-  <si>
-    <t>RQNF-15</t>
-  </si>
-  <si>
-    <t>La configuración de CORS lee FRONTEND_URL (index.js:45-48), pero el callback devuelve permitido también para orígenes que no están en la lista (index.js:54), con credentials: true.</t>
-  </si>
-  <si>
-    <t>Rechazar los orígenes que no estén en FRONTEND_URL (cambiar index.js:54). El PR #4 lo marcaba Implementado.</t>
-  </si>
-  <si>
-    <t>EV-54</t>
-  </si>
-  <si>
-    <t>El sistema debe restringir las solicitudes entre orígenes (CORS) a los dominios configurados.</t>
-  </si>
-  <si>
-    <t>Acción propuesta</t>
-  </si>
-  <si>
-    <t>Responsable</t>
-  </si>
-  <si>
-    <t>Esfuerzo</t>
-  </si>
-  <si>
-    <t>Puntos que suma</t>
-  </si>
-  <si>
-    <t>Avance global acumulado</t>
-  </si>
-  <si>
-    <t>Rechazar en CORS los orígenes que no estén en FRONTEND_URL (index.js:54)</t>
-  </si>
-  <si>
-    <t>Santiago</t>
-  </si>
-  <si>
-    <t>Bajo</t>
-  </si>
-  <si>
-    <t>Un SAVEPOINT por cada safe() y no insertar en auditoria lo que se borra; probar la eliminación</t>
-  </si>
-  <si>
-    <t>Relanzar el error en sendWhatsAppText para que un envío fallido no quede como exitoso</t>
-  </si>
-  <si>
-    <t>No marcar el aviso como enviado si WhatsApp no está listo (reintentar) y llevar los días a Configuración</t>
-  </si>
-  <si>
-    <t>Límite de intentos en verify-reset-code y reset-password</t>
-  </si>
-  <si>
-    <t>Prueba de usabilidad del check-in manual con 3 personas sin formación técnica</t>
-  </si>
-  <si>
-    <t>Luis</t>
-  </si>
-  <si>
-    <t>Lista de verificación con capturas en Chrome, Firefox y Edge</t>
-  </si>
-  <si>
-    <t>Cierre de sesión por inactividad en el frontend y expiración real del JWT</t>
-  </si>
-  <si>
-    <t>Gráfica de horas pico y refresco automático del dashboard</t>
-  </si>
-  <si>
-    <t>Registrar el acceso bloqueado y mostrarlo en la campana del administrador</t>
-  </si>
-  <si>
-    <t>Cerrar la fuga de vista.js, exigir rol de personal en /api/asistencia y quitar scryptSync del recorrido del check-in</t>
-  </si>
-  <si>
-    <t>Medio</t>
-  </si>
-  <si>
-    <t>Con la búsqueda del QR ya corregida (paso anterior), medir el check-in con un volumen realista (unos 200 miembros)</t>
-  </si>
-  <si>
-    <t>Luis o Santiago</t>
-  </si>
-  <si>
-    <t>Editar y desactivar cuentas del personal</t>
-  </si>
-  <si>
-    <t>Congelar y descongelar membresías</t>
-  </si>
-  <si>
-    <t>Motor diario con Alerta Amarilla / Roja y umbrales editables</t>
-  </si>
-  <si>
-    <t>Script test, pruebas de check-in y alertas hasta ≥ 70 % de cobertura</t>
-  </si>
-  <si>
-    <t>Migración que cree vista_miembros_activos, auditoria y las columnas que usa el código</t>
-  </si>
-  <si>
-    <t>Cálculo de rachas, hitos y mensaje en el check-in</t>
-  </si>
-  <si>
-    <t>Monitor externo de disponibilidad con reporte (depende del plan de Render)</t>
-  </si>
-  <si>
-    <t>CRUD de retos, progreso automático y aviso al completar</t>
-  </si>
-  <si>
-    <t>Alto</t>
-  </si>
-  <si>
-    <t>Módulo de campañas y plantillas</t>
-  </si>
-  <si>
-    <t>Orden de menor a mayor esfuerzo. «Avance global acumulado» suma los puntos de cada acción, en orden, sobre el avance actual y se pone verde al llegar a la meta. Lo decide Luis; las implementaciones las hace Santiago.</t>
-  </si>
-  <si>
-    <t>RQF-25 no suma en la ruta: repite RQF-03 y es un defecto de seguridad, no una función; su arreglo cuenta en RQNF-05. Luis decide si se retira, junto con RQF-23, RQF-24 y RQF-26.</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Requisito</t>
-  </si>
-  <si>
-    <t>Ubicación (archivo:línea, endpoint o enlace)</t>
-  </si>
-  <si>
-    <t>Qué demuestra</t>
-  </si>
-  <si>
-    <t>Fecha de verificación</t>
-  </si>
-  <si>
-    <t>Verificado por</t>
-  </si>
-  <si>
-    <t>EV-01</t>
-  </si>
-  <si>
-    <t>backend/src/routes/staff.js:109, :198, :227, :329, :384</t>
-  </si>
-  <si>
-    <t>Invitar, listar y revocar personal; aceptar la invitación crea la cuenta.</t>
-  </si>
-  <si>
-    <t>2026-10-16</t>
-  </si>
-  <si>
-    <t>Agente ejecutor (Claude)</t>
-  </si>
-  <si>
-    <t>EV-02</t>
-  </si>
-  <si>
-    <t>backend/src/routes/staff.js:112; miembros.js:667; checkin.js:57; middleware/auth.js:29</t>
-  </si>
-  <si>
-    <t>Permisos distintos para Administrador y Recepcionista.</t>
-  </si>
-  <si>
-    <t>EV-03</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:200, :231, :295; frontend/src/context/AuthContext.jsx:95</t>
-  </si>
-  <si>
-    <t>Login con bcrypt + JWT y cierre de sesión manual.</t>
-  </si>
-  <si>
-    <t>EV-04</t>
-  </si>
-  <si>
-    <t>Código (hallazgo)</t>
-  </si>
-  <si>
-    <t>backend/src/lib/auth-helpers.js:102-113</t>
-  </si>
-  <si>
-    <t>generarToken no aplica JWT_EXPIRES_IN: el token del personal no expira.</t>
-  </si>
-  <si>
-    <t>EV-05</t>
-  </si>
-  <si>
-    <t>backend/src/routes/miembros.js:357-369, :371-379</t>
-  </si>
-  <si>
-    <t>Rechazo de documento / correo duplicado y QR único.</t>
-  </si>
-  <si>
-    <t>EV-06</t>
-  </si>
-  <si>
-    <t>backend/src/routes/miembros.js:607, :664-675; frontend/src/pages/MiembrosPage.jsx:627, :919, :442</t>
-  </si>
-  <si>
-    <t>Editar y desactivar (soft delete) desde la pantalla de miembros.</t>
-  </si>
-  <si>
-    <t>EV-07</t>
-  </si>
-  <si>
-    <t>backend/src/routes/miembros.js:185, :382, :276-284, :754</t>
-  </si>
-  <si>
-    <t>Fecha de vencimiento automática, estado vencido / por vencer y renovación.</t>
-  </si>
-  <si>
-    <t>EV-08</t>
-  </si>
-  <si>
-    <t>Esquema</t>
-  </si>
-  <si>
-    <t>backend/migrations/002_esquema_inicial.sql:217</t>
-  </si>
-  <si>
-    <t>congelacion_membresia existe pero no se usa (falta Congelada).</t>
-  </si>
-  <si>
-    <t>EV-09</t>
-  </si>
-  <si>
-    <t>frontend/src/pages/CheckinPage.jsx:66, :221-223, :329-331</t>
-  </si>
-  <si>
-    <t>Lectura HID tipo teclado (autoFocus + Enter) y por cámara.</t>
-  </si>
-  <si>
-    <t>EV-10</t>
-  </si>
-  <si>
-    <t>Código / esquema</t>
-  </si>
-  <si>
-    <t>backend/src/routes/checkin.js:54, :167-172; backend/migrations/002_esquema_inicial.sql:100</t>
-  </si>
-  <si>
-    <t>Inserción del ingreso con marca de tiempo automática.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/checkin.js:116-136; frontend/src/pages/CheckinPage.jsx:133-143</t>
-  </si>
-  <si>
-    <t>Bloqueo de membresía vencida; no hay aviso del intento al administrador.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/dashboard.js:123, :128, :146, :189, :204; frontend/src/pages/DashboardPage.jsx:165-179, :446-473</t>
-  </si>
-  <si>
-    <t>KPIs del día y próximos vencimientos; gráfica por día de semana; carga única.</t>
-  </si>
-  <si>
-    <t>EV-13</t>
-  </si>
-  <si>
-    <t>backend/src/routes/notificaciones.js:38, :66, :125-137; dashboard.js:161, :182; miembros.js:263</t>
-  </si>
-  <si>
-    <t>Lista de miembros en riesgo calculada al consultar, un solo umbral.</t>
-  </si>
-  <si>
-    <t>EV-14</t>
-  </si>
-  <si>
-    <t>backend/src/jobs/scheduler.js:46</t>
-  </si>
-  <si>
-    <t>El único cron programado es el de vencimientos (no hay motor de abandono).</t>
-  </si>
-  <si>
-    <t>frontend/src/components/MenuNotificaciones.jsx:86-90; MiembrosPage.jsx:796-802; backend/src/routes/notificaciones.js:188-224</t>
-  </si>
-  <si>
-    <t>Envío por WhatsApp y registro en envio_mensaje con fecha y estado.</t>
-  </si>
-  <si>
-    <t>backend/migrations/002_esquema_inicial.sql:171-202</t>
-  </si>
-  <si>
-    <t>Tablas de campañas y plantillas sin rutas ni pantalla.</t>
-  </si>
-  <si>
-    <t>Código / datos</t>
-  </si>
-  <si>
-    <t>backend/src/routes/cliente.js:340-381; ConsultasDB/Poblar_Tablas.sql:384-419</t>
-  </si>
-  <si>
-    <t>Hitos solo de lectura, cargados por SQL; no hay cálculo de rachas.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/cliente.js:392-418; ConsultasDB/Poblar_Tablas.sql:456-490</t>
-  </si>
-  <si>
-    <t>Retos solo de lectura, cargados por SQL; sin CRUD ni progreso automático.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/admin-contrato.js:76-160, :167, :195; backend/migrations/008_contrato_enviado.sql; frontend/src/pages/MiembrosPage.jsx:855-880</t>
-  </si>
-  <si>
-    <t>Envío del contrato por WhatsApp con registro de cada intento.</t>
-  </si>
-  <si>
-    <t>EV-20</t>
-  </si>
-  <si>
-    <t>backend/src/jobs/scheduler.js:46; backend/src/jobs/expiracion.js:43, :74, :94, :117, :151</t>
-  </si>
-  <si>
-    <t>Aviso diario automático de vencimiento, sin duplicados.</t>
-  </si>
-  <si>
-    <t>EV-21</t>
-  </si>
-  <si>
-    <t>backend/src/routes/jobs.js:27, :38; backend/migrations/006_gimnasio_dias_aviso.sql; 007_alerta_vencimiento_enviada.sql</t>
-  </si>
-  <si>
-    <t>Ejecución manual y vista previa; días de aviso y anti-duplicado en BD.</t>
-  </si>
-  <si>
-    <t>EV-22</t>
-  </si>
-  <si>
-    <t>backend/src/routes/cliente.js:51, :88, :112, :227, :259, :292, :340, :392; backend/src/lib/auth-helpers.js:145</t>
-  </si>
-  <si>
-    <t>API de la app: login del miembro y consultas protegidas.</t>
-  </si>
-  <si>
-    <t>EV-23</t>
-  </si>
-  <si>
-    <t>Código (Flutter)</t>
-  </si>
-  <si>
-    <t>fitloyalty_cliente/lib/cliente/screens/login_screen.dart, qr_tab.dart, plan_tab.dart, asistencia_screen.dart, gamificacion_screen.dart; services/api_client.dart:41</t>
-  </si>
-  <si>
-    <t>Pantallas de la app móvil y almacenamiento seguro del token.</t>
-  </si>
-  <si>
-    <t>Código / configuración</t>
-  </si>
-  <si>
-    <t>backend/src/lib/trial.js:17, :52-74; backend/src/routes/billing.js:19; backend/src/routes/auth.js:126-138; render.yaml; frontend/src/components/AdminLayout.jsx:155</t>
-  </si>
-  <si>
-    <t>Prueba de 14 días, estado visible y bloqueo 402 al vencer.</t>
-  </si>
-  <si>
-    <t>EV-25</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:304, :360, :399, :447; backend/src/lib/email.js:289; frontend/src/pages/ForgotPasswordPage.jsx:121, :143, :161</t>
-  </si>
-  <si>
-    <t>Recuperación de contraseña con código por correo.</t>
-  </si>
-  <si>
-    <t>EV-26</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:337-346</t>
-  </si>
-  <si>
-    <t>El código se devuelve en la respuesta si el correo no sale.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/dashboard.js:31-50, :288-337; frontend/src/pages/DashboardPage.jsx:193-203</t>
-  </si>
-  <si>
-    <t>Exportación CSV de miembros activos con su membresía.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:100-190; frontend/src/pages/RegisterOwnerPage.jsx; frontend/src/App.jsx:38</t>
-  </si>
-  <si>
-    <t>Registro del gimnasio y de su administrador.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/config.js:20-30, :41, :77; frontend/src/pages/ConfigPage.jsx:26, :44; backend/src/routes/notificaciones.js:44-67</t>
-  </si>
-  <si>
-    <t>Configuración de precios y recordatorios por gimnasio.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/miembros.js:88-95, :439-450, :754; backend/migrations/004_extender_miembro_cobros.sql:54; frontend/src/pages/MiembrosPage.jsx:207-208, :349-350</t>
-  </si>
-  <si>
-    <t>Registro del plan y del pago por miembro.</t>
-  </si>
-  <si>
-    <t>EV-31</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:480-561 (safe() en :496-502); frontend/src/pages/EliminarCuentaPage.jsx:22</t>
-  </si>
-  <si>
-    <t>Flujo de eliminación; safe() sin SAVEPOINT.</t>
-  </si>
-  <si>
-    <t>EV-32</t>
-  </si>
-  <si>
-    <t>Prueba (verificador)</t>
-  </si>
-  <si>
-    <t>Informe del verificador, commit 70dd13c, docs/verificacion-requisitos.md §11.2.1</t>
-  </si>
-  <si>
-    <t>En PostgreSQL 18 la transacción aborta y el gimnasio no se borra (dos esquemas).</t>
-  </si>
-  <si>
-    <t>backend/src/routes/notificaciones.js:73-180; frontend/src/components/MenuNotificaciones.jsx:38, :86-90</t>
-  </si>
-  <si>
-    <t>Centro de avisos accionables en el encabezado.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/asistencia.js:21, :26-60; backend/src/routes/checkin.js:199-224; frontend/src/pages/CheckinPage.jsx:46</t>
-  </si>
-  <si>
-    <t>Listado de ingresos con resumen.</t>
-  </si>
-  <si>
-    <t>EV-35</t>
-  </si>
-  <si>
-    <t>backend/src/routes/vista.js:18, :27, :38</t>
-  </si>
-  <si>
-    <t>Sin filtro por gimnasio ni rol: expone datos personales de todos los gimnasios.</t>
-  </si>
-  <si>
-    <t>EV-36</t>
-  </si>
-  <si>
-    <t>ConsultasDB/Query_Inicial_Crear_Tablas.sql:473; backend/src/lib/planes.js:4-7</t>
-  </si>
-  <si>
-    <t>La vista no se crea en las migraciones y lee una tabla vacía.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/cliente.js:112, :171-225; fitloyalty_cliente/lib/cliente/screens/editar_perfil_screen.dart; services/perfil_service.dart</t>
-  </si>
-  <si>
-    <t>Edición del perfil desde la app.</t>
-  </si>
-  <si>
-    <t>Sin medición</t>
-  </si>
-  <si>
-    <t>— (riesgo en backend/src/routes/checkin.js:83-101)</t>
-  </si>
-  <si>
-    <t>No hay evidencia de tiempos; posible lentitud con muchos miembros.</t>
-  </si>
-  <si>
-    <t>backend/src/index.js:101, :103</t>
-  </si>
-  <si>
-    <t>Endpoints de salud disponibles para monitoreo; sin reporte.</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:145, :231, :447; staff.js:431; miembros.js:388, :625; cliente.js:88; frontend/src/api.js:26</t>
-  </si>
-  <si>
-    <t>bcrypt en todas las contraseñas y API por HTTPS.</t>
-  </si>
-  <si>
-    <t>frontend/src/pages/CheckinPage.jsx:221-223, :333, :341-347</t>
-  </si>
-  <si>
-    <t>Flujo manual de 2 interacciones (sin prueba con usuarios).</t>
+    <t>Medición</t>
+  </si>
+  <si>
+    <t>docs/evidencias/cobertura-backend-2026-10-16.txt</t>
+  </si>
+  <si>
+    <t>Cobertura 0 % en checkin.js y notificaciones.js; 23 pruebas, 2 fallan.</t>
   </si>
   <si>
     <t>EV-42</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:100, :134; miembros.js:358; checkin.js:76; dashboard.js:123; notificaciones.js:199; admin-contrato.js:92</t>
-  </si>
-  <si>
-    <t>Alta de gimnasios sin código y aislamiento por id_gimnasio.</t>
-  </si>
-  <si>
-    <t>EV-43</t>
-  </si>
-  <si>
-    <t>backend/src/routes/vista.js:27-42</t>
-  </si>
-  <si>
-    <t>Única consulta sin filtro de gimnasio encontrada.</t>
-  </si>
-  <si>
-    <t>Documento</t>
-  </si>
-  <si>
-    <t>Evidencias_Sustentacion/QA_Responsive_375px.md; frontend/package.json; vercel.json</t>
-  </si>
-  <si>
-    <t>App web sin instalación; sin prueba en los 3 navegadores.</t>
-  </si>
-  <si>
-    <t>EV-45</t>
-  </si>
-  <si>
-    <t>Medición</t>
-  </si>
-  <si>
-    <t>docs/evidencias/cobertura-backend-2026-10-16.txt</t>
-  </si>
-  <si>
-    <t>Cobertura 0 % en checkin.js y notificaciones.js; 23 pruebas, 2 fallan.</t>
-  </si>
-  <si>
-    <t>EV-46</t>
   </si>
   <si>
     <t>backend/src/{routes,lib,middleware,jobs,db}; backend/package.json (sin script test); backend/jest.config.js:15-18</t>
@@ -1821,20 +1725,20 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.65384615384615385</c:v>
+                  <c:v>0.63636363636363635</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.63414634146341464</c:v>
+                  <c:v>0.6216216216216216</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0931-4DEE-89A7-4145FEF1F2A3}"/>
+              <c16:uniqueId val="{00000000-76E4-481D-9F73-2DE1AA6E4B6D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1991,20 +1895,20 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>19</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E8DD-4F3D-82C8-6DFC9450FF5F}"/>
+              <c16:uniqueId val="{00000000-8554-49DA-AE64-EDB3BB66324A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2450,11 +2354,11 @@
       </c>
       <c r="C6" s="8">
         <f>COUNTA(RF!$A$2:$A$100)</f>
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
@@ -2462,11 +2366,11 @@
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.65384615384615385</v>
+        <v>0.63636363636363635</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2474,14 +2378,14 @@
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>3.8000000000000007</v>
+        <v>3.6000000000000014</v>
       </c>
       <c r="J6" t="s">
         <v>13</v>
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
@@ -2530,11 +2434,11 @@
       </c>
       <c r="C8" s="13">
         <f>C6+C7</f>
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
@@ -2542,11 +2446,11 @@
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.63414634146341464</v>
+        <v>0.6216216216216216</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2554,14 +2458,14 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>6.8000000000000043</v>
+        <v>6.6000000000000014</v>
       </c>
       <c r="J8" t="s">
         <v>17</v>
       </c>
       <c r="K8">
         <f>F8</f>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
@@ -2720,7 +2624,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -3229,7 +3133,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
         <v>127</v>
       </c>
@@ -3493,140 +3397,8 @@
         <v>175</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="B24" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C24" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>177</v>
-      </c>
-      <c r="E24" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="F24" s="25">
-        <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C24,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>1</v>
-      </c>
-      <c r="G24" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="H24" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="I24" s="23" t="s">
-        <v>179</v>
-      </c>
-      <c r="J24" s="23" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="22" t="s">
-        <v>181</v>
-      </c>
-      <c r="B25" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>182</v>
-      </c>
-      <c r="E25" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="F25" s="25">
-        <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C25,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>1</v>
-      </c>
-      <c r="G25" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="H25" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="I25" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="J25" s="23" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="C26" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>188</v>
-      </c>
-      <c r="E26" s="23" t="s">
-        <v>189</v>
-      </c>
-      <c r="F26" s="25">
-        <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C26,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G26" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="H26" s="23" t="s">
-        <v>190</v>
-      </c>
-      <c r="I26" s="23" t="s">
-        <v>191</v>
-      </c>
-      <c r="J26" s="23" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="22" t="s">
-        <v>193</v>
-      </c>
-      <c r="B27" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="C27" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>194</v>
-      </c>
-      <c r="E27" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="F27" s="25">
-        <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C27,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>1</v>
-      </c>
-      <c r="G27" s="24" t="s">
-        <v>117</v>
-      </c>
-      <c r="H27" s="23" t="s">
-        <v>195</v>
-      </c>
-      <c r="I27" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="J27" s="23" t="s">
-        <v>197</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J27" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <autoFilter ref="A1:J23" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <conditionalFormatting sqref="C2:C100">
     <cfRule type="cellIs" dxfId="9" priority="1" operator="equal">
       <formula>"Implementado"</formula>
@@ -3701,19 +3473,19 @@
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3726,27 +3498,27 @@
         <v>63</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>202</v>
+        <v>180</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>17</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>206</v>
+        <v>184</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>207</v>
+        <v>185</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3759,27 +3531,27 @@
         <v>63</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>13</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3792,27 +3564,27 @@
         <v>63</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>214</v>
+        <v>192</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>215</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>217</v>
+        <v>195</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>15</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3822,30 +3594,30 @@
         <v>37</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>221</v>
+        <v>199</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>222</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>225</v>
+        <v>203</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>226</v>
+        <v>204</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3858,27 +3630,27 @@
         <v>138</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>229</v>
+        <v>207</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>230</v>
+        <v>208</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>15</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>231</v>
+        <v>209</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3891,27 +3663,27 @@
         <v>63</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>233</v>
+        <v>211</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>234</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>15</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3924,27 +3696,27 @@
         <v>63</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>239</v>
+        <v>217</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>240</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>241</v>
+        <v>219</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>13</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>243</v>
+        <v>221</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>244</v>
+        <v>222</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3957,27 +3729,27 @@
         <v>63</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>245</v>
+        <v>223</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>246</v>
+        <v>224</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>247</v>
+        <v>225</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>15</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>248</v>
+        <v>226</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3990,27 +3762,27 @@
         <v>63</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>250</v>
+        <v>228</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>251</v>
+        <v>229</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>252</v>
+        <v>230</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>15</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>253</v>
+        <v>231</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
@@ -4023,27 +3795,27 @@
         <v>63</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>255</v>
+        <v>233</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>256</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>257</v>
+        <v>235</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>13</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>258</v>
+        <v>236</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>259</v>
+        <v>237</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -4056,15 +3828,15 @@
         <v>63</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>260</v>
+        <v>238</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>261</v>
+        <v>239</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>262</v>
+        <v>240</v>
       </c>
       <c r="B13" s="23" t="s">
         <v>170</v>
@@ -4073,7 +3845,7 @@
         <v>13</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>263</v>
+        <v>241</v>
       </c>
       <c r="E13" s="23" t="s">
         <v>63</v>
@@ -4089,24 +3861,24 @@
         <v>63</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>264</v>
+        <v>242</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>265</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>266</v>
+        <v>244</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>267</v>
+        <v>245</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>13</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>63</v>
@@ -4122,24 +3894,24 @@
         <v>63</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>269</v>
+        <v>247</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>270</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>271</v>
+        <v>249</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>272</v>
+        <v>250</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>63</v>
@@ -4155,27 +3927,27 @@
         <v>63</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>273</v>
+        <v>251</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>274</v>
+        <v>252</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>17</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>276</v>
+        <v>254</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
@@ -4188,10 +3960,10 @@
         <v>63</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>278</v>
+        <v>256</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>279</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>
@@ -4221,7 +3993,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4245,40 +4017,40 @@
         <v>17</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>280</v>
+        <v>258</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>281</v>
+        <v>259</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>282</v>
+        <v>260</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>283</v>
+        <v>261</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>284</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>275</v>
+        <v>253</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>277</v>
+        <v>255</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4286,7 +4058,7 @@
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.65853658536585369</v>
+        <v>0.64864864864864868</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -4301,13 +4073,13 @@
         <v>172</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>288</v>
+        <v>266</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4315,7 +4087,7 @@
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.68292682926829273</v>
+        <v>0.67567567567567566</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
@@ -4330,13 +4102,13 @@
         <v>116</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4344,7 +4116,7 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.69512195121951215</v>
+        <v>0.68918918918918914</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="72" x14ac:dyDescent="0.3">
@@ -4359,13 +4131,13 @@
         <v>123</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4373,28 +4145,28 @@
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.70731707317073167</v>
+        <v>0.70270270270270274</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>247</v>
+        <v>225</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>249</v>
+        <v>227</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>291</v>
+        <v>269</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4402,28 +4174,28 @@
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.71951219512195119</v>
+        <v>0.71621621621621623</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>292</v>
+        <v>270</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4431,28 +4203,28 @@
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.73170731707317072</v>
+        <v>0.72972972972972971</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>229</v>
+        <v>207</v>
       </c>
       <c r="B8" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4460,7 +4232,7 @@
       </c>
       <c r="H8" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.74390243902439024</v>
+        <v>0.7432432432432432</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4475,13 +4247,13 @@
         <v>43</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>295</v>
+        <v>273</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
@@ -4489,7 +4261,7 @@
       </c>
       <c r="H9" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.75609756097560976</v>
+        <v>0.7567567567567568</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4504,13 +4276,13 @@
         <v>76</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>296</v>
+        <v>274</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
@@ -4518,7 +4290,7 @@
       </c>
       <c r="H10" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.76829268292682928</v>
+        <v>0.77027027027027029</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4533,13 +4305,13 @@
         <v>69</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>297</v>
+        <v>275</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
@@ -4547,28 +4319,28 @@
       </c>
       <c r="H11" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.78048780487804881</v>
+        <v>0.78378378378378377</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="B12" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>226</v>
+        <v>204</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>298</v>
+        <v>276</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4576,28 +4348,28 @@
       </c>
       <c r="H12" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>0.79268292682926833</v>
+        <v>0.79729729729729726</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="B13" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>300</v>
+        <v>278</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>301</v>
+        <v>279</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G13" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
@@ -4605,7 +4377,7 @@
       </c>
       <c r="H13" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G13))/Resumen!$C$8</f>
-        <v>0.81707317073170727</v>
+        <v>0.82432432432432434</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4620,13 +4392,13 @@
         <v>36</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>302</v>
+        <v>280</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G14" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
@@ -4634,7 +4406,7 @@
       </c>
       <c r="H14" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G14))/Resumen!$C$8</f>
-        <v>0.82926829268292679</v>
+        <v>0.83783783783783783</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4649,13 +4421,13 @@
         <v>56</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>303</v>
+        <v>281</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G15" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
@@ -4663,7 +4435,7 @@
       </c>
       <c r="H15" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G15))/Resumen!$C$8</f>
-        <v>0.84146341463414631</v>
+        <v>0.85135135135135132</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4678,13 +4450,13 @@
         <v>83</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>304</v>
+        <v>282</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G16" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
@@ -4692,28 +4464,28 @@
       </c>
       <c r="H16" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G16))/Resumen!$C$8</f>
-        <v>0.85365853658536583</v>
+        <v>0.86486486486486491</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="B17" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>305</v>
+        <v>283</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G17" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
@@ -4721,28 +4493,28 @@
       </c>
       <c r="H17" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G17))/Resumen!$C$8</f>
-        <v>0.86585365853658536</v>
+        <v>0.8783783783783784</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>252</v>
+        <v>230</v>
       </c>
       <c r="B18" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>254</v>
+        <v>232</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>306</v>
+        <v>284</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G18" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
@@ -4750,7 +4522,7 @@
       </c>
       <c r="H18" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G18))/Resumen!$C$8</f>
-        <v>0.87804878048780488</v>
+        <v>0.89189189189189189</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4765,13 +4537,13 @@
         <v>103</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>307</v>
+        <v>285</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G19" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
@@ -4779,28 +4551,28 @@
       </c>
       <c r="H19" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G19))/Resumen!$C$8</f>
-        <v>0.90243902439024393</v>
+        <v>0.91891891891891897</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="B20" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>207</v>
+        <v>185</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>308</v>
+        <v>286</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
       <c r="G20" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
@@ -4808,7 +4580,7 @@
       </c>
       <c r="H20" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G20))/Resumen!$C$8</f>
-        <v>0.92682926829268297</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -4823,13 +4595,13 @@
         <v>109</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>309</v>
+        <v>287</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F21" s="24" t="s">
-        <v>310</v>
+        <v>288</v>
       </c>
       <c r="G21" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A21,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A21,RNF!$A$2:$A$100,0)))</f>
@@ -4837,7 +4609,7 @@
       </c>
       <c r="H21" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G21))/Resumen!$C$8</f>
-        <v>0.95121951219512191</v>
+        <v>0.97297297297297303</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
@@ -4852,13 +4624,13 @@
         <v>96</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>311</v>
+        <v>289</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F22" s="24" t="s">
-        <v>310</v>
+        <v>288</v>
       </c>
       <c r="G22" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A22,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A22,RNF!$A$2:$A$100,0)))</f>
@@ -4866,17 +4638,12 @@
       </c>
       <c r="H22" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G22))/Resumen!$C$8</f>
-        <v>0.97560975609756095</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" s="17" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
-        <v>313</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>
@@ -4922,7 +4689,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4936,30 +4703,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>315</v>
+        <v>292</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>316</v>
+        <v>293</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>317</v>
+        <v>294</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>318</v>
+        <v>295</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>319</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>320</v>
+        <v>297</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>33</v>
@@ -4968,21 +4735,21 @@
         <v>24</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>321</v>
+        <v>298</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>322</v>
+        <v>299</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>325</v>
+        <v>302</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>33</v>
@@ -4991,21 +4758,21 @@
         <v>24</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>326</v>
+        <v>303</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>327</v>
+        <v>304</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>328</v>
+        <v>305</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>41</v>
@@ -5014,44 +4781,44 @@
         <v>24</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>329</v>
+        <v>306</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>331</v>
+        <v>308</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>41</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>332</v>
+        <v>309</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>333</v>
+        <v>310</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>334</v>
+        <v>311</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>335</v>
+        <v>312</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>47</v>
@@ -5060,21 +4827,21 @@
         <v>24</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>336</v>
+        <v>313</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>337</v>
+        <v>314</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>338</v>
+        <v>315</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>47</v>
@@ -5083,21 +4850,21 @@
         <v>24</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>339</v>
+        <v>316</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>340</v>
+        <v>317</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>341</v>
+        <v>318</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>54</v>
@@ -5106,44 +4873,44 @@
         <v>24</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>342</v>
+        <v>319</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>343</v>
+        <v>320</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>344</v>
+        <v>321</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>54</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>345</v>
+        <v>322</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>346</v>
+        <v>323</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>347</v>
+        <v>324</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>348</v>
+        <v>325</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>60</v>
@@ -5152,39 +4919,39 @@
         <v>24</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>349</v>
+        <v>326</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>350</v>
+        <v>327</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>351</v>
+        <v>328</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>60</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>352</v>
+        <v>329</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>353</v>
+        <v>330</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>354</v>
+        <v>331</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5198,16 +4965,16 @@
         <v>24</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>356</v>
+        <v>333</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5221,21 +4988,21 @@
         <v>24</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>357</v>
+        <v>334</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>358</v>
+        <v>335</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>359</v>
+        <v>336</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>80</v>
@@ -5244,21 +5011,21 @@
         <v>24</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>360</v>
+        <v>337</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>361</v>
+        <v>338</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>362</v>
+        <v>339</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>80</v>
@@ -5267,16 +5034,16 @@
         <v>24</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>363</v>
+        <v>340</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>364</v>
+        <v>341</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5290,16 +5057,16 @@
         <v>24</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>365</v>
+        <v>342</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -5310,19 +5077,19 @@
         <v>93</v>
       </c>
       <c r="C17" s="23" t="s">
+        <v>322</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>344</v>
+      </c>
+      <c r="E17" s="23" t="s">
         <v>345</v>
       </c>
-      <c r="D17" s="23" t="s">
-        <v>367</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>368</v>
-      </c>
       <c r="F17" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -5333,19 +5100,19 @@
         <v>100</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>369</v>
+        <v>346</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>370</v>
+        <v>347</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>371</v>
+        <v>348</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5356,19 +5123,19 @@
         <v>107</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>369</v>
+        <v>346</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>372</v>
+        <v>349</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>373</v>
+        <v>350</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5379,24 +5146,24 @@
         <v>113</v>
       </c>
       <c r="C20" s="23" t="s">
+        <v>329</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>351</v>
+      </c>
+      <c r="E20" s="23" t="s">
         <v>352</v>
       </c>
-      <c r="D20" s="23" t="s">
-        <v>374</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>375</v>
-      </c>
       <c r="F20" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>376</v>
+        <v>353</v>
       </c>
       <c r="B21" s="23" t="s">
         <v>121</v>
@@ -5405,44 +5172,44 @@
         <v>24</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>379</v>
+        <v>356</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>121</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>352</v>
+        <v>329</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>380</v>
+        <v>357</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>381</v>
+        <v>358</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>382</v>
+        <v>359</v>
       </c>
       <c r="B23" s="23" t="s">
         <v>127</v>
@@ -5451,761 +5218,669 @@
         <v>24</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>383</v>
+        <v>360</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>384</v>
+        <v>361</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>385</v>
+        <v>362</v>
       </c>
       <c r="B24" s="23" t="s">
         <v>127</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>386</v>
+        <v>363</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>387</v>
+        <v>364</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>388</v>
+        <v>365</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
+        <v>366</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>367</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>368</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B26" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="C25" s="23" t="s">
-        <v>389</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>390</v>
-      </c>
-      <c r="E25" s="23" t="s">
-        <v>391</v>
-      </c>
-      <c r="F25" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G25" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="22" t="s">
-        <v>392</v>
-      </c>
-      <c r="B26" s="23" t="s">
-        <v>141</v>
-      </c>
       <c r="C26" s="23" t="s">
-        <v>24</v>
+        <v>369</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>393</v>
+        <v>370</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>394</v>
+        <v>371</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>395</v>
+        <v>372</v>
       </c>
       <c r="B27" s="23" t="s">
         <v>141</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>332</v>
+        <v>24</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>396</v>
+        <v>373</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>397</v>
+        <v>374</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>150</v>
+        <v>375</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>24</v>
+        <v>309</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>398</v>
+        <v>376</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>399</v>
+        <v>377</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>24</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>400</v>
+        <v>378</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>401</v>
+        <v>379</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>24</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>402</v>
+        <v>380</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>403</v>
+        <v>381</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="B31" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>382</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>383</v>
+      </c>
+      <c r="F31" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="G31" s="23" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="22" t="s">
         <v>167</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B32" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="C31" s="23" t="s">
-        <v>352</v>
-      </c>
-      <c r="D31" s="23" t="s">
-        <v>404</v>
-      </c>
-      <c r="E31" s="23" t="s">
-        <v>405</v>
-      </c>
-      <c r="F31" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G31" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A32" s="22" t="s">
-        <v>406</v>
-      </c>
-      <c r="B32" s="23" t="s">
-        <v>169</v>
-      </c>
       <c r="C32" s="23" t="s">
-        <v>24</v>
+        <v>329</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>407</v>
+        <v>384</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>408</v>
+        <v>385</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>409</v>
+        <v>386</v>
       </c>
       <c r="B33" s="23" t="s">
         <v>169</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>410</v>
+        <v>24</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>411</v>
+        <v>387</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>412</v>
+        <v>388</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>179</v>
+        <v>389</v>
       </c>
       <c r="B34" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="C34" s="23" t="s">
+        <v>390</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>391</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>392</v>
+      </c>
+      <c r="F34" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="G34" s="23" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="B35" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="C34" s="23" t="s">
+      <c r="C35" s="23" t="s">
+        <v>393</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>394</v>
+      </c>
+      <c r="E35" s="23" t="s">
+        <v>395</v>
+      </c>
+      <c r="F35" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="G35" s="23" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="C36" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="D34" s="23" t="s">
-        <v>413</v>
-      </c>
-      <c r="E34" s="23" t="s">
-        <v>414</v>
-      </c>
-      <c r="F34" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G34" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A35" s="22" t="s">
-        <v>185</v>
-      </c>
-      <c r="B35" s="23" t="s">
-        <v>181</v>
-      </c>
-      <c r="C35" s="23" t="s">
+      <c r="D36" s="23" t="s">
+        <v>396</v>
+      </c>
+      <c r="E36" s="23" t="s">
+        <v>397</v>
+      </c>
+      <c r="F36" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="G36" s="23" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A37" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="B37" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="C37" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="D35" s="23" t="s">
-        <v>415</v>
-      </c>
-      <c r="E35" s="23" t="s">
-        <v>416</v>
-      </c>
-      <c r="F35" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G35" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A36" s="22" t="s">
-        <v>417</v>
-      </c>
-      <c r="B36" s="23" t="s">
-        <v>187</v>
-      </c>
-      <c r="C36" s="23" t="s">
-        <v>332</v>
-      </c>
-      <c r="D36" s="23" t="s">
-        <v>418</v>
-      </c>
-      <c r="E36" s="23" t="s">
-        <v>419</v>
-      </c>
-      <c r="F36" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="22" t="s">
-        <v>420</v>
-      </c>
-      <c r="B37" s="23" t="s">
-        <v>187</v>
-      </c>
-      <c r="C37" s="23" t="s">
-        <v>345</v>
-      </c>
       <c r="D37" s="23" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>24</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>202</v>
+        <v>402</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>425</v>
+        <v>24</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="F39" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>208</v>
+        <v>405</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>24</v>
+        <v>309</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>428</v>
+        <v>406</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>429</v>
+        <v>407</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>24</v>
+        <v>408</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>430</v>
+        <v>409</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>431</v>
+        <v>410</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>221</v>
+        <v>411</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>24</v>
+        <v>412</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>432</v>
+        <v>413</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>433</v>
+        <v>414</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>434</v>
+        <v>415</v>
       </c>
       <c r="B43" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="C43" s="23" t="s">
+        <v>369</v>
+      </c>
+      <c r="D43" s="23" t="s">
+        <v>416</v>
+      </c>
+      <c r="E43" s="23" t="s">
+        <v>417</v>
+      </c>
+      <c r="F43" s="23" t="s">
+        <v>300</v>
+      </c>
+      <c r="G43" s="23" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A44" s="22" t="s">
         <v>223</v>
       </c>
-      <c r="C43" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D43" s="23" t="s">
-        <v>435</v>
-      </c>
-      <c r="E43" s="23" t="s">
-        <v>436</v>
-      </c>
-      <c r="F43" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G43" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="22" t="s">
-        <v>437</v>
-      </c>
       <c r="B44" s="23" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>332</v>
+        <v>157</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>438</v>
+        <v>418</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>439</v>
+        <v>419</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>440</v>
+        <v>24</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>441</v>
+        <v>420</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>442</v>
+        <v>421</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>443</v>
+        <v>233</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>444</v>
+        <v>24</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>445</v>
+        <v>422</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>446</v>
+        <v>423</v>
       </c>
       <c r="F46" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>447</v>
+        <v>238</v>
       </c>
       <c r="B47" s="23" t="s">
         <v>235</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>389</v>
+        <v>424</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>448</v>
+        <v>425</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>449</v>
+        <v>426</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>157</v>
+        <v>24</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>450</v>
+        <v>427</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>451</v>
+        <v>428</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>24</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>452</v>
+        <v>429</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>453</v>
+        <v>430</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>24</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>454</v>
+        <v>431</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>455</v>
+        <v>432</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>456</v>
+        <v>309</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>457</v>
+        <v>433</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>458</v>
+        <v>434</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>323</v>
+        <v>300</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A52" s="22" t="s">
-        <v>264</v>
-      </c>
-      <c r="B52" s="23" t="s">
-        <v>262</v>
-      </c>
-      <c r="C52" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D52" s="23" t="s">
-        <v>459</v>
-      </c>
-      <c r="E52" s="23" t="s">
-        <v>460</v>
-      </c>
-      <c r="F52" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G52" s="23" t="s">
-        <v>324</v>
+        <v>301</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A53" s="22" t="s">
-        <v>269</v>
-      </c>
-      <c r="B53" s="23" t="s">
-        <v>266</v>
-      </c>
-      <c r="C53" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D53" s="23" t="s">
-        <v>461</v>
-      </c>
-      <c r="E53" s="23" t="s">
-        <v>462</v>
-      </c>
-      <c r="F53" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G53" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A54" s="22" t="s">
-        <v>273</v>
-      </c>
-      <c r="B54" s="23" t="s">
-        <v>271</v>
-      </c>
-      <c r="C54" s="23" t="s">
-        <v>24</v>
-      </c>
-      <c r="D54" s="23" t="s">
-        <v>463</v>
-      </c>
-      <c r="E54" s="23" t="s">
-        <v>464</v>
-      </c>
-      <c r="F54" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G54" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A55" s="22" t="s">
-        <v>278</v>
-      </c>
-      <c r="B55" s="23" t="s">
-        <v>275</v>
-      </c>
-      <c r="C55" s="23" t="s">
-        <v>332</v>
-      </c>
-      <c r="D55" s="23" t="s">
-        <v>465</v>
-      </c>
-      <c r="E55" s="23" t="s">
-        <v>466</v>
-      </c>
-      <c r="F55" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="G55" s="23" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" s="17" t="s">
-        <v>467</v>
+      <c r="A53" s="17" t="s">
+        <v>435</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G55" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G51" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(avance): RQF-22 y RQNF-05 pasan a Implementado en el Excel (66,2 %)
Tras fusionar en develop los PR #9, #11, #14 y #15 (1ddcb24):
- RQF-22 Implementado (PR #15, verificador 94d5fbb sec. 16).
- RQNF-05 Implementado (PR #11, verificador 386d168 sec. 14.5).
- RQF-13 sigue Parcial: el contrato no sale tras un reinicio (sec. 14.3).
- RQNF-10 sigue Parcial: envio_mensaje y notificacion difieren de
  produccion (sec. 15).

Editado con Excel por COM para conservar graficos, formato condicional
y formulas. Avance: 24,5 de 37 puntos = 66,2 % (RF 68,2 %, RNF 63,3 %).
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C26BE2-6673-44F3-8F95-488B0B4EF963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6E09B9-5837-448A-8214-DDF52AE5FF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,14 +42,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="861" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="441">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
   <si>
-    <t>Estado de implementación verificado contra el código el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
-  </si>
-  <si>
     <t>Tipo</t>
   </si>
   <si>
@@ -389,12 +386,6 @@
     <t>Contratos</t>
   </si>
   <si>
-    <t>POST /api/admin/miembros/:id/contrato/enviar con control de gimnasio (admin-contrato.js:76-92); si el cliente de WhatsApp no está listo, lo informa y registra exito = false (:107-128); vista previa e historial por API (:167, :195); botón «Enviar contrato» (MiembrosPage.jsx:855-880, :1735).</t>
-  </si>
-  <si>
-    <t>Con el cliente listo, un envío que falla queda registrado como exitoso: sendWhatsAppText se traga el error (whatsapp.js:244-246) y el catch de admin-contrato.js:132-138 nunca se ejecuta. Arreglo: relanzar el error en sendWhatsAppText.</t>
-  </si>
-  <si>
     <t>Nuevo</t>
   </si>
   <si>
@@ -557,12 +548,6 @@
     <t>Cumplimiento</t>
   </si>
   <si>
-    <t>DELETE /api/auth/account (auth.js:480-561) borra en una transacción con safe(), que solo ignora el código 42P01 y no usa SAVEPOINT (auth.js:496-502). En PostgreSQL cualquier error, incluso el ignorado, aborta la transacción: con las migraciones falla en DELETE FROM auditoria (ninguna migración crea esa tabla) y con el esquema de ConsultasDB el INSERT en auditoria viola la llave foránea hacia el usuario borrado. En los dos casos el gimnasio queda intacto y la API responde 500. Probado en PostgreSQL 18 en el informe del verificador (70dd13c, sección 11.2.1).</t>
-  </si>
-  <si>
-    <t>Un SAVEPOINT por cada safe() (o quitar las tablas que no existen) y no insertar en auditoria filas que apunten al usuario y al gimnasio que se borran. Si se corrige y se prueba, puede volver a Implementado. El PR #4 y mi versión anterior lo daban por Implementado leyendo solo el código.</t>
-  </si>
-  <si>
     <t>HU-63</t>
   </si>
   <si>
@@ -581,9 +566,6 @@
     <t>No hay medición registrada.</t>
   </si>
   <si>
-    <t>Primero corregir la búsqueda del QR (paso 11 de «Trabajo pendiente»): si el QR no coincide directo, checkin.js:83-101 descifra en memoria los QR de todos los miembros del gimnasio. Después, medir el check-in con un volumen realista (unos 200 miembros) y registrar el tiempo de respuesta de POST /api/admin/checkin.</t>
-  </si>
-  <si>
     <t>EV-34</t>
   </si>
   <si>
@@ -653,12 +635,6 @@
     <t>Escalabilidad</t>
   </si>
   <si>
-    <t>Cada gimnasio nuevo se crea por registro, sin tocar código (auth.js:100, :134); casi todas las consultas filtran por el id_gimnasio del token (p. ej. miembros.js:358, checkin.js:76, dashboard.js:123, notificaciones.js:199; admin-contrato.js:92).</t>
-  </si>
-  <si>
-    <t>GET /api/vista/miembros-activos no filtra por gimnasio (vista.js:27-42) y rompe el aislamiento entre gimnasios. No hay prueba de carga que respalde «sin degradación del rendimiento».</t>
-  </si>
-  <si>
     <t>EV-38, EV-39</t>
   </si>
   <si>
@@ -737,12 +713,6 @@
     <t>RQNF-10</t>
   </si>
   <si>
-    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 008 en backend/migrations.</t>
-  </si>
-  <si>
-    <t>Una base creada solo con backend/migrations no tiene vista_miembros_activos ni auditoria, y reto tiene meta en lugar de meta_asistencias (002_esquema_inicial.sql:278-290); el esquema de producción salió de ConsultasDB/ y de cambios manuales. Probado en el informe del verificador (70dd13c, sección 11.2.1). Además hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica.</t>
-  </si>
-  <si>
     <t>EV-45</t>
   </si>
   <si>
@@ -842,12 +812,6 @@
     <t>Bajo</t>
   </si>
   <si>
-    <t>Un SAVEPOINT por cada safe() y no insertar en auditoria lo que se borra; probar la eliminación</t>
-  </si>
-  <si>
-    <t>Relanzar el error en sendWhatsAppText para que un envío fallido no quede como exitoso</t>
-  </si>
-  <si>
     <t>No marcar el aviso como enviado si WhatsApp no está listo (reintentar) y llevar los días a Configuración</t>
   </si>
   <si>
@@ -872,15 +836,9 @@
     <t>Registrar el acceso bloqueado y mostrarlo en la campana del administrador</t>
   </si>
   <si>
-    <t>Cerrar la fuga de vista.js, exigir rol de personal en /api/asistencia y quitar scryptSync del recorrido del check-in</t>
-  </si>
-  <si>
     <t>Medio</t>
   </si>
   <si>
-    <t>Con la búsqueda del QR ya corregida (paso anterior), medir el check-in con un volumen realista (unos 200 miembros)</t>
-  </si>
-  <si>
     <t>Luis o Santiago</t>
   </si>
   <si>
@@ -896,9 +854,6 @@
     <t>Script test, pruebas de check-in y alertas hasta ≥ 70 % de cobertura</t>
   </si>
   <si>
-    <t>Migración que cree vista_miembros_activos, auditoria y las columnas que usa el código</t>
-  </si>
-  <si>
     <t>Cálculo de rachas, hitos y mensaje en el check-in</t>
   </si>
   <si>
@@ -914,9 +869,6 @@
     <t>Módulo de campañas y plantillas</t>
   </si>
   <si>
-    <t>Orden de menor a mayor esfuerzo. «Avance global acumulado» suma los puntos de cada acción, en orden, sobre el avance actual y se pone verde al llegar a la meta. Lo decide Luis; las implementaciones las hace Santiago.</t>
-  </si>
-  <si>
     <t>ID</t>
   </si>
   <si>
@@ -1097,12 +1049,6 @@
     <t>Retos solo de lectura, cargados por SQL; sin CRUD ni progreso automático.</t>
   </si>
   <si>
-    <t>backend/src/routes/admin-contrato.js:76-160, :167, :195; backend/migrations/008_contrato_enviado.sql; frontend/src/pages/MiembrosPage.jsx:855-880</t>
-  </si>
-  <si>
-    <t>Envío del contrato por WhatsApp con registro de cada intento.</t>
-  </si>
-  <si>
     <t>EV-20</t>
   </si>
   <si>
@@ -1205,24 +1151,12 @@
     <t>EV-32</t>
   </si>
   <si>
-    <t>backend/src/routes/auth.js:480-561 (safe() en :496-502); frontend/src/pages/EliminarCuentaPage.jsx:22</t>
-  </si>
-  <si>
-    <t>Flujo de eliminación; safe() sin SAVEPOINT.</t>
-  </si>
-  <si>
     <t>EV-33</t>
   </si>
   <si>
     <t>Prueba (verificador)</t>
   </si>
   <si>
-    <t>Informe del verificador, commit 70dd13c, docs/verificacion-requisitos.md §11.2.1</t>
-  </si>
-  <si>
-    <t>En PostgreSQL 18 la transacción aborta y el gimnasio no se borra (dos esquemas).</t>
-  </si>
-  <si>
     <t>Sin medición</t>
   </si>
   <si>
@@ -1253,21 +1187,9 @@
     <t>EV-38</t>
   </si>
   <si>
-    <t>backend/src/routes/auth.js:100, :134; miembros.js:358; checkin.js:76; dashboard.js:123; notificaciones.js:199; admin-contrato.js:92</t>
-  </si>
-  <si>
-    <t>Alta de gimnasios sin código y aislamiento por id_gimnasio.</t>
-  </si>
-  <si>
     <t>EV-39</t>
   </si>
   <si>
-    <t>backend/src/routes/vista.js:27-42</t>
-  </si>
-  <si>
-    <t>Única consulta sin filtro de gimnasio encontrada.</t>
-  </si>
-  <si>
     <t>Documento</t>
   </si>
   <si>
@@ -1310,12 +1232,6 @@
     <t>Límites de intentos por IP en los endpoints sensibles.</t>
   </si>
   <si>
-    <t>backend/src/db/migrate.js:15-56; backend/src/index.js:128-132; backend/migrations/</t>
-  </si>
-  <si>
-    <t>Migraciones versionadas aplicadas al iniciar.</t>
-  </si>
-  <si>
     <t>Configuración / ejecución</t>
   </si>
   <si>
@@ -1350,6 +1266,105 @@
   </si>
   <si>
     <t>Rutas relativas a la raíz del repositorio en main @ 54b19fa (el CI de RQNF-11 en 8acab31). No se hicieron pruebas en vivo: la verificación es por lectura de código, pruebas existentes y CI.</t>
+  </si>
+  <si>
+    <t>POST /api/admin/miembros/:id/contrato/enviar con control de gimnasio (admin-contrato.js:76-92); vista previa e historial por API (:167, :195); botón «Enviar contrato» (MiembrosPage.jsx:855-880, :1735). Desde el PR #9, sendWhatsAppText lanza un error si el módulo está apagado, el cliente no está listo, el teléfono no es válido o el envío falla (whatsapp.js:223-246), y admin-contrato.js:130-138 registra exito = false; 5 pruebas en backend/tests/whatsapp-text.test.js.</t>
+  </si>
+  <si>
+    <t>Sigue Parcial (criterio del 2026-10-18): el aviso al administrador y el registro de cada intento ya son correctos, pero tras cada reinicio del servidor el contrato no sale. admin-contrato.js:107 pregunta isWhatsAppReady() antes de enviar y el cliente se inicia de forma perezosa (whatsapp.js:146), así que responde «no autenticado» sin llegar a iniciar el cliente ni a mostrar el QR que pide escanear; solo funciona si otro flujo lo inició antes (alta de un miembro con teléfono). Arreglo: quitar esa comprobación previa (sendWhatsAppText ya lanza el error) o iniciar el cliente antes, junto con la corrección del PR #10. Verificador: 386d168, sección 14.3.</t>
+  </si>
+  <si>
+    <t>DELETE /api/auth/account (auth.js:548), solo para el administrador (403 en :554). Borra en una transacción los 29 pasos de PASOS_ELIMINAR_CUENTA (:493) con un SAVEPOINT por paso (borrarPaso, :534), que solo omite una tabla o columna inexistente (42P01 y 42703, :527); el gimnasio se borra al final (:567), responde 404 si ya no existe (:570) y el rastro queda en el log del servidor (:575). Ya no inserta en auditoria. PR #15.</t>
+  </si>
+  <si>
+    <t>Probado por el verificador con el handler real sobre PostgreSQL 18 (94d5fbb, sección 16): en las bases Docker, Docker + 009 y tipo producción responde 200, no deja filas del gimnasio y no toca las de otro; si una FK desconocida lo bloquea, responde 500 y no borra nada. Riesgo anotado: cualquier usuario con rol admin, también un administrador invitado, puede eliminar el gimnasio sin volver a escribir su contraseña; conviene pedirla. EliminarCuentaPage.jsx:46 todavía promete cancelar la facturación, y el sistema no cobra.</t>
+  </si>
+  <si>
+    <t>Cada gimnasio nuevo se crea por registro, sin tocar código (auth.js:100, :134); las consultas filtran por el id_gimnasio del token (p. ej. miembros.js:358, checkin.js:76, dashboard.js:123, notificaciones.js:199). Desde el PR #11: vista.js exige rol de personal (:20), rechaza al personal sin gimnasio (:28) y filtra por gimnasio (:32, :46) sobre la vista de la migración 011; asistencia.js exige rol de personal (:22); checkin.js deriva la clave del QR una sola vez (:26, :31). 9 pruebas en backend/tests/aislamiento.test.js.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-18): ya no queda ninguna consulta sin filtro de gimnasio y el check-in dejó de derivar la clave del QR por cada miembro (verificador: 386d168, sección 14.5). La medición del tiempo de respuesta con volumen realista queda en RQNF-01. Menor: la vista lee membresia y plan_membresia, que el alta no llena, así que sus columnas de plan salen en NULL.</t>
+  </si>
+  <si>
+    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 009 y 011: la 009 (PR #14) crea auditoria y agrega las columnas y restricciones de gamificación de producción, y la 011 (PR #11) recrea vista_miembros_activos con id_gimnasio.</t>
+  </si>
+  <si>
+    <t>Sigue Parcial (verificador: 94d5fbb, sección 15): una base hecha solo con migraciones todavía difiere de producción en 15 tablas, y el código usa dos de ellas: notificaciones.js:211 escribe envio_mensaje.canal y :217 notificacion.leido, que no existen en el esquema de producción (allí son id_canal y leida). Pasa a Implementado con una migración que reconcilie esas dos tablas (o un cambio del código), probada contra la copia de producción. Además hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica.</t>
+  </si>
+  <si>
+    <t>La búsqueda del QR ya no deriva la clave por cada miembro (PR #11, checkin.js:26, :31): hace un descifrado AES por miembro. Falta medir el check-in con un volumen realista (unos 200 miembros) y registrar el tiempo de respuesta de POST /api/admin/checkin.</t>
+  </si>
+  <si>
+    <t>Código / prueba</t>
+  </si>
+  <si>
+    <t>backend/src/routes/admin-contrato.js:76-160, :107, :130-138, :167, :195; backend/src/lib/whatsapp.js:146, :223-246; backend/tests/whatsapp-text.test.js; backend/migrations/008_contrato_enviado.sql; frontend/src/pages/MiembrosPage.jsx:855-880</t>
+  </si>
+  <si>
+    <t>Envío del contrato con registro de cada intento; el error del envío ya llega al registro (exito = false). Tras un reinicio no se inicia el cliente (admin-contrato.js:107).</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:493, :527, :534, :548-585 (403 en :554, gimnasio en :567, 404 en :570); frontend/src/pages/EliminarCuentaPage.jsx</t>
+  </si>
+  <si>
+    <t>Eliminación de cuenta con un SAVEPOINT por paso, solo para el administrador y atómica (PR #15).</t>
+  </si>
+  <si>
+    <t>Informe del verificador, commit 94d5fbb, docs/verificacion-requisitos.md §16</t>
+  </si>
+  <si>
+    <t>Con el handler real en PostgreSQL 18 y tres esquemas: 200, sin filas del gimnasio y sin tocar el otro; 500 sin borrar nada si una FK desconocida lo bloquea.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:100, :134; vista.js:20, :28, :32, :46; asistencia.js:22; checkin.js:26, :31, :76; miembros.js:358; dashboard.js:123; notificaciones.js:199</t>
+  </si>
+  <si>
+    <t>Alta de gimnasios sin código; aislamiento por id_gimnasio en todas las consultas, también en la vista y en asistencia (PR #11).</t>
+  </si>
+  <si>
+    <t>Prueba / esquema</t>
+  </si>
+  <si>
+    <t>backend/tests/aislamiento.test.js (9 pruebas); backend/migrations/011_vista_miembros_activos_gimnasio.sql; informe del verificador, commit 386d168, §14.5</t>
+  </si>
+  <si>
+    <t>La vista y asistencia rechazan tokens de miembro y filtran por gimnasio; la 011 expone id_gimnasio.</t>
+  </si>
+  <si>
+    <t>backend/src/db/migrate.js:15-56; backend/src/index.js:128-132; backend/migrations/ (009_auditoria_y_gamificacion.sql y 011_vista_miembros_activos_gimnasio.sql)</t>
+  </si>
+  <si>
+    <t>Migraciones versionadas aplicadas al iniciar; la 009 cierra auditoría y gamificación. Quedan diferencias en envio_mensaje y notificacion (verificador 94d5fbb §15).</t>
+  </si>
+  <si>
+    <t>Tras un reinicio el contrato no sale: admin-contrato.js:107 pregunta isWhatsAppReady() y nunca inicia el cliente de WhatsApp (whatsapp.js:146).</t>
+  </si>
+  <si>
+    <t>Quitar la comprobación previa de admin-contrato.js:107 (o iniciar el cliente antes de preguntar), junto con el arreglo del PR #10</t>
+  </si>
+  <si>
+    <t>Medir el check-in con un volumen realista (unos 200 miembros)</t>
+  </si>
+  <si>
+    <t>notificaciones.js:211 y :217 escriben envio_mensaje.canal y notificacion.leido, que no existen en el esquema de producción (verificador, sección 15).</t>
+  </si>
+  <si>
+    <t>Migración que reconcilie envio_mensaje y notificacion con producción (o cambio del código), probada contra la copia de producción</t>
+  </si>
+  <si>
+    <t>Luis (PR #16)</t>
+  </si>
+  <si>
+    <t>Luis (PR #17)</t>
+  </si>
+  <si>
+    <t>Estado actualizado el 2026-10-18 con los PR fusionados en develop @ 1ddcb24 (#9, #11, #14 y #15); la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
+  </si>
+  <si>
+    <t>Orden de menor a mayor esfuerzo. «Avance global acumulado» suma los puntos de cada acción, en orden, sobre el avance actual y se pone verde al llegar a la meta. Lo decide Luis; el reparto de tareas está en docs/plan-trabajo.md.</t>
+  </si>
+  <si>
+    <t>2026-10-18</t>
   </si>
 </sst>
 </file>
@@ -1457,7 +1472,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1524,6 +1539,9 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1725,13 +1743,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.63636363636363635</c:v>
+                  <c:v>0.68181818181818177</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.6</c:v>
+                  <c:v>0.6333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.6216216216216216</c:v>
+                  <c:v>0.66216216216216217</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1895,13 +1913,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>14</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2313,44 +2331,44 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>1</v>
+        <v>438</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" s="8">
         <f>COUNTA(RF!$A$2:$A$100)</f>
@@ -2358,7 +2376,7 @@
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
@@ -2366,11 +2384,11 @@
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.63636363636363635</v>
+        <v>0.68181818181818177</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2378,19 +2396,19 @@
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>3.6000000000000014</v>
+        <v>2.6000000000000032</v>
       </c>
       <c r="J6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B7" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7" s="8">
         <f>COUNTA(RNF!$A$2:$A$100)</f>
@@ -2398,11 +2416,11 @@
       </c>
       <c r="D7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Implementado")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Parcial")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Pendiente")</f>
@@ -2410,7 +2428,7 @@
       </c>
       <c r="G7" s="9">
         <f>IF(C7=0,0,SUM(RNF!$F$2:$F$100)/C7)</f>
-        <v>0.6</v>
+        <v>0.6333333333333333</v>
       </c>
       <c r="H7" s="10">
         <f>Resumen!$C$40</f>
@@ -2418,19 +2436,19 @@
       </c>
       <c r="I7" s="11">
         <f>MAX(0,H7*C7-G7*C7)</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="J7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K7">
         <f>E8</f>
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B8" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C8" s="13">
         <f>C6+C7</f>
@@ -2438,19 +2456,19 @@
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.6216216216216216</v>
+        <v>0.66216216216216217</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2458,49 +2476,49 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>6.6000000000000014</v>
+        <v>5.1000000000000014</v>
       </c>
       <c r="J8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8">
         <f>F8</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B10" s="17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B29" s="18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B30" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="D30" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="G30" s="6" t="s">
         <v>6</v>
-      </c>
-      <c r="G30" s="6" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B31" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C31" s="8">
         <f>COUNTIFS(RF!$A$2:$A$100,"RQ*",RF!$G$2:$G$100,"Original")</f>
@@ -2525,7 +2543,7 @@
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B32" s="7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C32" s="8">
         <f>COUNTIFS(RNF!$A$2:$A$100,"RQ*",RNF!$G$2:$G$100,"Original")</f>
@@ -2533,11 +2551,11 @@
       </c>
       <c r="D32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Implementado",RNF!$G$2:$G$100,"Original")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Parcial",RNF!$G$2:$G$100,"Original")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Pendiente",RNF!$G$2:$G$100,"Original")</f>
@@ -2545,12 +2563,12 @@
       </c>
       <c r="G32" s="9">
         <f>IF(C32=0,0,SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original")/C32)</f>
-        <v>0.5</v>
+        <v>0.5625</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B33" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C33" s="13">
         <f>C31+C32</f>
@@ -2558,11 +2576,11 @@
       </c>
       <c r="D33" s="13">
         <f>D31+D32</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E33" s="13">
         <f>E31+E32</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F33" s="13">
         <f>F31+F32</f>
@@ -2570,28 +2588,28 @@
       </c>
       <c r="G33" s="14">
         <f>IF(C33=0,0,(SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")+SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original"))/C33)</f>
-        <v>0.5</v>
+        <v>0.52500000000000002</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B35" s="18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B36" s="19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C36" s="20">
         <v>1</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B37" s="19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C37" s="20">
         <v>0.5</v>
@@ -2599,7 +2617,7 @@
     </row>
     <row r="38" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B38" s="19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C38" s="20">
         <v>0</v>
@@ -2607,13 +2625,13 @@
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B40" s="18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C40" s="21">
         <v>0.8</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -2641,760 +2659,760 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="C2" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="23" t="s">
+      <c r="E2" s="23" t="s">
         <v>35</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>36</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G2" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="H2" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="I2" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="J2" s="23" t="s">
         <v>39</v>
-      </c>
-      <c r="J2" s="23" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="23" t="s">
+      <c r="E3" s="23" t="s">
         <v>42</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>43</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H3" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="I3" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="J3" s="23" t="s">
         <v>45</v>
-      </c>
-      <c r="J3" s="23" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="C4" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="C4" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="23" t="s">
+      <c r="E4" s="23" t="s">
         <v>49</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>50</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H4" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="I4" s="23" t="s">
         <v>51</v>
       </c>
-      <c r="I4" s="23" t="s">
+      <c r="J4" s="23" t="s">
         <v>52</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="B5" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="23" t="s">
+      <c r="E5" s="23" t="s">
         <v>55</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>56</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H5" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="J5" s="23" t="s">
         <v>58</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="C6" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="23" t="s">
+      <c r="E6" s="23" t="s">
         <v>62</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>63</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H6" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="I6" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="J6" s="23" t="s">
         <v>65</v>
-      </c>
-      <c r="J6" s="23" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="23" t="s">
+      <c r="E7" s="23" t="s">
         <v>68</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>69</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H7" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="J7" s="23" t="s">
         <v>71</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="23" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="C8" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="C8" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="23" t="s">
+      <c r="E8" s="23" t="s">
         <v>75</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>76</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H8" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="J8" s="23" t="s">
         <v>78</v>
-      </c>
-      <c r="J8" s="23" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="C9" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="23" t="s">
+      <c r="E9" s="23" t="s">
         <v>82</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>83</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H9" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="I9" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="J9" s="23" t="s">
         <v>85</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="23" t="s">
-        <v>81</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="23" t="s">
+      <c r="E10" s="23" t="s">
         <v>88</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>89</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H10" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="I10" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="I10" s="23" t="s">
+      <c r="J10" s="23" t="s">
         <v>91</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B11" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="C11" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="C11" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="23" t="s">
+      <c r="E11" s="23" t="s">
         <v>95</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>96</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H11" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="I11" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="J11" s="23" t="s">
         <v>98</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="C12" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="C12" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="23" t="s">
+      <c r="E12" s="23" t="s">
         <v>102</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>103</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H12" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="I12" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="I12" s="23" t="s">
+      <c r="J12" s="23" t="s">
         <v>105</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="B13" s="23" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="B13" s="23" t="s">
-        <v>101</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="23" t="s">
+      <c r="E13" s="23" t="s">
         <v>108</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>109</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H13" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="I13" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="I13" s="23" t="s">
+      <c r="J13" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="J13" s="23" t="s">
+    </row>
+    <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
+      <c r="A14" s="22" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
+      <c r="B14" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="23" t="s">
-        <v>114</v>
-      </c>
       <c r="C14" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>115</v>
+        <v>408</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>116</v>
+        <v>409</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="J14" s="23" t="s">
         <v>117</v>
-      </c>
-      <c r="H14" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="E16" s="23" t="s">
         <v>127</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>130</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="E17" s="23" t="s">
         <v>134</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>135</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>137</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I17" s="23" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I18" s="23" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C19" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F19" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C19,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="I19" s="23" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C20" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F20" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C20,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="E21" s="23" t="s">
         <v>156</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="C21" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="E21" s="23" t="s">
-        <v>159</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="I21" s="23" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C22" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="I22" s="23" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C23" s="24" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>171</v>
+        <v>410</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>172</v>
+        <v>411</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -3441,529 +3459,529 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>179</v>
+        <v>416</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>203</v>
+        <v>412</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>204</v>
+        <v>413</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>231</v>
+        <v>414</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>232</v>
+        <v>415</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -3993,7 +4011,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4008,49 +4026,49 @@
   <sheetData>
     <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
+        <v>245</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>253</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>255</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>263</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>264</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>265</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4058,57 +4076,57 @@
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.64864864864864868</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.68918918918918914</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>169</v>
+        <v>112</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>172</v>
+        <v>431</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>266</v>
+        <v>432</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.67567567567567566</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.70270270270270274</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4116,28 +4134,28 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.68918918918918914</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+        <v>0.71621621621621623</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>121</v>
+        <v>217</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>123</v>
+        <v>219</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4145,28 +4163,28 @@
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.70270270270270274</v>
+        <v>0.72972972972972971</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>225</v>
+        <v>188</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>227</v>
+        <v>191</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4174,28 +4192,28 @@
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.71621621621621623</v>
+        <v>0.7432432432432432</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4203,28 +4221,28 @@
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.72972972972972971</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.7567567567567568</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>207</v>
+        <v>40</v>
       </c>
       <c r="B8" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>210</v>
+        <v>42</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4232,28 +4250,28 @@
       </c>
       <c r="H8" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.7432432432432432</v>
+        <v>0.77027027027027029</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>264</v>
+        <v>436</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
@@ -4261,28 +4279,28 @@
       </c>
       <c r="H9" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.7567567567567568</v>
+        <v>0.78378378378378377</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B10" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
@@ -4290,57 +4308,57 @@
       </c>
       <c r="H10" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.77027027027027029</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.79729729729729726</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>67</v>
+        <v>171</v>
       </c>
       <c r="B11" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>69</v>
+        <v>416</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>275</v>
+        <v>433</v>
       </c>
       <c r="E11" s="23" t="s">
+        <v>265</v>
+      </c>
+      <c r="F11" s="24" t="s">
         <v>264</v>
-      </c>
-      <c r="F11" s="24" t="s">
-        <v>265</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H11" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.78378378378378377</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.82432432432432434</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>201</v>
+        <v>32</v>
       </c>
       <c r="B12" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>204</v>
+        <v>35</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="E12" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="F12" s="24" t="s">
         <v>264</v>
-      </c>
-      <c r="F12" s="24" t="s">
-        <v>277</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4348,57 +4366,57 @@
       </c>
       <c r="H12" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>0.79729729729729726</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.83783783783783783</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>176</v>
+        <v>53</v>
       </c>
       <c r="B13" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>179</v>
+        <v>55</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>279</v>
+        <v>437</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>277</v>
+        <v>264</v>
       </c>
       <c r="G13" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H13" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G13))/Resumen!$C$8</f>
-        <v>0.82432432432432434</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.85135135135135132</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="B14" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="E14" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="F14" s="24" t="s">
         <v>264</v>
-      </c>
-      <c r="F14" s="24" t="s">
-        <v>277</v>
       </c>
       <c r="G14" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
@@ -4406,28 +4424,28 @@
       </c>
       <c r="H14" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G14))/Resumen!$C$8</f>
-        <v>0.83783783783783783</v>
+        <v>0.86486486486486491</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>54</v>
+        <v>205</v>
       </c>
       <c r="B15" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>56</v>
+        <v>208</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="E15" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="F15" s="24" t="s">
         <v>264</v>
-      </c>
-      <c r="F15" s="24" t="s">
-        <v>277</v>
       </c>
       <c r="G15" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
@@ -4435,28 +4453,28 @@
       </c>
       <c r="H15" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G15))/Resumen!$C$8</f>
-        <v>0.85135135135135132</v>
+        <v>0.8783783783783784</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>80</v>
+        <v>222</v>
       </c>
       <c r="B16" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>83</v>
+        <v>434</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>282</v>
+        <v>435</v>
       </c>
       <c r="E16" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="F16" s="24" t="s">
         <v>264</v>
-      </c>
-      <c r="F16" s="24" t="s">
-        <v>277</v>
       </c>
       <c r="G16" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
@@ -4464,86 +4482,86 @@
       </c>
       <c r="H16" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G16))/Resumen!$C$8</f>
-        <v>0.86486486486486491</v>
+        <v>0.89189189189189189</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>213</v>
+        <v>99</v>
       </c>
       <c r="B17" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>216</v>
+        <v>102</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
       <c r="E17" s="23" t="s">
+        <v>254</v>
+      </c>
+      <c r="F17" s="24" t="s">
         <v>264</v>
-      </c>
-      <c r="F17" s="24" t="s">
-        <v>277</v>
       </c>
       <c r="G17" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H17" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G17))/Resumen!$C$8</f>
-        <v>0.8783783783783784</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
+        <v>0.91891891891891897</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>230</v>
+        <v>176</v>
       </c>
       <c r="B18" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>232</v>
+        <v>179</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
       <c r="E18" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="F18" s="24" t="s">
         <v>264</v>
-      </c>
-      <c r="F18" s="24" t="s">
-        <v>277</v>
       </c>
       <c r="G18" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H18" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G18))/Resumen!$C$8</f>
-        <v>0.89189189189189189</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B19" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="G19" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
@@ -4551,28 +4569,28 @@
       </c>
       <c r="H19" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G19))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.97297297297297303</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>182</v>
+        <v>92</v>
       </c>
       <c r="B20" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>185</v>
+        <v>95</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="G20" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
@@ -4580,74 +4598,16 @@
       </c>
       <c r="H20" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G20))/Resumen!$C$8</f>
-        <v>0.94594594594594594</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
-        <v>107</v>
-      </c>
-      <c r="B21" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A21,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A21,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C21" s="23" t="s">
-        <v>109</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>287</v>
-      </c>
-      <c r="E21" s="23" t="s">
-        <v>264</v>
-      </c>
-      <c r="F21" s="24" t="s">
-        <v>288</v>
-      </c>
-      <c r="G21" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A21,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A21,RNF!$A$2:$A$100,0)))</f>
         <v>1</v>
       </c>
-      <c r="H21" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G21))/Resumen!$C$8</f>
-        <v>0.97297297297297303</v>
-      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="B22" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A22,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A22,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C22" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>289</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>264</v>
-      </c>
-      <c r="F22" s="24" t="s">
-        <v>288</v>
-      </c>
-      <c r="G22" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A22,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A22,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
-      </c>
-      <c r="H22" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G22))/Resumen!$C$8</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A24" s="17" t="s">
-        <v>290</v>
+      <c r="A22" s="17" t="s">
+        <v>439</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B22">
+  <conditionalFormatting sqref="B2:B20">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Implementado"</formula>
     </cfRule>
@@ -4679,7 +4639,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H2:H22</xm:sqref>
+          <xm:sqref>H2:H20</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4703,1180 +4663,1180 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>291</v>
+        <v>275</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>292</v>
+        <v>276</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>294</v>
+        <v>278</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>296</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>297</v>
+        <v>281</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>298</v>
+        <v>282</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>299</v>
+        <v>283</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>303</v>
+        <v>287</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>304</v>
+        <v>288</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>305</v>
+        <v>289</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>306</v>
+        <v>290</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>307</v>
+        <v>291</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>308</v>
+        <v>292</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>310</v>
+        <v>294</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>311</v>
+        <v>295</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>312</v>
+        <v>296</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>313</v>
+        <v>297</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>314</v>
+        <v>298</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>315</v>
+        <v>299</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>316</v>
+        <v>300</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>317</v>
+        <v>301</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>318</v>
+        <v>302</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>319</v>
+        <v>303</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>320</v>
+        <v>304</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>321</v>
+        <v>305</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>322</v>
+        <v>306</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>323</v>
+        <v>307</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>324</v>
+        <v>308</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>325</v>
+        <v>309</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>326</v>
+        <v>310</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>327</v>
+        <v>311</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>328</v>
+        <v>312</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>330</v>
+        <v>314</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>331</v>
+        <v>315</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>332</v>
+        <v>316</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>333</v>
+        <v>317</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>334</v>
+        <v>318</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>336</v>
+        <v>320</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>338</v>
+        <v>322</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>339</v>
+        <v>323</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>340</v>
+        <v>324</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>341</v>
+        <v>325</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>342</v>
+        <v>326</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>343</v>
+        <v>327</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>322</v>
+        <v>306</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>344</v>
+        <v>328</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>345</v>
+        <v>329</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>347</v>
+        <v>331</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>348</v>
+        <v>332</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>349</v>
+        <v>333</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>350</v>
+        <v>334</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>329</v>
+        <v>417</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>351</v>
+        <v>418</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>352</v>
-      </c>
-      <c r="F20" s="23" t="s">
-        <v>300</v>
+        <v>419</v>
+      </c>
+      <c r="F20" s="27" t="s">
+        <v>440</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>353</v>
+        <v>335</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>354</v>
+        <v>336</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>355</v>
+        <v>337</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>356</v>
+        <v>338</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>357</v>
+        <v>339</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>358</v>
+        <v>340</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>359</v>
+        <v>341</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>360</v>
+        <v>342</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>361</v>
+        <v>343</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>362</v>
+        <v>344</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>363</v>
+        <v>345</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>364</v>
+        <v>346</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>365</v>
+        <v>347</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>366</v>
+        <v>348</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>367</v>
+        <v>349</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>370</v>
+        <v>352</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>371</v>
+        <v>353</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>372</v>
+        <v>354</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>373</v>
+        <v>355</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>374</v>
+        <v>356</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>375</v>
+        <v>357</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>376</v>
+        <v>358</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>377</v>
+        <v>359</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>378</v>
+        <v>360</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>379</v>
+        <v>361</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>380</v>
+        <v>362</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>381</v>
+        <v>363</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>382</v>
+        <v>364</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>383</v>
+        <v>365</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>384</v>
+        <v>366</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>385</v>
+        <v>367</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>386</v>
+        <v>368</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>387</v>
+        <v>420</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>388</v>
-      </c>
-      <c r="F33" s="23" t="s">
-        <v>300</v>
+        <v>421</v>
+      </c>
+      <c r="F33" s="27" t="s">
+        <v>440</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>389</v>
+        <v>369</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>390</v>
+        <v>370</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>391</v>
+        <v>422</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>392</v>
-      </c>
-      <c r="F34" s="23" t="s">
-        <v>300</v>
+        <v>423</v>
+      </c>
+      <c r="F34" s="27" t="s">
+        <v>440</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>393</v>
+        <v>371</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>394</v>
+        <v>372</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>395</v>
+        <v>373</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>396</v>
+        <v>374</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>397</v>
+        <v>375</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>398</v>
+        <v>376</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>399</v>
+        <v>377</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>400</v>
+        <v>378</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>401</v>
+        <v>379</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>402</v>
+        <v>380</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>403</v>
+        <v>424</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>404</v>
-      </c>
-      <c r="F39" s="23" t="s">
-        <v>300</v>
+        <v>425</v>
+      </c>
+      <c r="F39" s="27" t="s">
+        <v>440</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>405</v>
+        <v>381</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>309</v>
+        <v>426</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>406</v>
+        <v>427</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>407</v>
-      </c>
-      <c r="F40" s="23" t="s">
-        <v>300</v>
+        <v>428</v>
+      </c>
+      <c r="F40" s="27" t="s">
+        <v>440</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>408</v>
+        <v>382</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>409</v>
+        <v>383</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>410</v>
+        <v>384</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>411</v>
+        <v>385</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>412</v>
+        <v>386</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>413</v>
+        <v>387</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>414</v>
+        <v>388</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>415</v>
+        <v>389</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>416</v>
+        <v>390</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>417</v>
+        <v>391</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>418</v>
+        <v>392</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>419</v>
+        <v>393</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>420</v>
+        <v>394</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>421</v>
+        <v>395</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>423</v>
-      </c>
-      <c r="F46" s="23" t="s">
-        <v>300</v>
+        <v>430</v>
+      </c>
+      <c r="F46" s="27" t="s">
+        <v>440</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>424</v>
+        <v>396</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>425</v>
+        <v>397</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>426</v>
+        <v>398</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>427</v>
+        <v>399</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>428</v>
+        <v>400</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>429</v>
+        <v>401</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>430</v>
+        <v>402</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>431</v>
+        <v>403</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>432</v>
+        <v>404</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>433</v>
+        <v>405</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>434</v>
+        <v>406</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>435</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): observaciones de RQF-04 (check-in congelado) y RQF-09 (columnas por confirmar)
- RQF-04: el check-in de una membresia congelada queda pendiente del
  cambio de Santiago (estado CONGELADO, decision de Luis); no pasa a
  Implementado hasta que esten fusionados el PR #17 y ese cambio.
- RQF-09: sin cambio de estado; falta confirmar en la copia de produccion
  si envio_mensaje tiene canal y notificacion tiene leido.
- estado.md anota los secretos quitados de COMO_CORRER.md y que hay que
  rotarlos.
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6E09B9-5837-448A-8214-DDF52AE5FF3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188FFDD2-7E40-4CCF-86D3-76E34894F530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="442">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -209,9 +209,6 @@
     <t>Cálculo automático de fecha_fin según el plan (miembros.js:185, :382); estado vencido / por vencer contra la fecha actual (miembros.js:276-284); renovación del plan (miembros.js:754).</t>
   </si>
   <si>
-    <t>Estado Congelada: la tabla congelacion_membresia existe (migración 002:217) pero ninguna ruta ni pantalla la usa.</t>
-  </si>
-  <si>
     <t>HU-11, HU-12, HU-13, HU-35..HU-40</t>
   </si>
   <si>
@@ -308,9 +305,6 @@
     <t>Botón de WhatsApp con el mensaje armado para miembros en riesgo (MenuNotificaciones.jsx:86-90, MiembrosPage.jsx:796-802); POST /api/admin/notificaciones/enviado guarda canal, estado ENVIADO y fecha en envio_mensaje (notificaciones.js:188-224).</t>
   </si>
   <si>
-    <t>Observación: solo WhatsApp por enlace wa.me; el estado no confirma la entrega y el correo no se usa para retención.</t>
-  </si>
-  <si>
     <t>HU-19, HU-20, HU-52</t>
   </si>
   <si>
@@ -845,9 +839,6 @@
     <t>Editar y desactivar cuentas del personal</t>
   </si>
   <si>
-    <t>Congelar y descongelar membresías</t>
-  </si>
-  <si>
     <t>Motor diario con Alerta Amarilla / Roja y umbrales editables</t>
   </si>
   <si>
@@ -1355,9 +1346,6 @@
     <t>Luis (PR #16)</t>
   </si>
   <si>
-    <t>Luis (PR #17)</t>
-  </si>
-  <si>
     <t>Estado actualizado el 2026-10-18 con los PR fusionados en develop @ 1ddcb24 (#9, #11, #14 y #15); la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
   </si>
   <si>
@@ -1365,6 +1353,21 @@
   </si>
   <si>
     <t>2026-10-18</t>
+  </si>
+  <si>
+    <t>Estado Congelada: la tabla congelacion_membresia existe (migración 002:217) pero ninguna ruta ni pantalla la usa. En revisión: el PR #17 (sin fusionar) agrega congelar y descongelar sobre plan_cobro (migración 010). El check-in de una membresía congelada está pendiente de un cambio de Santiago en checkin.js y CheckinPage.jsx: por decisión de Luis (2026-10-18) no entra, con estado CONGELADO y el mensaje «Tu membresía está congelada. Pide en recepción que la reactiven para poder ingresar.». RQF-04 no pasa a Implementado hasta que los dos cambios estén fusionados y verificados.</t>
+  </si>
+  <si>
+    <t>Observación: solo WhatsApp por enlace wa.me; el estado no confirma la entrega y el correo no se usa para retención. Pendiente de confirmar en la copia de producción si envio_mensaje tiene la columna canal y notificacion la columna leido (verificador: 94d5fbb, sección 15). Si no las tiene, POST /api/admin/notificaciones/enviado falla siempre (el frontend oculta el error, MiembrosPage.jsx:802-808) y RQF-09 baja a Parcial. Santiago lo consulta.</t>
+  </si>
+  <si>
+    <t>Estado Congelada: congelar y descongelar en revisión en el PR #17; falta que el check-in rechace una membresía congelada (estado CONGELADO, cambio de Santiago en checkin.js y CheckinPage.jsx).</t>
+  </si>
+  <si>
+    <t>Congelar y descongelar membresías (PR #17) y check-in con estado CONGELADO</t>
+  </si>
+  <si>
+    <t>Luis (PR #17) y Santiago (check-in)</t>
   </si>
 </sst>
 </file>
@@ -2331,7 +2334,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2788,7 +2791,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>53</v>
       </c>
@@ -2802,7 +2805,7 @@
         <v>54</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>55</v>
+        <v>437</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2812,30 +2815,30 @@
         <v>36</v>
       </c>
       <c r="H5" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="J5" s="23" t="s">
         <v>57</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>59</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>60</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6" s="23" t="s">
         <v>61</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>62</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2845,30 +2848,30 @@
         <v>36</v>
       </c>
       <c r="H6" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="I6" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="J6" s="23" t="s">
         <v>64</v>
-      </c>
-      <c r="J6" s="23" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>67</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>68</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2878,30 +2881,30 @@
         <v>36</v>
       </c>
       <c r="H7" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="I7" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="J7" s="23" t="s">
         <v>70</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="23" t="s">
         <v>72</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>73</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="E8" s="23" t="s">
         <v>74</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>75</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2911,30 +2914,30 @@
         <v>36</v>
       </c>
       <c r="H8" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="I8" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="J8" s="23" t="s">
         <v>77</v>
-      </c>
-      <c r="J8" s="23" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" s="23" t="s">
         <v>79</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>80</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>81</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>82</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2944,30 +2947,30 @@
         <v>36</v>
       </c>
       <c r="H9" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="I9" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="J9" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="J9" s="23" t="s">
+    </row>
+    <row r="10" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="22" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
-        <v>86</v>
-      </c>
       <c r="B10" s="23" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>88</v>
+        <v>438</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2977,30 +2980,30 @@
         <v>36</v>
       </c>
       <c r="H10" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="J10" s="23" t="s">
         <v>89</v>
-      </c>
-      <c r="I10" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3010,30 +3013,30 @@
         <v>36</v>
       </c>
       <c r="H11" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="J11" s="23" t="s">
         <v>96</v>
-      </c>
-      <c r="I11" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3043,30 +3046,30 @@
         <v>36</v>
       </c>
       <c r="H12" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="J12" s="23" t="s">
         <v>103</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3076,51 +3079,51 @@
         <v>36</v>
       </c>
       <c r="H13" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="J13" s="23" t="s">
         <v>109</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>110</v>
-      </c>
-      <c r="J13" s="23" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="I14" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="J14" s="23" t="s">
         <v>115</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>116</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>47</v>
@@ -3129,97 +3132,97 @@
         <v>14</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H15" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="J15" s="23" t="s">
         <v>121</v>
-      </c>
-      <c r="I15" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="J15" s="23" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H16" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="J16" s="23" t="s">
         <v>128</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>129</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H17" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="J17" s="23" t="s">
         <v>135</v>
-      </c>
-      <c r="I17" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="J17" s="23" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>33</v>
@@ -3228,64 +3231,64 @@
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H18" s="23" t="s">
+        <v>139</v>
+      </c>
+      <c r="I18" s="23" t="s">
+        <v>140</v>
+      </c>
+      <c r="J18" s="23" t="s">
         <v>141</v>
-      </c>
-      <c r="I18" s="23" t="s">
-        <v>142</v>
-      </c>
-      <c r="J18" s="23" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F19" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C19,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H19" s="23" t="s">
+        <v>144</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="J19" s="23" t="s">
         <v>146</v>
-      </c>
-      <c r="I19" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="J19" s="23" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>33</v>
@@ -3294,64 +3297,64 @@
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F20" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C20,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H21" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="I21" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="J21" s="23" t="s">
         <v>157</v>
-      </c>
-      <c r="I21" s="23" t="s">
-        <v>158</v>
-      </c>
-      <c r="J21" s="23" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>47</v>
@@ -3360,59 +3363,59 @@
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H22" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="I22" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="J22" s="23" t="s">
         <v>163</v>
-      </c>
-      <c r="I22" s="23" t="s">
-        <v>164</v>
-      </c>
-      <c r="J22" s="23" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H23" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="J23" s="23" t="s">
         <v>168</v>
-      </c>
-      <c r="I23" s="23" t="s">
-        <v>169</v>
-      </c>
-      <c r="J23" s="23" t="s">
-        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -3491,19 +3494,19 @@
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3513,30 +3516,30 @@
         <v>36</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3546,30 +3549,30 @@
         <v>36</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3579,30 +3582,30 @@
         <v>36</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3612,30 +3615,30 @@
         <v>36</v>
       </c>
       <c r="H5" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="I5" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="J5" s="23" t="s">
         <v>192</v>
-      </c>
-      <c r="I5" s="23" t="s">
-        <v>193</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3645,30 +3648,30 @@
         <v>36</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3678,30 +3681,30 @@
         <v>36</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3711,30 +3714,30 @@
         <v>36</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3744,244 +3747,244 @@
         <v>36</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -4035,40 +4038,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>250</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D2" s="23" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>252</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>253</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>254</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>255</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4081,23 +4084,23 @@
     </row>
     <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4110,23 +4113,23 @@
     </row>
     <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4139,23 +4142,23 @@
     </row>
     <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4168,23 +4171,23 @@
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4197,23 +4200,23 @@
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4236,13 +4239,13 @@
         <v>42</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4255,23 +4258,23 @@
     </row>
     <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
@@ -4284,23 +4287,23 @@
     </row>
     <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B10" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
@@ -4313,23 +4316,23 @@
     </row>
     <row r="11" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B11" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
@@ -4352,13 +4355,13 @@
         <v>35</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4369,7 +4372,7 @@
         <v>0.83783783783783783</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
         <v>53</v>
       </c>
@@ -4378,16 +4381,16 @@
         <v>Parcial</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>55</v>
+        <v>439</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>267</v>
+        <v>440</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G13" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
@@ -4400,23 +4403,23 @@
     </row>
     <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B14" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G14" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
@@ -4429,23 +4432,23 @@
     </row>
     <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B15" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G15" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
@@ -4458,23 +4461,23 @@
     </row>
     <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B16" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G16" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
@@ -4487,23 +4490,23 @@
     </row>
     <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B17" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G17" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
@@ -4516,23 +4519,23 @@
     </row>
     <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B18" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G18" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
@@ -4545,23 +4548,23 @@
     </row>
     <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B19" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G19" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
@@ -4574,23 +4577,23 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B20" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="F20" s="24" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G20" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
@@ -4603,7 +4606,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="17" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
     </row>
   </sheetData>
@@ -4663,30 +4666,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>277</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4695,21 +4698,21 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
+        <v>279</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>280</v>
+      </c>
+      <c r="F2" s="23" t="s">
+        <v>281</v>
+      </c>
+      <c r="G2" s="23" t="s">
         <v>282</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>283</v>
-      </c>
-      <c r="F2" s="23" t="s">
-        <v>284</v>
-      </c>
-      <c r="G2" s="23" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
@@ -4718,21 +4721,21 @@
         <v>23</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>40</v>
@@ -4741,44 +4744,44 @@
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>40</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>46</v>
@@ -4787,21 +4790,21 @@
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>46</v>
@@ -4810,21 +4813,21 @@
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>53</v>
@@ -4833,1010 +4836,1010 @@
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="F8" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>53</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C10" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
+        <v>309</v>
+      </c>
+      <c r="B11" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>310</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>311</v>
+      </c>
+      <c r="E11" s="23" t="s">
         <v>312</v>
       </c>
-      <c r="B11" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>313</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>314</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>315</v>
-      </c>
       <c r="F11" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C14" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C15" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C19" s="23" t="s">
+        <v>327</v>
+      </c>
+      <c r="D19" s="23" t="s">
         <v>330</v>
       </c>
-      <c r="D19" s="23" t="s">
-        <v>333</v>
-      </c>
       <c r="E19" s="23" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
+        <v>341</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>342</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>343</v>
+      </c>
+      <c r="E24" s="23" t="s">
         <v>344</v>
       </c>
-      <c r="B24" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>345</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>346</v>
-      </c>
-      <c r="E24" s="23" t="s">
-        <v>347</v>
-      </c>
       <c r="F24" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C36" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
+        <v>382</v>
+      </c>
+      <c r="B42" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="C42" s="23" t="s">
+        <v>383</v>
+      </c>
+      <c r="D42" s="23" t="s">
+        <v>384</v>
+      </c>
+      <c r="E42" s="23" t="s">
         <v>385</v>
       </c>
-      <c r="B42" s="23" t="s">
-        <v>205</v>
-      </c>
-      <c r="C42" s="23" t="s">
-        <v>386</v>
-      </c>
-      <c r="D42" s="23" t="s">
-        <v>387</v>
-      </c>
-      <c r="E42" s="23" t="s">
-        <v>388</v>
-      </c>
       <c r="F42" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): RQF-07 Implementado y evidencia del #17 y el #21 en el Excel (67,6 %)
- RQF-07 Implementado con el PR #16 (verificador 1be53f7, sec. 19 y 21.1).
- RQF-04 sigue Parcial con el #17 fusionado: faltan el job de vencimientos
  y el check-in que salten las congeladas (decision de Luis).
- RQF-22: solo el dueno, con su contrasena (PR #21); falta el limite de
  intentos en DELETE /api/auth/account. Sin la frase de la facturacion.
- RQF-14 anota que el job no salta las congeladas.
- Responsables: RQF-02 Luis (PR #18), RQF-01 Luis (PR #19), RQF-04 Santiago.

Editado con Excel por COM. Avance: 25 de 37 = 67,6 % (RF 70,5 %, RNF 63,3 %).
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188FFDD2-7E40-4CCF-86D3-76E34894F530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A94D9E-0220-4960-A9E0-2FC2D458BDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="442">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -206,9 +206,6 @@
     <t>RQF-04</t>
   </si>
   <si>
-    <t>Cálculo automático de fecha_fin según el plan (miembros.js:185, :382); estado vencido / por vencer contra la fecha actual (miembros.js:276-284); renovación del plan (miembros.js:754).</t>
-  </si>
-  <si>
     <t>HU-11, HU-12, HU-13, HU-35..HU-40</t>
   </si>
   <si>
@@ -263,12 +260,6 @@
     <t>Dashboard</t>
   </si>
   <si>
-    <t>GET /api/admin/dashboard: miembros activos (dashboard.js:123, :146), entradas de hoy (:128) y próximos vencimientos a 30 días (:204); listado en DashboardPage.jsx:446-473.</t>
-  </si>
-  <si>
-    <t>Gráfica de horas pico (la gráfica agrupa por día de la semana, dashboard.js:189) y actualización automática (el panel se carga una sola vez, DashboardPage.jsx:165-179).</t>
-  </si>
-  <si>
     <t>HU-16, HU-34, HU-41, HU-42, HU-43</t>
   </si>
   <si>
@@ -824,9 +815,6 @@
     <t>Cierre de sesión por inactividad en el frontend y expiración real del JWT</t>
   </si>
   <si>
-    <t>Gráfica de horas pico y refresco automático del dashboard</t>
-  </si>
-  <si>
     <t>Registrar el acceso bloqueado y mostrarlo en la campana del administrador</t>
   </si>
   <si>
@@ -944,9 +932,6 @@
     <t>EV-07</t>
   </si>
   <si>
-    <t>backend/src/routes/miembros.js:185, :382, :276-284, :754</t>
-  </si>
-  <si>
     <t>Fecha de vencimiento automática, estado vencido / por vencer y renovación.</t>
   </si>
   <si>
@@ -956,12 +941,6 @@
     <t>Esquema</t>
   </si>
   <si>
-    <t>backend/migrations/002_esquema_inicial.sql:217</t>
-  </si>
-  <si>
-    <t>congelacion_membresia existe pero no se usa (falta Congelada).</t>
-  </si>
-  <si>
     <t>EV-09</t>
   </si>
   <si>
@@ -989,12 +968,6 @@
     <t>Bloqueo de membresía vencida; no hay aviso del intento al administrador.</t>
   </si>
   <si>
-    <t>backend/src/routes/dashboard.js:123, :128, :146, :189, :204; frontend/src/pages/DashboardPage.jsx:165-179, :446-473</t>
-  </si>
-  <si>
-    <t>KPIs del día y próximos vencimientos; gráfica por día de semana; carga única.</t>
-  </si>
-  <si>
     <t>EV-13</t>
   </si>
   <si>
@@ -1265,12 +1238,6 @@
     <t>Sigue Parcial (criterio del 2026-10-18): el aviso al administrador y el registro de cada intento ya son correctos, pero tras cada reinicio del servidor el contrato no sale. admin-contrato.js:107 pregunta isWhatsAppReady() antes de enviar y el cliente se inicia de forma perezosa (whatsapp.js:146), así que responde «no autenticado» sin llegar a iniciar el cliente ni a mostrar el QR que pide escanear; solo funciona si otro flujo lo inició antes (alta de un miembro con teléfono). Arreglo: quitar esa comprobación previa (sendWhatsAppText ya lanza el error) o iniciar el cliente antes, junto con la corrección del PR #10. Verificador: 386d168, sección 14.3.</t>
   </si>
   <si>
-    <t>DELETE /api/auth/account (auth.js:548), solo para el administrador (403 en :554). Borra en una transacción los 29 pasos de PASOS_ELIMINAR_CUENTA (:493) con un SAVEPOINT por paso (borrarPaso, :534), que solo omite una tabla o columna inexistente (42P01 y 42703, :527); el gimnasio se borra al final (:567), responde 404 si ya no existe (:570) y el rastro queda en el log del servidor (:575). Ya no inserta en auditoria. PR #15.</t>
-  </si>
-  <si>
-    <t>Probado por el verificador con el handler real sobre PostgreSQL 18 (94d5fbb, sección 16): en las bases Docker, Docker + 009 y tipo producción responde 200, no deja filas del gimnasio y no toca las de otro; si una FK desconocida lo bloquea, responde 500 y no borra nada. Riesgo anotado: cualquier usuario con rol admin, también un administrador invitado, puede eliminar el gimnasio sin volver a escribir su contraseña; conviene pedirla. EliminarCuentaPage.jsx:46 todavía promete cancelar la facturación, y el sistema no cobra.</t>
-  </si>
-  <si>
     <t>Cada gimnasio nuevo se crea por registro, sin tocar código (auth.js:100, :134); las consultas filtran por el id_gimnasio del token (p. ej. miembros.js:358, checkin.js:76, dashboard.js:123, notificaciones.js:199). Desde el PR #11: vista.js exige rol de personal (:20), rechaza al personal sin gimnasio (:28) y filtra por gimnasio (:32, :46) sobre la vista de la migración 011; asistencia.js exige rol de personal (:22); checkin.js deriva la clave del QR una sola vez (:26, :31). 9 pruebas en backend/tests/aislamiento.test.js.</t>
   </si>
   <si>
@@ -1295,18 +1262,6 @@
     <t>Envío del contrato con registro de cada intento; el error del envío ya llega al registro (exito = false). Tras un reinicio no se inicia el cliente (admin-contrato.js:107).</t>
   </si>
   <si>
-    <t>backend/src/routes/auth.js:493, :527, :534, :548-585 (403 en :554, gimnasio en :567, 404 en :570); frontend/src/pages/EliminarCuentaPage.jsx</t>
-  </si>
-  <si>
-    <t>Eliminación de cuenta con un SAVEPOINT por paso, solo para el administrador y atómica (PR #15).</t>
-  </si>
-  <si>
-    <t>Informe del verificador, commit 94d5fbb, docs/verificacion-requisitos.md §16</t>
-  </si>
-  <si>
-    <t>Con el handler real en PostgreSQL 18 y tres esquemas: 200, sin filas del gimnasio y sin tocar el otro; 500 sin borrar nada si una FK desconocida lo bloquea.</t>
-  </si>
-  <si>
     <t>backend/src/routes/auth.js:100, :134; vista.js:20, :28, :32, :46; asistencia.js:22; checkin.js:26, :31, :76; miembros.js:358; dashboard.js:123; notificaciones.js:199</t>
   </si>
   <si>
@@ -1343,31 +1298,76 @@
     <t>Migración que reconcilie envio_mensaje y notificacion con producción (o cambio del código), probada contra la copia de producción</t>
   </si>
   <si>
-    <t>Luis (PR #16)</t>
-  </si>
-  <si>
-    <t>Estado actualizado el 2026-10-18 con los PR fusionados en develop @ 1ddcb24 (#9, #11, #14 y #15); la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
-  </si>
-  <si>
     <t>Orden de menor a mayor esfuerzo. «Avance global acumulado» suma los puntos de cada acción, en orden, sobre el avance actual y se pone verde al llegar a la meta. Lo decide Luis; el reparto de tareas está en docs/plan-trabajo.md.</t>
   </si>
   <si>
     <t>2026-10-18</t>
   </si>
   <si>
-    <t>Estado Congelada: la tabla congelacion_membresia existe (migración 002:217) pero ninguna ruta ni pantalla la usa. En revisión: el PR #17 (sin fusionar) agrega congelar y descongelar sobre plan_cobro (migración 010). El check-in de una membresía congelada está pendiente de un cambio de Santiago en checkin.js y CheckinPage.jsx: por decisión de Luis (2026-10-18) no entra, con estado CONGELADO y el mensaje «Tu membresía está congelada. Pide en recepción que la reactiven para poder ingresar.». RQF-04 no pasa a Implementado hasta que los dos cambios estén fusionados y verificados.</t>
-  </si>
-  <si>
     <t>Observación: solo WhatsApp por enlace wa.me; el estado no confirma la entrega y el correo no se usa para retención. Pendiente de confirmar en la copia de producción si envio_mensaje tiene la columna canal y notificacion la columna leido (verificador: 94d5fbb, sección 15). Si no las tiene, POST /api/admin/notificaciones/enviado falla siempre (el frontend oculta el error, MiembrosPage.jsx:802-808) y RQF-09 baja a Parcial. Santiago lo consulta.</t>
   </si>
   <si>
-    <t>Estado Congelada: congelar y descongelar en revisión en el PR #17; falta que el check-in rechace una membresía congelada (estado CONGELADO, cambio de Santiago en checkin.js y CheckinPage.jsx).</t>
-  </si>
-  <si>
-    <t>Congelar y descongelar membresías (PR #17) y check-in con estado CONGELADO</t>
-  </si>
-  <si>
-    <t>Luis (PR #17) y Santiago (check-in)</t>
+    <t>GET /api/admin/dashboard: miembros activos (dashboard.js:150, :174), entradas de hoy con el día cortado en hora de Colombia (:155; ayudantes enHoraLocal e inicioLocal en :69 y :74), semana desde el lunes de Colombia (:217) y próximos vencimientos a 30 días (:232). GET /api/admin/dashboard/horas-pico (:327; periodos en :320 y hora local en :339): entradas por hora y hora pico. DashboardPage.jsx: gráfica BarsHoras (:172), que abre en «Hoy» (:226); refresco cada 60 s con la pestaña visible y al volver a ella (REFRESCO_MS :49, :279-288), sin cargas en paralelo (:239-246); listado de próximos vencimientos (:610-626). PR #16.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-18; verificador 1be53f7, secciones 19 y 21.1): se cumplen las cuatro partes del texto y el día se corta en hora de Colombia. Observaciones: las comparaciones con columnas DATE (próximas a vencer y vencen en 7 días) siguen con CURRENT_DATE en UTC, así que de 19:00 a 24:00 en Colombia hay un día de desfase; y vencen7 y proximos todavía cuentan las membresías congeladas (va en un PR aparte).</t>
+  </si>
+  <si>
+    <t>Cálculo automático de fecha_fin según el plan (miembros.js:193, :395); estado vencido / por vencer contra la fecha actual (:286-290); renovación del plan (:926). Estado Congelada (PR #17, migración 010): POST /api/admin/miembros/:id/congelar (:810) y /descongelar (:869), que corre fecha_fin y la próxima fecha de cobro los días congelados (:892), con historial en congelacion_plan; la lista marca la membresía congelada y no la cuenta como vencida (:286); pantalla en MiembrosPage.jsx:238, :742, :1907.</t>
+  </si>
+  <si>
+    <t>Sigue Parcial (decisión de Luis, 2026-10-18): congelar y descongelar ya están en develop (PR #17; verificador 1be53f7, sección 18.2), pero falta que Santiago haga que el job de avisos de vencimiento (expiracion.js) y el check-in salten las membresías congeladas. El check-in debe negar el ingreso con estado CONGELADO y el mensaje «Tu membresía está congelada. Pide en recepción que la reactiven para poder ingresar.». Hoy el job le mandaría a un miembro congelado el aviso de que su plan vence, y el check-in lo deja entrar. Pasa a Implementado cuando esos dos cambios estén fusionados y verificados. Menores: congelar entre las 19:00 y las 24:00 de Colombia toma la fecha del día siguiente (CURRENT_DATE en UTC), y renovar el plan mientras está congelado conserva congelado_desde.</t>
+  </si>
+  <si>
+    <t>DELETE /api/auth/account (auth.js:558): solo el administrador (403 NOT_ADMIN en :565) y solo el dueño, que es el primer usuario del gimnasio (:575-590, 403 NOT_OWNER), confirmando con su contraseña (:493, :592-593, 403 WRONG_PASSWORD) antes de abrir la transacción (:598). Borra los pasos de PASOS_ELIMINAR_CUENTA (:503) con un SAVEPOINT por paso (borrarPaso, :544), que solo omite una tabla o columna inexistente (42P01 y 42703, :537); el gimnasio se borra al final (:605), responde 404 si ya no existe (:608) y el rastro queda en el log (:613). La página pide la contraseña (EliminarCuentaPage.jsx:12, :124-126). PR #15 y #21.</t>
+  </si>
+  <si>
+    <t>Solo el dueño, con su contraseña (PR #21). Probado por el verificador con el handler real sobre PostgreSQL 18 (94d5fbb, sección 16; 1be53f7, sección 21.2): responde 200 sin dejar filas del gimnasio ni tocar las de otro, 403 al administrador invitado y con la contraseña mala, y 500 sin borrar nada si una FK desconocida lo bloquea. Falta el límite de intentos en DELETE /api/auth/account: con un token robado del dueño se puede probar su contraseña sin freno. Es una línea en index.js (zona de Daniel), antes de la :81.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:193, :395, :286-290, :926</t>
+  </si>
+  <si>
+    <t>backend/migrations/010_congelar_membresia.sql; backend/src/routes/miembros.js:810, :869, :892; frontend/src/pages/MiembrosPage.jsx:238, :742, :1907</t>
+  </si>
+  <si>
+    <t>Congelar y descongelar con historial y corrimiento del vencimiento (PR #17). Falta que el job y el check-in salten las congeladas.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/dashboard.js:69, :74, :150, :155, :174, :217, :232, :320, :327, :339; frontend/src/pages/DashboardPage.jsx:49, :172, :226, :239-246, :279-288, :610-626</t>
+  </si>
+  <si>
+    <t>KPIs del día con el corte en hora de Colombia, gráfica de horas pico, próximos vencimientos y refresco automático cada 60 s (PR #16).</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:493, :503, :537, :544, :558-623 (NOT_ADMIN :565, NOT_OWNER :588, WRONG_PASSWORD :593, BEGIN :598); frontend/src/pages/EliminarCuentaPage.jsx:12, :124-126</t>
+  </si>
+  <si>
+    <t>Eliminación de cuenta solo por el dueño y con su contraseña, con un SAVEPOINT por paso y atómica (PR #15 y #21).</t>
+  </si>
+  <si>
+    <t>Informe del verificador: commit 94d5fbb, docs/verificacion-requisitos.md §16; commit 1be53f7, §21.2</t>
+  </si>
+  <si>
+    <t>Con el handler real en PostgreSQL 18: 200 sin filas del gimnasio y sin tocar el otro; 403 al admin invitado y con la contraseña mala; 500 sin borrar nada si una FK desconocida lo bloquea.</t>
+  </si>
+  <si>
+    <t>Que el job de vencimientos y el check-in salten las membresías congeladas (check-in con estado CONGELADO); congelar y descongelar ya están en develop (PR #17).</t>
+  </si>
+  <si>
+    <t>Job de vencimientos y check-in que salten las membresías congeladas (check-in con estado CONGELADO)</t>
+  </si>
+  <si>
+    <t>Luis (PR #18)</t>
+  </si>
+  <si>
+    <t>Luis (PR #19)</t>
+  </si>
+  <si>
+    <t>Si WhatsApp no está listo, sendWhatsAppText vuelve sin error (whatsapp.js:228-231) y el job marca el aviso como enviado (expiracion.js:206-207), así que nunca lo reintenta; en Render no hay Chrome (whatsapp.js:7-25). Los días de anticipación (gimnasio.dias_aviso_vencimiento) solo se cambian en la base de datos: PUT /admin/config no los acepta (config.js:20-30). Además, el job no salta las membresías congeladas (expiracion.js:43-65; verificador 1be53f7, sección 18.2): le avisaría a un miembro congelado que su plan vence.</t>
+  </si>
+  <si>
+    <t>Estado actualizado el 2026-10-18 con los PR fusionados en develop @ f3d323c (#9, #11, #14, #15, #16, #17 y #21); la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
   </si>
 </sst>
 </file>
@@ -1475,7 +1475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1544,6 +1544,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1746,13 +1749,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.68181818181818177</c:v>
+                  <c:v>0.70454545454545459</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.6333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.66216216216216217</c:v>
+                  <c:v>0.67567567567567566</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1916,10 +1919,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>18</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>6</c:v>
@@ -2334,7 +2337,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2379,11 +2382,11 @@
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
@@ -2391,7 +2394,7 @@
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.68181818181818177</v>
+        <v>0.70454545454545459</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2399,14 +2402,14 @@
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>2.6000000000000032</v>
+        <v>2.1000000000000014</v>
       </c>
       <c r="J6" t="s">
         <v>12</v>
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
@@ -2446,7 +2449,7 @@
       </c>
       <c r="K7">
         <f>E8</f>
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
@@ -2459,11 +2462,11 @@
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
@@ -2471,7 +2474,7 @@
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.66216216216216217</v>
+        <v>0.67567567567567566</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2479,7 +2482,7 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>5.1000000000000014</v>
+        <v>4.6000000000000014</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
@@ -2529,11 +2532,11 @@
       </c>
       <c r="D31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Implementado",RF!$G$2:$G$100,"Original")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Parcial",RF!$G$2:$G$100,"Original")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Pendiente",RF!$G$2:$G$100,"Original")</f>
@@ -2541,7 +2544,7 @@
       </c>
       <c r="G31" s="9">
         <f>IF(C31=0,0,SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")/C31)</f>
-        <v>0.5</v>
+        <v>0.54166666666666663</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
@@ -2579,11 +2582,11 @@
       </c>
       <c r="D33" s="13">
         <f>D31+D32</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E33" s="13">
         <f>E31+E32</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F33" s="13">
         <f>F31+F32</f>
@@ -2591,7 +2594,7 @@
       </c>
       <c r="G33" s="14">
         <f>IF(C33=0,0,(SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")+SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original"))/C33)</f>
-        <v>0.52500000000000002</v>
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
@@ -2791,7 +2794,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>53</v>
       </c>
@@ -2802,10 +2805,10 @@
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>54</v>
+        <v>423</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>437</v>
+        <v>424</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2815,30 +2818,30 @@
         <v>36</v>
       </c>
       <c r="H5" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="I5" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="J5" s="23" t="s">
         <v>56</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>58</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>59</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" s="23" t="s">
         <v>60</v>
-      </c>
-      <c r="E6" s="23" t="s">
-        <v>61</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2848,30 +2851,30 @@
         <v>36</v>
       </c>
       <c r="H6" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="I6" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="J6" s="23" t="s">
         <v>63</v>
-      </c>
-      <c r="J6" s="23" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>66</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>67</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2881,63 +2884,63 @@
         <v>36</v>
       </c>
       <c r="H7" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="I7" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="J7" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="J7" s="23" t="s">
+    </row>
+    <row r="8" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="22" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
+      <c r="B8" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="23" t="s">
-        <v>72</v>
-      </c>
       <c r="C8" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>73</v>
+        <v>421</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>74</v>
+        <v>422</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G8" s="24" t="s">
         <v>36</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2947,30 +2950,30 @@
         <v>36</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>438</v>
+        <v>420</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2980,30 +2983,30 @@
         <v>36</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3013,30 +3016,30 @@
         <v>36</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3046,30 +3049,30 @@
         <v>36</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3079,51 +3082,51 @@
         <v>36</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="J14" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="H14" s="23" t="s">
+    </row>
+    <row r="15" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="22" t="s">
         <v>113</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>116</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>47</v>
@@ -3132,97 +3135,97 @@
         <v>14</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>118</v>
+        <v>440</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I17" s="23" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>33</v>
@@ -3231,64 +3234,64 @@
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="I18" s="23" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F19" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C19,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I19" s="23" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>33</v>
@@ -3297,64 +3300,64 @@
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F20" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C20,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I21" s="23" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>47</v>
@@ -3363,59 +3366,59 @@
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H22" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="I22" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="J22" s="23" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A23" s="22" t="s">
         <v>161</v>
       </c>
-      <c r="I22" s="23" t="s">
+      <c r="B23" s="23" t="s">
         <v>162</v>
-      </c>
-      <c r="J22" s="23" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="B23" s="23" t="s">
-        <v>165</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>407</v>
+        <v>425</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>408</v>
+        <v>426</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -3494,19 +3497,19 @@
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>413</v>
+        <v>402</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3516,30 +3519,30 @@
         <v>36</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3549,30 +3552,30 @@
         <v>36</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3582,30 +3585,30 @@
         <v>36</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3615,30 +3618,30 @@
         <v>36</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>409</v>
+        <v>398</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3648,30 +3651,30 @@
         <v>36</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3681,30 +3684,30 @@
         <v>36</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3714,30 +3717,30 @@
         <v>36</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3747,244 +3750,244 @@
         <v>36</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>412</v>
+        <v>401</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -4014,7 +4017,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4038,40 +4041,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>247</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>249</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4079,28 +4082,28 @@
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.68918918918918914</v>
+        <v>0.70270270270270274</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>428</v>
+        <v>413</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>429</v>
+        <v>414</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4108,28 +4111,28 @@
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.70270270270270274</v>
+        <v>0.71621621621621623</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4137,28 +4140,28 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.71621621621621623</v>
+        <v>0.72972972972972971</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4166,28 +4169,28 @@
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.72972972972972971</v>
+        <v>0.7432432432432432</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4195,28 +4198,28 @@
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.7432432432432432</v>
+        <v>0.7567567567567568</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4224,7 +4227,7 @@
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.7567567567567568</v>
+        <v>0.77027027027027029</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
@@ -4239,13 +4242,13 @@
         <v>42</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>252</v>
+        <v>438</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4253,28 +4256,28 @@
       </c>
       <c r="H8" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.77027027027027029</v>
+        <v>0.78378378378378377</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>433</v>
+        <v>249</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
@@ -4282,86 +4285,86 @@
       </c>
       <c r="H9" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.78378378378378377</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.79729729729729726</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>65</v>
+        <v>166</v>
       </c>
       <c r="B10" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>67</v>
+        <v>402</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>261</v>
+        <v>415</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H10" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.79729729729729726</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.82432432432432434</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>169</v>
+        <v>32</v>
       </c>
       <c r="B11" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>413</v>
+        <v>35</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>430</v>
+        <v>260</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>263</v>
+        <v>439</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H11" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.82432432432432434</v>
+        <v>0.83783783783783783</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>32</v>
+        <v>53</v>
       </c>
       <c r="B12" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>35</v>
+        <v>436</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>264</v>
+        <v>437</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4369,28 +4372,28 @@
       </c>
       <c r="H12" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>0.83783783783783783</v>
+        <v>0.85135135135135132</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>53</v>
+        <v>75</v>
       </c>
       <c r="B13" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>439</v>
+        <v>78</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>440</v>
+        <v>261</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>441</v>
+        <v>249</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G13" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
@@ -4398,28 +4401,28 @@
       </c>
       <c r="H13" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G13))/Resumen!$C$8</f>
-        <v>0.85135135135135132</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.86486486486486491</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>78</v>
+        <v>200</v>
       </c>
       <c r="B14" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>81</v>
+        <v>203</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G14" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
@@ -4427,28 +4430,28 @@
       </c>
       <c r="H14" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G14))/Resumen!$C$8</f>
-        <v>0.86486486486486491</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.8783783783783784</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>203</v>
+        <v>217</v>
       </c>
       <c r="B15" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>206</v>
+        <v>416</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>266</v>
+        <v>417</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G15" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
@@ -4456,57 +4459,57 @@
       </c>
       <c r="H15" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G15))/Resumen!$C$8</f>
-        <v>0.8783783783783784</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.89189189189189189</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>220</v>
+        <v>94</v>
       </c>
       <c r="B16" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>431</v>
+        <v>97</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>432</v>
+        <v>263</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G16" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H16" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G16))/Resumen!$C$8</f>
-        <v>0.89189189189189189</v>
+        <v>0.91891891891891897</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>97</v>
+        <v>171</v>
       </c>
       <c r="B17" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>100</v>
+        <v>174</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="G17" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
@@ -4514,28 +4517,28 @@
       </c>
       <c r="H17" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G17))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>174</v>
+        <v>101</v>
       </c>
       <c r="B18" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>177</v>
+        <v>103</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="F18" s="24" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="G18" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
@@ -4543,28 +4546,28 @@
       </c>
       <c r="H18" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G18))/Resumen!$C$8</f>
-        <v>0.94594594594594594</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.97297297297297303</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="B19" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>106</v>
+        <v>90</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="G19" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
@@ -4572,45 +4575,16 @@
       </c>
       <c r="H19" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G19))/Resumen!$C$8</f>
-        <v>0.97297297297297303</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B20" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>271</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>252</v>
-      </c>
-      <c r="F20" s="24" t="s">
-        <v>270</v>
-      </c>
-      <c r="G20" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A20,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A20,RNF!$A$2:$A$100,0)))</f>
         <v>1</v>
       </c>
-      <c r="H20" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G20))/Resumen!$C$8</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A22" s="17" t="s">
-        <v>435</v>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="17" t="s">
+        <v>418</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B20">
+  <conditionalFormatting sqref="B2:B19">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Implementado"</formula>
     </cfRule>
@@ -4642,7 +4616,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H2:H20</xm:sqref>
+          <xm:sqref>H2:H19</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4666,30 +4640,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4698,21 +4672,21 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="F2" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
@@ -4721,21 +4695,21 @@
         <v>23</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="F3" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>40</v>
@@ -4744,44 +4718,44 @@
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="F4" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>40</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>46</v>
@@ -4790,21 +4764,21 @@
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>294</v>
+        <v>290</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>46</v>
@@ -4813,21 +4787,21 @@
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>53</v>
@@ -4836,21 +4810,21 @@
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>300</v>
+        <v>427</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>301</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>281</v>
+        <v>296</v>
+      </c>
+      <c r="F8" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>53</v>
@@ -4859,987 +4833,987 @@
         <v>303</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>304</v>
+        <v>428</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>305</v>
-      </c>
-      <c r="F9" s="23" t="s">
-        <v>281</v>
+        <v>429</v>
+      </c>
+      <c r="F9" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>315</v>
+        <v>430</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>316</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>281</v>
+        <v>431</v>
+      </c>
+      <c r="F13" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C14" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C15" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C16" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>415</v>
+        <v>404</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>416</v>
+        <v>405</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>349</v>
+        <v>340</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>350</v>
+        <v>341</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>351</v>
+        <v>342</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>352</v>
+        <v>343</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>353</v>
+        <v>344</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>354</v>
+        <v>345</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>355</v>
+        <v>346</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>357</v>
+        <v>348</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>358</v>
+        <v>349</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>359</v>
+        <v>350</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>360</v>
+        <v>351</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>362</v>
+        <v>353</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>363</v>
+        <v>354</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>364</v>
+        <v>355</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>365</v>
+        <v>356</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>417</v>
+        <v>432</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="D34" s="23" t="s">
+        <v>434</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>435</v>
+      </c>
+      <c r="F34" s="27" t="s">
         <v>419</v>
       </c>
-      <c r="E34" s="23" t="s">
-        <v>420</v>
-      </c>
-      <c r="F34" s="27" t="s">
-        <v>436</v>
-      </c>
       <c r="G34" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>369</v>
+        <v>360</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>370</v>
+        <v>361</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C36" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>371</v>
+        <v>362</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>372</v>
+        <v>363</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>373</v>
+        <v>364</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>374</v>
+        <v>365</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>375</v>
+        <v>366</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>376</v>
+        <v>367</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>377</v>
+        <v>368</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>421</v>
+        <v>406</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>378</v>
+        <v>369</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>423</v>
+        <v>408</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>424</v>
+        <v>409</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>425</v>
+        <v>410</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>348</v>
+        <v>339</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>426</v>
+        <v>411</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>427</v>
+        <v>412</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>436</v>
+        <v>419</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>401</v>
+        <v>392</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>402</v>
+        <v>393</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): RQF-01 y RQF-02 Implementados en el Excel (70,3 %)
- RQF-02 Implementado con el PR #18 (verificador b8f99d2, sec. 22 y 25.4);
  observaciones: CheckinPage no llama a marcarActividad, render.yaml 24h y
  docker-compose 7d.
- RQF-01 Implementado con el PR #19 (sec. 25); observacion: FK compuesta
  recomendada para gimnasio.id_dueno.
- RQF-07: sin la observacion de las congeladas (PR #22).
- RQF-22: el dueno es gimnasio.id_dueno (PR #19).
- RQF-01 y RQF-02 salen de la ruta.

Editado con Excel por COM. Avance: 26 de 37 = 70,3 % (RF 75,0 %, RNF 63,3 %).
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83A94D9E-0220-4960-A9E0-2FC2D458BDC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{692AE4A1-D0E1-4736-A0C2-7811DBB69D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="438">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -146,12 +146,6 @@
     <t>Gestión de Usuarios</t>
   </si>
   <si>
-    <t>Crear (por invitación), listar personal y revocar invitaciones: staff.js:109, :198, :227, :329; aceptar la invitación crea la cuenta: staff.js:384. Roles diferenciados: authorize('admin') en staff.js:112 y miembros.js:667 frente a authorize('admin', 'receptionist') en checkin.js:57.</t>
-  </si>
-  <si>
-    <t>Editar y eliminar o desactivar cuentas de personal existentes: no hay PUT/DELETE en /api/admin/staff ni acciones en StaffPage.jsx.</t>
-  </si>
-  <si>
     <t>Original</t>
   </si>
   <si>
@@ -167,12 +161,6 @@
     <t>RQF-02</t>
   </si>
   <si>
-    <t>POST /api/auth/login compara con bcrypt y emite JWT (auth.js:200, :231); cierre manual (auth.js:295, AuthContext.jsx:95); límite de 5 intentos por minuto (index.js:63, :79).</t>
-  </si>
-  <si>
-    <t>Cierre automático por inactividad (no existe en frontend ni backend). Hallazgo: el JWT del personal no expira, generarToken no aplica JWT_EXPIRES_IN (auth-helpers.js:102-113).</t>
-  </si>
-  <si>
     <t>HU-05, HU-06</t>
   </si>
   <si>
@@ -812,9 +800,6 @@
     <t>Lista de verificación con capturas en Chrome, Firefox y Edge</t>
   </si>
   <si>
-    <t>Cierre de sesión por inactividad en el frontend y expiración real del JWT</t>
-  </si>
-  <si>
     <t>Registrar el acceso bloqueado y mostrarlo en la campana del administrador</t>
   </si>
   <si>
@@ -824,9 +809,6 @@
     <t>Luis o Santiago</t>
   </si>
   <si>
-    <t>Editar y desactivar cuentas del personal</t>
-  </si>
-  <si>
     <t>Motor diario con Alerta Amarilla / Roja y umbrales editables</t>
   </si>
   <si>
@@ -869,12 +851,6 @@
     <t>EV-01</t>
   </si>
   <si>
-    <t>backend/src/routes/staff.js:109, :198, :227, :329, :384</t>
-  </si>
-  <si>
-    <t>Invitar, listar y revocar personal; aceptar la invitación crea la cuenta.</t>
-  </si>
-  <si>
     <t>2026-10-16</t>
   </si>
   <si>
@@ -884,33 +860,15 @@
     <t>EV-02</t>
   </si>
   <si>
-    <t>backend/src/routes/staff.js:112; miembros.js:667; checkin.js:57; middleware/auth.js:29</t>
-  </si>
-  <si>
-    <t>Permisos distintos para Administrador y Recepcionista.</t>
-  </si>
-  <si>
     <t>EV-03</t>
   </si>
   <si>
-    <t>backend/src/routes/auth.js:200, :231, :295; frontend/src/context/AuthContext.jsx:95</t>
-  </si>
-  <si>
-    <t>Login con bcrypt + JWT y cierre de sesión manual.</t>
-  </si>
-  <si>
     <t>EV-04</t>
   </si>
   <si>
     <t>Código (hallazgo)</t>
   </si>
   <si>
-    <t>backend/src/lib/auth-helpers.js:102-113</t>
-  </si>
-  <si>
-    <t>generarToken no aplica JWT_EXPIRES_IN: el token del personal no expira.</t>
-  </si>
-  <si>
     <t>EV-05</t>
   </si>
   <si>
@@ -1307,24 +1265,12 @@
     <t>Observación: solo WhatsApp por enlace wa.me; el estado no confirma la entrega y el correo no se usa para retención. Pendiente de confirmar en la copia de producción si envio_mensaje tiene la columna canal y notificacion la columna leido (verificador: 94d5fbb, sección 15). Si no las tiene, POST /api/admin/notificaciones/enviado falla siempre (el frontend oculta el error, MiembrosPage.jsx:802-808) y RQF-09 baja a Parcial. Santiago lo consulta.</t>
   </si>
   <si>
-    <t>GET /api/admin/dashboard: miembros activos (dashboard.js:150, :174), entradas de hoy con el día cortado en hora de Colombia (:155; ayudantes enHoraLocal e inicioLocal en :69 y :74), semana desde el lunes de Colombia (:217) y próximos vencimientos a 30 días (:232). GET /api/admin/dashboard/horas-pico (:327; periodos en :320 y hora local en :339): entradas por hora y hora pico. DashboardPage.jsx: gráfica BarsHoras (:172), que abre en «Hoy» (:226); refresco cada 60 s con la pestaña visible y al volver a ella (REFRESCO_MS :49, :279-288), sin cargas en paralelo (:239-246); listado de próximos vencimientos (:610-626). PR #16.</t>
-  </si>
-  <si>
-    <t>Implementado (2026-10-18; verificador 1be53f7, secciones 19 y 21.1): se cumplen las cuatro partes del texto y el día se corta en hora de Colombia. Observaciones: las comparaciones con columnas DATE (próximas a vencer y vencen en 7 días) siguen con CURRENT_DATE en UTC, así que de 19:00 a 24:00 en Colombia hay un día de desfase; y vencen7 y proximos todavía cuentan las membresías congeladas (va en un PR aparte).</t>
-  </si>
-  <si>
     <t>Cálculo automático de fecha_fin según el plan (miembros.js:193, :395); estado vencido / por vencer contra la fecha actual (:286-290); renovación del plan (:926). Estado Congelada (PR #17, migración 010): POST /api/admin/miembros/:id/congelar (:810) y /descongelar (:869), que corre fecha_fin y la próxima fecha de cobro los días congelados (:892), con historial en congelacion_plan; la lista marca la membresía congelada y no la cuenta como vencida (:286); pantalla en MiembrosPage.jsx:238, :742, :1907.</t>
   </si>
   <si>
     <t>Sigue Parcial (decisión de Luis, 2026-10-18): congelar y descongelar ya están en develop (PR #17; verificador 1be53f7, sección 18.2), pero falta que Santiago haga que el job de avisos de vencimiento (expiracion.js) y el check-in salten las membresías congeladas. El check-in debe negar el ingreso con estado CONGELADO y el mensaje «Tu membresía está congelada. Pide en recepción que la reactiven para poder ingresar.». Hoy el job le mandaría a un miembro congelado el aviso de que su plan vence, y el check-in lo deja entrar. Pasa a Implementado cuando esos dos cambios estén fusionados y verificados. Menores: congelar entre las 19:00 y las 24:00 de Colombia toma la fecha del día siguiente (CURRENT_DATE en UTC), y renovar el plan mientras está congelado conserva congelado_desde.</t>
   </si>
   <si>
-    <t>DELETE /api/auth/account (auth.js:558): solo el administrador (403 NOT_ADMIN en :565) y solo el dueño, que es el primer usuario del gimnasio (:575-590, 403 NOT_OWNER), confirmando con su contraseña (:493, :592-593, 403 WRONG_PASSWORD) antes de abrir la transacción (:598). Borra los pasos de PASOS_ELIMINAR_CUENTA (:503) con un SAVEPOINT por paso (borrarPaso, :544), que solo omite una tabla o columna inexistente (42P01 y 42703, :537); el gimnasio se borra al final (:605), responde 404 si ya no existe (:608) y el rastro queda en el log (:613). La página pide la contraseña (EliminarCuentaPage.jsx:12, :124-126). PR #15 y #21.</t>
-  </si>
-  <si>
-    <t>Solo el dueño, con su contraseña (PR #21). Probado por el verificador con el handler real sobre PostgreSQL 18 (94d5fbb, sección 16; 1be53f7, sección 21.2): responde 200 sin dejar filas del gimnasio ni tocar las de otro, 403 al administrador invitado y con la contraseña mala, y 500 sin borrar nada si una FK desconocida lo bloquea. Falta el límite de intentos en DELETE /api/auth/account: con un token robado del dueño se puede probar su contraseña sin freno. Es una línea en index.js (zona de Daniel), antes de la :81.</t>
-  </si>
-  <si>
     <t>backend/src/routes/miembros.js:193, :395, :286-290, :926</t>
   </si>
   <si>
@@ -1334,18 +1280,6 @@
     <t>Congelar y descongelar con historial y corrimiento del vencimiento (PR #17). Falta que el job y el check-in salten las congeladas.</t>
   </si>
   <si>
-    <t>backend/src/routes/dashboard.js:69, :74, :150, :155, :174, :217, :232, :320, :327, :339; frontend/src/pages/DashboardPage.jsx:49, :172, :226, :239-246, :279-288, :610-626</t>
-  </si>
-  <si>
-    <t>KPIs del día con el corte en hora de Colombia, gráfica de horas pico, próximos vencimientos y refresco automático cada 60 s (PR #16).</t>
-  </si>
-  <si>
-    <t>backend/src/routes/auth.js:493, :503, :537, :544, :558-623 (NOT_ADMIN :565, NOT_OWNER :588, WRONG_PASSWORD :593, BEGIN :598); frontend/src/pages/EliminarCuentaPage.jsx:12, :124-126</t>
-  </si>
-  <si>
-    <t>Eliminación de cuenta solo por el dueño y con su contraseña, con un SAVEPOINT por paso y atómica (PR #15 y #21).</t>
-  </si>
-  <si>
     <t>Informe del verificador: commit 94d5fbb, docs/verificacion-requisitos.md §16; commit 1be53f7, §21.2</t>
   </si>
   <si>
@@ -1358,16 +1292,70 @@
     <t>Job de vencimientos y check-in que salten las membresías congeladas (check-in con estado CONGELADO)</t>
   </si>
   <si>
-    <t>Luis (PR #18)</t>
-  </si>
-  <si>
-    <t>Luis (PR #19)</t>
-  </si>
-  <si>
     <t>Si WhatsApp no está listo, sendWhatsAppText vuelve sin error (whatsapp.js:228-231) y el job marca el aviso como enviado (expiracion.js:206-207), así que nunca lo reintenta; en Render no hay Chrome (whatsapp.js:7-25). Los días de anticipación (gimnasio.dias_aviso_vencimiento) solo se cambian en la base de datos: PUT /admin/config no los acepta (config.js:20-30). Además, el job no salta las membresías congeladas (expiracion.js:43-65; verificador 1be53f7, sección 18.2): le avisaría a un miembro congelado que su plan vence.</t>
   </si>
   <si>
-    <t>Estado actualizado el 2026-10-18 con los PR fusionados en develop @ f3d323c (#9, #11, #14, #15, #16, #17 y #21); la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
+    <t>Crear cuentas por invitación (POST /api/admin/staff/invite, staff.js:133), listar el personal (:357) y las invitaciones (:222), revocarlas (:251) y aceptar la invitación, que crea la cuenta (:499). PATCH /api/admin/staff/:id (:388) edita el nombre y el rol y desactiva o reactiva la cuenta; protege al dueño (OWNER_PROTECTED, :424) y no deja que uno se quite el acceso a sí mismo (SELF_LOCKOUT, :421). authenticate vuelve a leer al personal en cada petición (middleware/auth.js:10, :78): una cuenta desactivada o movida de gimnasio pierde el acceso en la siguiente petición, y el rol sale de la base. Dueño explícito en gimnasio.id_dueno (migración 013; registro en auth.js:157-162; sqlIdDueno en auth-helpers.js:188). Pantalla: StaffPage.jsx:138 (editar), :421 y :434 (desactivar y reactivar). PR #19.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-18; verificador b8f99d2, secciones 25.1 y 25.4). Observaciones abiertas: id_dueno puede apuntar a un usuario de otro gimnasio, porque la FK es solo id_dueno → usuario; se recomienda una FK compuesta (id_dueno, id_gimnasio) → usuario (id_usuario, id_gimnasio) (sección 25.2). El segundo bloque del relleno de la 013 debería exigir id_rol IS NULL. El PATCH no tiene pruebas automáticas ni escribe en auditoria (criterio 4 de HU-04, que el texto de RQF-01 no pide).</t>
+  </si>
+  <si>
+    <t>POST /api/auth/login con bcrypt (auth.js:212, :243) y límite de 5 intentos por minuto (index.js:63, :79); cierre manual (auth.js:313, AuthContext.jsx:223). El JWT del personal siempre vence: 8 h por defecto o JWT_EXPIRES_IN, y 8 h si la configuración no es válida (vigenciaTokenPersonal y generarToken, auth-helpers.js:113, :135-143); authenticate rechaza los tokens sin vencimiento (401 TOKEN_SIN_VENCIMIENTO, middleware/auth.js:63). Cierre automático tras 30 min sin actividad, compartido entre pestañas (AuthContext.jsx:23-27, :40, :150-178), al vencer el token y ante un 401 (api.js:115). PR #18.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-18; verificador b8f99d2, secciones 22.6 y 25.4). Observaciones: CheckinPage.jsx (zona de Santiago) todavía no llama a marcarActividad() (AuthContext.jsx:219), así que un kiosco que solo usa la cámara se cierra a los 30 min. La vigencia no está alineada: render.yaml:19 usa 24h y docker-compose.yml:61, 7d (se recomienda 8h). Con JWT_EXPIRES_IN en 0 o negativo el token nace vencido. 4 pruebas de aislamiento.test.js firman tokens sin vencimiento y fallan (arreglo de una línea de Santiago).</t>
+  </si>
+  <si>
+    <t>GET /api/admin/dashboard: miembros activos (dashboard.js:165, :190), entradas de hoy con el día cortado en hora de Colombia (:170; ayudantes enHoraLocal e inicioLocal en :69 y :74), semana desde el lunes de Colombia (:233) y próximos vencimientos a 30 días (:248), sin las membresías congeladas (:85, :187, :256). GET /api/admin/dashboard/horas-pico (:344; periodos en :337 y hora local en :356): entradas por hora y hora pico. DashboardPage.jsx: gráfica BarsHoras (:172), que abre en «Hoy» (:226); refresco cada 60 s con la pestaña visible y al volver a ella (REFRESCO_MS :49, :279-288), sin cargas en paralelo (:239-246); listado de próximos vencimientos (:610-626). PR #16 y #22.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-18; verificador 1be53f7, secciones 19 y 21.1). Desde el PR #22, «Vencen en 7 días» y «Próximos vencimientos» no cuentan las membresías congeladas. Observación: las comparaciones con columnas DATE (próximas a vencer y vencen en 7 días) siguen con CURRENT_DATE en UTC, así que de 19:00 a 24:00 en Colombia hay un día de desfase.</t>
+  </si>
+  <si>
+    <t>DELETE /api/auth/account (auth.js:576): solo el administrador (403 NOT_ADMIN en :583) y solo el dueño, que es gimnasio.id_dueno (sqlIdDueno, auth-helpers.js:188; :594, 403 NOT_OWNER en :606), confirmando con su contraseña (:511, :611, 403 WRONG_PASSWORD) antes de abrir la transacción (:616). Borra los pasos de PASOS_ELIMINAR_CUENTA (:521) con un SAVEPOINT por paso (borrarPaso, :562), que solo omite una tabla o columna inexistente (42P01 y 42703, :555); el gimnasio se borra al final (:623), responde 404 si ya no existe (:626) y el rastro queda en el log (:631). La página pide la contraseña (EliminarCuentaPage.jsx:12, :124-126). PR #15, #21 y #19 (id_dueno).</t>
+  </si>
+  <si>
+    <t>Solo el dueño, con su contraseña (PR #21); el dueño es gimnasio.id_dueno desde el PR #19. Probado por el verificador con el handler real sobre PostgreSQL 18 (94d5fbb, sección 16; 1be53f7, sección 21.2; b8f99d2, sección 25.2): responde 200 sin dejar filas del gimnasio ni tocar las de otro, 403 al administrador invitado y con la contraseña mala, y 500 sin borrar nada si una FK desconocida lo bloquea. Falta el límite de intentos en DELETE /api/auth/account: con un token robado del dueño se puede probar su contraseña sin freno. Es una línea en index.js (zona de Daniel), antes de la :81.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/staff.js:133, :222, :251, :357, :388, :421, :424, :499; frontend/src/pages/StaffPage.jsx:138, :421, :434</t>
+  </si>
+  <si>
+    <t>Invitar, listar, revocar, editar, desactivar y reactivar al personal; el dueño queda protegido (PR #19).</t>
+  </si>
+  <si>
+    <t>backend/src/middleware/auth.js:10, :78; backend/migrations/013_gimnasio_id_dueno.sql; backend/src/lib/auth-helpers.js:188</t>
+  </si>
+  <si>
+    <t>El rol y el acceso se leen de la base en cada petición; dueño explícito en gimnasio.id_dueno.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:212, :243, :313; backend/src/index.js:63, :79; frontend/src/context/AuthContext.jsx:23-27, :40, :150-178, :223; frontend/src/api.js:115</t>
+  </si>
+  <si>
+    <t>Login con bcrypt y límite de intentos, cierre manual y cierre automático por inactividad, vencimiento o 401 (PR #18).</t>
+  </si>
+  <si>
+    <t>backend/src/lib/auth-helpers.js:113, :135-143; backend/src/middleware/auth.js:63</t>
+  </si>
+  <si>
+    <t>El token del personal siempre vence (8 h por defecto) y se rechazan los tokens sin vencimiento (PR #18).</t>
+  </si>
+  <si>
+    <t>backend/src/routes/dashboard.js:69, :74, :85, :165, :170, :190, :233, :248, :337, :344, :356; frontend/src/pages/DashboardPage.jsx:49, :172, :226, :239-246, :279-288, :610-626</t>
+  </si>
+  <si>
+    <t>KPIs del día con el corte en hora de Colombia, gráfica de horas pico, próximos vencimientos sin congeladas y refresco automático cada 60 s (PR #16 y #22).</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:511, :521, :555, :562, :576-641 (NOT_ADMIN :583, NOT_OWNER :606, WRONG_PASSWORD :611, BEGIN :616); backend/src/lib/auth-helpers.js:188; frontend/src/pages/EliminarCuentaPage.jsx:12, :124-126</t>
+  </si>
+  <si>
+    <t>Eliminación de cuenta solo por el dueño (gimnasio.id_dueno) y con su contraseña, con un SAVEPOINT por paso y atómica (PR #15, #21 y #19).</t>
+  </si>
+  <si>
+    <t>Estado actualizado el 2026-10-18 con los PR fusionados en develop @ bdf987b (#9, #11, #14 a #19, #21 y #22); la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
   </si>
 </sst>
 </file>
@@ -1749,13 +1737,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.70454545454545459</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.6333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.67567567567567566</c:v>
+                  <c:v>0.70270270270270274</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1919,10 +1907,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>19</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>6</c:v>
@@ -2337,7 +2325,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2382,11 +2370,11 @@
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
@@ -2394,7 +2382,7 @@
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.70454545454545459</v>
+        <v>0.75</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2402,14 +2390,14 @@
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>2.1000000000000014</v>
+        <v>1.1000000000000014</v>
       </c>
       <c r="J6" t="s">
         <v>12</v>
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
@@ -2449,7 +2437,7 @@
       </c>
       <c r="K7">
         <f>E8</f>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
@@ -2462,11 +2450,11 @@
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
@@ -2474,7 +2462,7 @@
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.67567567567567566</v>
+        <v>0.70270270270270274</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2482,7 +2470,7 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>4.6000000000000014</v>
+        <v>3.6000000000000014</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
@@ -2532,11 +2520,11 @@
       </c>
       <c r="D31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Implementado",RF!$G$2:$G$100,"Original")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Parcial",RF!$G$2:$G$100,"Original")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Pendiente",RF!$G$2:$G$100,"Original")</f>
@@ -2544,7 +2532,7 @@
       </c>
       <c r="G31" s="9">
         <f>IF(C31=0,0,SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")/C31)</f>
-        <v>0.54166666666666663</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
@@ -2582,11 +2570,11 @@
       </c>
       <c r="D33" s="13">
         <f>D31+D32</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E33" s="13">
         <f>E31+E32</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F33" s="13">
         <f>F31+F32</f>
@@ -2594,7 +2582,7 @@
       </c>
       <c r="G33" s="14">
         <f>IF(C33=0,0,(SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")+SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original"))/C33)</f>
-        <v>0.55000000000000004</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
@@ -2695,7 +2683,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
         <v>32</v>
       </c>
@@ -2703,202 +2691,202 @@
         <v>33</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>34</v>
+        <v>417</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>35</v>
+        <v>418</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G2" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="J2" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="I2" s="23" t="s">
+    </row>
+    <row r="3" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="22" t="s">
         <v>38</v>
-      </c>
-      <c r="J2" s="23" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="22" t="s">
-        <v>40</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>33</v>
       </c>
       <c r="C3" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>41</v>
+        <v>419</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>42</v>
+        <v>420</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>423</v>
+        <v>407</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>424</v>
+        <v>408</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H7" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="J7" s="23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="23" t="s">
         <v>67</v>
-      </c>
-      <c r="I7" s="23" t="s">
-        <v>68</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>71</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>12</v>
@@ -2914,318 +2902,318 @@
         <v>1</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>420</v>
+        <v>406</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>396</v>
+        <v>382</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>397</v>
+        <v>383</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>440</v>
+        <v>416</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I17" s="23" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>33</v>
@@ -3234,64 +3222,64 @@
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="I18" s="23" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F19" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C19,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="I19" s="23" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>33</v>
@@ -3300,125 +3288,125 @@
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F20" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C20,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="I21" s="23" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C22" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I22" s="23" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -3497,497 +3485,497 @@
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>401</v>
+        <v>387</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -4017,7 +4005,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4041,40 +4029,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="H1" s="6" t="s">
         <v>243</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4082,28 +4070,28 @@
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.70270270270270274</v>
+        <v>0.72972972972972971</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4111,28 +4099,28 @@
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.71621621621621623</v>
+        <v>0.7432432432432432</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4140,28 +4128,28 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.72972972972972971</v>
+        <v>0.7567567567567568</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4169,28 +4157,28 @@
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.7432432432432432</v>
+        <v>0.77027027027027029</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4198,28 +4186,28 @@
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.7567567567567568</v>
+        <v>0.78378378378378377</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4227,28 +4215,28 @@
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.77027027027027029</v>
+        <v>0.79729729729729726</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="B8" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>438</v>
+        <v>245</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4256,86 +4244,86 @@
       </c>
       <c r="H8" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.78378378378378377</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.81081081081081086</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>64</v>
+        <v>162</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>66</v>
+        <v>388</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>257</v>
+        <v>401</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H9" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.79729729729729726</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.83783783783783783</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>166</v>
+        <v>49</v>
       </c>
       <c r="B10" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="D10" s="23" t="s">
         <v>415</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H10" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.82432432432432434</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.85135135135135132</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
       <c r="B11" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>35</v>
+        <v>74</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>439</v>
+        <v>245</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
@@ -4343,28 +4331,28 @@
       </c>
       <c r="H11" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.83783783783783783</v>
+        <v>0.86486486486486491</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>53</v>
+        <v>196</v>
       </c>
       <c r="B12" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>436</v>
+        <v>199</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>437</v>
+        <v>256</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4372,28 +4360,28 @@
       </c>
       <c r="H12" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>0.85135135135135132</v>
+        <v>0.8783783783783784</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>75</v>
+        <v>213</v>
       </c>
       <c r="B13" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>78</v>
+        <v>402</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>261</v>
+        <v>403</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="G13" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
@@ -4401,86 +4389,86 @@
       </c>
       <c r="H13" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G13))/Resumen!$C$8</f>
-        <v>0.86486486486486491</v>
+        <v>0.89189189189189189</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>200</v>
+        <v>90</v>
       </c>
       <c r="B14" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>203</v>
+        <v>93</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="G14" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H14" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G14))/Resumen!$C$8</f>
-        <v>0.8783783783783784</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.91891891891891897</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>217</v>
+        <v>167</v>
       </c>
       <c r="B15" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>416</v>
+        <v>170</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>417</v>
+        <v>258</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="G15" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H15" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G15))/Resumen!$C$8</f>
-        <v>0.89189189189189189</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B16" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="G16" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
@@ -4488,28 +4476,28 @@
       </c>
       <c r="H16" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G16))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.97297297297297303</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>171</v>
+        <v>83</v>
       </c>
       <c r="B17" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>174</v>
+        <v>86</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="G17" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
@@ -4517,74 +4505,16 @@
       </c>
       <c r="H17" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G17))/Resumen!$C$8</f>
-        <v>0.94594594594594594</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="B18" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>103</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>265</v>
-      </c>
-      <c r="E18" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="F18" s="24" t="s">
-        <v>266</v>
-      </c>
-      <c r="G18" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
         <v>1</v>
       </c>
-      <c r="H18" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G18))/Resumen!$C$8</f>
-        <v>0.97297297297297303</v>
-      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>267</v>
-      </c>
-      <c r="E19" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="F19" s="24" t="s">
-        <v>266</v>
-      </c>
-      <c r="G19" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A19,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A19,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
-      </c>
-      <c r="H19" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G19))/Resumen!$C$8</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="17" t="s">
-        <v>418</v>
+      <c r="A19" s="17" t="s">
+        <v>404</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B19">
+  <conditionalFormatting sqref="B2:B17">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Implementado"</formula>
     </cfRule>
@@ -4616,7 +4546,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H2:H19</xm:sqref>
+          <xm:sqref>H2:H17</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4640,30 +4570,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4672,1148 +4602,1148 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>275</v>
+        <v>425</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>276</v>
-      </c>
-      <c r="F2" s="23" t="s">
-        <v>277</v>
+        <v>426</v>
+      </c>
+      <c r="F2" s="28" t="s">
+        <v>405</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>23</v>
+        <v>289</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>280</v>
+        <v>427</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>281</v>
-      </c>
-      <c r="F3" s="23" t="s">
-        <v>277</v>
+        <v>428</v>
+      </c>
+      <c r="F3" s="28" t="s">
+        <v>405</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>283</v>
+        <v>429</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>284</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>277</v>
+        <v>430</v>
+      </c>
+      <c r="F4" s="28" t="s">
+        <v>405</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>286</v>
+        <v>23</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>287</v>
+        <v>431</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>288</v>
-      </c>
-      <c r="F5" s="23" t="s">
-        <v>277</v>
+        <v>432</v>
+      </c>
+      <c r="F5" s="28" t="s">
+        <v>405</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>289</v>
+        <v>275</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C6" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>291</v>
+        <v>277</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>292</v>
+        <v>278</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C7" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>293</v>
+        <v>279</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>294</v>
+        <v>280</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>295</v>
+        <v>281</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C8" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>427</v>
+        <v>409</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>296</v>
+        <v>282</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>297</v>
+        <v>283</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>428</v>
+        <v>410</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>429</v>
+        <v>411</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>299</v>
+        <v>285</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C10" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>300</v>
+        <v>286</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>301</v>
+        <v>287</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>304</v>
+        <v>290</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>305</v>
+        <v>291</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>306</v>
+        <v>292</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>307</v>
+        <v>293</v>
       </c>
       <c r="F12" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>308</v>
+        <v>294</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C14" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>309</v>
+        <v>295</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>310</v>
+        <v>296</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>311</v>
+        <v>297</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C15" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>312</v>
+        <v>298</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>313</v>
+        <v>299</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C16" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>314</v>
+        <v>300</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>315</v>
+        <v>301</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>298</v>
+        <v>284</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>316</v>
+        <v>302</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>317</v>
+        <v>303</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>319</v>
+        <v>305</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>320</v>
+        <v>306</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>318</v>
+        <v>304</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>321</v>
+        <v>307</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>322</v>
+        <v>308</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>404</v>
+        <v>390</v>
       </c>
       <c r="E20" s="23" t="s">
+        <v>391</v>
+      </c>
+      <c r="F20" s="27" t="s">
         <v>405</v>
       </c>
-      <c r="F20" s="27" t="s">
-        <v>419</v>
-      </c>
       <c r="G20" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>323</v>
+        <v>309</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>324</v>
+        <v>310</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>325</v>
+        <v>311</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>326</v>
+        <v>312</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>327</v>
+        <v>313</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>328</v>
+        <v>314</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>330</v>
+        <v>316</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>331</v>
+        <v>317</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>332</v>
+        <v>318</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>333</v>
+        <v>319</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>334</v>
+        <v>320</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>337</v>
+        <v>323</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>338</v>
+        <v>324</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>340</v>
+        <v>326</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>341</v>
+        <v>327</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>342</v>
+        <v>328</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>343</v>
+        <v>329</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>344</v>
+        <v>330</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>345</v>
+        <v>331</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>346</v>
+        <v>332</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>347</v>
+        <v>333</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>348</v>
+        <v>334</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>349</v>
+        <v>335</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>350</v>
+        <v>336</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>351</v>
+        <v>337</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>352</v>
+        <v>338</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>353</v>
+        <v>339</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>303</v>
+        <v>289</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>354</v>
+        <v>340</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>355</v>
+        <v>341</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>356</v>
+        <v>342</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>357</v>
+        <v>343</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>358</v>
+        <v>344</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>434</v>
+        <v>412</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>435</v>
+        <v>413</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>359</v>
+        <v>345</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>360</v>
+        <v>346</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>361</v>
+        <v>347</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C36" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>362</v>
+        <v>348</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>363</v>
+        <v>349</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>365</v>
+        <v>351</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>366</v>
+        <v>352</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>367</v>
+        <v>353</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>368</v>
+        <v>354</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>369</v>
+        <v>355</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>370</v>
+        <v>356</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>371</v>
+        <v>357</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>372</v>
+        <v>358</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>373</v>
+        <v>359</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>374</v>
+        <v>360</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>375</v>
+        <v>361</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>376</v>
+        <v>362</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>377</v>
+        <v>363</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>339</v>
+        <v>325</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>378</v>
+        <v>364</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>379</v>
+        <v>365</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>380</v>
+        <v>366</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>381</v>
+        <v>367</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>382</v>
+        <v>368</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>383</v>
+        <v>369</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>419</v>
+        <v>405</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>384</v>
+        <v>370</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>385</v>
+        <v>371</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>386</v>
+        <v>372</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>387</v>
+        <v>373</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>388</v>
+        <v>374</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>389</v>
+        <v>375</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>390</v>
+        <v>376</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>391</v>
+        <v>377</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>392</v>
+        <v>378</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>393</v>
+        <v>379</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>394</v>
+        <v>380</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>395</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): RQF-09 pasa a Parcial en el Excel (68,9 %)
Santiago confirmo contra una copia de la base real (issue #24) que
POST /api/admin/notificaciones/enviado no guarda nada: envio_mensaje usa
id_canal (FK a canal_comunicacion, sin filas para los gimnasios reales) y
exige mensaje_copiado. RQF-09 vuelve a la ruta al 80 % y RQNF-10 cita la
confirmacion. RQF-06 y RQF-14 no cambian (PR #23 y #10 en revision).

Editado con Excel por COM. Avance: 25,5 de 37 = 68,9 % (RF 72,7 %, RNF 63,3 %).
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{692AE4A1-D0E1-4736-A0C2-7811DBB69D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8D538E-11DB-4081-A0A9-4E811A40A7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="438">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="442">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -281,9 +281,6 @@
     <t>RQF-09</t>
   </si>
   <si>
-    <t>Botón de WhatsApp con el mensaje armado para miembros en riesgo (MenuNotificaciones.jsx:86-90, MiembrosPage.jsx:796-802); POST /api/admin/notificaciones/enviado guarda canal, estado ENVIADO y fecha en envio_mensaje (notificaciones.js:188-224).</t>
-  </si>
-  <si>
     <t>HU-19, HU-20, HU-52</t>
   </si>
   <si>
@@ -944,12 +941,6 @@
     <t>El único cron programado es el de vencimientos (no hay motor de abandono).</t>
   </si>
   <si>
-    <t>frontend/src/components/MenuNotificaciones.jsx:86-90; MiembrosPage.jsx:796-802; backend/src/routes/notificaciones.js:188-224</t>
-  </si>
-  <si>
-    <t>Envío por WhatsApp y registro en envio_mensaje con fecha y estado.</t>
-  </si>
-  <si>
     <t>backend/migrations/002_esquema_inicial.sql:171-202</t>
   </si>
   <si>
@@ -1202,12 +1193,6 @@
     <t>Implementado (2026-10-18): ya no queda ninguna consulta sin filtro de gimnasio y el check-in dejó de derivar la clave del QR por cada miembro (verificador: 386d168, sección 14.5). La medición del tiempo de respuesta con volumen realista queda en RQNF-01. Menor: la vista lee membresia y plan_membresia, que el alta no llena, así que sus columnas de plan salen en NULL.</t>
   </si>
   <si>
-    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 009 y 011: la 009 (PR #14) crea auditoria y agrega las columnas y restricciones de gamificación de producción, y la 011 (PR #11) recrea vista_miembros_activos con id_gimnasio.</t>
-  </si>
-  <si>
-    <t>Sigue Parcial (verificador: 94d5fbb, sección 15): una base hecha solo con migraciones todavía difiere de producción en 15 tablas, y el código usa dos de ellas: notificaciones.js:211 escribe envio_mensaje.canal y :217 notificacion.leido, que no existen en el esquema de producción (allí son id_canal y leida). Pasa a Implementado con una migración que reconcilie esas dos tablas (o un cambio del código), probada contra la copia de producción. Además hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica.</t>
-  </si>
-  <si>
     <t>La búsqueda del QR ya no deriva la clave por cada miembro (PR #11, checkin.js:26, :31): hace un descifrado AES por miembro. Falta medir el check-in con un volumen realista (unos 200 miembros) y registrar el tiempo de respuesta de POST /api/admin/checkin.</t>
   </si>
   <si>
@@ -1235,12 +1220,6 @@
     <t>La vista y asistencia rechazan tokens de miembro y filtran por gimnasio; la 011 expone id_gimnasio.</t>
   </si>
   <si>
-    <t>backend/src/db/migrate.js:15-56; backend/src/index.js:128-132; backend/migrations/ (009_auditoria_y_gamificacion.sql y 011_vista_miembros_activos_gimnasio.sql)</t>
-  </si>
-  <si>
-    <t>Migraciones versionadas aplicadas al iniciar; la 009 cierra auditoría y gamificación. Quedan diferencias en envio_mensaje y notificacion (verificador 94d5fbb §15).</t>
-  </si>
-  <si>
     <t>Tras un reinicio el contrato no sale: admin-contrato.js:107 pregunta isWhatsAppReady() y nunca inicia el cliente de WhatsApp (whatsapp.js:146).</t>
   </si>
   <si>
@@ -1250,9 +1229,6 @@
     <t>Medir el check-in con un volumen realista (unos 200 miembros)</t>
   </si>
   <si>
-    <t>notificaciones.js:211 y :217 escriben envio_mensaje.canal y notificacion.leido, que no existen en el esquema de producción (verificador, sección 15).</t>
-  </si>
-  <si>
     <t>Migración que reconcilie envio_mensaje y notificacion con producción (o cambio del código), probada contra la copia de producción</t>
   </si>
   <si>
@@ -1262,9 +1238,6 @@
     <t>2026-10-18</t>
   </si>
   <si>
-    <t>Observación: solo WhatsApp por enlace wa.me; el estado no confirma la entrega y el correo no se usa para retención. Pendiente de confirmar en la copia de producción si envio_mensaje tiene la columna canal y notificacion la columna leido (verificador: 94d5fbb, sección 15). Si no las tiene, POST /api/admin/notificaciones/enviado falla siempre (el frontend oculta el error, MiembrosPage.jsx:802-808) y RQF-09 baja a Parcial. Santiago lo consulta.</t>
-  </si>
-  <si>
     <t>Cálculo automático de fecha_fin según el plan (miembros.js:193, :395); estado vencido / por vencer contra la fecha actual (:286-290); renovación del plan (:926). Estado Congelada (PR #17, migración 010): POST /api/admin/miembros/:id/congelar (:810) y /descongelar (:869), que corre fecha_fin y la próxima fecha de cobro los días congelados (:892), con historial en congelacion_plan; la lista marca la membresía congelada y no la cuenta como vencida (:286); pantalla en MiembrosPage.jsx:238, :742, :1907.</t>
   </si>
   <si>
@@ -1355,7 +1328,46 @@
     <t>Eliminación de cuenta solo por el dueño (gimnasio.id_dueno) y con su contraseña, con un SAVEPOINT por paso y atómica (PR #15, #21 y #19).</t>
   </si>
   <si>
-    <t>Estado actualizado el 2026-10-18 con los PR fusionados en develop @ bdf987b (#9, #11, #14 a #19, #21 y #22); la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
+    <t>Botón de WhatsApp con el mensaje armado para los miembros en riesgo (MenuNotificaciones.jsx:84-99, MiembrosPage.jsx:836-849). El registro de cada envío lo hace POST /api/admin/notificaciones/enviado (notificaciones.js:189), que inserta en envio_mensaje (:211) y en notificacion (:217).</t>
+  </si>
+  <si>
+    <t>Parcial (2026-10-19): el registro de la fecha y el estado de cada envío no funciona con el esquema real. Santiago lo confirmó contra una copia de la base real (issue #24): envio_mensaje no tiene la columna canal (usa id_canal, con FK a canal_comunicacion, y exige mensaje_copiado NOT NULL; también tiene enviado_por), y canal_comunicacion solo tiene filas para los 3 gimnasios de ejemplo, así que no hay un id_canal válido. El endpoint responde 503 y el frontend oculta el error (MiembrosPage.jsx:847-849, MenuNotificaciones.jsx:95-98). El insert en notificacion (leido/leida y tipo) se corrige en el PR #23. Falta decidir cómo se crea el canal WhatsApp de cada gimnasio (bajo demanda o al registrarlo), qué se guarda en mensaje_copiado (el texto que se abrió en WhatsApp) y si enviado_por es el usuario del token. Además: solo WhatsApp por enlace wa.me; el estado no confirma la entrega y el correo no se usa para retención.</t>
+  </si>
+  <si>
+    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 011 y 013: la 009 (PR #14) crea auditoria y agrega las columnas y restricciones de gamificación de producción, la 010 (PR #17) el congelamiento, la 011 (PR #11) recrea vista_miembros_activos con id_gimnasio y la 013 (PR #19) agrega gimnasio.id_dueno.</t>
+  </si>
+  <si>
+    <t>Sigue Parcial (verificador: 94d5fbb, sección 15; confirmado contra una copia de la base real en el issue #24): una base hecha solo con migraciones todavía difiere de producción en 15 tablas, y el código usa dos de ellas. notificaciones.js:211 escribe envio_mensaje.canal, que en producción no existe (allí hay id_canal, con FK a canal_comunicacion, y mensaje_copiado NOT NULL); :217 escribe notificacion.leido, que allí es leida (lo corrige el PR #23, en revisión). Pasa a Implementado con una migración que reconcilie esas tablas, o un cambio del código, probado contra la copia de producción. Además hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica.</t>
+  </si>
+  <si>
+    <t>Código / hallazgo</t>
+  </si>
+  <si>
+    <t>frontend/src/components/MenuNotificaciones.jsx:84-99; frontend/src/pages/MiembrosPage.jsx:836-849; backend/src/routes/notificaciones.js:189, :211, :217; issue #24</t>
+  </si>
+  <si>
+    <t>Envío por WhatsApp; el registro en envio_mensaje falla con el esquema real (issue #24).</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>backend/src/db/migrate.js:15-56; backend/src/index.js:128-132; backend/migrations/ (009, 010, 011 y 013); issue #24</t>
+  </si>
+  <si>
+    <t>Migraciones versionadas aplicadas al iniciar. Quedan diferencias con producción en envio_mensaje y notificacion (verificador 94d5fbb §15; issue #24).</t>
+  </si>
+  <si>
+    <t>notificaciones.js:211 escribe envio_mensaje.canal, que no existe en el esquema de producción (issue #24); notificacion.leido lo corrige el PR #23.</t>
+  </si>
+  <si>
+    <t>Estado actualizado el 2026-10-19 con los PR fusionados en develop @ dcda269 (#9, #11 y #14 a #22) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
+  </si>
+  <si>
+    <t>POST /api/admin/notificaciones/enviado no guarda nada con el esquema real: envio_mensaje usa id_canal (FK a canal_comunicacion, sin filas para los gimnasios reales) y exige mensaje_copiado (issue #24).</t>
+  </si>
+  <si>
+    <t>Buscar o crear el canal WhatsApp del gimnasio, mandar el mensaje desde el frontend e insertar en envio_mensaje con id_canal, mensaje_copiado y enviado_por, con una prueba contra el esquema real (issue #24)</t>
   </si>
 </sst>
 </file>
@@ -1737,13 +1749,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.75</c:v>
+                  <c:v>0.72727272727272729</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0.6333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.70270270270270274</c:v>
+                  <c:v>0.68918918918918914</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1907,10 +1919,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>21</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>6</c:v>
@@ -2325,7 +2337,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2370,11 +2382,11 @@
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
@@ -2382,7 +2394,7 @@
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.75</v>
+        <v>0.72727272727272729</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2390,14 +2402,14 @@
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>1.1000000000000014</v>
+        <v>1.6000000000000014</v>
       </c>
       <c r="J6" t="s">
         <v>12</v>
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
@@ -2437,7 +2449,7 @@
       </c>
       <c r="K7">
         <f>E8</f>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
@@ -2450,11 +2462,11 @@
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
@@ -2462,7 +2474,7 @@
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.70270270270270274</v>
+        <v>0.68918918918918914</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2470,7 +2482,7 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>3.6000000000000014</v>
+        <v>4.1000000000000014</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
@@ -2520,11 +2532,11 @@
       </c>
       <c r="D31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Implementado",RF!$G$2:$G$100,"Original")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Parcial",RF!$G$2:$G$100,"Original")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Pendiente",RF!$G$2:$G$100,"Original")</f>
@@ -2532,7 +2544,7 @@
       </c>
       <c r="G31" s="9">
         <f>IF(C31=0,0,SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")/C31)</f>
-        <v>0.625</v>
+        <v>0.58333333333333337</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
@@ -2570,11 +2582,11 @@
       </c>
       <c r="D33" s="13">
         <f>D31+D32</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E33" s="13">
         <f>E31+E32</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F33" s="13">
         <f>F31+F32</f>
@@ -2582,7 +2594,7 @@
       </c>
       <c r="G33" s="14">
         <f>IF(C33=0,0,(SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")+SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original"))/C33)</f>
-        <v>0.6</v>
+        <v>0.57499999999999996</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
@@ -2694,10 +2706,10 @@
         <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2727,10 +2739,10 @@
         <v>12</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2793,10 +2805,10 @@
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2892,10 +2904,10 @@
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2947,7 +2959,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="216" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
         <v>78</v>
       </c>
@@ -2955,46 +2967,46 @@
         <v>72</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>79</v>
+        <v>428</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>406</v>
+        <v>429</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
         <v>34</v>
       </c>
       <c r="H10" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="I10" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="I10" s="23" t="s">
+      <c r="J10" s="23" t="s">
         <v>81</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" s="23" t="s">
         <v>83</v>
-      </c>
-      <c r="B11" s="23" t="s">
-        <v>84</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="E11" s="23" t="s">
         <v>85</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>86</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3004,30 +3016,30 @@
         <v>34</v>
       </c>
       <c r="H11" s="23" t="s">
+        <v>86</v>
+      </c>
+      <c r="I11" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="I11" s="23" t="s">
+      <c r="J11" s="23" t="s">
         <v>88</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="23" t="s">
         <v>90</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>91</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="E12" s="23" t="s">
         <v>92</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>93</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3037,30 +3049,30 @@
         <v>34</v>
       </c>
       <c r="H12" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="I12" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="I12" s="23" t="s">
+      <c r="J12" s="23" t="s">
         <v>95</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="E13" s="23" t="s">
         <v>98</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>99</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3070,51 +3082,51 @@
         <v>34</v>
       </c>
       <c r="H13" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="I13" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="I13" s="23" t="s">
+      <c r="J13" s="23" t="s">
         <v>101</v>
-      </c>
-      <c r="J13" s="23" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>103</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>104</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="H14" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="I14" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="I14" s="23" t="s">
+      <c r="J14" s="23" t="s">
         <v>107</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>43</v>
@@ -3123,97 +3135,97 @@
         <v>14</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H15" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="I15" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="I15" s="23" t="s">
+      <c r="J15" s="23" t="s">
         <v>113</v>
-      </c>
-      <c r="J15" s="23" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="B16" s="23" t="s">
         <v>115</v>
-      </c>
-      <c r="B16" s="23" t="s">
-        <v>116</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="E16" s="23" t="s">
         <v>117</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>118</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H16" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="I16" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="I16" s="23" t="s">
+      <c r="J16" s="23" t="s">
         <v>120</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="23" t="s">
         <v>122</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>123</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" s="23" t="s">
         <v>124</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>125</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H17" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="I17" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="I17" s="23" t="s">
+      <c r="J17" s="23" t="s">
         <v>127</v>
-      </c>
-      <c r="J17" s="23" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>33</v>
@@ -3222,31 +3234,31 @@
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="E18" s="23" t="s">
         <v>130</v>
-      </c>
-      <c r="E18" s="23" t="s">
-        <v>131</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H18" s="23" t="s">
+        <v>131</v>
+      </c>
+      <c r="I18" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="I18" s="23" t="s">
+      <c r="J18" s="23" t="s">
         <v>133</v>
-      </c>
-      <c r="J18" s="23" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B19" s="23" t="s">
         <v>67</v>
@@ -3255,7 +3267,7 @@
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E19" s="23" t="s">
         <v>56</v>
@@ -3265,21 +3277,21 @@
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H19" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="I19" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="I19" s="23" t="s">
+      <c r="J19" s="23" t="s">
         <v>138</v>
-      </c>
-      <c r="J19" s="23" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>33</v>
@@ -3288,7 +3300,7 @@
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E20" s="23" t="s">
         <v>56</v>
@@ -3298,54 +3310,54 @@
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I20" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="J20" s="23" t="s">
         <v>142</v>
-      </c>
-      <c r="J20" s="23" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="B21" s="23" t="s">
         <v>144</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>145</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="E21" s="23" t="s">
         <v>146</v>
-      </c>
-      <c r="E21" s="23" t="s">
-        <v>147</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H21" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="I21" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="I21" s="23" t="s">
+      <c r="J21" s="23" t="s">
         <v>149</v>
-      </c>
-      <c r="J21" s="23" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>43</v>
@@ -3354,59 +3366,59 @@
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="E22" s="23" t="s">
         <v>152</v>
-      </c>
-      <c r="E22" s="23" t="s">
-        <v>153</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H22" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="I22" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="I22" s="23" t="s">
+      <c r="J22" s="23" t="s">
         <v>155</v>
-      </c>
-      <c r="J22" s="23" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
+        <v>156</v>
+      </c>
+      <c r="B23" s="23" t="s">
         <v>157</v>
-      </c>
-      <c r="B23" s="23" t="s">
-        <v>158</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H23" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="I23" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="I23" s="23" t="s">
+      <c r="J23" s="23" t="s">
         <v>160</v>
-      </c>
-      <c r="J23" s="23" t="s">
-        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -3485,19 +3497,19 @@
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" s="23" t="s">
         <v>162</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>163</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3510,27 +3522,27 @@
         <v>56</v>
       </c>
       <c r="I2" s="23" t="s">
+        <v>164</v>
+      </c>
+      <c r="J2" s="23" t="s">
         <v>165</v>
-      </c>
-      <c r="J2" s="23" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" s="23" t="s">
         <v>167</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>168</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
+        <v>168</v>
+      </c>
+      <c r="E3" s="23" t="s">
         <v>169</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>170</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3543,27 +3555,27 @@
         <v>56</v>
       </c>
       <c r="I3" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="J3" s="23" t="s">
         <v>171</v>
-      </c>
-      <c r="J3" s="23" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>173</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>174</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
+        <v>174</v>
+      </c>
+      <c r="E4" s="23" t="s">
         <v>175</v>
-      </c>
-      <c r="E4" s="23" t="s">
-        <v>176</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3576,27 +3588,27 @@
         <v>56</v>
       </c>
       <c r="I4" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="J4" s="23" t="s">
         <v>177</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
+        <v>178</v>
+      </c>
+      <c r="B5" s="23" t="s">
         <v>179</v>
-      </c>
-      <c r="B5" s="23" t="s">
-        <v>180</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="E5" s="23" t="s">
         <v>181</v>
-      </c>
-      <c r="E5" s="23" t="s">
-        <v>182</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3606,30 +3618,30 @@
         <v>34</v>
       </c>
       <c r="H5" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="I5" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="J5" s="23" t="s">
         <v>184</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" s="23" t="s">
         <v>186</v>
-      </c>
-      <c r="B6" s="23" t="s">
-        <v>187</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3639,30 +3651,30 @@
         <v>34</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I6" s="23" t="s">
+        <v>187</v>
+      </c>
+      <c r="J6" s="23" t="s">
         <v>188</v>
-      </c>
-      <c r="J6" s="23" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
+        <v>189</v>
+      </c>
+      <c r="B7" s="23" t="s">
         <v>190</v>
-      </c>
-      <c r="B7" s="23" t="s">
-        <v>191</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
+        <v>191</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>192</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>193</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3675,27 +3687,27 @@
         <v>56</v>
       </c>
       <c r="I7" s="23" t="s">
+        <v>193</v>
+      </c>
+      <c r="J7" s="23" t="s">
         <v>194</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
+        <v>195</v>
+      </c>
+      <c r="B8" s="23" t="s">
         <v>196</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>197</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E8" s="23" t="s">
         <v>198</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>199</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3708,27 +3720,27 @@
         <v>56</v>
       </c>
       <c r="I8" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="J8" s="23" t="s">
         <v>200</v>
-      </c>
-      <c r="J8" s="23" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
+        <v>201</v>
+      </c>
+      <c r="B9" s="23" t="s">
         <v>202</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>203</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
+        <v>203</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>204</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>205</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3741,123 +3753,123 @@
         <v>56</v>
       </c>
       <c r="I9" s="23" t="s">
+        <v>205</v>
+      </c>
+      <c r="J9" s="23" t="s">
         <v>206</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="E10" s="23" t="s">
         <v>209</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>210</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H10" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I10" s="23" t="s">
+        <v>210</v>
+      </c>
+      <c r="J10" s="23" t="s">
         <v>211</v>
       </c>
-      <c r="J10" s="23" t="s">
+    </row>
+    <row r="11" spans="1:10" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>213</v>
-      </c>
       <c r="B11" s="23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>386</v>
+        <v>430</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>387</v>
+        <v>431</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H11" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I11" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="J11" s="23" t="s">
         <v>214</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="E12" s="23" t="s">
         <v>217</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>218</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H12" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I12" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="J12" s="23" t="s">
         <v>219</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E13" s="23" t="s">
         <v>56</v>
@@ -3867,30 +3879,30 @@
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H13" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I13" s="23" t="s">
+        <v>222</v>
+      </c>
+      <c r="J13" s="23" t="s">
         <v>223</v>
-      </c>
-      <c r="J13" s="23" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
+        <v>224</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>225</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>226</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>56</v>
@@ -3900,30 +3912,30 @@
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H14" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I14" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="J14" s="23" t="s">
         <v>228</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>56</v>
@@ -3933,49 +3945,49 @@
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H15" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I15" s="23" t="s">
+        <v>231</v>
+      </c>
+      <c r="J15" s="23" t="s">
         <v>232</v>
-      </c>
-      <c r="J15" s="23" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
+        <v>234</v>
+      </c>
+      <c r="E16" s="23" t="s">
         <v>235</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>236</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H16" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="J16" s="23" t="s">
         <v>237</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -4005,7 +4017,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4029,40 +4041,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>242</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D2" s="23" t="s">
+        <v>243</v>
+      </c>
+      <c r="E2" s="23" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="F2" s="24" t="s">
         <v>245</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>246</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4070,28 +4082,28 @@
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.72972972972972971</v>
+        <v>0.71621621621621623</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>399</v>
+        <v>392</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>400</v>
+        <v>393</v>
       </c>
       <c r="E3" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="F3" s="24" t="s">
         <v>245</v>
-      </c>
-      <c r="F3" s="24" t="s">
-        <v>246</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4099,28 +4111,28 @@
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.7432432432432432</v>
+        <v>0.72972972972972971</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E4" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="F4" s="24" t="s">
         <v>245</v>
-      </c>
-      <c r="F4" s="24" t="s">
-        <v>246</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4128,28 +4140,28 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.7567567567567568</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.7432432432432432</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>208</v>
+        <v>78</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>210</v>
+        <v>440</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>248</v>
+        <v>441</v>
       </c>
       <c r="E5" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="F5" s="24" t="s">
         <v>245</v>
-      </c>
-      <c r="F5" s="24" t="s">
-        <v>246</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4157,28 +4169,28 @@
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.77027027027027029</v>
+        <v>0.7567567567567568</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>179</v>
+        <v>207</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>182</v>
+        <v>209</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4186,28 +4198,28 @@
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.78378378378378377</v>
+        <v>0.77027027027027029</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4215,28 +4227,28 @@
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.79729729729729726</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.78378378378378377</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>60</v>
+        <v>189</v>
       </c>
       <c r="B8" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>62</v>
+        <v>192</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E8" s="23" t="s">
+        <v>249</v>
+      </c>
+      <c r="F8" s="24" t="s">
         <v>245</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>246</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4244,86 +4256,86 @@
       </c>
       <c r="H8" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.81081081081081086</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.79729729729729726</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>162</v>
+        <v>60</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>388</v>
+        <v>62</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>401</v>
+        <v>251</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H9" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.83783783783783783</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.81081081081081086</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>49</v>
+        <v>161</v>
       </c>
       <c r="B10" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>414</v>
+        <v>383</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>415</v>
+        <v>394</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H10" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.85135135135135132</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.83783783783783783</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>71</v>
+        <v>49</v>
       </c>
       <c r="B11" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>74</v>
+        <v>405</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>255</v>
+        <v>406</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
@@ -4331,28 +4343,28 @@
       </c>
       <c r="H11" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.86486486486486491</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.85135135135135132</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>196</v>
+        <v>71</v>
       </c>
       <c r="B12" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>199</v>
+        <v>74</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4360,28 +4372,28 @@
       </c>
       <c r="H12" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>0.8783783783783784</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.86486486486486491</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>213</v>
+        <v>195</v>
       </c>
       <c r="B13" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>402</v>
+        <v>198</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>403</v>
+        <v>255</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G13" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
@@ -4389,57 +4401,57 @@
       </c>
       <c r="H13" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G13))/Resumen!$C$8</f>
-        <v>0.89189189189189189</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.8783783783783784</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>90</v>
+        <v>212</v>
       </c>
       <c r="B14" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>93</v>
+        <v>438</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>257</v>
+        <v>395</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G14" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H14" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G14))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
+        <v>0.89189189189189189</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>167</v>
+        <v>89</v>
       </c>
       <c r="B15" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>170</v>
+        <v>92</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G15" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
@@ -4447,28 +4459,28 @@
       </c>
       <c r="H15" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G15))/Resumen!$C$8</f>
-        <v>0.94594594594594594</v>
+        <v>0.91891891891891897</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>97</v>
+        <v>166</v>
       </c>
       <c r="B16" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>99</v>
+        <v>169</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="G16" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
@@ -4476,28 +4488,28 @@
       </c>
       <c r="H16" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G16))/Resumen!$C$8</f>
-        <v>0.97297297297297303</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+        <v>0.94594594594594594</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="B17" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G17" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
@@ -4505,16 +4517,45 @@
       </c>
       <c r="H17" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G17))/Resumen!$C$8</f>
+        <v>0.97297297297297303</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="24" t="str">
+        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
+        <v>Pendiente</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>260</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>244</v>
+      </c>
+      <c r="F18" s="24" t="s">
+        <v>259</v>
+      </c>
+      <c r="G18" s="25">
+        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
-        <v>404</v>
+      <c r="H18" s="26">
+        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G18))/Resumen!$C$8</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="17" t="s">
+        <v>396</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B17">
+  <conditionalFormatting sqref="B2:B18">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Implementado"</formula>
     </cfRule>
@@ -4546,7 +4587,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H2:H17</xm:sqref>
+          <xm:sqref>H2:H18</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4570,30 +4611,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>262</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>263</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>266</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4602,44 +4643,44 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>425</v>
+        <v>416</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>38</v>
@@ -4648,21 +4689,21 @@
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>38</v>
@@ -4671,21 +4712,21 @@
         <v>23</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>432</v>
+        <v>423</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>42</v>
@@ -4694,21 +4735,21 @@
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
+        <v>275</v>
+      </c>
+      <c r="E6" s="23" t="s">
         <v>276</v>
       </c>
-      <c r="E6" s="23" t="s">
-        <v>277</v>
-      </c>
       <c r="F6" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G6" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>42</v>
@@ -4717,21 +4758,21 @@
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
+        <v>278</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>279</v>
       </c>
-      <c r="E7" s="23" t="s">
-        <v>280</v>
-      </c>
       <c r="F7" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G7" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>49</v>
@@ -4740,44 +4781,44 @@
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>49</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>53</v>
@@ -4786,39 +4827,39 @@
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
+        <v>285</v>
+      </c>
+      <c r="E10" s="23" t="s">
         <v>286</v>
       </c>
-      <c r="E10" s="23" t="s">
-        <v>287</v>
-      </c>
       <c r="F10" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G10" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>53</v>
       </c>
       <c r="C11" s="23" t="s">
+        <v>288</v>
+      </c>
+      <c r="D11" s="23" t="s">
         <v>289</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="E11" s="23" t="s">
         <v>290</v>
       </c>
-      <c r="E11" s="23" t="s">
-        <v>291</v>
-      </c>
       <c r="F11" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G11" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4832,16 +4873,16 @@
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="E12" s="23" t="s">
         <v>292</v>
       </c>
-      <c r="E12" s="23" t="s">
-        <v>293</v>
-      </c>
       <c r="F12" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G12" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G12" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4855,21 +4896,21 @@
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>434</v>
+        <v>425</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>71</v>
@@ -4878,21 +4919,21 @@
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
+        <v>294</v>
+      </c>
+      <c r="E14" s="23" t="s">
         <v>295</v>
       </c>
-      <c r="E14" s="23" t="s">
-        <v>296</v>
-      </c>
       <c r="F14" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G14" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>71</v>
@@ -4901,849 +4942,849 @@
         <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
+        <v>297</v>
+      </c>
+      <c r="E15" s="23" t="s">
         <v>298</v>
       </c>
-      <c r="E15" s="23" t="s">
-        <v>299</v>
-      </c>
       <c r="F15" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G15" s="23" t="s">
         <v>269</v>
       </c>
-      <c r="G15" s="23" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B16" s="23" t="s">
         <v>78</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>23</v>
+        <v>432</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>300</v>
+        <v>433</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>301</v>
-      </c>
-      <c r="F16" s="23" t="s">
+        <v>434</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>435</v>
+      </c>
+      <c r="G16" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G16" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="F17" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G17" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G17" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="F18" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G18" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G18" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C19" s="23" t="s">
+        <v>301</v>
+      </c>
+      <c r="D19" s="23" t="s">
         <v>304</v>
       </c>
-      <c r="D19" s="23" t="s">
-        <v>307</v>
-      </c>
       <c r="E19" s="23" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F19" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G19" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="F21" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G21" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G21" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="F22" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G22" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G22" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F23" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G23" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G23" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
+        <v>315</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>316</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>317</v>
+      </c>
+      <c r="E24" s="23" t="s">
         <v>318</v>
       </c>
-      <c r="B24" s="23" t="s">
-        <v>115</v>
-      </c>
-      <c r="C24" s="23" t="s">
-        <v>319</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>320</v>
-      </c>
-      <c r="E24" s="23" t="s">
-        <v>321</v>
-      </c>
       <c r="F24" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G24" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G24" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="F25" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G25" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G25" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="F26" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G26" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G26" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="F27" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G27" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G27" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F28" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G28" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G28" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="F29" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G29" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G29" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F30" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G30" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G30" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F31" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G31" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G31" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="F32" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G32" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G32" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>435</v>
+        <v>426</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>436</v>
+        <v>427</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="F35" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G35" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G35" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C36" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F36" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G36" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F37" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G37" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F38" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G38" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G38" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>396</v>
+        <v>391</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>405</v>
+        <v>397</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="F41" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G41" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G41" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
+        <v>356</v>
+      </c>
+      <c r="B42" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="C42" s="23" t="s">
+        <v>357</v>
+      </c>
+      <c r="D42" s="23" t="s">
+        <v>358</v>
+      </c>
+      <c r="E42" s="23" t="s">
         <v>359</v>
       </c>
-      <c r="B42" s="23" t="s">
-        <v>196</v>
-      </c>
-      <c r="C42" s="23" t="s">
-        <v>360</v>
-      </c>
-      <c r="D42" s="23" t="s">
-        <v>361</v>
-      </c>
-      <c r="E42" s="23" t="s">
-        <v>362</v>
-      </c>
       <c r="F42" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G42" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G42" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="F43" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G43" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G43" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="F44" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G44" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G44" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="F45" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G45" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G45" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>397</v>
+        <v>436</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>398</v>
+        <v>437</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>405</v>
+        <v>435</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="F47" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G47" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G47" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="F48" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G48" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G48" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="F49" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G49" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G49" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="F50" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G50" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G50" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F51" s="23" t="s">
+        <v>268</v>
+      </c>
+      <c r="G51" s="23" t="s">
         <v>269</v>
-      </c>
-      <c r="G51" s="23" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): RQNF-10 y RQF-06 Implementados en el Excel (71,6 %)
- RQNF-10 Implementado con la migracion 014 (PR #27): el pg_dump de
  notificacion y envio_mensaje sale identico al de produccion (verificador
  54b3cce, sec. 29.1 y 31). Observaciones: 13 tablas que aun difieren,
  prefijos 004/005 repetidos y src/db/migrations/001 sin aplicar.
- RQF-06 Implementado con el PR #23 (sec. 27.1, 29.2 y 31). Observaciones:
  un congelado con plan vigente todavia entra (RQF-04) y la deduplicacion
  es de 10 minutos.
- Trabajo pendiente: la migracion de RQNF-10 queda hecha por Luis (L1,
  PR #27), no Santiago; RQF-06 sale de la ruta.

Editado con Excel por COM. Avance: 26,5 de 37 = 71,6 % (RF 75,0 %, RNF 66,7 %).
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8D538E-11DB-4081-A0A9-4E811A40A7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F1B7FA-EDA1-4A10-AECB-607D0EC61349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="841" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="442">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -227,12 +227,6 @@
     <t>RQF-06</t>
   </si>
   <si>
-    <t>Valida el último plan y responde VENCIDO sin registrar el ingreso (checkin.js:116-136); la pantalla muestra «Acceso denegado» (CheckinPage.jsx:133-143).</t>
-  </si>
-  <si>
-    <t>Notificar al administrador del intento bloqueado: el intento no se guarda y la campana (notificaciones.js:96-108) solo lista membresías vencidas, no accesos denegados.</t>
-  </si>
-  <si>
     <t>HU-15</t>
   </si>
   <si>
@@ -797,9 +791,6 @@
     <t>Lista de verificación con capturas en Chrome, Firefox y Edge</t>
   </si>
   <si>
-    <t>Registrar el acceso bloqueado y mostrarlo en la campana del administrador</t>
-  </si>
-  <si>
     <t>Medio</t>
   </si>
   <si>
@@ -917,12 +908,6 @@
     <t>Inserción del ingreso con marca de tiempo automática.</t>
   </si>
   <si>
-    <t>backend/src/routes/checkin.js:116-136; frontend/src/pages/CheckinPage.jsx:133-143</t>
-  </si>
-  <si>
-    <t>Bloqueo de membresía vencida; no hay aviso del intento al administrador.</t>
-  </si>
-  <si>
     <t>EV-13</t>
   </si>
   <si>
@@ -1229,9 +1214,6 @@
     <t>Medir el check-in con un volumen realista (unos 200 miembros)</t>
   </si>
   <si>
-    <t>Migración que reconcilie envio_mensaje y notificacion con producción (o cambio del código), probada contra la copia de producción</t>
-  </si>
-  <si>
     <t>Orden de menor a mayor esfuerzo. «Avance global acumulado» suma los puntos de cada acción, en orden, sobre el avance actual y se pone verde al llegar a la meta. Lo decide Luis; el reparto de tareas está en docs/plan-trabajo.md.</t>
   </si>
   <si>
@@ -1334,12 +1316,6 @@
     <t>Parcial (2026-10-19): el registro de la fecha y el estado de cada envío no funciona con el esquema real. Santiago lo confirmó contra una copia de la base real (issue #24): envio_mensaje no tiene la columna canal (usa id_canal, con FK a canal_comunicacion, y exige mensaje_copiado NOT NULL; también tiene enviado_por), y canal_comunicacion solo tiene filas para los 3 gimnasios de ejemplo, así que no hay un id_canal válido. El endpoint responde 503 y el frontend oculta el error (MiembrosPage.jsx:847-849, MenuNotificaciones.jsx:95-98). El insert en notificacion (leido/leida y tipo) se corrige en el PR #23. Falta decidir cómo se crea el canal WhatsApp de cada gimnasio (bajo demanda o al registrarlo), qué se guarda en mensaje_copiado (el texto que se abrió en WhatsApp) y si enviado_por es el usuario del token. Además: solo WhatsApp por enlace wa.me; el estado no confirma la entrega y el correo no se usa para retención.</t>
   </si>
   <si>
-    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 011 y 013: la 009 (PR #14) crea auditoria y agrega las columnas y restricciones de gamificación de producción, la 010 (PR #17) el congelamiento, la 011 (PR #11) recrea vista_miembros_activos con id_gimnasio y la 013 (PR #19) agrega gimnasio.id_dueno.</t>
-  </si>
-  <si>
-    <t>Sigue Parcial (verificador: 94d5fbb, sección 15; confirmado contra una copia de la base real en el issue #24): una base hecha solo con migraciones todavía difiere de producción en 15 tablas, y el código usa dos de ellas. notificaciones.js:211 escribe envio_mensaje.canal, que en producción no existe (allí hay id_canal, con FK a canal_comunicacion, y mensaje_copiado NOT NULL); :217 escribe notificacion.leido, que allí es leida (lo corrige el PR #23, en revisión). Pasa a Implementado con una migración que reconcilie esas tablas, o un cambio del código, probado contra la copia de producción. Además hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica.</t>
-  </si>
-  <si>
     <t>Código / hallazgo</t>
   </si>
   <si>
@@ -1352,22 +1328,46 @@
     <t>2026-10-19</t>
   </si>
   <si>
-    <t>backend/src/db/migrate.js:15-56; backend/src/index.js:128-132; backend/migrations/ (009, 010, 011 y 013); issue #24</t>
-  </si>
-  <si>
-    <t>Migraciones versionadas aplicadas al iniciar. Quedan diferencias con producción en envio_mensaje y notificacion (verificador 94d5fbb §15; issue #24).</t>
-  </si>
-  <si>
-    <t>notificaciones.js:211 escribe envio_mensaje.canal, que no existe en el esquema de producción (issue #24); notificacion.leido lo corrige el PR #23.</t>
-  </si>
-  <si>
-    <t>Estado actualizado el 2026-10-19 con los PR fusionados en develop @ dcda269 (#9, #11 y #14 a #22) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
-  </si>
-  <si>
     <t>POST /api/admin/notificaciones/enviado no guarda nada con el esquema real: envio_mensaje usa id_canal (FK a canal_comunicacion, sin filas para los gimnasios reales) y exige mensaje_copiado (issue #24).</t>
   </si>
   <si>
     <t>Buscar o crear el canal WhatsApp del gimnasio, mandar el mensaje desde el frontend e insertar en envio_mensaje con id_canal, mensaje_copiado y enviado_por, con una prueba contra el esquema real (issue #24)</t>
+  </si>
+  <si>
+    <t>Valida el último plan en el check-in (checkin.js:123-131) y, si está vencido o no hay plan, bloquea y responde VENCIDO sin registrar asistencia (:133-147; el INSERT en checkin de :182 queda fuera de ese camino); la pantalla muestra «Acceso denegado» (CheckinPage.jsx:134-135, :187-188). Avisa al administrador: registrarAccesoBloqueado (lib/accesos.js:33) guarda el intento en notificacion sin repetirlo en 10 minutos (:20, :39-49) y la campana lo muestra primero (notificaciones.js:74-109, :168-182), con «Visto» (:216-231) y refresco cada 30 s (MenuNotificaciones.jsx:52, :72). PR #23, con la migración 014 (PR #27) para Docker.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-19; verificador 54b3cce, secciones 27.1, 29.2 y 31). Observaciones: un miembro congelado con el plan vigente todavía entra (la parte de RQF-04 que le falta a Santiago) y uno congelado con el plan vencido aparece como «Membresía vencida»; la deduplicación es de 10 minutos y la campana no agrupa por miembro.</t>
+  </si>
+  <si>
+    <t>applyMigrations lee backend/migrations en orden, aplica solo las pendientes y las registra en schema_migrations (migrate.js:15-56); se ejecuta al arrancar (index.js:128-132). Migraciones 002 a 011, 013 y 014: la 009 (PR #14) crea auditoria y las columnas de gamificación de producción, la 010 (PR #17) el congelamiento, la 011 (PR #11) recrea vista_miembros_activos con id_gimnasio, la 013 (PR #19) agrega gimnasio.id_dueno y la 014 (PR #27) reconstruye notificacion y envio_mensaje con el DDL de ConsultasDB (014:118, :267): el pg_dump -s de esas dos tablas y sus secuencias sale idéntico al de producción, sin perder filas.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-19; verificador 54b3cce, secciones 29.1 y 31): las migraciones describen el esquema de producción en las dos tablas que el código escribe, con el pg_dump idéntico. Observaciones: todavía difieren 13 tablas que el código no usa (sección 15); hay prefijos repetidos (004 y 005) y backend/src/db/migrations/001_invitacion_staff.sql no se aplica. Antes de desplegar, correr la 014 en una copia de producción dentro de BEGIN; … ROLLBACK; y confirmar que imprime dos veces «sin cambios».</t>
+  </si>
+  <si>
+    <t>backend/src/routes/checkin.js:123-147, :182; backend/src/lib/accesos.js:20, :33-52; backend/src/routes/notificaciones.js:74-109, :168-182, :216-231; frontend/src/components/MenuNotificaciones.jsx:52, :72; frontend/src/pages/CheckinPage.jsx:134-135</t>
+  </si>
+  <si>
+    <t>Bloqueo sin contar asistencia y aviso al administrador en la campana, sin repetirse en 10 minutos (PR #23).</t>
+  </si>
+  <si>
+    <t>backend/src/db/migrate.js:15-56; backend/src/index.js:128-132; backend/migrations/ (009, 010, 011, 013 y 014); informe del verificador, commit 54b3cce, §29.1 y §31</t>
+  </si>
+  <si>
+    <t>Migraciones versionadas aplicadas al iniciar; con la 014, notificacion y envio_mensaje quedan como en producción (pg_dump idéntico).</t>
+  </si>
+  <si>
+    <t>Hecho: la migración 014 reconcilia envio_mensaje y notificacion con producción (pg_dump idéntico). Estaba asignada por error a Santiago; la hizo Luis en la tarea L1.</t>
+  </si>
+  <si>
+    <t>Migración que reconcilie envio_mensaje y notificacion con producción (hecha: 014, PR #27)</t>
+  </si>
+  <si>
+    <t>Luis (L1, PR #27)</t>
+  </si>
+  <si>
+    <t>Estado actualizado el 2026-10-19 con los PR fusionados en develop @ 66186d7 (#9, #11, #14 a #23, #25 y #27) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
   </si>
 </sst>
 </file>
@@ -1749,13 +1749,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.72727272727272729</c:v>
+                  <c:v>0.75</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.6333333333333333</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.68918918918918914</c:v>
+                  <c:v>0.71621621621621623</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1919,10 +1919,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>11</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>6</c:v>
@@ -2337,7 +2337,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2382,11 +2382,11 @@
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.72727272727272729</v>
+        <v>0.75</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2402,14 +2402,14 @@
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>1.6000000000000014</v>
+        <v>1.1000000000000014</v>
       </c>
       <c r="J6" t="s">
         <v>12</v>
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
@@ -2422,11 +2422,11 @@
       </c>
       <c r="D7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Implementado")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Parcial")</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Pendiente")</f>
@@ -2434,7 +2434,7 @@
       </c>
       <c r="G7" s="9">
         <f>IF(C7=0,0,SUM(RNF!$F$2:$F$100)/C7)</f>
-        <v>0.6333333333333333</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="H7" s="10">
         <f>Resumen!$C$40</f>
@@ -2442,14 +2442,14 @@
       </c>
       <c r="I7" s="11">
         <f>MAX(0,H7*C7-G7*C7)</f>
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="J7" t="s">
         <v>14</v>
       </c>
       <c r="K7">
         <f>E8</f>
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
@@ -2462,11 +2462,11 @@
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.68918918918918914</v>
+        <v>0.71621621621621623</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>4.1000000000000014</v>
+        <v>3.1000000000000014</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
@@ -2532,11 +2532,11 @@
       </c>
       <c r="D31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Implementado",RF!$G$2:$G$100,"Original")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Parcial",RF!$G$2:$G$100,"Original")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Pendiente",RF!$G$2:$G$100,"Original")</f>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="G31" s="9">
         <f>IF(C31=0,0,SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")/C31)</f>
-        <v>0.58333333333333337</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
@@ -2582,11 +2582,11 @@
       </c>
       <c r="D33" s="13">
         <f>D31+D32</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E33" s="13">
         <f>E31+E32</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F33" s="13">
         <f>F31+F32</f>
@@ -2594,7 +2594,7 @@
       </c>
       <c r="G33" s="14">
         <f>IF(C33=0,0,(SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")+SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original"))/C33)</f>
-        <v>0.57499999999999996</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
@@ -2706,10 +2706,10 @@
         <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2739,10 +2739,10 @@
         <v>12</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2805,10 +2805,10 @@
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2860,7 +2860,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
         <v>60</v>
       </c>
@@ -2868,46 +2868,46 @@
         <v>54</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>61</v>
+        <v>430</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>62</v>
+        <v>431</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G7" s="24" t="s">
         <v>34</v>
       </c>
       <c r="H7" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="23" t="s">
+        <v>62</v>
+      </c>
+      <c r="J7" s="23" t="s">
         <v>63</v>
-      </c>
-      <c r="I7" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2917,30 +2917,30 @@
         <v>34</v>
       </c>
       <c r="H8" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="I8" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="23" t="s">
         <v>68</v>
-      </c>
-      <c r="I8" s="23" t="s">
-        <v>69</v>
-      </c>
-      <c r="J8" s="23" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2950,30 +2950,30 @@
         <v>34</v>
       </c>
       <c r="H9" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="J9" s="23" t="s">
         <v>75</v>
-      </c>
-      <c r="I9" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="216" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2983,30 +2983,30 @@
         <v>34</v>
       </c>
       <c r="H10" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="J10" s="23" t="s">
         <v>79</v>
-      </c>
-      <c r="I10" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3016,30 +3016,30 @@
         <v>34</v>
       </c>
       <c r="H11" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="J11" s="23" t="s">
         <v>86</v>
-      </c>
-      <c r="I11" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3049,30 +3049,30 @@
         <v>34</v>
       </c>
       <c r="H12" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="J12" s="23" t="s">
         <v>93</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3082,51 +3082,51 @@
         <v>34</v>
       </c>
       <c r="H13" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="J13" s="23" t="s">
         <v>99</v>
-      </c>
-      <c r="I13" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="J13" s="23" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="I14" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="J14" s="23" t="s">
         <v>105</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>43</v>
@@ -3135,97 +3135,97 @@
         <v>14</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H15" s="23" t="s">
+        <v>109</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="J15" s="23" t="s">
         <v>111</v>
-      </c>
-      <c r="I15" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="J15" s="23" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H16" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="J16" s="23" t="s">
         <v>118</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>119</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H17" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>124</v>
+      </c>
+      <c r="J17" s="23" t="s">
         <v>125</v>
-      </c>
-      <c r="I17" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="J17" s="23" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>33</v>
@@ -3234,40 +3234,40 @@
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H18" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="I18" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="J18" s="23" t="s">
         <v>131</v>
-      </c>
-      <c r="I18" s="23" t="s">
-        <v>132</v>
-      </c>
-      <c r="J18" s="23" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E19" s="23" t="s">
         <v>56</v>
@@ -3277,21 +3277,21 @@
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H19" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="I19" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="J19" s="23" t="s">
         <v>136</v>
-      </c>
-      <c r="I19" s="23" t="s">
-        <v>137</v>
-      </c>
-      <c r="J19" s="23" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>33</v>
@@ -3300,7 +3300,7 @@
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E20" s="23" t="s">
         <v>56</v>
@@ -3310,54 +3310,54 @@
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H21" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="J21" s="23" t="s">
         <v>147</v>
-      </c>
-      <c r="I21" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="J21" s="23" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>43</v>
@@ -3366,59 +3366,59 @@
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H22" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="I22" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="J22" s="23" t="s">
         <v>153</v>
-      </c>
-      <c r="I22" s="23" t="s">
-        <v>154</v>
-      </c>
-      <c r="J22" s="23" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H23" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="I23" s="23" t="s">
+        <v>157</v>
+      </c>
+      <c r="J23" s="23" t="s">
         <v>158</v>
-      </c>
-      <c r="I23" s="23" t="s">
-        <v>159</v>
-      </c>
-      <c r="J23" s="23" t="s">
-        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -3497,19 +3497,19 @@
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3522,27 +3522,27 @@
         <v>56</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3555,27 +3555,27 @@
         <v>56</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3588,27 +3588,27 @@
         <v>56</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3618,30 +3618,30 @@
         <v>34</v>
       </c>
       <c r="H5" s="23" t="s">
+        <v>180</v>
+      </c>
+      <c r="I5" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="J5" s="23" t="s">
         <v>182</v>
-      </c>
-      <c r="I5" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3651,30 +3651,30 @@
         <v>34</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3687,27 +3687,27 @@
         <v>56</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3720,27 +3720,27 @@
         <v>56</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3753,123 +3753,123 @@
         <v>56</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H10" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I10" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="J10" s="23" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="J10" s="23" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="158.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>212</v>
-      </c>
       <c r="B11" s="23" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C11" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H11" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H12" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E13" s="23" t="s">
         <v>56</v>
@@ -3879,30 +3879,30 @@
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H13" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>56</v>
@@ -3912,30 +3912,30 @@
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H14" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>56</v>
@@ -3945,49 +3945,49 @@
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H15" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H16" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -4017,7 +4017,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4041,40 +4041,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>240</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D2" s="23" t="s">
+        <v>241</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>242</v>
+      </c>
+      <c r="F2" s="24" t="s">
         <v>243</v>
-      </c>
-      <c r="E2" s="23" t="s">
-        <v>244</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>245</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4082,28 +4082,28 @@
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.71621621621621623</v>
+        <v>0.7432432432432432</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>393</v>
+        <v>388</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4111,28 +4111,28 @@
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.72972972972972971</v>
+        <v>0.7567567567567568</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4140,28 +4140,28 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.7432432432432432</v>
+        <v>0.77027027027027029</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>440</v>
+        <v>428</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>441</v>
+        <v>429</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4169,28 +4169,28 @@
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.7567567567567568</v>
+        <v>0.78378378378378377</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4198,28 +4198,28 @@
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.77027027027027029</v>
+        <v>0.79729729729729726</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4227,28 +4227,28 @@
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.78378378378378377</v>
+        <v>0.81081081081081086</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B8" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4256,86 +4256,86 @@
       </c>
       <c r="H8" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.79729729729729726</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.82432432432432434</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>60</v>
+        <v>159</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>62</v>
+        <v>378</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>251</v>
+        <v>389</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H9" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.81081081081081086</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.85135135135135132</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>161</v>
+        <v>49</v>
       </c>
       <c r="B10" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>383</v>
+        <v>399</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H10" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.83783783783783783</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.86486486486486491</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="B11" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>405</v>
+        <v>72</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>406</v>
+        <v>251</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
@@ -4343,28 +4343,28 @@
       </c>
       <c r="H11" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.85135135135135132</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.8783783783783784</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>71</v>
+        <v>193</v>
       </c>
       <c r="B12" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>74</v>
+        <v>196</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4372,86 +4372,86 @@
       </c>
       <c r="H12" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>0.86486486486486491</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.89189189189189189</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="B13" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Implementado</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>198</v>
+        <v>438</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>255</v>
+        <v>439</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>244</v>
+        <v>440</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G13" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H13" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G13))/Resumen!$C$8</f>
-        <v>0.8783783783783784</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.89189189189189189</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>212</v>
+        <v>87</v>
       </c>
       <c r="B14" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>438</v>
+        <v>90</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>395</v>
+        <v>253</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G14" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H14" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G14))/Resumen!$C$8</f>
-        <v>0.89189189189189189</v>
+        <v>0.91891891891891897</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>89</v>
+        <v>164</v>
       </c>
       <c r="B15" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>92</v>
+        <v>167</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G15" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
@@ -4459,28 +4459,28 @@
       </c>
       <c r="H15" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G15))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>166</v>
+        <v>94</v>
       </c>
       <c r="B16" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>169</v>
+        <v>96</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="G16" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
@@ -4488,28 +4488,28 @@
       </c>
       <c r="H16" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G16))/Resumen!$C$8</f>
-        <v>0.94594594594594594</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.97297297297297303</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="B17" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="G17" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
@@ -4517,45 +4517,16 @@
       </c>
       <c r="H17" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G17))/Resumen!$C$8</f>
-        <v>0.97297297297297303</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="B18" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C18" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D18" s="23" t="s">
-        <v>260</v>
-      </c>
-      <c r="E18" s="23" t="s">
-        <v>244</v>
-      </c>
-      <c r="F18" s="24" t="s">
-        <v>259</v>
-      </c>
-      <c r="G18" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A18,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A18,RNF!$A$2:$A$100,0)))</f>
         <v>1</v>
       </c>
-      <c r="H18" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G18))/Resumen!$C$8</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="17" t="s">
-        <v>396</v>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="17" t="s">
+        <v>390</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B18">
+  <conditionalFormatting sqref="B2:B17">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Implementado"</formula>
     </cfRule>
@@ -4587,7 +4558,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H2:H18</xm:sqref>
+          <xm:sqref>H2:H17</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4611,30 +4582,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="G1" s="6" t="s">
         <v>263</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>264</v>
-      </c>
-      <c r="F1" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4643,44 +4614,44 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>38</v>
@@ -4689,21 +4660,21 @@
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>38</v>
@@ -4712,21 +4683,21 @@
         <v>23</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>42</v>
@@ -4735,21 +4706,21 @@
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>42</v>
@@ -4758,21 +4729,21 @@
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>49</v>
@@ -4781,44 +4752,44 @@
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>49</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>53</v>
@@ -4827,44 +4798,44 @@
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>53</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B12" s="23" t="s">
         <v>60</v>
@@ -4873,783 +4844,783 @@
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>291</v>
+        <v>434</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>292</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>268</v>
+        <v>435</v>
+      </c>
+      <c r="F12" s="28" t="s">
+        <v>427</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C14" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C15" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>432</v>
+        <v>424</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>433</v>
+        <v>425</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>434</v>
+        <v>426</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>386</v>
+        <v>381</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C36" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>387</v>
+        <v>382</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="E40" s="23" t="s">
+        <v>386</v>
+      </c>
+      <c r="F40" s="27" t="s">
         <v>391</v>
       </c>
-      <c r="F40" s="27" t="s">
-        <v>397</v>
-      </c>
       <c r="G40" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="F42" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
@@ -5661,130 +5632,130 @@
         <v>437</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>435</v>
+        <v>427</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): RQF-13, RQF-14, RQF-04, RQF-11 y RQNF-07 Implementados en el Excel (79,7 %)
- RQF-14 y RQF-13 (PR #10), con la limitacion de despliegue que decidio
  Luis: Render y la imagen Docker no tienen Chrome, asi que WhatsApp solo
  envia en un equipo con Chrome, el QR escaneado y ENABLE_WHATSAPP activo.
- RQF-04 (PR #30): el check-in niega a las congeladas y el job las salta.
- RQF-11 (PR #32), desde Pendiente: rachas, hitos y su configuracion.
- RQNF-07 (PR #33): script test y 122 pruebas; nueva evidencia
  docs/evidencias/cobertura-backend-2026-10-20.txt.
- RQF-02 cierra la observacion del kiosco (marcarActividad en el check-in).
- Salen de la ruta los cinco que quedaron Implementados.

Editado con Excel por COM. Avance: 29,5 de 37 = 79,7 % (RF 86,4 %, RNF 70,0 %).
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77F1B7FA-EDA1-4A10-AECB-607D0EC61349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9AFFD6-E7B4-44E4-A840-6571AC1291F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="836" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="435">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -311,12 +311,6 @@
     <t>Gamificación</t>
   </si>
   <si>
-    <t>La app del miembro lee hitos y su estado (cliente.js:340-381, gamificacion_screen.dart), pero ningún archivo calcula rachas ni escribe hito_miembro; los datos que existen vienen del script ConsultasDB/Poblar_Tablas.sql:384-419.</t>
-  </si>
-  <si>
-    <t>Cálculo de rachas en cada check-in, otorgar hitos, mensaje en la pantalla de check-in y configuración de hitos por el administrador.</t>
-  </si>
-  <si>
     <t>HU-25, HU-26, HU-27, HU-47, HU-48</t>
   </si>
   <si>
@@ -365,12 +359,6 @@
     <t>RQF-14</t>
   </si>
   <si>
-    <t>Cron diario a las 9:00 a.m. America/Bogota (scheduler.js:46); selección de planes por vencer y control de duplicados (expiracion.js:43, :74, :94, :117); 0 días desactiva el aviso (expiracion.js:151); POST /api/jobs/expiracion/run y GET /api/jobs/expiracion/preview (jobs.js:27, :38); migraciones 006 y 007.</t>
-  </si>
-  <si>
-    <t>Si WhatsApp no está listo, sendWhatsAppText vuelve sin error (whatsapp.js:228-231) y el job marca el aviso como enviado (expiracion.js:206-207), así que nunca lo reintenta; en Render no hay Chrome (whatsapp.js:7-25). Los días de anticipación (gimnasio.dias_aviso_vencimiento) solo se cambian en la base de datos: PUT /admin/config no los acepta (config.js:20-30).</t>
-  </si>
-  <si>
     <t>HU-55</t>
   </si>
   <si>
@@ -629,12 +617,6 @@
     <t>Mantenibilidad</t>
   </si>
   <si>
-    <t>Capas en backend/src (routes, lib, middleware, jobs, db) y diagrama de arquitectura en el documento (sección 8). Cobertura medida el 2026-10-16: 0 % en routes/checkin.js y routes/notificaciones.js, 1,48 % de líneas en todo el backend; 23 pruebas, 2 fallan.</t>
-  </si>
-  <si>
-    <t>Script «test» en backend/package.json, pruebas de check-in y alertas hasta ≥ 70 % y corregir las 2 pruebas que fallan.</t>
-  </si>
-  <si>
     <t>EV-41, EV-42</t>
   </si>
   <si>
@@ -776,9 +758,6 @@
     <t>Bajo</t>
   </si>
   <si>
-    <t>No marcar el aviso como enviado si WhatsApp no está listo (reintentar) y llevar los días a Configuración</t>
-  </si>
-  <si>
     <t>Límite de intentos en verify-reset-code y reset-password</t>
   </si>
   <si>
@@ -800,12 +779,6 @@
     <t>Motor diario con Alerta Amarilla / Roja y umbrales editables</t>
   </si>
   <si>
-    <t>Script test, pruebas de check-in y alertas hasta ≥ 70 % de cobertura</t>
-  </si>
-  <si>
-    <t>Cálculo de rachas, hitos y mensaje en el check-in</t>
-  </si>
-  <si>
     <t>Monitor externo de disponibilidad con reporte (depende del plan de Render)</t>
   </si>
   <si>
@@ -935,12 +908,6 @@
     <t>Código / datos</t>
   </si>
   <si>
-    <t>backend/src/routes/cliente.js:340-381; ConsultasDB/Poblar_Tablas.sql:384-419</t>
-  </si>
-  <si>
-    <t>Hitos solo de lectura, cargados por SQL; no hay cálculo de rachas.</t>
-  </si>
-  <si>
     <t>backend/src/routes/cliente.js:392-418; ConsultasDB/Poblar_Tablas.sql:456-490</t>
   </si>
   <si>
@@ -950,21 +917,9 @@
     <t>EV-20</t>
   </si>
   <si>
-    <t>backend/src/jobs/scheduler.js:46; backend/src/jobs/expiracion.js:43, :74, :94, :117, :151</t>
-  </si>
-  <si>
-    <t>Aviso diario automático de vencimiento, sin duplicados.</t>
-  </si>
-  <si>
     <t>EV-21</t>
   </si>
   <si>
-    <t>backend/src/routes/jobs.js:27, :38; backend/migrations/006_gimnasio_dias_aviso.sql; 007_alerta_vencimiento_enviada.sql</t>
-  </si>
-  <si>
-    <t>Ejecución manual y vista previa; días de aviso y anti-duplicado en BD.</t>
-  </si>
-  <si>
     <t>EV-22</t>
   </si>
   <si>
@@ -1103,21 +1058,9 @@
     <t>Medición</t>
   </si>
   <si>
-    <t>docs/evidencias/cobertura-backend-2026-10-16.txt</t>
-  </si>
-  <si>
-    <t>Cobertura 0 % en checkin.js y notificaciones.js; 23 pruebas, 2 fallan.</t>
-  </si>
-  <si>
     <t>EV-42</t>
   </si>
   <si>
-    <t>backend/src/{routes,lib,middleware,jobs,db}; backend/package.json (sin script test); backend/jest.config.js:15-18</t>
-  </si>
-  <si>
-    <t>Arquitectura en capas; las pruebas no se ejecutan con npm test.</t>
-  </si>
-  <si>
     <t>backend/Dockerfile; frontend/Dockerfile; frontend/nginx.conf; docker-compose.yml; render.yaml; vercel.json</t>
   </si>
   <si>
@@ -1166,12 +1109,6 @@
     <t>Rutas relativas a la raíz del repositorio en main @ 54b19fa (el CI de RQNF-11 en 8acab31). No se hicieron pruebas en vivo: la verificación es por lectura de código, pruebas existentes y CI.</t>
   </si>
   <si>
-    <t>POST /api/admin/miembros/:id/contrato/enviar con control de gimnasio (admin-contrato.js:76-92); vista previa e historial por API (:167, :195); botón «Enviar contrato» (MiembrosPage.jsx:855-880, :1735). Desde el PR #9, sendWhatsAppText lanza un error si el módulo está apagado, el cliente no está listo, el teléfono no es válido o el envío falla (whatsapp.js:223-246), y admin-contrato.js:130-138 registra exito = false; 5 pruebas en backend/tests/whatsapp-text.test.js.</t>
-  </si>
-  <si>
-    <t>Sigue Parcial (criterio del 2026-10-18): el aviso al administrador y el registro de cada intento ya son correctos, pero tras cada reinicio del servidor el contrato no sale. admin-contrato.js:107 pregunta isWhatsAppReady() antes de enviar y el cliente se inicia de forma perezosa (whatsapp.js:146), así que responde «no autenticado» sin llegar a iniciar el cliente ni a mostrar el QR que pide escanear; solo funciona si otro flujo lo inició antes (alta de un miembro con teléfono). Arreglo: quitar esa comprobación previa (sendWhatsAppText ya lanza el error) o iniciar el cliente antes, junto con la corrección del PR #10. Verificador: 386d168, sección 14.3.</t>
-  </si>
-  <si>
     <t>Cada gimnasio nuevo se crea por registro, sin tocar código (auth.js:100, :134); las consultas filtran por el id_gimnasio del token (p. ej. miembros.js:358, checkin.js:76, dashboard.js:123, notificaciones.js:199). Desde el PR #11: vista.js exige rol de personal (:20), rechaza al personal sin gimnasio (:28) y filtra por gimnasio (:32, :46) sobre la vista de la migración 011; asistencia.js exige rol de personal (:22); checkin.js deriva la clave del QR una sola vez (:26, :31). 9 pruebas en backend/tests/aislamiento.test.js.</t>
   </si>
   <si>
@@ -1184,12 +1121,6 @@
     <t>Código / prueba</t>
   </si>
   <si>
-    <t>backend/src/routes/admin-contrato.js:76-160, :107, :130-138, :167, :195; backend/src/lib/whatsapp.js:146, :223-246; backend/tests/whatsapp-text.test.js; backend/migrations/008_contrato_enviado.sql; frontend/src/pages/MiembrosPage.jsx:855-880</t>
-  </si>
-  <si>
-    <t>Envío del contrato con registro de cada intento; el error del envío ya llega al registro (exito = false). Tras un reinicio no se inicia el cliente (admin-contrato.js:107).</t>
-  </si>
-  <si>
     <t>backend/src/routes/auth.js:100, :134; vista.js:20, :28, :32, :46; asistencia.js:22; checkin.js:26, :31, :76; miembros.js:358; dashboard.js:123; notificaciones.js:199</t>
   </si>
   <si>
@@ -1205,12 +1136,6 @@
     <t>La vista y asistencia rechazan tokens de miembro y filtran por gimnasio; la 011 expone id_gimnasio.</t>
   </si>
   <si>
-    <t>Tras un reinicio el contrato no sale: admin-contrato.js:107 pregunta isWhatsAppReady() y nunca inicia el cliente de WhatsApp (whatsapp.js:146).</t>
-  </si>
-  <si>
-    <t>Quitar la comprobación previa de admin-contrato.js:107 (o iniciar el cliente antes de preguntar), junto con el arreglo del PR #10</t>
-  </si>
-  <si>
     <t>Medir el check-in con un volumen realista (unos 200 miembros)</t>
   </si>
   <si>
@@ -1220,36 +1145,15 @@
     <t>2026-10-18</t>
   </si>
   <si>
-    <t>Cálculo automático de fecha_fin según el plan (miembros.js:193, :395); estado vencido / por vencer contra la fecha actual (:286-290); renovación del plan (:926). Estado Congelada (PR #17, migración 010): POST /api/admin/miembros/:id/congelar (:810) y /descongelar (:869), que corre fecha_fin y la próxima fecha de cobro los días congelados (:892), con historial en congelacion_plan; la lista marca la membresía congelada y no la cuenta como vencida (:286); pantalla en MiembrosPage.jsx:238, :742, :1907.</t>
-  </si>
-  <si>
-    <t>Sigue Parcial (decisión de Luis, 2026-10-18): congelar y descongelar ya están en develop (PR #17; verificador 1be53f7, sección 18.2), pero falta que Santiago haga que el job de avisos de vencimiento (expiracion.js) y el check-in salten las membresías congeladas. El check-in debe negar el ingreso con estado CONGELADO y el mensaje «Tu membresía está congelada. Pide en recepción que la reactiven para poder ingresar.». Hoy el job le mandaría a un miembro congelado el aviso de que su plan vence, y el check-in lo deja entrar. Pasa a Implementado cuando esos dos cambios estén fusionados y verificados. Menores: congelar entre las 19:00 y las 24:00 de Colombia toma la fecha del día siguiente (CURRENT_DATE en UTC), y renovar el plan mientras está congelado conserva congelado_desde.</t>
-  </si>
-  <si>
     <t>backend/src/routes/miembros.js:193, :395, :286-290, :926</t>
   </si>
   <si>
-    <t>backend/migrations/010_congelar_membresia.sql; backend/src/routes/miembros.js:810, :869, :892; frontend/src/pages/MiembrosPage.jsx:238, :742, :1907</t>
-  </si>
-  <si>
-    <t>Congelar y descongelar con historial y corrimiento del vencimiento (PR #17). Falta que el job y el check-in salten las congeladas.</t>
-  </si>
-  <si>
     <t>Informe del verificador: commit 94d5fbb, docs/verificacion-requisitos.md §16; commit 1be53f7, §21.2</t>
   </si>
   <si>
     <t>Con el handler real en PostgreSQL 18: 200 sin filas del gimnasio y sin tocar el otro; 403 al admin invitado y con la contraseña mala; 500 sin borrar nada si una FK desconocida lo bloquea.</t>
   </si>
   <si>
-    <t>Que el job de vencimientos y el check-in salten las membresías congeladas (check-in con estado CONGELADO); congelar y descongelar ya están en develop (PR #17).</t>
-  </si>
-  <si>
-    <t>Job de vencimientos y check-in que salten las membresías congeladas (check-in con estado CONGELADO)</t>
-  </si>
-  <si>
-    <t>Si WhatsApp no está listo, sendWhatsAppText vuelve sin error (whatsapp.js:228-231) y el job marca el aviso como enviado (expiracion.js:206-207), así que nunca lo reintenta; en Render no hay Chrome (whatsapp.js:7-25). Los días de anticipación (gimnasio.dias_aviso_vencimiento) solo se cambian en la base de datos: PUT /admin/config no los acepta (config.js:20-30). Además, el job no salta las membresías congeladas (expiracion.js:43-65; verificador 1be53f7, sección 18.2): le avisaría a un miembro congelado que su plan vence.</t>
-  </si>
-  <si>
     <t>Crear cuentas por invitación (POST /api/admin/staff/invite, staff.js:133), listar el personal (:357) y las invitaciones (:222), revocarlas (:251) y aceptar la invitación, que crea la cuenta (:499). PATCH /api/admin/staff/:id (:388) edita el nombre y el rol y desactiva o reactiva la cuenta; protege al dueño (OWNER_PROTECTED, :424) y no deja que uno se quite el acceso a sí mismo (SELF_LOCKOUT, :421). authenticate vuelve a leer al personal en cada petición (middleware/auth.js:10, :78): una cuenta desactivada o movida de gimnasio pierde el acceso en la siguiente petición, y el rol sale de la base. Dueño explícito en gimnasio.id_dueno (migración 013; registro en auth.js:157-162; sqlIdDueno en auth-helpers.js:188). Pantalla: StaffPage.jsx:138 (editar), :421 y :434 (desactivar y reactivar). PR #19.</t>
   </si>
   <si>
@@ -1259,9 +1163,6 @@
     <t>POST /api/auth/login con bcrypt (auth.js:212, :243) y límite de 5 intentos por minuto (index.js:63, :79); cierre manual (auth.js:313, AuthContext.jsx:223). El JWT del personal siempre vence: 8 h por defecto o JWT_EXPIRES_IN, y 8 h si la configuración no es válida (vigenciaTokenPersonal y generarToken, auth-helpers.js:113, :135-143); authenticate rechaza los tokens sin vencimiento (401 TOKEN_SIN_VENCIMIENTO, middleware/auth.js:63). Cierre automático tras 30 min sin actividad, compartido entre pestañas (AuthContext.jsx:23-27, :40, :150-178), al vencer el token y ante un 401 (api.js:115). PR #18.</t>
   </si>
   <si>
-    <t>Implementado (2026-10-18; verificador b8f99d2, secciones 22.6 y 25.4). Observaciones: CheckinPage.jsx (zona de Santiago) todavía no llama a marcarActividad() (AuthContext.jsx:219), así que un kiosco que solo usa la cámara se cierra a los 30 min. La vigencia no está alineada: render.yaml:19 usa 24h y docker-compose.yml:61, 7d (se recomienda 8h). Con JWT_EXPIRES_IN en 0 o negativo el token nace vencido. 4 pruebas de aislamiento.test.js firman tokens sin vencimiento y fallan (arreglo de una línea de Santiago).</t>
-  </si>
-  <si>
     <t>GET /api/admin/dashboard: miembros activos (dashboard.js:165, :190), entradas de hoy con el día cortado en hora de Colombia (:170; ayudantes enHoraLocal e inicioLocal en :69 y :74), semana desde el lunes de Colombia (:233) y próximos vencimientos a 30 días (:248), sin las membresías congeladas (:85, :187, :256). GET /api/admin/dashboard/horas-pico (:344; periodos en :337 y hora local en :356): entradas por hora y hora pico. DashboardPage.jsx: gráfica BarsHoras (:172), que abre en «Hoy» (:226); refresco cada 60 s con la pestaña visible y al volver a ella (REFRESCO_MS :49, :279-288), sin cargas en paralelo (:239-246); listado de próximos vencimientos (:610-626). PR #16 y #22.</t>
   </si>
   <si>
@@ -1286,12 +1187,6 @@
     <t>El rol y el acceso se leen de la base en cada petición; dueño explícito en gimnasio.id_dueno.</t>
   </si>
   <si>
-    <t>backend/src/routes/auth.js:212, :243, :313; backend/src/index.js:63, :79; frontend/src/context/AuthContext.jsx:23-27, :40, :150-178, :223; frontend/src/api.js:115</t>
-  </si>
-  <si>
-    <t>Login con bcrypt y límite de intentos, cierre manual y cierre automático por inactividad, vencimiento o 401 (PR #18).</t>
-  </si>
-  <si>
     <t>backend/src/lib/auth-helpers.js:113, :135-143; backend/src/middleware/auth.js:63</t>
   </si>
   <si>
@@ -1367,7 +1262,91 @@
     <t>Luis (L1, PR #27)</t>
   </si>
   <si>
-    <t>Estado actualizado el 2026-10-19 con los PR fusionados en develop @ 66186d7 (#9, #11, #14 a #23, #25 y #27) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
+    <t>POST /api/admin/miembros/:id/contrato/enviar con control de gimnasio (admin-contrato.js:76-92); vista previa e historial por API (:153, :181); botón «Enviar contrato» (MiembrosPage.jsx:901, :1784). Desde el PR #10 ya no se pregunta isWhatsAppReady() antes de enviar: sendWhatsAppText inicia el cliente perezoso y, si no queda listo, lanza WHATSAPP_NO_LISTO (whatsapp.js:229-238); admin-contrato.js:105-116 registra exito = false con la guía del QR y cliente_listo (:145). Pruebas en backend/tests/contrato.test.js y whatsapp-text.test.js.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, sección 33.1). Limitación de despliegue, por decisión de Luis: Render (render.yaml, entorno node) y la imagen Docker (Dockerfile:13, :29, PUPPETEER_SKIP_DOWNLOAD=true, sin chromium) no tienen Chrome, así que el envío por WhatsApp solo funciona en un equipo con Chrome, con el QR escaneado y ENABLE_WHATSAPP activo. En el entorno desplegado el contrato no sale, pero el intento queda registrado con exito = false.</t>
+  </si>
+  <si>
+    <t>Cron a las 9:00 y a las 15:00 (reintento) en America/Bogota (scheduler.js:62-63); selección de planes por vencer sin las membresías congeladas (expiracion.js:43-62); un aviso al entrar en la ventana y otro el día 0, y si el servidor estuvo dormido ese día sale al siguiente (:101-103, :156-168); el aviso solo se marca si el envío no falla (:217-218), y sendWhatsAppText inicia el cliente y lanza WHATSAPP_NO_LISTO si no queda listo (whatsapp.js:229-238). Días de aviso por gimnasio desde Configuración, entre 0 y 30 (config.js:33, :119; ConfigPage.jsx:236-239). POST /api/jobs/expiracion/run y GET /api/jobs/expiracion/preview (jobs.js:27, :38); migraciones 006 y 007. Pruebas en backend/tests/expiracion.test.js. PR #10 y #30.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, secciones 33.1 y 33.2). Limitación de despliegue, por decisión de Luis: Render (render.yaml, entorno node) y la imagen Docker (Dockerfile:13, :29, PUPPETEER_SKIP_DOWNLOAD=true, sin chromium) no tienen Chrome, así que el envío por WhatsApp solo funciona en un equipo con Chrome, con el QR escaneado y ENABLE_WHATSAPP activo. En el entorno desplegado los avisos no se marcan como enviados y se reintentan en la corrida siguiente. Además, el cron vive dentro del proceso web: si Render tiene el servicio dormido a las 9:00 y a las 15:00, no corre.</t>
+  </si>
+  <si>
+    <t>Cálculo automático de fecha_fin según el plan (miembros.js:193, :395); estado vencido / por vencer contra la fecha actual (:286-290); renovación del plan (:926). Estado Congelada (PR #17, migración 010): POST /api/admin/miembros/:id/congelar (:810) y /descongelar (:869), que corre fecha_fin y la próxima fecha de cobro los días congelados (:892), con historial en congelacion_plan; pantalla en MiembrosPage.jsx:238, :742, :1907. Desde el PR #30, el check-in niega el ingreso de una membresía congelada con estado CONGELADO, sin registrar asistencia (checkin.js:125-149); el job de avisos la excluye (expiracion.js:62) y la campana la muestra como acceso bloqueado (notificaciones.js:101-107); ULTIMO_PLAN trae congelado_desde (lib/planes.js:30).</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, sección 33.2): ya están las dos cosas que pedía la decisión de Luis. Observaciones: congelar entre las 19:00 y las 24:00 de Colombia toma el día siguiente (CURRENT_DATE en UTC), y renovar el plan mientras está congelada conserva congelado_desde.</t>
+  </si>
+  <si>
+    <t>En cada check-in correcto (checkin.js:211-217), calcularGamificacion (lib/gamificacion.js:54) calcula la racha de días seguidos en hora de Colombia (:18, :25), otorga los hitos alcanzados sin repetirlos (ON CONFLICT, :90-94) y arma el mensaje (:41-46), que la pantalla de check-in muestra con la racha y los hitos logrados (CheckinPage.jsx:393-402). El administrador configura los hitos con GET, POST, PUT y DELETE /api/admin/hitos (config.js:190-280) y la pantalla HitosConfig en Configuración (ConfigPage.jsx:289). 12 pruebas en backend/tests/gamificacion.test.js. PR #32.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, sección 33.3), desde Pendiente. Menores: el mensaje dice «Te faltan 1» sin aclarar si son días o visitas; con dos hitos a la vez solo muestra el mensaje del primero; PUT /admin/hitos/:id con un id no numérico da 503 en vez de 400.</t>
+  </si>
+  <si>
+    <t>Capas en backend/src (routes, lib, middleware, jobs, db) y diagrama de arquitectura en el documento (sección 8). Scripts test y test:cov en backend/package.json (:8-9); jest.config.js mide src/lib, src/middleware, routes/checkin.js y routes/notificaciones.js (:15-19). Medición del 2026-10-20 sobre develop @ 3c35d53: 8 suites y 122 pruebas, todas pasan; cobertura de líneas de 97,72 % en routes/checkin.js y 90,32 % en routes/notificaciones.js (docs/evidencias/cobertura-backend-2026-10-20.txt). PR #33.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, sección 34): están el script test, las pruebas de check-in y alertas por encima del 70 % y las 2 pruebas que fallaban. Observaciones: el CI todavía no corre npm test (queda para la parte 2), así que una regresión podría entrar a develop sin que nadie lo note; el total del conjunto medido es 67,81 % por archivos de lib sin pruebas (whatsapp.js, email.js); la prueba de /enviado espera la columna canal, que no existe en el esquema real (issue #24).</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-18; verificador b8f99d2, secciones 22.6 y 25.4). Desde el PR #30, CheckinPage.jsx llama a marcarActividad() después de cada check-in correcto (:170, :225), así que un kiosco que solo usa la cámara ya no se cierra a los 30 min (verificador 47dde34, sección 33.2). Observaciones: la vigencia no está alineada: render.yaml:19 usa 24h y docker-compose.yml:61, 7d (se recomienda 8h). Con JWT_EXPIRES_IN en 0 o negativo el token nace vencido.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/admin-contrato.js:76-92, :105-116, :145, :153, :181; backend/src/lib/whatsapp.js:146, :229-238; backend/tests/contrato.test.js; backend/tests/whatsapp-text.test.js; frontend/src/pages/MiembrosPage.jsx:901, :1784</t>
+  </si>
+  <si>
+    <t>Envío del contrato sin comprobar antes isWhatsAppReady(): el cliente se inicia al enviar y cada intento queda registrado (PR #10).</t>
+  </si>
+  <si>
+    <t>2026-10-20</t>
+  </si>
+  <si>
+    <t>backend/src/jobs/scheduler.js:62-63; backend/src/jobs/expiracion.js:43-62, :101-103, :156-168, :217-218; backend/tests/expiracion.test.js</t>
+  </si>
+  <si>
+    <t>Aviso diario a las 9:00 con reintento a las 15:00, sin congeladas, una vez por etapa y marcado solo si se envía (PR #10 y #30).</t>
+  </si>
+  <si>
+    <t>backend/src/routes/config.js:33, :119; frontend/src/pages/ConfigPage.jsx:236-239; backend/src/routes/jobs.js:27, :38; backend/migrations/006_gimnasio_dias_aviso.sql; 007_alerta_vencimiento_enviada.sql</t>
+  </si>
+  <si>
+    <t>Días de aviso por gimnasio desde Configuración; ejecución manual y vista previa.</t>
+  </si>
+  <si>
+    <t>backend/migrations/010_congelar_membresia.sql; backend/src/routes/miembros.js:810, :869, :892; frontend/src/pages/MiembrosPage.jsx:238, :742, :1907; backend/src/routes/checkin.js:125-149; backend/src/jobs/expiracion.js:62</t>
+  </si>
+  <si>
+    <t>Congelar y descongelar (PR #17); el check-in niega el ingreso con CONGELADO y el job la excluye (PR #30).</t>
+  </si>
+  <si>
+    <t>backend/src/lib/gamificacion.js:18-122; backend/src/routes/checkin.js:211-217; backend/src/routes/config.js:190-280; frontend/src/pages/CheckinPage.jsx:393-402; frontend/src/components/HitosConfig.jsx; backend/tests/gamificacion.test.js</t>
+  </si>
+  <si>
+    <t>Racha en hora de Colombia, hitos otorgados sin repetir y configurables por el administrador (PR #32).</t>
+  </si>
+  <si>
+    <t>docs/evidencias/cobertura-backend-2026-10-20.txt (la medición inicial está en cobertura-backend-2026-10-16.txt)</t>
+  </si>
+  <si>
+    <t>122 de 122 pruebas; cobertura de líneas de 97,72 % en checkin.js y 90,32 % en notificaciones.js.</t>
+  </si>
+  <si>
+    <t>backend/src/{routes,lib,middleware,jobs,db}; backend/package.json:8-9 (test y test:cov); backend/jest.config.js:15-19; backend/tests/ (8 suites)</t>
+  </si>
+  <si>
+    <t>Arquitectura en capas, script de pruebas y cobertura configurada sobre check-in y alertas (PR #33).</t>
+  </si>
+  <si>
+    <t>backend/src/routes/auth.js:212, :243, :313; backend/src/index.js:63, :79; frontend/src/context/AuthContext.jsx:23-27, :40, :150-178, :223; frontend/src/api.js:115; frontend/src/pages/CheckinPage.jsx:170, :225 (marcarActividad)</t>
+  </si>
+  <si>
+    <t>Login con bcrypt y límite de intentos, cierre manual y cierre automático por inactividad, vencimiento o 401; el check-in cuenta como actividad (PR #18 y #30).</t>
+  </si>
+  <si>
+    <t>Estado actualizado el 2026-10-20 con los PR fusionados en develop hasta ese día (develop @ 3c35d53) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
   </si>
 </sst>
 </file>
@@ -1749,13 +1728,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.75</c:v>
+                  <c:v>0.86363636363636365</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.66666666666666663</c:v>
+                  <c:v>0.7</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.71621621621621623</c:v>
+                  <c:v>0.79729729729729726</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1919,13 +1898,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>22</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2337,7 +2316,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>441</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2382,19 +2361,19 @@
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.75</v>
+        <v>0.86363636363636365</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2402,14 +2381,14 @@
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>1.1000000000000014</v>
+        <v>0</v>
       </c>
       <c r="J6" t="s">
         <v>12</v>
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
@@ -2422,11 +2401,11 @@
       </c>
       <c r="D7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Implementado")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Parcial")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Pendiente")</f>
@@ -2434,7 +2413,7 @@
       </c>
       <c r="G7" s="9">
         <f>IF(C7=0,0,SUM(RNF!$F$2:$F$100)/C7)</f>
-        <v>0.66666666666666663</v>
+        <v>0.7</v>
       </c>
       <c r="H7" s="10">
         <f>Resumen!$C$40</f>
@@ -2442,14 +2421,14 @@
       </c>
       <c r="I7" s="11">
         <f>MAX(0,H7*C7-G7*C7)</f>
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J7" t="s">
         <v>14</v>
       </c>
       <c r="K7">
         <f>E8</f>
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
@@ -2462,19 +2441,19 @@
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.71621621621621623</v>
+        <v>0.79729729729729726</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2482,14 +2461,14 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>3.1000000000000014</v>
+        <v>0.10000000000000142</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
       </c>
       <c r="K8">
         <f>F8</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
@@ -2532,19 +2511,19 @@
       </c>
       <c r="D31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Implementado",RF!$G$2:$G$100,"Original")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Parcial",RF!$G$2:$G$100,"Original")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Pendiente",RF!$G$2:$G$100,"Original")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G31" s="9">
         <f>IF(C31=0,0,SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")/C31)</f>
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
@@ -2557,11 +2536,11 @@
       </c>
       <c r="D32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Implementado",RNF!$G$2:$G$100,"Original")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Parcial",RNF!$G$2:$G$100,"Original")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Pendiente",RNF!$G$2:$G$100,"Original")</f>
@@ -2569,7 +2548,7 @@
       </c>
       <c r="G32" s="9">
         <f>IF(C32=0,0,SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original")/C32)</f>
-        <v>0.5625</v>
+        <v>0.625</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.3">
@@ -2582,19 +2561,19 @@
       </c>
       <c r="D33" s="13">
         <f>D31+D32</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E33" s="13">
         <f>E31+E32</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F33" s="13">
         <f>F31+F32</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G33" s="14">
         <f>IF(C33=0,0,(SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")+SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original"))/C33)</f>
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
@@ -2706,10 +2685,10 @@
         <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>402</v>
+        <v>370</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>403</v>
+        <v>371</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2739,10 +2718,10 @@
         <v>12</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>404</v>
+        <v>372</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>405</v>
+        <v>416</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2794,7 +2773,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
         <v>49</v>
       </c>
@@ -2802,17 +2781,17 @@
         <v>43</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>392</v>
+        <v>410</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>393</v>
+        <v>411</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G5" s="24" t="s">
         <v>34</v>
@@ -2871,10 +2850,10 @@
         <v>12</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>430</v>
+        <v>395</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>431</v>
+        <v>396</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2904,10 +2883,10 @@
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>406</v>
+        <v>373</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>407</v>
+        <v>374</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2970,10 +2949,10 @@
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>422</v>
+        <v>387</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>423</v>
+        <v>388</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3025,7 +3004,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>87</v>
       </c>
@@ -3033,34 +3012,34 @@
         <v>88</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>89</v>
+        <v>412</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>90</v>
+        <v>413</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
         <v>34</v>
       </c>
       <c r="H12" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" s="23" t="s">
         <v>91</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B13" s="23" t="s">
         <v>88</v>
@@ -3069,10 +3048,10 @@
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3082,150 +3061,150 @@
         <v>34</v>
       </c>
       <c r="H13" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="J13" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="I13" s="23" t="s">
+    </row>
+    <row r="14" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="J13" s="23" t="s">
+      <c r="B14" s="23" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>100</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>101</v>
-      </c>
       <c r="C14" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>374</v>
+        <v>406</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>375</v>
+        <v>407</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>101</v>
+      </c>
+      <c r="I14" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="J14" s="23" t="s">
         <v>103</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>43</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>107</v>
+        <v>408</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="I17" s="23" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>33</v>
@@ -3234,31 +3213,31 @@
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I18" s="23" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B19" s="23" t="s">
         <v>65</v>
@@ -3267,7 +3246,7 @@
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E19" s="23" t="s">
         <v>56</v>
@@ -3277,21 +3256,21 @@
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I19" s="23" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>33</v>
@@ -3300,7 +3279,7 @@
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E20" s="23" t="s">
         <v>56</v>
@@ -3310,54 +3289,54 @@
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="I21" s="23" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>43</v>
@@ -3366,59 +3345,59 @@
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I22" s="23" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>408</v>
+        <v>375</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>409</v>
+        <v>376</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>
@@ -3497,19 +3476,19 @@
     </row>
     <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>378</v>
+        <v>357</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3522,27 +3501,27 @@
         <v>56</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3555,27 +3534,27 @@
         <v>56</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3588,27 +3567,27 @@
         <v>56</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3618,30 +3597,30 @@
         <v>34</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>376</v>
+        <v>355</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>377</v>
+        <v>356</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3651,30 +3630,30 @@
         <v>34</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3687,31 +3666,31 @@
         <v>56</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>195</v>
+        <v>414</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>196</v>
+        <v>415</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G8" s="24" t="s">
         <v>34</v>
@@ -3720,27 +3699,27 @@
         <v>56</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3753,123 +3732,123 @@
         <v>56</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H10" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>432</v>
+        <v>397</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>433</v>
+        <v>398</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H11" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H12" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="E13" s="23" t="s">
         <v>56</v>
@@ -3879,30 +3858,30 @@
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H13" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>56</v>
@@ -3912,30 +3891,30 @@
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H14" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>56</v>
@@ -3945,49 +3924,49 @@
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H15" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H16" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -4017,7 +3996,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4041,40 +4020,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4082,28 +4061,28 @@
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.7432432432432432</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.82432432432432434</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>100</v>
+        <v>76</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4111,28 +4090,28 @@
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.7567567567567568</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
+        <v>0.83783783783783783</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>106</v>
+        <v>199</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>108</v>
+        <v>201</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4140,28 +4119,28 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.77027027027027029</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.85135135135135132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>76</v>
+        <v>172</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>428</v>
+        <v>175</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>429</v>
+        <v>239</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4169,28 +4148,28 @@
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.78378378378378377</v>
+        <v>0.86486486486486491</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4198,57 +4177,57 @@
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.79729729729729726</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.8783783783783784</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>176</v>
+        <v>155</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>179</v>
+        <v>357</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>246</v>
+        <v>364</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.81081081081081086</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.90540540540540537</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>187</v>
+        <v>69</v>
       </c>
       <c r="B8" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>190</v>
+        <v>72</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4256,277 +4235,132 @@
       </c>
       <c r="H8" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.82432432432432434</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.91891891891891897</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>159</v>
+        <v>204</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Implementado</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>378</v>
+        <v>403</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>250</v>
+        <v>405</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.85135135135135132</v>
+        <v>0.91891891891891897</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>49</v>
+        <v>160</v>
       </c>
       <c r="B10" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>399</v>
+        <v>163</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>400</v>
+        <v>245</v>
       </c>
       <c r="E10" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="F10" s="24" t="s">
         <v>242</v>
-      </c>
-      <c r="F10" s="24" t="s">
-        <v>249</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H10" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.86486486486486491</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+        <v>0.94594594594594594</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="B11" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H11" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.8783783783783784</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.97297297297297303</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>193</v>
+        <v>80</v>
       </c>
       <c r="B12" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>196</v>
+        <v>83</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H12" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>0.89189189189189189</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="22" t="s">
-        <v>210</v>
-      </c>
-      <c r="B13" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
-        <v>Implementado</v>
-      </c>
-      <c r="C13" s="23" t="s">
-        <v>438</v>
-      </c>
-      <c r="D13" s="23" t="s">
-        <v>439</v>
-      </c>
-      <c r="E13" s="23" t="s">
-        <v>440</v>
-      </c>
-      <c r="F13" s="24" t="s">
-        <v>249</v>
-      </c>
-      <c r="G13" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A13,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A13,RNF!$A$2:$A$100,0)))</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G13))/Resumen!$C$8</f>
-        <v>0.89189189189189189</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C14" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="D14" s="23" t="s">
-        <v>253</v>
-      </c>
-      <c r="E14" s="23" t="s">
-        <v>242</v>
-      </c>
-      <c r="F14" s="24" t="s">
-        <v>249</v>
-      </c>
-      <c r="G14" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A14,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A14,RNF!$A$2:$A$100,0)))</f>
         <v>1</v>
       </c>
-      <c r="H14" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G14))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="B15" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C15" s="23" t="s">
-        <v>167</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>254</v>
-      </c>
-      <c r="E15" s="23" t="s">
-        <v>247</v>
-      </c>
-      <c r="F15" s="24" t="s">
-        <v>249</v>
-      </c>
-      <c r="G15" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A15,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A15,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
-      </c>
-      <c r="H15" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G15))/Resumen!$C$8</f>
-        <v>0.94594594594594594</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="B16" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C16" s="23" t="s">
-        <v>96</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>242</v>
-      </c>
-      <c r="F16" s="24" t="s">
-        <v>256</v>
-      </c>
-      <c r="G16" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A16,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A16,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
-      </c>
-      <c r="H16" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G16))/Resumen!$C$8</f>
-        <v>0.97297297297297303</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="B17" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>257</v>
-      </c>
-      <c r="E17" s="23" t="s">
-        <v>242</v>
-      </c>
-      <c r="F17" s="24" t="s">
-        <v>256</v>
-      </c>
-      <c r="G17" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A17,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A17,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
-      </c>
-      <c r="H17" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G17))/Resumen!$C$8</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
-        <v>390</v>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B17">
+  <conditionalFormatting sqref="B2:B12">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Implementado"</formula>
     </cfRule>
@@ -4558,7 +4392,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H2:H17</xm:sqref>
+          <xm:sqref>H2:H12</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4582,30 +4416,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4614,44 +4448,44 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>410</v>
+        <v>377</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>411</v>
+        <v>378</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>412</v>
+        <v>379</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>413</v>
+        <v>380</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>38</v>
@@ -4660,21 +4494,21 @@
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>414</v>
+        <v>432</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>415</v>
+        <v>433</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>391</v>
+        <v>419</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>38</v>
@@ -4683,21 +4517,21 @@
         <v>23</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>416</v>
+        <v>381</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>417</v>
+        <v>382</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>42</v>
@@ -4706,21 +4540,21 @@
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>42</v>
@@ -4729,21 +4563,21 @@
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>49</v>
@@ -4752,44 +4586,44 @@
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>394</v>
+        <v>367</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>49</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>395</v>
+        <v>424</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>396</v>
+        <v>425</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>391</v>
+        <v>419</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>53</v>
@@ -4798,39 +4632,39 @@
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>53</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4844,16 +4678,16 @@
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>434</v>
+        <v>399</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>435</v>
+        <v>400</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>427</v>
+        <v>392</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4867,21 +4701,21 @@
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>418</v>
+        <v>383</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>419</v>
+        <v>384</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>69</v>
@@ -4890,21 +4724,21 @@
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>69</v>
@@ -4913,16 +4747,16 @@
         <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="F15" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4933,19 +4767,19 @@
         <v>76</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>424</v>
+        <v>389</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>425</v>
+        <v>390</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>426</v>
+        <v>391</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>427</v>
+        <v>392</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -4956,806 +4790,806 @@
         <v>80</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>87</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>296</v>
+        <v>358</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>297</v>
+        <v>426</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>298</v>
-      </c>
-      <c r="F18" s="23" t="s">
-        <v>265</v>
+        <v>427</v>
+      </c>
+      <c r="F18" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>287</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>288</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>256</v>
+      </c>
+      <c r="G19" s="23" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="B20" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="B19" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="C19" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="D19" s="23" t="s">
-        <v>299</v>
-      </c>
-      <c r="E19" s="23" t="s">
-        <v>300</v>
-      </c>
-      <c r="F19" s="23" t="s">
-        <v>265</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="22" t="s">
+      <c r="C20" s="23" t="s">
+        <v>358</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>417</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>418</v>
+      </c>
+      <c r="F20" s="27" t="s">
+        <v>419</v>
+      </c>
+      <c r="G20" s="23" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="22" t="s">
+        <v>290</v>
+      </c>
+      <c r="B21" s="23" t="s">
         <v>104</v>
-      </c>
-      <c r="B20" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="C20" s="23" t="s">
-        <v>379</v>
-      </c>
-      <c r="D20" s="23" t="s">
-        <v>380</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>381</v>
-      </c>
-      <c r="F20" s="27" t="s">
-        <v>391</v>
-      </c>
-      <c r="G20" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="22" t="s">
-        <v>301</v>
-      </c>
-      <c r="B21" s="23" t="s">
-        <v>106</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>302</v>
+        <v>420</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>303</v>
-      </c>
-      <c r="F21" s="23" t="s">
-        <v>265</v>
+        <v>421</v>
+      </c>
+      <c r="F21" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>305</v>
+        <v>422</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>306</v>
-      </c>
-      <c r="F22" s="23" t="s">
-        <v>265</v>
+        <v>423</v>
+      </c>
+      <c r="F22" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>307</v>
+        <v>292</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>308</v>
+        <v>293</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>310</v>
+        <v>295</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>311</v>
+        <v>296</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>312</v>
+        <v>297</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>313</v>
+        <v>298</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>314</v>
+        <v>299</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>325</v>
+        <v>310</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>327</v>
+        <v>312</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>331</v>
+        <v>316</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>333</v>
+        <v>318</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>420</v>
+        <v>385</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>421</v>
+        <v>386</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>335</v>
+        <v>320</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>336</v>
+        <v>321</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>397</v>
+        <v>368</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>398</v>
+        <v>369</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>337</v>
+        <v>322</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>338</v>
+        <v>323</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>339</v>
+        <v>324</v>
       </c>
       <c r="F35" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C36" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>340</v>
+        <v>325</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>341</v>
+        <v>326</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>342</v>
+        <v>327</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>343</v>
+        <v>328</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>344</v>
+        <v>329</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>345</v>
+        <v>330</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>346</v>
+        <v>331</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>382</v>
+        <v>359</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>383</v>
+        <v>360</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>347</v>
+        <v>332</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>384</v>
+        <v>361</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>385</v>
+        <v>362</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>386</v>
+        <v>363</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>391</v>
+        <v>366</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>348</v>
+        <v>333</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>349</v>
+        <v>334</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>350</v>
+        <v>335</v>
       </c>
       <c r="F41" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>351</v>
+        <v>336</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>353</v>
+        <v>428</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>354</v>
-      </c>
-      <c r="F42" s="23" t="s">
-        <v>265</v>
+        <v>429</v>
+      </c>
+      <c r="F42" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>355</v>
+        <v>338</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>356</v>
+        <v>430</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>357</v>
-      </c>
-      <c r="F43" s="23" t="s">
-        <v>265</v>
+        <v>431</v>
+      </c>
+      <c r="F43" s="28" t="s">
+        <v>419</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>358</v>
+        <v>339</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>359</v>
+        <v>340</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>360</v>
+        <v>341</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>361</v>
+        <v>342</v>
       </c>
       <c r="F45" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>436</v>
+        <v>401</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>437</v>
+        <v>402</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>427</v>
+        <v>392</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>362</v>
+        <v>343</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>363</v>
+        <v>344</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>364</v>
+        <v>345</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>365</v>
+        <v>346</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>366</v>
+        <v>347</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>367</v>
+        <v>348</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>368</v>
+        <v>349</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>369</v>
+        <v>350</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>370</v>
+        <v>351</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>371</v>
+        <v>352</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>372</v>
+        <v>353</v>
       </c>
       <c r="F51" s="23" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>373</v>
+        <v>354</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): rutas nuevas del PR #34 en los documentos de seguimiento
Evidencias_Sustentacion/ pasa a docs/sustentacion/evidencias/ y
COMO_CORRER.md a docs/guias/COMO_CORRER.md en estado.md (5 menciones), la
matriz (RQNF-06) y el Excel (RNF!D7 y EV-40, editado por COM). El docx no
tenia rutas viejas. No queda ninguna de las rutas que movio el #34.
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC9AFFD6-E7B4-44E4-A840-6571AC1291F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D99D01E-29BC-459C-8083-F58E5270E86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -599,9 +599,6 @@
     <t>Compatibilidad</t>
   </si>
   <si>
-    <t>Aplicación web React / Vite servida por Vercel que solo requiere navegador (frontend/package.json, vercel.json); QA responsive a 375 px (Evidencias_Sustentacion/QA_Responsive_375px.md).</t>
-  </si>
-  <si>
     <t>Prueba documentada en Chrome, Firefox y Edge (lista de verificación de las pantallas principales con capturas).</t>
   </si>
   <si>
@@ -1046,9 +1043,6 @@
     <t>Documento</t>
   </si>
   <si>
-    <t>Evidencias_Sustentacion/QA_Responsive_375px.md; frontend/package.json; vercel.json</t>
-  </si>
-  <si>
     <t>App web sin instalación; sin prueba en los 3 navegadores.</t>
   </si>
   <si>
@@ -1347,6 +1341,12 @@
   </si>
   <si>
     <t>Estado actualizado el 2026-10-20 con los PR fusionados en develop hasta ese día (develop @ 3c35d53) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
+  </si>
+  <si>
+    <t>Aplicación web React / Vite servida por Vercel que solo requiere navegador (frontend/package.json, vercel.json); QA responsive a 375 px (docs/sustentacion/evidencias/QA_Responsive_375px.md).</t>
+  </si>
+  <si>
+    <t>docs/sustentacion/evidencias/QA_Responsive_375px.md; frontend/package.json; vercel.json</t>
   </si>
 </sst>
 </file>
@@ -2316,7 +2316,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2685,10 +2685,10 @@
         <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2718,10 +2718,10 @@
         <v>12</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2784,10 +2784,10 @@
         <v>12</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2850,10 +2850,10 @@
         <v>12</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2883,10 +2883,10 @@
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2949,10 +2949,10 @@
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3015,10 +3015,10 @@
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3081,10 +3081,10 @@
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3114,10 +3114,10 @@
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3378,10 +3378,10 @@
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3488,7 +3488,7 @@
         <v>157</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3617,10 +3617,10 @@
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3650,10 +3650,10 @@
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
+        <v>433</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>185</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>186</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3666,27 +3666,27 @@
         <v>56</v>
       </c>
       <c r="I7" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="J7" s="23" t="s">
         <v>187</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="23" t="s">
         <v>189</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>190</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3699,27 +3699,27 @@
         <v>56</v>
       </c>
       <c r="I8" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="J8" s="23" t="s">
         <v>191</v>
-      </c>
-      <c r="J8" s="23" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
+        <v>192</v>
+      </c>
+      <c r="B9" s="23" t="s">
         <v>193</v>
-      </c>
-      <c r="B9" s="23" t="s">
-        <v>194</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>195</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>196</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3732,15 +3732,15 @@
         <v>56</v>
       </c>
       <c r="I9" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="J9" s="23" t="s">
         <v>197</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>167</v>
@@ -3749,10 +3749,10 @@
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="E10" s="23" t="s">
         <v>200</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>201</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3765,27 +3765,27 @@
         <v>56</v>
       </c>
       <c r="I10" s="23" t="s">
+        <v>201</v>
+      </c>
+      <c r="J10" s="23" t="s">
         <v>202</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3798,27 +3798,27 @@
         <v>56</v>
       </c>
       <c r="I11" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="J11" s="23" t="s">
         <v>205</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
+        <v>207</v>
+      </c>
+      <c r="E12" s="23" t="s">
         <v>208</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>209</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3831,15 +3831,15 @@
         <v>56</v>
       </c>
       <c r="I12" s="23" t="s">
+        <v>209</v>
+      </c>
+      <c r="J12" s="23" t="s">
         <v>210</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B13" s="23" t="s">
         <v>151</v>
@@ -3848,7 +3848,7 @@
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E13" s="23" t="s">
         <v>56</v>
@@ -3864,24 +3864,24 @@
         <v>56</v>
       </c>
       <c r="I13" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="J13" s="23" t="s">
         <v>214</v>
-      </c>
-      <c r="J13" s="23" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
+        <v>215</v>
+      </c>
+      <c r="B14" s="23" t="s">
         <v>216</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>217</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>56</v>
@@ -3897,24 +3897,24 @@
         <v>56</v>
       </c>
       <c r="I14" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="J14" s="23" t="s">
         <v>219</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>56</v>
@@ -3930,15 +3930,15 @@
         <v>56</v>
       </c>
       <c r="I15" s="23" t="s">
+        <v>222</v>
+      </c>
+      <c r="J15" s="23" t="s">
         <v>223</v>
-      </c>
-      <c r="J15" s="23" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B16" s="23" t="s">
         <v>167</v>
@@ -3947,10 +3947,10 @@
         <v>16</v>
       </c>
       <c r="D16" s="23" t="s">
+        <v>225</v>
+      </c>
+      <c r="E16" s="23" t="s">
         <v>226</v>
-      </c>
-      <c r="E16" s="23" t="s">
-        <v>227</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3963,10 +3963,10 @@
         <v>56</v>
       </c>
       <c r="I16" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="J16" s="23" t="s">
         <v>228</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>229</v>
       </c>
     </row>
   </sheetData>
@@ -4020,40 +4020,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>233</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D2" s="23" t="s">
+        <v>234</v>
+      </c>
+      <c r="E2" s="23" t="s">
         <v>235</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="F2" s="24" t="s">
         <v>236</v>
-      </c>
-      <c r="F2" s="24" t="s">
-        <v>237</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4073,16 +4073,16 @@
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="E3" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="F3" s="24" t="s">
         <v>236</v>
-      </c>
-      <c r="F3" s="24" t="s">
-        <v>237</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4095,23 +4095,23 @@
     </row>
     <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E4" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="F4" s="24" t="s">
         <v>236</v>
-      </c>
-      <c r="F4" s="24" t="s">
-        <v>237</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4134,13 +4134,13 @@
         <v>175</v>
       </c>
       <c r="D5" s="23" t="s">
+        <v>238</v>
+      </c>
+      <c r="E5" s="23" t="s">
         <v>239</v>
       </c>
-      <c r="E5" s="23" t="s">
-        <v>240</v>
-      </c>
       <c r="F5" s="24" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4160,16 +4160,16 @@
         <v>Parcial</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4189,16 +4189,16 @@
         <v>Pendiente</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4221,13 +4221,13 @@
         <v>72</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G8" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
@@ -4240,23 +4240,23 @@
     </row>
     <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B9" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
         <v>Implementado</v>
       </c>
       <c r="C9" s="23" t="s">
+        <v>401</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>402</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>403</v>
       </c>
-      <c r="D9" s="23" t="s">
-        <v>404</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>405</v>
-      </c>
       <c r="F9" s="24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G9" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
@@ -4279,13 +4279,13 @@
         <v>163</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G10" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
@@ -4308,13 +4308,13 @@
         <v>94</v>
       </c>
       <c r="D11" s="23" t="s">
+        <v>245</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>235</v>
+      </c>
+      <c r="F11" s="24" t="s">
         <v>246</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>236</v>
-      </c>
-      <c r="F11" s="24" t="s">
-        <v>247</v>
       </c>
       <c r="G11" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
@@ -4337,13 +4337,13 @@
         <v>83</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G12" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
@@ -4356,7 +4356,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="17" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
   </sheetData>
@@ -4416,30 +4416,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>249</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>250</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="F1" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>253</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4448,44 +4448,44 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>38</v>
@@ -4494,21 +4494,21 @@
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>38</v>
@@ -4517,21 +4517,21 @@
         <v>23</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>42</v>
@@ -4540,21 +4540,21 @@
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="E6" s="23" t="s">
         <v>263</v>
       </c>
-      <c r="E6" s="23" t="s">
-        <v>264</v>
-      </c>
       <c r="F6" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G6" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G6" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>42</v>
@@ -4563,21 +4563,21 @@
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
+        <v>265</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>266</v>
       </c>
-      <c r="E7" s="23" t="s">
-        <v>267</v>
-      </c>
       <c r="F7" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G7" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>49</v>
@@ -4586,44 +4586,44 @@
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>49</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>53</v>
@@ -4632,39 +4632,39 @@
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
+        <v>272</v>
+      </c>
+      <c r="E10" s="23" t="s">
         <v>273</v>
       </c>
-      <c r="E10" s="23" t="s">
-        <v>274</v>
-      </c>
       <c r="F10" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G10" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G10" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>53</v>
       </c>
       <c r="C11" s="23" t="s">
+        <v>275</v>
+      </c>
+      <c r="D11" s="23" t="s">
         <v>276</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="E11" s="23" t="s">
         <v>277</v>
       </c>
-      <c r="E11" s="23" t="s">
-        <v>278</v>
-      </c>
       <c r="F11" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G11" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G11" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4678,16 +4678,16 @@
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4701,21 +4701,21 @@
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>69</v>
@@ -4724,21 +4724,21 @@
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
+        <v>279</v>
+      </c>
+      <c r="E14" s="23" t="s">
         <v>280</v>
       </c>
-      <c r="E14" s="23" t="s">
-        <v>281</v>
-      </c>
       <c r="F14" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G14" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G14" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>69</v>
@@ -4747,16 +4747,16 @@
         <v>23</v>
       </c>
       <c r="D15" s="23" t="s">
+        <v>282</v>
+      </c>
+      <c r="E15" s="23" t="s">
         <v>283</v>
       </c>
-      <c r="E15" s="23" t="s">
-        <v>284</v>
-      </c>
       <c r="F15" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G15" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G15" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4767,19 +4767,19 @@
         <v>76</v>
       </c>
       <c r="C16" s="23" t="s">
+        <v>387</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>388</v>
+      </c>
+      <c r="E16" s="23" t="s">
         <v>389</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="F16" s="28" t="s">
         <v>390</v>
       </c>
-      <c r="E16" s="23" t="s">
-        <v>391</v>
-      </c>
-      <c r="F16" s="28" t="s">
-        <v>392</v>
-      </c>
       <c r="G16" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
@@ -4790,19 +4790,19 @@
         <v>80</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D17" s="23" t="s">
+        <v>284</v>
+      </c>
+      <c r="E17" s="23" t="s">
         <v>285</v>
       </c>
-      <c r="E17" s="23" t="s">
-        <v>286</v>
-      </c>
       <c r="F17" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G17" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G17" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4813,19 +4813,19 @@
         <v>87</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -4836,19 +4836,19 @@
         <v>92</v>
       </c>
       <c r="C19" s="23" t="s">
+        <v>286</v>
+      </c>
+      <c r="D19" s="23" t="s">
         <v>287</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="E19" s="23" t="s">
         <v>288</v>
       </c>
-      <c r="E19" s="23" t="s">
-        <v>289</v>
-      </c>
       <c r="F19" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G19" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G19" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4859,24 +4859,24 @@
         <v>98</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D20" s="23" t="s">
+        <v>415</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>416</v>
+      </c>
+      <c r="F20" s="27" t="s">
         <v>417</v>
       </c>
-      <c r="E20" s="23" t="s">
-        <v>418</v>
-      </c>
-      <c r="F20" s="27" t="s">
-        <v>419</v>
-      </c>
       <c r="G20" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B21" s="23" t="s">
         <v>104</v>
@@ -4885,44 +4885,44 @@
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="F21" s="28" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>104</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="F22" s="28" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B23" s="23" t="s">
         <v>108</v>
@@ -4931,44 +4931,44 @@
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
+        <v>292</v>
+      </c>
+      <c r="E23" s="23" t="s">
         <v>293</v>
       </c>
-      <c r="E23" s="23" t="s">
-        <v>294</v>
-      </c>
       <c r="F23" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G23" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G23" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B24" s="23" t="s">
         <v>108</v>
       </c>
       <c r="C24" s="23" t="s">
+        <v>295</v>
+      </c>
+      <c r="D24" s="23" t="s">
         <v>296</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="E24" s="23" t="s">
         <v>297</v>
       </c>
-      <c r="E24" s="23" t="s">
-        <v>298</v>
-      </c>
       <c r="F24" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G24" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G24" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="B25" s="23" t="s">
         <v>108</v>
@@ -4977,16 +4977,16 @@
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
+        <v>299</v>
+      </c>
+      <c r="E25" s="23" t="s">
         <v>300</v>
       </c>
-      <c r="E25" s="23" t="s">
-        <v>301</v>
-      </c>
       <c r="F25" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G25" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G25" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4997,24 +4997,24 @@
         <v>115</v>
       </c>
       <c r="C26" s="23" t="s">
+        <v>301</v>
+      </c>
+      <c r="D26" s="23" t="s">
         <v>302</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="E26" s="23" t="s">
         <v>303</v>
       </c>
-      <c r="E26" s="23" t="s">
-        <v>304</v>
-      </c>
       <c r="F26" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G26" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G26" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="B27" s="23" t="s">
         <v>122</v>
@@ -5023,39 +5023,39 @@
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
+        <v>305</v>
+      </c>
+      <c r="E27" s="23" t="s">
         <v>306</v>
       </c>
-      <c r="E27" s="23" t="s">
-        <v>307</v>
-      </c>
       <c r="F27" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G27" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G27" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B28" s="23" t="s">
         <v>122</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D28" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="E28" s="23" t="s">
         <v>309</v>
       </c>
-      <c r="E28" s="23" t="s">
-        <v>310</v>
-      </c>
       <c r="F28" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G28" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G28" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5069,16 +5069,16 @@
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
+        <v>310</v>
+      </c>
+      <c r="E29" s="23" t="s">
         <v>311</v>
       </c>
-      <c r="E29" s="23" t="s">
-        <v>312</v>
-      </c>
       <c r="F29" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G29" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G29" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5092,16 +5092,16 @@
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
+        <v>312</v>
+      </c>
+      <c r="E30" s="23" t="s">
         <v>313</v>
       </c>
-      <c r="E30" s="23" t="s">
-        <v>314</v>
-      </c>
       <c r="F30" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G30" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G30" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5115,16 +5115,16 @@
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
+        <v>314</v>
+      </c>
+      <c r="E31" s="23" t="s">
         <v>315</v>
       </c>
-      <c r="E31" s="23" t="s">
-        <v>316</v>
-      </c>
       <c r="F31" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G31" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G31" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -5135,24 +5135,24 @@
         <v>144</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D32" s="23" t="s">
+        <v>316</v>
+      </c>
+      <c r="E32" s="23" t="s">
         <v>317</v>
       </c>
-      <c r="E32" s="23" t="s">
-        <v>318</v>
-      </c>
       <c r="F32" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G32" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G32" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="B33" s="23" t="s">
         <v>150</v>
@@ -5161,39 +5161,39 @@
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="B34" s="23" t="s">
         <v>150</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
@@ -5204,19 +5204,19 @@
         <v>155</v>
       </c>
       <c r="C35" s="23" t="s">
+        <v>321</v>
+      </c>
+      <c r="D35" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="E35" s="23" t="s">
         <v>323</v>
       </c>
-      <c r="E35" s="23" t="s">
-        <v>324</v>
-      </c>
       <c r="F35" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G35" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G35" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -5230,16 +5230,16 @@
         <v>23</v>
       </c>
       <c r="D36" s="23" t="s">
+        <v>324</v>
+      </c>
+      <c r="E36" s="23" t="s">
         <v>325</v>
       </c>
-      <c r="E36" s="23" t="s">
-        <v>326</v>
-      </c>
       <c r="F36" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G36" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G36" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -5253,16 +5253,16 @@
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="E37" s="23" t="s">
         <v>327</v>
       </c>
-      <c r="E37" s="23" t="s">
-        <v>328</v>
-      </c>
       <c r="F37" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G37" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
@@ -5276,21 +5276,21 @@
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
+        <v>328</v>
+      </c>
+      <c r="E38" s="23" t="s">
         <v>329</v>
       </c>
-      <c r="E38" s="23" t="s">
-        <v>330</v>
-      </c>
       <c r="F38" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G38" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G38" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="B39" s="23" t="s">
         <v>179</v>
@@ -5299,297 +5299,297 @@
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B40" s="23" t="s">
         <v>179</v>
       </c>
       <c r="C40" s="23" t="s">
+        <v>359</v>
+      </c>
+      <c r="D40" s="23" t="s">
+        <v>360</v>
+      </c>
+      <c r="E40" s="23" t="s">
         <v>361</v>
       </c>
-      <c r="D40" s="23" t="s">
-        <v>362</v>
-      </c>
-      <c r="E40" s="23" t="s">
-        <v>363</v>
-      </c>
       <c r="F40" s="27" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B41" s="23" t="s">
         <v>183</v>
       </c>
       <c r="C41" s="23" t="s">
+        <v>332</v>
+      </c>
+      <c r="D41" s="23" t="s">
+        <v>434</v>
+      </c>
+      <c r="E41" s="23" t="s">
         <v>333</v>
       </c>
-      <c r="D41" s="23" t="s">
-        <v>334</v>
-      </c>
-      <c r="E41" s="23" t="s">
-        <v>335</v>
-      </c>
       <c r="F41" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G41" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G41" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="F42" s="28" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="F43" s="28" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C44" s="23" t="s">
         <v>138</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="F44" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G44" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G44" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F45" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G45" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G45" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C47" s="23" t="s">
+        <v>341</v>
+      </c>
+      <c r="D47" s="23" t="s">
+        <v>342</v>
+      </c>
+      <c r="E47" s="23" t="s">
         <v>343</v>
       </c>
-      <c r="D47" s="23" t="s">
-        <v>344</v>
-      </c>
-      <c r="E47" s="23" t="s">
-        <v>345</v>
-      </c>
       <c r="F47" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G47" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G47" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="F48" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G48" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G48" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="F49" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G49" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G49" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="F50" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G50" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G50" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F51" s="23" t="s">
+        <v>255</v>
+      </c>
+      <c r="G51" s="23" t="s">
         <v>256</v>
-      </c>
-      <c r="G51" s="23" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): RQF-08, RQNF-01, RQNF-15 y RQNF-09 Implementados en el Excel (87,8 %)
- RQF-08 (PR #39), decision de Luis, con sus observaciones (campana del
  job diario, Render a las 8:00, tres calculos de en riesgo, dias en UTC).
- RQNF-01 (PR #40): check-in con 200 miembros, p95 de milisegundos.
- RQNF-15 y RQNF-09 (PR #28): 403 CORS_BLOCKED y tres limitadores; regla
  de no poner previews en FRONTEND_URL (buildAcceptUrl).
- RQNF-07 cierra la observacion del CI (PR #41); RQNF-02 con el monitor
  activo y su calendario (PR #42); RQNF-06 con la evidencia del #43.
- RQF-13 y RQF-14: el monitor mantiene despierto a Render en horario.
- RQF-22 y RQF-17: el #28 agrega los limites de intentos que faltaban.
- Trabajo pendiente: quedan RQF-09, RQNF-04, RQNF-06, RQNF-02, RQF-12 y
  RQF-10; RQF-09 y RQNF-04 pasan el 90 %.

Editado con Excel por COM. Avance: 32,5 de 37 = 87,8 % (RF 88,6 %, RNF 86,7 %).
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D99D01E-29BC-459C-8083-F58E5270E86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A87A8E-20E6-4FEE-90F5-103A34653237}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="434">
   <si>
     <t>FitLoyalty — Seguimiento de requisitos</t>
   </si>
@@ -257,12 +257,6 @@
     <t>Alertas de Abandono</t>
   </si>
   <si>
-    <t>Lista de miembros sin ingresar en N días calculada al consultar: campana de avisos (notificaciones.js:125-137; umbral del gimnasio, 15 por defecto, :38 y :66), dashboard (dashboard.js:161, :182) y filtro «En riesgo» de miembros (miembros.js:263, MiembrosPage.jsx:939).</t>
-  </si>
-  <si>
-    <t>Ejecución diaria del motor (el scheduler solo programa vencimientos, scheduler.js:46), los dos niveles Amarilla / Roja, registro en alerta_abandono (tabla sin uso) y pantalla para configurar el umbral (el dashboard usa 15 días fijos).</t>
-  </si>
-  <si>
     <t>HU-17, HU-18, HU-44, HU-64</t>
   </si>
   <si>
@@ -416,9 +410,6 @@
     <t>POST /api/auth/forgot-password genera un código de 6 dígitos con vigencia de 15 minutos y lo envía (auth.js:304-340, email.js:289); POST /verify-reset-code (auth.js:360) y POST /reset-password con bcrypt (auth.js:399, :447); pantalla ForgotPasswordPage.jsx:121, :143, :161; límite de 3 solicitudes por minuto solo en forgot-password (index.js:68, :80).</t>
   </si>
   <si>
-    <t>Riesgo de seguridad: si el correo no sale (o con SHOW_DEV_CODE_IN_UI=true), la API devuelve el código en la respuesta (auth.js:337-346), así que cualquiera que sepa el correo de un usuario puede cambiarle la contraseña; además verify-reset-code y reset-password no tienen límite de intentos (ver RQNF-09).</t>
-  </si>
-  <si>
     <t>HU-59</t>
   </si>
   <si>
@@ -515,9 +506,6 @@
     <t>Rendimiento</t>
   </si>
   <si>
-    <t>No hay medición registrada.</t>
-  </si>
-  <si>
     <t>EV-34</t>
   </si>
   <si>
@@ -530,12 +518,6 @@
     <t>Disponibilidad</t>
   </si>
   <si>
-    <t>Existen /api/healthz y /api/health (index.js:101, :103), pero no hay monitoreo ni reporte de disponibilidad.</t>
-  </si>
-  <si>
-    <t>Monitor externo sobre /api/healthz con reporte del período; el plan gratuito de Render suspende el servicio por inactividad (scheduler.js:9-10).</t>
-  </si>
-  <si>
     <t>EV-35</t>
   </si>
   <si>
@@ -599,9 +581,6 @@
     <t>Compatibilidad</t>
   </si>
   <si>
-    <t>Prueba documentada en Chrome, Firefox y Edge (lista de verificación de las pantallas principales con capturas).</t>
-  </si>
-  <si>
     <t>EV-40</t>
   </si>
   <si>
@@ -641,12 +620,6 @@
     <t>RQNF-09</t>
   </si>
   <si>
-    <t>express-rate-limit: inicio de sesión 5 por minuto, recuperación de contraseña 3 por minuto y login de la app 10 por minuto (index.js:63-77, :79-80, :94); trust proxy para tomar la IP real detrás de Render (index.js:43).</t>
-  </si>
-  <si>
-    <t>verify-reset-code (auth.js:360) y reset-password (auth.js:399) no tienen límite: el código de 6 dígitos se puede probar sin límite durante sus 15 minutos de vida.</t>
-  </si>
-  <si>
     <t>EV-44</t>
   </si>
   <si>
@@ -719,12 +692,6 @@
     <t>RQNF-15</t>
   </si>
   <si>
-    <t>La configuración de CORS lee FRONTEND_URL (index.js:45-48), pero el callback devuelve permitido también para orígenes que no están en la lista (index.js:54), con credentials: true.</t>
-  </si>
-  <si>
-    <t>Rechazar los orígenes que no estén en FRONTEND_URL (cambiar index.js:54). El PR #4 lo marcaba Implementado.</t>
-  </si>
-  <si>
     <t>EV-50</t>
   </si>
   <si>
@@ -746,39 +713,15 @@
     <t>Avance global acumulado</t>
   </si>
   <si>
-    <t>Rechazar en CORS los orígenes que no estén en FRONTEND_URL (index.js:54)</t>
-  </si>
-  <si>
     <t>Santiago</t>
   </si>
   <si>
     <t>Bajo</t>
   </si>
   <si>
-    <t>Límite de intentos en verify-reset-code y reset-password</t>
-  </si>
-  <si>
-    <t>Prueba de usabilidad del check-in manual con 3 personas sin formación técnica</t>
-  </si>
-  <si>
-    <t>Luis</t>
-  </si>
-  <si>
-    <t>Lista de verificación con capturas en Chrome, Firefox y Edge</t>
-  </si>
-  <si>
     <t>Medio</t>
   </si>
   <si>
-    <t>Luis o Santiago</t>
-  </si>
-  <si>
-    <t>Motor diario con Alerta Amarilla / Roja y umbrales editables</t>
-  </si>
-  <si>
-    <t>Monitor externo de disponibilidad con reporte (depende del plan de Render)</t>
-  </si>
-  <si>
     <t>CRUD de retos, progreso automático y aviso al completar</t>
   </si>
   <si>
@@ -881,21 +824,9 @@
     <t>EV-13</t>
   </si>
   <si>
-    <t>backend/src/routes/notificaciones.js:38, :66, :125-137; dashboard.js:161, :182; miembros.js:263</t>
-  </si>
-  <si>
-    <t>Lista de miembros en riesgo calculada al consultar, un solo umbral.</t>
-  </si>
-  <si>
     <t>EV-14</t>
   </si>
   <si>
-    <t>backend/src/jobs/scheduler.js:46</t>
-  </si>
-  <si>
-    <t>El único cron programado es el de vencimientos (no hay motor de abandono).</t>
-  </si>
-  <si>
     <t>backend/migrations/002_esquema_inicial.sql:171-202</t>
   </si>
   <si>
@@ -1007,21 +938,6 @@
     <t>Prueba (verificador)</t>
   </si>
   <si>
-    <t>Sin medición</t>
-  </si>
-  <si>
-    <t>— (riesgo en backend/src/routes/checkin.js:83-101)</t>
-  </si>
-  <si>
-    <t>No hay evidencia de tiempos; posible lentitud con muchos miembros.</t>
-  </si>
-  <si>
-    <t>backend/src/index.js:101, :103</t>
-  </si>
-  <si>
-    <t>Endpoints de salud disponibles para monitoreo; sin reporte.</t>
-  </si>
-  <si>
     <t>backend/src/routes/auth.js:145, :231, :447; staff.js:431; miembros.js:388, :625; cliente.js:88; frontend/src/api.js:26</t>
   </si>
   <si>
@@ -1040,12 +956,6 @@
     <t>EV-39</t>
   </si>
   <si>
-    <t>Documento</t>
-  </si>
-  <si>
-    <t>App web sin instalación; sin prueba en los 3 navegadores.</t>
-  </si>
-  <si>
     <t>EV-41</t>
   </si>
   <si>
@@ -1061,12 +971,6 @@
     <t>Contenedores definidos y despliegue en nube.</t>
   </si>
   <si>
-    <t>backend/src/index.js:43, :63-80, :94</t>
-  </si>
-  <si>
-    <t>Límites de intentos por IP en los endpoints sensibles.</t>
-  </si>
-  <si>
     <t>Configuración / ejecución</t>
   </si>
   <si>
@@ -1094,12 +998,6 @@
     <t>Errores manejados de forma centralizada.</t>
   </si>
   <si>
-    <t>backend/src/index.js:45-57</t>
-  </si>
-  <si>
-    <t>CORS acepta cualquier origen.</t>
-  </si>
-  <si>
     <t>Rutas relativas a la raíz del repositorio en main @ 54b19fa (el CI de RQNF-11 en 8acab31). No se hicieron pruebas en vivo: la verificación es por lectura de código, pruebas existentes y CI.</t>
   </si>
   <si>
@@ -1109,9 +1007,6 @@
     <t>Implementado (2026-10-18): ya no queda ninguna consulta sin filtro de gimnasio y el check-in dejó de derivar la clave del QR por cada miembro (verificador: 386d168, sección 14.5). La medición del tiempo de respuesta con volumen realista queda en RQNF-01. Menor: la vista lee membresia y plan_membresia, que el alta no llena, así que sus columnas de plan salen en NULL.</t>
   </si>
   <si>
-    <t>La búsqueda del QR ya no deriva la clave por cada miembro (PR #11, checkin.js:26, :31): hace un descifrado AES por miembro. Falta medir el check-in con un volumen realista (unos 200 miembros) y registrar el tiempo de respuesta de POST /api/admin/checkin.</t>
-  </si>
-  <si>
     <t>Código / prueba</t>
   </si>
   <si>
@@ -1130,9 +1025,6 @@
     <t>La vista y asistencia rechazan tokens de miembro y filtran por gimnasio; la 011 expone id_gimnasio.</t>
   </si>
   <si>
-    <t>Medir el check-in con un volumen realista (unos 200 miembros)</t>
-  </si>
-  <si>
     <t>Orden de menor a mayor esfuerzo. «Avance global acumulado» suma los puntos de cada acción, en orden, sobre el avance actual y se pone verde al llegar a la meta. Lo decide Luis; el reparto de tareas está en docs/plan-trabajo.md.</t>
   </si>
   <si>
@@ -1166,9 +1058,6 @@
     <t>DELETE /api/auth/account (auth.js:576): solo el administrador (403 NOT_ADMIN en :583) y solo el dueño, que es gimnasio.id_dueno (sqlIdDueno, auth-helpers.js:188; :594, 403 NOT_OWNER en :606), confirmando con su contraseña (:511, :611, 403 WRONG_PASSWORD) antes de abrir la transacción (:616). Borra los pasos de PASOS_ELIMINAR_CUENTA (:521) con un SAVEPOINT por paso (borrarPaso, :562), que solo omite una tabla o columna inexistente (42P01 y 42703, :555); el gimnasio se borra al final (:623), responde 404 si ya no existe (:626) y el rastro queda en el log (:631). La página pide la contraseña (EliminarCuentaPage.jsx:12, :124-126). PR #15, #21 y #19 (id_dueno).</t>
   </si>
   <si>
-    <t>Solo el dueño, con su contraseña (PR #21); el dueño es gimnasio.id_dueno desde el PR #19. Probado por el verificador con el handler real sobre PostgreSQL 18 (94d5fbb, sección 16; 1be53f7, sección 21.2; b8f99d2, sección 25.2): responde 200 sin dejar filas del gimnasio ni tocar las de otro, 403 al administrador invitado y con la contraseña mala, y 500 sin borrar nada si una FK desconocida lo bloquea. Falta el límite de intentos en DELETE /api/auth/account: con un token robado del dueño se puede probar su contraseña sin freno. Es una línea en index.js (zona de Daniel), antes de la :81.</t>
-  </si>
-  <si>
     <t>backend/src/routes/staff.js:133, :222, :251, :357, :388, :421, :424, :499; frontend/src/pages/StaffPage.jsx:138, :421, :434</t>
   </si>
   <si>
@@ -1247,27 +1136,12 @@
     <t>Migraciones versionadas aplicadas al iniciar; con la 014, notificacion y envio_mensaje quedan como en producción (pg_dump idéntico).</t>
   </si>
   <si>
-    <t>Hecho: la migración 014 reconcilia envio_mensaje y notificacion con producción (pg_dump idéntico). Estaba asignada por error a Santiago; la hizo Luis en la tarea L1.</t>
-  </si>
-  <si>
-    <t>Migración que reconcilie envio_mensaje y notificacion con producción (hecha: 014, PR #27)</t>
-  </si>
-  <si>
-    <t>Luis (L1, PR #27)</t>
-  </si>
-  <si>
     <t>POST /api/admin/miembros/:id/contrato/enviar con control de gimnasio (admin-contrato.js:76-92); vista previa e historial por API (:153, :181); botón «Enviar contrato» (MiembrosPage.jsx:901, :1784). Desde el PR #10 ya no se pregunta isWhatsAppReady() antes de enviar: sendWhatsAppText inicia el cliente perezoso y, si no queda listo, lanza WHATSAPP_NO_LISTO (whatsapp.js:229-238); admin-contrato.js:105-116 registra exito = false con la guía del QR y cliente_listo (:145). Pruebas en backend/tests/contrato.test.js y whatsapp-text.test.js.</t>
   </si>
   <si>
-    <t>Implementado (2026-10-20; verificador 47dde34, sección 33.1). Limitación de despliegue, por decisión de Luis: Render (render.yaml, entorno node) y la imagen Docker (Dockerfile:13, :29, PUPPETEER_SKIP_DOWNLOAD=true, sin chromium) no tienen Chrome, así que el envío por WhatsApp solo funciona en un equipo con Chrome, con el QR escaneado y ENABLE_WHATSAPP activo. En el entorno desplegado el contrato no sale, pero el intento queda registrado con exito = false.</t>
-  </si>
-  <si>
     <t>Cron a las 9:00 y a las 15:00 (reintento) en America/Bogota (scheduler.js:62-63); selección de planes por vencer sin las membresías congeladas (expiracion.js:43-62); un aviso al entrar en la ventana y otro el día 0, y si el servidor estuvo dormido ese día sale al siguiente (:101-103, :156-168); el aviso solo se marca si el envío no falla (:217-218), y sendWhatsAppText inicia el cliente y lanza WHATSAPP_NO_LISTO si no queda listo (whatsapp.js:229-238). Días de aviso por gimnasio desde Configuración, entre 0 y 30 (config.js:33, :119; ConfigPage.jsx:236-239). POST /api/jobs/expiracion/run y GET /api/jobs/expiracion/preview (jobs.js:27, :38); migraciones 006 y 007. Pruebas en backend/tests/expiracion.test.js. PR #10 y #30.</t>
   </si>
   <si>
-    <t>Implementado (2026-10-20; verificador 47dde34, secciones 33.1 y 33.2). Limitación de despliegue, por decisión de Luis: Render (render.yaml, entorno node) y la imagen Docker (Dockerfile:13, :29, PUPPETEER_SKIP_DOWNLOAD=true, sin chromium) no tienen Chrome, así que el envío por WhatsApp solo funciona en un equipo con Chrome, con el QR escaneado y ENABLE_WHATSAPP activo. En el entorno desplegado los avisos no se marcan como enviados y se reintentan en la corrida siguiente. Además, el cron vive dentro del proceso web: si Render tiene el servicio dormido a las 9:00 y a las 15:00, no corre.</t>
-  </si>
-  <si>
     <t>Cálculo automático de fecha_fin según el plan (miembros.js:193, :395); estado vencido / por vencer contra la fecha actual (:286-290); renovación del plan (:926). Estado Congelada (PR #17, migración 010): POST /api/admin/miembros/:id/congelar (:810) y /descongelar (:869), que corre fecha_fin y la próxima fecha de cobro los días congelados (:892), con historial en congelacion_plan; pantalla en MiembrosPage.jsx:238, :742, :1907. Desde el PR #30, el check-in niega el ingreso de una membresía congelada con estado CONGELADO, sin registrar asistencia (checkin.js:125-149); el job de avisos la excluye (expiracion.js:62) y la campana la muestra como acceso bloqueado (notificaciones.js:101-107); ULTIMO_PLAN trae congelado_desde (lib/planes.js:30).</t>
   </si>
   <si>
@@ -1280,12 +1154,6 @@
     <t>Implementado (2026-10-20; verificador 47dde34, sección 33.3), desde Pendiente. Menores: el mensaje dice «Te faltan 1» sin aclarar si son días o visitas; con dos hitos a la vez solo muestra el mensaje del primero; PUT /admin/hitos/:id con un id no numérico da 503 en vez de 400.</t>
   </si>
   <si>
-    <t>Capas en backend/src (routes, lib, middleware, jobs, db) y diagrama de arquitectura en el documento (sección 8). Scripts test y test:cov en backend/package.json (:8-9); jest.config.js mide src/lib, src/middleware, routes/checkin.js y routes/notificaciones.js (:15-19). Medición del 2026-10-20 sobre develop @ 3c35d53: 8 suites y 122 pruebas, todas pasan; cobertura de líneas de 97,72 % en routes/checkin.js y 90,32 % en routes/notificaciones.js (docs/evidencias/cobertura-backend-2026-10-20.txt). PR #33.</t>
-  </si>
-  <si>
-    <t>Implementado (2026-10-20; verificador 47dde34, sección 34): están el script test, las pruebas de check-in y alertas por encima del 70 % y las 2 pruebas que fallaban. Observaciones: el CI todavía no corre npm test (queda para la parte 2), así que una regresión podría entrar a develop sin que nadie lo note; el total del conjunto medido es 67,81 % por archivos de lib sin pruebas (whatsapp.js, email.js); la prueba de /enviado espera la columna canal, que no existe en el esquema real (issue #24).</t>
-  </si>
-  <si>
     <t>Implementado (2026-10-18; verificador b8f99d2, secciones 22.6 y 25.4). Desde el PR #30, CheckinPage.jsx llama a marcarActividad() después de cada check-in correcto (:170, :225), así que un kiosco que solo usa la cámara ya no se cierra a los 30 min (verificador 47dde34, sección 33.2). Observaciones: la vigencia no está alineada: render.yaml:19 usa 24h y docker-compose.yml:61, 7d (se recomienda 8h). Con JWT_EXPIRES_IN en 0 o negativo el token nace vencido.</t>
   </si>
   <si>
@@ -1328,25 +1196,154 @@
     <t>122 de 122 pruebas; cobertura de líneas de 97,72 % en checkin.js y 90,32 % en notificaciones.js.</t>
   </si>
   <si>
-    <t>backend/src/{routes,lib,middleware,jobs,db}; backend/package.json:8-9 (test y test:cov); backend/jest.config.js:15-19; backend/tests/ (8 suites)</t>
-  </si>
-  <si>
-    <t>Arquitectura en capas, script de pruebas y cobertura configurada sobre check-in y alertas (PR #33).</t>
-  </si>
-  <si>
     <t>backend/src/routes/auth.js:212, :243, :313; backend/src/index.js:63, :79; frontend/src/context/AuthContext.jsx:23-27, :40, :150-178, :223; frontend/src/api.js:115; frontend/src/pages/CheckinPage.jsx:170, :225 (marcarActividad)</t>
   </si>
   <si>
     <t>Login con bcrypt y límite de intentos, cierre manual y cierre automático por inactividad, vencimiento o 401; el check-in cuenta como actividad (PR #18 y #30).</t>
   </si>
   <si>
-    <t>Estado actualizado el 2026-10-20 con los PR fusionados en develop hasta ese día (develop @ 3c35d53) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
-  </si>
-  <si>
-    <t>Aplicación web React / Vite servida por Vercel que solo requiere navegador (frontend/package.json, vercel.json); QA responsive a 375 px (docs/sustentacion/evidencias/QA_Responsive_375px.md).</t>
-  </si>
-  <si>
-    <t>docs/sustentacion/evidencias/QA_Responsive_375px.md; frontend/package.json; vercel.json</t>
+    <t>Motor diario (jobs/abandono.js:97, runJob) programado a las 8:00 en hora de Colombia (scheduler.js:71): clasifica en AMARILLA desde umbral_alerta_amarilla días sin ingresar (7 por defecto) y en ROJA desde umbral_alerta_roja (15) (abandono.js:35-37), y deja una sola alerta PENDIENTE por miembro en alerta_abandono: la sube de nivel, la cierra como GESTIONADA si vuelve e IGNORADA si deja de aplicar (congela, vence o se da de baja) (abandono.js:19-22). Umbrales por gimnasio con validación (config.js:36-60; ConfigPage.jsx:18-19, :45-46); la campana los lista, ROJA primero (notificaciones.js:149-207); ejecución manual con POST /api/jobs/abandono/run (jobs.js:46). La migración 012 alinea alerta_abandono con producción. 28 pruebas en backend/tests/abandono.test.js. PR #39.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-25, decisión de Luis; verificador 61df91a, sección 36.1). Observaciones: la campana muestra lo que dejó el job diario, así que un miembro que congela o vuelve hoy sigue «en riesgo» hasta el día siguiente; si Render duerme a las 8:00 el job no corre, aunque el monitor del #42 lo mantiene despierto de 4:50 a 22:00. Santiago hará en un PR de seguimiento el filtro de la campana y correr el job al arrancar. Hay tres cálculos distintos de «en riesgo» (dashboard, Miembros y job) y los días se cuentan en UTC.</t>
+  </si>
+  <si>
+    <t>backend/scripts/medir-checkin.js (npm run medir:checkin) mide POST /api/admin/checkin contra una base local con 200 y 2000 miembros, por documento, QR directo y QR cifrado, y se niega a correr contra una base que no sea local. Resultado (docs/evidencias/rqnf-01-checkin.md): con 200 miembros el peor caso fue de 15 ms y el p95 de 13 ms; con 2000, de 60 ms. El verificador lo reprodujo con p95 de 6 a 8 ms, 0 errores y 181 respuestas 201 (61df91a, sección 36.2). PR #40.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-25; verificador 61df91a, sección 36.2): el límite es de 2 s y el check-in responde en milisegundos. Observaciones: mide solo el backend, no el lector HID ni el navegador; se midió en local, sin la red de Render y Neon; el documento debería aclarar que usa el esquema de Docker.</t>
+  </si>
+  <si>
+    <t>CORS rechaza con 403 CORS_BLOCKED los orígenes que no están en FRONTEND_URL (index.js:57); las peticiones sin Origin (app Flutter, curl, healthz) pasan. 9 pruebas en backend/tests/cors-limites.test.js. PR #28.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-25; verificador 61df91a, sección 37.1). Regla de despliegue: no poner previews de Vercel en FRONTEND_URL, porque buildAcceptUrl (staff.js:66-67) arma el enlace de invitación con esa variable entera. Los previews de Vercel y Docker por 127.0.0.1 o desde la red local reciben 403.</t>
+  </si>
+  <si>
+    <t>express-rate-limit: inicio de sesión 5 por minuto, recuperación de contraseña 3 por minuto, verify-reset-code, reset-password y DELETE /api/auth/account 5 cada 15 minutos, y login de la app 10 por minuto (index.js:66-91, :97-101, :116); trust proxy para tomar la IP real detrás de Render (index.js:44). Pruebas en backend/tests/cors-limites.test.js. PR #28.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-25; verificador 61df91a, sección 37.1): los tres limitadores nuevos responden 429 después de 5 intentos, cada uno con su propio contador.</t>
+  </si>
+  <si>
+    <t>Capas en backend/src (routes, lib, middleware, jobs, db) y diagrama de arquitectura en el documento (sección 8). Scripts test y test:cov en backend/package.json (:8-9); jest.config.js mide src/lib, src/middleware, routes/checkin.js y routes/notificaciones.js (:15-19). Medición del 2026-10-20 sobre develop @ 3c35d53: 122 pruebas, todas pasan; cobertura de líneas de 97,72 % en routes/checkin.js y 90,32 % en routes/notificaciones.js (docs/evidencias/cobertura-backend-2026-10-20.txt). Desde el PR #41, el paso «Pruebas» del CI corre npm test en cada PR (.github/workflows/ci.yml:47-48). PR #33 y #41.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, sección 34). Desde el PR #41 el CI corre npm test en cada PR, con 214 pruebas (verificador 61df91a, sección 36.3), así que se cierra la observación de que no lo hacía. Observaciones: no hay coverageThreshold, así que el CI no frena si la cobertura de check-in y alertas bajara del 70 %; jest.config.js no incluye src/jobs/abandono.js; la prueba de /enviado espera la columna canal, que no existe en el esquema real (issue #24).</t>
+  </si>
+  <si>
+    <t>Existen /api/healthz y /api/health (index.js:123, :125). Monitor externo activo desde el 2026-10-25 (PR #42): .github/workflows/availability-monitor.yml consulta /api/healthz cada 5 minutos de 5:02 a 21:57 de Colombia (204 mediciones al día) y calienta el servicio a las 4:50; el reporte y la receta de conteo están en docs/evidencias/rqnf-02-disponibilidad.md.</t>
+  </si>
+  <si>
+    <t>Sigue Pendiente (verificador 61df91a, sección 37.2): el monitor empezó hoy y todavía no hay historial. Calendario: Parcial el lunes 26 en la noche, con un día operativo completo; Implementado como pronto el domingo 1/11, con 7 días seguidos (de lunes a domingo) al 99 % o más. Si da menos de 99 %, queda en Parcial.</t>
+  </si>
+  <si>
+    <t>Aplicación web React / Vite servida por Vercel que solo requiere navegador (frontend/package.json, vercel.json); QA responsive a 375 px (docs/sustentacion/evidencias/QA_Responsive_375px.md). Prueba del 2026-10-22 en Chrome 155, Firefox 157 y Edge 155: portada y formulario de inicio de sesión sin errores ni desbordamiento, con capturas (docs/evidencias/rqnf-06-navegadores.md, PR #43); el build de Vite 5 apunta a chrome87, firefox78 y edge88.</t>
+  </si>
+  <si>
+    <t>Sigue Parcial (verificador 61df91a, sección 37.3): la prueba del #43 solo cubre la portada y el login, sin backend. Falta repetirla con el backend en las pantallas principales (inicio de sesión, dashboard, miembros, check-in y configuración) en Chrome, Firefox y Edge, con capturas (Daniel, D4).</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, sección 33.1). Limitación de despliegue, por decisión de Luis: Render (render.yaml, entorno node) y la imagen Docker (Dockerfile:13, :29, PUPPETEER_SKIP_DOWNLOAD=true, sin chromium) no tienen Chrome, así que el envío por WhatsApp solo funciona en un equipo con Chrome, con el QR escaneado y ENABLE_WHATSAPP activo. En el entorno desplegado el contrato no sale, pero el intento queda registrado con exito = false. Desde el PR #42, el monitor de disponibilidad mantiene despierto a Render de 4:50 a unas 22:12, lo que ayuda a que corran los crons de avisos; la limitación de Chrome sigue igual.</t>
+  </si>
+  <si>
+    <t>Implementado (2026-10-20; verificador 47dde34, secciones 33.1 y 33.2). Limitación de despliegue, por decisión de Luis: Render (render.yaml, entorno node) y la imagen Docker (Dockerfile:13, :29, PUPPETEER_SKIP_DOWNLOAD=true, sin chromium) no tienen Chrome, así que el envío por WhatsApp solo funciona en un equipo con Chrome, con el QR escaneado y ENABLE_WHATSAPP activo. En el entorno desplegado los avisos no se marcan como enviados y se reintentan en la corrida siguiente. Además, el cron vive dentro del proceso web: si Render tiene el servicio dormido a las 9:00 y a las 15:00, no corre. Desde el PR #42, el monitor de disponibilidad mantiene despierto a Render de 4:50 a unas 22:12, lo que ayuda a que corran los crons de avisos; la limitación de Chrome sigue igual.</t>
+  </si>
+  <si>
+    <t>Riesgo de seguridad: si el correo no sale (o con SHOW_DEV_CODE_IN_UI=true), la API devuelve el código en la respuesta (auth.js:355-362), así que cualquiera que sepa el correo de un usuario puede cambiarle la contraseña; desde el PR #28, verify-reset-code y reset-password tienen un límite de 5 intentos cada 15 minutos (ver RQNF-09).</t>
+  </si>
+  <si>
+    <t>Solo el dueño, con su contraseña (PR #21); el dueño es gimnasio.id_dueno desde el PR #19. Probado por el verificador con el handler real sobre PostgreSQL 18 (94d5fbb, sección 16; 1be53f7, sección 21.2; b8f99d2, sección 25.2): responde 200 sin dejar filas del gimnasio ni tocar las de otro, 403 al administrador invitado y con la contraseña mala, y 500 sin borrar nada si una FK desconocida lo bloquea. Desde el PR #28, DELETE /api/auth/account tiene un límite de 5 intentos cada 15 minutos (index.js:86, :101), así que ya no se puede probar la contraseña del dueño sin freno.</t>
+  </si>
+  <si>
+    <t>backend/src/jobs/abandono.js:19-37, :97; backend/src/jobs/scheduler.js:71; backend/src/routes/config.js:36-60; backend/src/routes/notificaciones.js:149-207; backend/src/routes/jobs.js:46; frontend/src/pages/ConfigPage.jsx:18-19, :45-46</t>
+  </si>
+  <si>
+    <t>Motor diario de alertas Amarilla y Roja con umbrales por gimnasio, registro en alerta_abandono y campana (PR #39).</t>
+  </si>
+  <si>
+    <t>2026-10-25</t>
+  </si>
+  <si>
+    <t>Esquema / prueba</t>
+  </si>
+  <si>
+    <t>backend/migrations/012_alerta_abandono_como_produccion.sql; backend/tests/abandono.test.js (28 pruebas); informe del verificador, commit 61df91a, §36.1</t>
+  </si>
+  <si>
+    <t>Migración que alinea alerta_abandono con producción y pruebas del motor.</t>
+  </si>
+  <si>
+    <t>docs/evidencias/rqnf-01-checkin.md; backend/scripts/medir-checkin.js (npm run medir:checkin)</t>
+  </si>
+  <si>
+    <t>Check-in con 200 miembros: peor caso de 15 ms y p95 de 13 ms, frente a un límite de 2 s (PR #40).</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>.github/workflows/availability-monitor.yml; docs/evidencias/rqnf-02-disponibilidad.md; backend/src/index.js:123, :125</t>
+  </si>
+  <si>
+    <t>Monitor de /api/healthz cada 5 minutos en horario operativo, activo desde el 2026-10-25; todavía sin historial (PR #42).</t>
+  </si>
+  <si>
+    <t>Documento / capturas</t>
+  </si>
+  <si>
+    <t>docs/evidencias/rqnf-06-navegadores.md y docs/evidencias/capturas/; docs/sustentacion/evidencias/QA_Responsive_375px.md; frontend/package.json; vercel.json</t>
+  </si>
+  <si>
+    <t>Portada y login en Chrome, Firefox y Edge con capturas (PR #43); faltan las pantallas principales con backend.</t>
+  </si>
+  <si>
+    <t>backend/src/{routes,lib,middleware,jobs,db}; backend/package.json:8-9 (test y test:cov); backend/jest.config.js:15-19; backend/tests/; .github/workflows/ci.yml:47-48 (npm test en el CI)</t>
+  </si>
+  <si>
+    <t>Arquitectura en capas, script de pruebas, cobertura sobre check-in y alertas, y pruebas en el CI (PR #33 y #41).</t>
+  </si>
+  <si>
+    <t>backend/src/index.js:44, :66-91, :97-101, :116; backend/tests/cors-limites.test.js</t>
+  </si>
+  <si>
+    <t>Límites de intentos en el login, la recuperación, verify-reset-code, reset-password, la eliminación de cuenta y el login de la app (PR #28).</t>
+  </si>
+  <si>
+    <t>backend/src/index.js:57 (403 CORS_BLOCKED); backend/tests/cors-limites.test.js</t>
+  </si>
+  <si>
+    <t>CORS rechaza con 403 los orígenes que no están en FRONTEND_URL (PR #28).</t>
+  </si>
+  <si>
+    <t>Santiago (issue #24)</t>
+  </si>
+  <si>
+    <t>Prueba de usabilidad del check-in manual con 3 personas sin formación técnica (D5)</t>
+  </si>
+  <si>
+    <t>Daniel (D5)</t>
+  </si>
+  <si>
+    <t>La prueba del #43 solo cubre la portada y el login sin backend; falta repetirla con el backend en las pantallas principales (inicio de sesión, dashboard, miembros, check-in y configuración) en los tres navegadores.</t>
+  </si>
+  <si>
+    <t>Repetir la prueba de navegadores con el backend en marcha, con capturas por pantalla (D4)</t>
+  </si>
+  <si>
+    <t>Daniel (D4)</t>
+  </si>
+  <si>
+    <t>Monitor activo desde el 2026-10-25 (PR #42); falta el historial. Parcial el lunes 26 en la noche, con un día operativo completo; Implementado como pronto el domingo 1/11, con 7 días seguidos al 99 % o más.</t>
+  </si>
+  <si>
+    <t>Juntar 7 días de mediciones del monitor y llenar el reporte del período (D3)</t>
+  </si>
+  <si>
+    <t>Daniel (D3)</t>
+  </si>
+  <si>
+    <t>Estado actualizado el 2026-10-25 con los PR fusionados en develop hasta ese día (develop @ 21e7e9c) y la confirmación del issue #24 sobre el esquema real; la verificación inicial fue el 2026-10-16 (main @ 54b19fa). Todas las cifras son fórmulas sobre las hojas RF y RNF.</t>
   </si>
 </sst>
 </file>
@@ -1728,13 +1725,13 @@
                 <c:formatCode>0.0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.86363636363636365</c:v>
+                  <c:v>0.88636363636363635</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.7</c:v>
+                  <c:v>0.8666666666666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.79729729729729726</c:v>
+                  <c:v>0.8783783783783784</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1898,13 +1895,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>27</c:v>
+                  <c:v>31</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2316,7 +2313,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2361,11 +2358,11 @@
       </c>
       <c r="D6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Implementado")</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Parcial")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F6" s="8">
         <f>COUNTIF(RF!$C$2:$C$100,"Pendiente")</f>
@@ -2373,7 +2370,7 @@
       </c>
       <c r="G6" s="9">
         <f>IF(C6=0,0,SUM(RF!$F$2:$F$100)/C6)</f>
-        <v>0.86363636363636365</v>
+        <v>0.88636363636363635</v>
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
@@ -2388,7 +2385,7 @@
       </c>
       <c r="K6">
         <f>D8</f>
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.3">
@@ -2401,19 +2398,19 @@
       </c>
       <c r="D7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Implementado")</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Parcial")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" s="8">
         <f>COUNTIF(RNF!$C$2:$C$100,"Pendiente")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G7" s="9">
         <f>IF(C7=0,0,SUM(RNF!$F$2:$F$100)/C7)</f>
-        <v>0.7</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="H7" s="10">
         <f>Resumen!$C$40</f>
@@ -2421,14 +2418,14 @@
       </c>
       <c r="I7" s="11">
         <f>MAX(0,H7*C7-G7*C7)</f>
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="J7" t="s">
         <v>14</v>
       </c>
       <c r="K7">
         <f>E8</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
@@ -2441,19 +2438,19 @@
       </c>
       <c r="D8" s="13">
         <f>D6+D7</f>
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E8" s="13">
         <f>E6+E7</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F8" s="13">
         <f>F6+F7</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G8" s="14">
         <f>IF(C8=0,0,(SUM(RF!$F$2:$F$100)+SUM(RNF!$F$2:$F$100))/C8)</f>
-        <v>0.79729729729729726</v>
+        <v>0.8783783783783784</v>
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
@@ -2461,14 +2458,14 @@
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>0.10000000000000142</v>
+        <v>0</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
       </c>
       <c r="K8">
         <f>F8</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.3">
@@ -2511,11 +2508,11 @@
       </c>
       <c r="D31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Implementado",RF!$G$2:$G$100,"Original")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Parcial",RF!$G$2:$G$100,"Original")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" s="8">
         <f>COUNTIFS(RF!$C$2:$C$100,"Pendiente",RF!$G$2:$G$100,"Original")</f>
@@ -2523,7 +2520,7 @@
       </c>
       <c r="G31" s="9">
         <f>IF(C31=0,0,SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")/C31)</f>
-        <v>0.75</v>
+        <v>0.79166666666666663</v>
       </c>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.3">
@@ -2536,7 +2533,7 @@
       </c>
       <c r="D32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Implementado",RNF!$G$2:$G$100,"Original")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Parcial",RNF!$G$2:$G$100,"Original")</f>
@@ -2544,11 +2541,11 @@
       </c>
       <c r="F32" s="8">
         <f>COUNTIFS(RNF!$C$2:$C$100,"Pendiente",RNF!$G$2:$G$100,"Original")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G32" s="9">
         <f>IF(C32=0,0,SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original")/C32)</f>
-        <v>0.625</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="33" spans="2:7" x14ac:dyDescent="0.3">
@@ -2561,19 +2558,19 @@
       </c>
       <c r="D33" s="13">
         <f>D31+D32</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E33" s="13">
         <f>E31+E32</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F33" s="13">
         <f>F31+F32</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G33" s="14">
         <f>IF(C33=0,0,(SUMIFS(RF!$F$2:$F$100,RF!$G$2:$G$100,"Original")+SUMIFS(RNF!$F$2:$F$100,RNF!$G$2:$G$100,"Original"))/C33)</f>
-        <v>0.7</v>
+        <v>0.77500000000000002</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
@@ -2685,10 +2682,10 @@
         <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>368</v>
+        <v>332</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>369</v>
+        <v>333</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2718,10 +2715,10 @@
         <v>12</v>
       </c>
       <c r="D3" s="23" t="s">
+        <v>334</v>
+      </c>
+      <c r="E3" s="23" t="s">
         <v>370</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>414</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2784,10 +2781,10 @@
         <v>12</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>408</v>
+        <v>366</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>409</v>
+        <v>367</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2850,10 +2847,10 @@
         <v>12</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>393</v>
+        <v>356</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>394</v>
+        <v>357</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2883,10 +2880,10 @@
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>371</v>
+        <v>335</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>372</v>
+        <v>336</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2905,7 +2902,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
         <v>69</v>
       </c>
@@ -2913,34 +2910,34 @@
         <v>70</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>71</v>
+        <v>386</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>72</v>
+        <v>387</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G9" s="24" t="s">
         <v>34</v>
       </c>
       <c r="H9" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="I9" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="J9" s="23" t="s">
         <v>73</v>
-      </c>
-      <c r="I9" s="23" t="s">
-        <v>74</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="216" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>70</v>
@@ -2949,10 +2946,10 @@
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>385</v>
+        <v>348</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>386</v>
+        <v>349</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2962,30 +2959,30 @@
         <v>34</v>
       </c>
       <c r="H10" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" s="23" t="s">
         <v>77</v>
-      </c>
-      <c r="I10" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="J10" s="23" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
@@ -2995,30 +2992,30 @@
         <v>34</v>
       </c>
       <c r="H11" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="I11" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="J11" s="23" t="s">
         <v>84</v>
-      </c>
-      <c r="I11" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="J11" s="23" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>410</v>
+        <v>368</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>411</v>
+        <v>369</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3028,30 +3025,30 @@
         <v>34</v>
       </c>
       <c r="H12" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="I12" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="J12" s="23" t="s">
         <v>89</v>
-      </c>
-      <c r="I12" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="J12" s="23" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3061,51 +3058,51 @@
         <v>34</v>
       </c>
       <c r="H13" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="I13" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="J13" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="I13" s="23" t="s">
+    </row>
+    <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
+      <c r="A14" s="22" t="s">
         <v>96</v>
       </c>
-      <c r="J13" s="23" t="s">
+      <c r="B14" s="23" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="B14" s="23" t="s">
-        <v>99</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>404</v>
+        <v>364</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="I14" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="H14" s="23" t="s">
+      <c r="J14" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="I14" s="23" t="s">
+    </row>
+    <row r="15" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="22" t="s">
         <v>102</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="22" t="s">
-        <v>104</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>43</v>
@@ -3114,97 +3111,97 @@
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>406</v>
+        <v>365</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H15" s="23" t="s">
+        <v>103</v>
+      </c>
+      <c r="I15" s="23" t="s">
+        <v>104</v>
+      </c>
+      <c r="J15" s="23" t="s">
         <v>105</v>
-      </c>
-      <c r="I15" s="23" t="s">
-        <v>106</v>
-      </c>
-      <c r="J15" s="23" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H16" s="23" t="s">
+        <v>110</v>
+      </c>
+      <c r="I16" s="23" t="s">
+        <v>111</v>
+      </c>
+      <c r="J16" s="23" t="s">
         <v>112</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>113</v>
-      </c>
-      <c r="J16" s="23" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H17" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="I17" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="J17" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="I17" s="23" t="s">
+    </row>
+    <row r="18" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="22" t="s">
         <v>120</v>
-      </c>
-      <c r="J17" s="23" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="72" x14ac:dyDescent="0.3">
-      <c r="A18" s="22" t="s">
-        <v>122</v>
       </c>
       <c r="B18" s="23" t="s">
         <v>33</v>
@@ -3213,31 +3210,31 @@
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>124</v>
+        <v>402</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="I18" s="23" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B19" s="23" t="s">
         <v>65</v>
@@ -3246,7 +3243,7 @@
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E19" s="23" t="s">
         <v>56</v>
@@ -3256,21 +3253,21 @@
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="I19" s="23" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B20" s="23" t="s">
         <v>33</v>
@@ -3279,7 +3276,7 @@
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E20" s="23" t="s">
         <v>56</v>
@@ -3289,54 +3286,54 @@
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I21" s="23" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B22" s="23" t="s">
         <v>43</v>
@@ -3345,59 +3342,59 @@
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I22" s="23" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>373</v>
+        <v>337</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>374</v>
+        <v>403</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -3474,25 +3471,25 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>157</v>
+        <v>388</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>355</v>
+        <v>389</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="24" t="s">
         <v>34</v>
@@ -3501,27 +3498,27 @@
         <v>56</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>162</v>
+        <v>396</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>163</v>
+        <v>397</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3534,27 +3531,27 @@
         <v>56</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3567,27 +3564,27 @@
         <v>56</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3597,30 +3594,30 @@
         <v>34</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>353</v>
+        <v>319</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>354</v>
+        <v>320</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3630,30 +3627,30 @@
         <v>34</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>433</v>
+        <v>398</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>185</v>
+        <v>399</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3666,27 +3663,27 @@
         <v>56</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>412</v>
+        <v>394</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>413</v>
+        <v>395</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3699,27 +3696,27 @@
         <v>56</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
@@ -3732,123 +3729,123 @@
         <v>56</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>199</v>
+        <v>392</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>200</v>
+        <v>393</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H10" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>395</v>
+        <v>358</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>396</v>
+        <v>359</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H11" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H12" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="E13" s="23" t="s">
         <v>56</v>
@@ -3858,30 +3855,30 @@
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H13" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>216</v>
+        <v>207</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="E14" s="23" t="s">
         <v>56</v>
@@ -3891,30 +3888,30 @@
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H14" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>56</v>
@@ -3924,49 +3921,49 @@
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H15" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C16" s="24" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>225</v>
+        <v>390</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>226</v>
+        <v>391</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H16" s="23" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -3996,7 +3993,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4020,69 +4017,69 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>224</v>
+        <v>74</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
+        <v>Parcial</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>226</v>
+        <v>354</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>234</v>
+        <v>355</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>235</v>
+        <v>424</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="H2" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G2))/Resumen!$C$8</f>
-        <v>0.82432432432432434</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.89189189189189189</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>76</v>
+        <v>166</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>391</v>
+        <v>169</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>392</v>
+        <v>425</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>235</v>
+        <v>426</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4090,28 +4087,28 @@
       </c>
       <c r="H3" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G3))/Resumen!$C$8</f>
-        <v>0.83783783783783783</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.90540540540540537</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>200</v>
+        <v>427</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>237</v>
+        <v>428</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>235</v>
+        <v>429</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>236</v>
+        <v>224</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4119,86 +4116,86 @@
       </c>
       <c r="H4" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G4))/Resumen!$C$8</f>
-        <v>0.85135135135135132</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+        <v>0.91891891891891897</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>175</v>
+        <v>430</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>238</v>
+        <v>431</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>239</v>
+        <v>432</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H5" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G5))/Resumen!$C$8</f>
-        <v>0.86486486486486491</v>
+        <v>0.94594594594594594</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>183</v>
+        <v>90</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
+        <v>Pendiente</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>185</v>
+        <v>92</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>240</v>
+        <v>226</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H6" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G6))/Resumen!$C$8</f>
-        <v>0.8783783783783784</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>0.97297297297297303</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>155</v>
+        <v>78</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>355</v>
+        <v>81</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>362</v>
+        <v>228</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>242</v>
+        <v>223</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>241</v>
+        <v>227</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4206,161 +4203,16 @@
       </c>
       <c r="H7" s="26">
         <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G7))/Resumen!$C$8</f>
-        <v>0.90540540540540537</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="B8" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
-        <v>Parcial</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>243</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="F8" s="24" t="s">
-        <v>241</v>
-      </c>
-      <c r="G8" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A8,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A8,RNF!$A$2:$A$100,0)))</f>
-        <v>0.5</v>
-      </c>
-      <c r="H8" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G8))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="22" t="s">
-        <v>203</v>
-      </c>
-      <c r="B9" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>Implementado</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>401</v>
-      </c>
-      <c r="D9" s="23" t="s">
-        <v>402</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>403</v>
-      </c>
-      <c r="F9" s="24" t="s">
-        <v>241</v>
-      </c>
-      <c r="G9" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A9,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A9,RNF!$A$2:$A$100,0)))</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G9))/Resumen!$C$8</f>
-        <v>0.91891891891891897</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="22" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>163</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>244</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>239</v>
-      </c>
-      <c r="F10" s="24" t="s">
-        <v>241</v>
-      </c>
-      <c r="G10" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A10,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A10,RNF!$A$2:$A$100,0)))</f>
         <v>1</v>
       </c>
-      <c r="H10" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G10))/Resumen!$C$8</f>
-        <v>0.94594594594594594</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="B11" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C11" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="D11" s="23" t="s">
-        <v>245</v>
-      </c>
-      <c r="E11" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="F11" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="G11" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A11,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A11,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
-      </c>
-      <c r="H11" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G11))/Resumen!$C$8</f>
-        <v>0.97297297297297303</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12" s="24" t="str">
-        <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
-        <v>Pendiente</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>83</v>
-      </c>
-      <c r="D12" s="23" t="s">
-        <v>247</v>
-      </c>
-      <c r="E12" s="23" t="s">
-        <v>235</v>
-      </c>
-      <c r="F12" s="24" t="s">
-        <v>246</v>
-      </c>
-      <c r="G12" s="25">
-        <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A12,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A12,RNF!$A$2:$A$100,0)))</f>
-        <v>1</v>
-      </c>
-      <c r="H12" s="26">
-        <f>(Resumen!$G$8*Resumen!$C$8+SUM($G$2:G12))/Resumen!$C$8</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="17" t="s">
-        <v>363</v>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>327</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B12">
+  <conditionalFormatting sqref="B2:B7">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
       <formula>"Implementado"</formula>
     </cfRule>
@@ -4392,7 +4244,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>H2:H12</xm:sqref>
+          <xm:sqref>H2:H7</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -4416,30 +4268,30 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>248</v>
+        <v>229</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>249</v>
+        <v>230</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>250</v>
+        <v>231</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>251</v>
+        <v>232</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>252</v>
+        <v>233</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>253</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>254</v>
+        <v>235</v>
       </c>
       <c r="B2" s="23" t="s">
         <v>32</v>
@@ -4448,44 +4300,44 @@
         <v>23</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>375</v>
+        <v>338</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>376</v>
+        <v>339</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>257</v>
+        <v>238</v>
       </c>
       <c r="B3" s="23" t="s">
         <v>32</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>377</v>
+        <v>340</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>378</v>
+        <v>341</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>258</v>
+        <v>239</v>
       </c>
       <c r="B4" s="23" t="s">
         <v>38</v>
@@ -4494,21 +4346,21 @@
         <v>23</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>430</v>
+        <v>384</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>431</v>
+        <v>385</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>417</v>
+        <v>373</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>259</v>
+        <v>240</v>
       </c>
       <c r="B5" s="23" t="s">
         <v>38</v>
@@ -4517,21 +4369,21 @@
         <v>23</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>379</v>
+        <v>342</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>380</v>
+        <v>343</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="B6" s="23" t="s">
         <v>42</v>
@@ -4540,21 +4392,21 @@
         <v>23</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>262</v>
+        <v>243</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>263</v>
+        <v>244</v>
       </c>
       <c r="F6" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>264</v>
+        <v>245</v>
       </c>
       <c r="B7" s="23" t="s">
         <v>42</v>
@@ -4563,21 +4415,21 @@
         <v>23</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>265</v>
+        <v>246</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>266</v>
+        <v>247</v>
       </c>
       <c r="F7" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>267</v>
+        <v>248</v>
       </c>
       <c r="B8" s="23" t="s">
         <v>49</v>
@@ -4586,44 +4438,44 @@
         <v>23</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>365</v>
+        <v>329</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>268</v>
+        <v>249</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>269</v>
+        <v>250</v>
       </c>
       <c r="B9" s="23" t="s">
         <v>49</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>422</v>
+        <v>378</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>423</v>
+        <v>379</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>417</v>
+        <v>373</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>271</v>
+        <v>252</v>
       </c>
       <c r="B10" s="23" t="s">
         <v>53</v>
@@ -4632,39 +4484,39 @@
         <v>23</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>272</v>
+        <v>253</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>273</v>
+        <v>254</v>
       </c>
       <c r="F10" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>274</v>
+        <v>255</v>
       </c>
       <c r="B11" s="23" t="s">
         <v>53</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>276</v>
+        <v>257</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>277</v>
+        <v>258</v>
       </c>
       <c r="F11" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -4678,16 +4530,16 @@
         <v>23</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>397</v>
+        <v>360</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>398</v>
+        <v>361</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>390</v>
+        <v>353</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
@@ -4701,21 +4553,21 @@
         <v>23</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>381</v>
+        <v>344</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>382</v>
+        <v>345</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>278</v>
+        <v>259</v>
       </c>
       <c r="B14" s="23" t="s">
         <v>69</v>
@@ -4724,872 +4576,872 @@
         <v>23</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>279</v>
+        <v>404</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>280</v>
-      </c>
-      <c r="F14" s="23" t="s">
-        <v>255</v>
+        <v>405</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>406</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>281</v>
+        <v>260</v>
       </c>
       <c r="B15" s="23" t="s">
         <v>69</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>23</v>
+        <v>407</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>282</v>
+        <v>408</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>283</v>
-      </c>
-      <c r="F15" s="23" t="s">
-        <v>255</v>
+        <v>409</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>406</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>387</v>
+        <v>350</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>388</v>
+        <v>351</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>389</v>
+        <v>352</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>390</v>
+        <v>353</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C17" s="23" t="s">
-        <v>270</v>
+        <v>251</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>284</v>
+        <v>261</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>285</v>
+        <v>262</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>356</v>
+        <v>321</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>424</v>
+        <v>380</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>425</v>
+        <v>381</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>417</v>
+        <v>373</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>286</v>
+        <v>263</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>287</v>
+        <v>264</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>356</v>
+        <v>321</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>415</v>
+        <v>371</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>416</v>
+        <v>372</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>417</v>
+        <v>373</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>289</v>
+        <v>266</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C21" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>418</v>
+        <v>374</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>419</v>
+        <v>375</v>
       </c>
       <c r="F21" s="28" t="s">
-        <v>417</v>
+        <v>373</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>290</v>
+        <v>267</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>420</v>
+        <v>376</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>421</v>
+        <v>377</v>
       </c>
       <c r="F22" s="28" t="s">
-        <v>417</v>
+        <v>373</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>291</v>
+        <v>268</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>292</v>
+        <v>269</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>293</v>
+        <v>270</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>294</v>
+        <v>271</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>295</v>
+        <v>272</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>296</v>
+        <v>273</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>297</v>
+        <v>274</v>
       </c>
       <c r="F24" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>298</v>
+        <v>275</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>299</v>
+        <v>276</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>300</v>
+        <v>277</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>301</v>
+        <v>278</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>302</v>
+        <v>279</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>303</v>
+        <v>280</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>304</v>
+        <v>281</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C27" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>305</v>
+        <v>282</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>306</v>
+        <v>283</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>307</v>
+        <v>284</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>260</v>
+        <v>241</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>308</v>
+        <v>285</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>309</v>
+        <v>286</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C29" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>310</v>
+        <v>287</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>311</v>
+        <v>288</v>
       </c>
       <c r="F29" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C30" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>312</v>
+        <v>289</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>313</v>
+        <v>290</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>314</v>
+        <v>291</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>315</v>
+        <v>292</v>
       </c>
       <c r="F31" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>316</v>
+        <v>293</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>317</v>
+        <v>294</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>318</v>
+        <v>295</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C33" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>383</v>
+        <v>346</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>384</v>
+        <v>347</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>319</v>
+        <v>296</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>320</v>
+        <v>297</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>366</v>
+        <v>330</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>367</v>
+        <v>331</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="B35" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>305</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>410</v>
+      </c>
+      <c r="E35" s="23" t="s">
+        <v>411</v>
+      </c>
+      <c r="F35" s="28" t="s">
+        <v>406</v>
+      </c>
+      <c r="G35" s="23" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="B35" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="C35" s="23" t="s">
-        <v>321</v>
-      </c>
-      <c r="D35" s="23" t="s">
-        <v>322</v>
-      </c>
-      <c r="E35" s="23" t="s">
-        <v>323</v>
-      </c>
-      <c r="F35" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="G35" s="23" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="22" t="s">
-        <v>164</v>
-      </c>
       <c r="B36" s="23" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>23</v>
+        <v>412</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>324</v>
+        <v>413</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>325</v>
-      </c>
-      <c r="F36" s="23" t="s">
-        <v>255</v>
+        <v>414</v>
+      </c>
+      <c r="F36" s="28" t="s">
+        <v>406</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C37" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>326</v>
+        <v>298</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>327</v>
+        <v>299</v>
       </c>
       <c r="F37" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C38" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>328</v>
+        <v>300</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>329</v>
+        <v>301</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>330</v>
+        <v>302</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C39" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>357</v>
+        <v>322</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>358</v>
+        <v>323</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>364</v>
+        <v>328</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>331</v>
+        <v>303</v>
       </c>
       <c r="B40" s="23" t="s">
+        <v>173</v>
+      </c>
+      <c r="C40" s="23" t="s">
+        <v>324</v>
+      </c>
+      <c r="D40" s="23" t="s">
+        <v>325</v>
+      </c>
+      <c r="E40" s="23" t="s">
+        <v>326</v>
+      </c>
+      <c r="F40" s="27" t="s">
+        <v>328</v>
+      </c>
+      <c r="G40" s="23" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A41" s="22" t="s">
         <v>179</v>
       </c>
-      <c r="C40" s="23" t="s">
-        <v>359</v>
-      </c>
-      <c r="D40" s="23" t="s">
-        <v>360</v>
-      </c>
-      <c r="E40" s="23" t="s">
-        <v>361</v>
-      </c>
-      <c r="F40" s="27" t="s">
-        <v>364</v>
-      </c>
-      <c r="G40" s="23" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="22" t="s">
-        <v>186</v>
-      </c>
       <c r="B41" s="23" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>332</v>
+        <v>415</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>434</v>
+        <v>416</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>333</v>
-      </c>
-      <c r="F41" s="23" t="s">
-        <v>255</v>
+        <v>417</v>
+      </c>
+      <c r="F41" s="28" t="s">
+        <v>406</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>334</v>
+        <v>304</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>335</v>
+        <v>305</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>426</v>
+        <v>382</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>427</v>
+        <v>383</v>
       </c>
       <c r="F42" s="28" t="s">
-        <v>417</v>
+        <v>373</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>336</v>
+        <v>306</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>301</v>
+        <v>278</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>428</v>
+        <v>418</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>429</v>
+        <v>419</v>
       </c>
       <c r="F43" s="28" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="B44" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="C44" s="23" t="s">
+        <v>135</v>
+      </c>
+      <c r="D44" s="23" t="s">
+        <v>307</v>
+      </c>
+      <c r="E44" s="23" t="s">
+        <v>308</v>
+      </c>
+      <c r="F44" s="23" t="s">
+        <v>236</v>
+      </c>
+      <c r="G44" s="23" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="22" t="s">
         <v>192</v>
       </c>
-      <c r="C44" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="D44" s="23" t="s">
-        <v>337</v>
-      </c>
-      <c r="E44" s="23" t="s">
-        <v>338</v>
-      </c>
-      <c r="F44" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="G44" s="23" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="22" t="s">
-        <v>201</v>
-      </c>
       <c r="B45" s="23" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C45" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>339</v>
+        <v>420</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>340</v>
-      </c>
-      <c r="F45" s="23" t="s">
-        <v>255</v>
+        <v>421</v>
+      </c>
+      <c r="F45" s="28" t="s">
+        <v>406</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="C46" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>399</v>
+        <v>362</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>400</v>
+        <v>363</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>390</v>
+        <v>353</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>206</v>
+        <v>197</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>341</v>
+        <v>309</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>342</v>
+        <v>310</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>343</v>
+        <v>311</v>
       </c>
       <c r="F47" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
       <c r="C48" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>344</v>
+        <v>312</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>345</v>
+        <v>313</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="C49" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>346</v>
+        <v>314</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>347</v>
+        <v>315</v>
       </c>
       <c r="F49" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="C50" s="23" t="s">
         <v>23</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>348</v>
+        <v>316</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>349</v>
+        <v>317</v>
       </c>
       <c r="F50" s="23" t="s">
-        <v>255</v>
+        <v>236</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>260</v>
+        <v>321</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>350</v>
+        <v>422</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>351</v>
-      </c>
-      <c r="F51" s="23" t="s">
-        <v>255</v>
+        <v>423</v>
+      </c>
+      <c r="F51" s="28" t="s">
+        <v>406</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>256</v>
+        <v>237</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>352</v>
+        <v>318</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(avance): meta del Excel al 90 % y citas de la fase 1 verificadas en develop
Meta: por decision de Luis, Resumen!C40 pasa de 0,8 a 0,9 (por COM, como
numero) y D40 dice que la del 80 % pedida para la entrega ya esta superada.
Puntos que faltan: 0,3 (RF), 0,5 (RNF) y 0,8 (total); graficos y formato
condicional sin cambios. La matriz marca la meta del 90 % en la ruta y da los
puntos que faltan por tipo; estado.md actualiza la seccion del 25 y
«Resultado» (las del 18 al 20 quedan como registro).

Citas de la fase 1 (main @ 54b19fa) mapeadas con git diff y verificadas por
contenido en develop @ 21e7e9c, en el Excel, el docx y la matriz: RQF-03 y
RQF-21 (miembros.js, MiembrosPage.jsx), RQF-05 (checkin.js,
CheckinPage.jsx), RQF-15 (auth-helpers.js) y RQF-18 (dashboard.js,
DashboardPage.jsx); tambien RQF-06, citado el 19 y corrido por #30 y #32.
RQF-12 queda igual: cliente.js y Poblar_Tablas.sql no cambiaron. Sigue en
87,8 %.
</commit_message>
<xml_diff>
--- a/docs/avance-requisitos.xlsx
+++ b/docs/avance-requisitos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Proyecto_FitLoyalty\.claude\worktrees\avance-requisitos-ca5ff0\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D485DDE-28AC-4CF7-85D1-1395B4373279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6023229-9EEF-4186-A584-DDA388B9850D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -110,9 +110,6 @@
     <t>Meta de avance (editable)</t>
   </si>
   <si>
-    <t>Meta del 80 % pedida por Luis para la entrega.</t>
-  </si>
-  <si>
     <t>Código</t>
   </si>
   <si>
@@ -176,9 +173,6 @@
     <t>Gestión de Miembros</t>
   </si>
   <si>
-    <t>POST /api/admin/miembros rechaza documento o correo duplicados (miembros.js:357-369) y genera un código QR único (:371-379); editar con PUT (:607); desactivar con activo = FALSE (:664-675); pantalla MiembrosPage.jsx:627, :919, :442.</t>
-  </si>
-  <si>
     <t>Observación: al editar no se vuelven a validar duplicados de documento o correo (criterio 2 de HU-09).</t>
   </si>
   <si>
@@ -209,9 +203,6 @@
     <t>Check-in y Asistencia</t>
   </si>
   <si>
-    <t>Campo con autoFocus que recibe la lectura del lector HID tipo teclado y envía con Enter (CheckinPage.jsx:221-223, :329-331); lectura por cámara (CheckinPage.jsx:66); POST /api/admin/checkin inserta el ingreso (checkin.js:54, :167-172); fecha_hora DEFAULT CURRENT_TIMESTAMP (migración 002:100).</t>
-  </si>
-  <si>
     <t>—</t>
   </si>
   <si>
@@ -368,9 +359,6 @@
     <t>App del miembro</t>
   </si>
   <si>
-    <t>POST /api/cliente/login con teléfono y contraseña bcrypt (cliente.js:51, :88) y JWT de 30 días (auth-helpers.js:145); rutas protegidas con requireClient (cliente.js:112); /qr, /membresia, /asistencia, /gamificacion y /retos (cliente.js:227, :259, :292, :340, :392); edición del perfil con PUT /api/cliente/me, que valida el correo único (cliente.js:171-225); app Flutter: login_screen.dart, qr_tab.dart, plan_tab.dart, asistencia_screen.dart, gamificacion_screen.dart, editar_perfil_screen.dart; token en FlutterSecureStorage (api_client.dart:41).</t>
-  </si>
-  <si>
     <t>Ajuste de redacción: el PR #4 decía «rachas», que no se calculan (ver RQF-11); la app muestra hitos y retos de solo lectura. Absorbe RQF-26 (edición del perfil), que el PR #4 contaba aparte. Sin pruebas automatizadas reales (widget_test.dart es una prueba mínima).</t>
   </si>
   <si>
@@ -413,9 +401,6 @@
     <t>RQF-18</t>
   </si>
   <si>
-    <t>GET /api/admin/dashboard/export arma un CSV RFC 4180 de miembros activos con su plan (dashboard.js:288-337, helpers :31-50); el panel lo descarga (DashboardPage.jsx:193-203).</t>
-  </si>
-  <si>
     <t>HU-60</t>
   </si>
   <si>
@@ -455,9 +440,6 @@
     <t>RQF-21</t>
   </si>
   <si>
-    <t>Esquema de alta con valor_total, valor_pagado, metodo_pago y estado_pago (miembros.js:88-95); inserción en plan_cobro (miembros.js:439-450, migración 004); edición del plan (miembros.js:754); validaciones en MiembrosPage.jsx:349-350.</t>
-  </si>
-  <si>
     <t>Ajuste de redacción: se acotó al pago, porque el plan y su vigencia ya están en RQF-04.</t>
   </si>
   <si>
@@ -740,18 +722,12 @@
     <t>EV-05</t>
   </si>
   <si>
-    <t>backend/src/routes/miembros.js:357-369, :371-379</t>
-  </si>
-  <si>
     <t>Rechazo de documento / correo duplicado y QR único.</t>
   </si>
   <si>
     <t>EV-06</t>
   </si>
   <si>
-    <t>backend/src/routes/miembros.js:607, :664-675; frontend/src/pages/MiembrosPage.jsx:627, :919, :442</t>
-  </si>
-  <si>
     <t>Editar y desactivar (soft delete) desde la pantalla de miembros.</t>
   </si>
   <si>
@@ -770,9 +746,6 @@
     <t>EV-09</t>
   </si>
   <si>
-    <t>frontend/src/pages/CheckinPage.jsx:66, :221-223, :329-331</t>
-  </si>
-  <si>
     <t>Lectura HID tipo teclado (autoFocus + Enter) y por cámara.</t>
   </si>
   <si>
@@ -782,9 +755,6 @@
     <t>Código / esquema</t>
   </si>
   <si>
-    <t>backend/src/routes/checkin.js:54, :167-172; backend/migrations/002_esquema_inicial.sql:100</t>
-  </si>
-  <si>
     <t>Inserción del ingreso con marca de tiempo automática.</t>
   </si>
   <si>
@@ -818,9 +788,6 @@
     <t>EV-22</t>
   </si>
   <si>
-    <t>backend/src/routes/cliente.js:51, :88, :112, :227, :259, :292, :340, :392; backend/src/lib/auth-helpers.js:145</t>
-  </si>
-  <si>
     <t>API de la app: login del miembro y consultas protegidas.</t>
   </si>
   <si>
@@ -863,9 +830,6 @@
     <t>El código se devuelve en la respuesta si el correo no sale.</t>
   </si>
   <si>
-    <t>backend/src/routes/dashboard.js:31-50, :288-337; frontend/src/pages/DashboardPage.jsx:193-203</t>
-  </si>
-  <si>
     <t>Exportación CSV de miembros activos con su membresía.</t>
   </si>
   <si>
@@ -875,9 +839,6 @@
     <t>Configuración de precios y recordatorios por gimnasio.</t>
   </si>
   <si>
-    <t>backend/src/routes/miembros.js:88-95, :439-450, :754; backend/migrations/004_extender_miembro_cobros.sql:54; frontend/src/pages/MiembrosPage.jsx:207-208, :349-350</t>
-  </si>
-  <si>
     <t>Registro del plan y del pago por miembro.</t>
   </si>
   <si>
@@ -1232,9 +1193,6 @@
     <t>Cálculo automático de fecha_fin según el plan (miembros.js:193, :395); estado vencido / por vencer contra la fecha actual (:286-290); renovación del plan (:926). Estado Congelada (PR #17, migración 010): POST /api/admin/miembros/:id/congelar (:810) y /descongelar (:869), que corre fecha_fin y la próxima fecha de cobro los días congelados (:892), con historial en congelacion_plan; pantalla en MiembrosPage.jsx:238, :742, :1907. Desde el PR #30, el check-in niega el ingreso de una membresía congelada con estado CONGELADO, sin registrar asistencia (checkin.js:125-149); el job de avisos la excluye (expiracion.js:62) y la campana la muestra como acceso bloqueado (notificaciones.js:106-112); ULTIMO_PLAN trae congelado_desde (lib/planes.js:30).</t>
   </si>
   <si>
-    <t>Valida el último plan en el check-in (checkin.js:123-131) y, si está vencido o no hay plan, bloquea y responde VENCIDO sin registrar asistencia (:133-147; el INSERT en checkin de :182 queda fuera de ese camino); la pantalla muestra «Acceso denegado» (CheckinPage.jsx:134-135, :187-188). Avisa al administrador: registrarAccesoBloqueado (lib/accesos.js:33) guarda el intento en notificacion sin repetirlo en 10 minutos (:20, :39-49) y la campana lo muestra primero (notificaciones.js:79-115, :175-190), con «Visto» (:226-241) y refresco cada 30 s (MenuNotificaciones.jsx:52, :72). PR #23, con la migración 014 (PR #27) para Docker.</t>
-  </si>
-  <si>
     <t>Motor diario (jobs/abandono.js:97, runJob) programado a las 8:00 en hora de Colombia (scheduler.js:71): clasifica en AMARILLA desde umbral_alerta_amarilla días sin ingresar (7 por defecto) y en ROJA desde umbral_alerta_roja (15) (abandono.js:35-37), y deja una sola alerta PENDIENTE por miembro en alerta_abandono: la sube de nivel, la cierra como GESTIONADA si vuelve e IGNORADA si deja de aplicar (congela, vence o se da de baja) (abandono.js:19-22). Umbrales por gimnasio con validación: la roja debe ser mayor que la amarilla o responde 400 (config.js:36-71; ConfigPage.jsx:18-19, :45-46); la campana los lista, ROJA primero (notificaciones.js:149-207); ejecución manual con POST /api/jobs/abandono/run (jobs.js:46). La migración 012 alinea alerta_abandono con producción. 28 pruebas en backend/tests/abandono.test.js. PR #39.</t>
   </si>
   <si>
@@ -1292,9 +1250,6 @@
     <t>backend/src/routes/auth.js:212, :243, :313; backend/src/index.js:66, :97; frontend/src/context/AuthContext.jsx:23-27, :40, :150-178, :223; frontend/src/api.js:115; frontend/src/pages/CheckinPage.jsx:170, :225 (marcarActividad)</t>
   </si>
   <si>
-    <t>backend/src/routes/checkin.js:123-147, :182; backend/src/lib/accesos.js:20, :33-52; backend/src/routes/notificaciones.js:79-115, :175-190, :226-241; frontend/src/components/MenuNotificaciones.jsx:52, :72; frontend/src/pages/CheckinPage.jsx:134-135</t>
-  </si>
-  <si>
     <t>backend/src/jobs/abandono.js:19-37, :97; backend/src/jobs/scheduler.js:71; backend/src/routes/config.js:36-71; backend/src/routes/notificaciones.js:149-207; backend/src/routes/jobs.js:46; frontend/src/pages/ConfigPage.jsx:18-19, :45-46</t>
   </si>
   <si>
@@ -1341,6 +1296,51 @@
   </si>
   <si>
     <t>backend/src/middleware/errorHandler.js:17-49; backend/src/lib/errors.js; backend/src/lib/asyncHandler.js; backend/src/index.js:135-139</t>
+  </si>
+  <si>
+    <t>POST /api/admin/miembros rechaza documento o correo duplicados (miembros.js:370-382) y genera un código QR único (:384-392); editar con PUT (:620); desactivar con activo = FALSE (:677-688); pantalla MiembrosPage.jsx:635, :961, :450.</t>
+  </si>
+  <si>
+    <t>Campo con autoFocus que recibe la lectura del lector HID tipo teclado y envía con Enter (CheckinPage.jsx:238-240, :346-348); lectura por cámara (CheckinPage.jsx:79); POST /api/admin/checkin inserta el ingreso (checkin.js:62, :203-208); fecha_hora DEFAULT CURRENT_TIMESTAMP (migración 002:100).</t>
+  </si>
+  <si>
+    <t>Valida el último plan en el check-in (checkin.js:124-132) y, si está vencido o no hay plan, bloquea y responde VENCIDO sin registrar asistencia (:155-169; el INSERT en checkin de :204 queda fuera de ese camino); la pantalla muestra «Acceso denegado» (CheckinPage.jsx:25-29). Avisa al administrador: registrarAccesoBloqueado (lib/accesos.js:34) guarda el intento en notificacion sin repetirlo en 10 minutos (:20, :40-50) y la campana lo muestra primero (notificaciones.js:79-115, :175-190), con «Visto» (:226-241) y refresco cada 30 s (MenuNotificaciones.jsx:52, :72). PR #23, con la migración 014 (PR #27) para Docker.</t>
+  </si>
+  <si>
+    <t>POST /api/cliente/login con teléfono y contraseña bcrypt (cliente.js:51, :88) y JWT de 30 días (auth-helpers.js:178); rutas protegidas con requireClient (cliente.js:112); /qr, /membresia, /asistencia, /gamificacion y /retos (cliente.js:227, :259, :292, :340, :392); edición del perfil con PUT /api/cliente/me, que valida el correo único (cliente.js:171-225); app Flutter: login_screen.dart, qr_tab.dart, plan_tab.dart, asistencia_screen.dart, gamificacion_screen.dart, editar_perfil_screen.dart; token en FlutterSecureStorage (api_client.dart:41).</t>
+  </si>
+  <si>
+    <t>GET /api/admin/dashboard/export arma un CSV RFC 4180 de miembros activos con su plan (dashboard.js:383-432, helpers :32-51); el panel lo descarga (DashboardPage.jsx:304-314).</t>
+  </si>
+  <si>
+    <t>Esquema de alta con valor_total, valor_pagado, metodo_pago y estado_pago (miembros.js:96-103); inserción en plan_cobro (miembros.js:452-463, migración 004); edición del plan (miembros.js:926); validaciones en MiembrosPage.jsx:357-358.</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:370-382, :384-392</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:620, :677-688; frontend/src/pages/MiembrosPage.jsx:635, :961, :450</t>
+  </si>
+  <si>
+    <t>frontend/src/pages/CheckinPage.jsx:79, :238-240, :346-348</t>
+  </si>
+  <si>
+    <t>backend/src/routes/checkin.js:62, :203-208; backend/migrations/002_esquema_inicial.sql:100</t>
+  </si>
+  <si>
+    <t>backend/src/routes/checkin.js:124-169, :204; backend/src/lib/accesos.js:20, :34-53; backend/src/routes/notificaciones.js:79-115, :175-190, :226-241; frontend/src/components/MenuNotificaciones.jsx:52, :72; frontend/src/pages/CheckinPage.jsx:25-29</t>
+  </si>
+  <si>
+    <t>backend/src/routes/cliente.js:51, :88, :112, :227, :259, :292, :340, :392; backend/src/lib/auth-helpers.js:178</t>
+  </si>
+  <si>
+    <t>backend/src/routes/dashboard.js:32-51, :383-432; frontend/src/pages/DashboardPage.jsx:304-314</t>
+  </si>
+  <si>
+    <t>backend/src/routes/miembros.js:96-103, :452-463, :926; backend/migrations/004_extender_miembro_cobros.sql:54; frontend/src/pages/MiembrosPage.jsx:208-209, :357-358</t>
+  </si>
+  <si>
+    <t>Meta del plan de trabajo (90 %); la del 80 % pedida por Luis para la entrega ya está superada.</t>
   </si>
 </sst>
 </file>
@@ -2310,7 +2310,7 @@
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
-        <v>393</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
@@ -2371,11 +2371,11 @@
       </c>
       <c r="H6" s="10">
         <f>Resumen!$C$40</f>
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I6" s="11">
         <f>MAX(0,H6*C6-G6*C6)</f>
-        <v>0</v>
+        <v>0.30000000000000071</v>
       </c>
       <c r="J6" t="s">
         <v>12</v>
@@ -2411,11 +2411,11 @@
       </c>
       <c r="H7" s="10">
         <f>Resumen!$C$40</f>
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I7" s="11">
         <f>MAX(0,H7*C7-G7*C7)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J7" t="s">
         <v>14</v>
@@ -2451,11 +2451,11 @@
       </c>
       <c r="H8" s="15">
         <f>Resumen!$C$40</f>
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I8" s="16">
         <f>MAX(0,H8*C8-G8*C8)</f>
-        <v>0</v>
+        <v>0.80000000000000426</v>
       </c>
       <c r="J8" t="s">
         <v>16</v>
@@ -2607,10 +2607,10 @@
         <v>21</v>
       </c>
       <c r="C40" s="21">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>22</v>
+        <v>432</v>
       </c>
     </row>
   </sheetData>
@@ -2638,760 +2638,760 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="23" t="s">
         <v>32</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>33</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>310</v>
+        <v>297</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>311</v>
+        <v>298</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G2" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H2" s="23" t="s">
+      <c r="I2" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="J2" s="23" t="s">
         <v>36</v>
-      </c>
-      <c r="J2" s="23" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>394</v>
+        <v>381</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>337</v>
+        <v>324</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H3" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="J3" s="23" t="s">
         <v>40</v>
-      </c>
-      <c r="J3" s="23" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="23" t="s">
         <v>42</v>
-      </c>
-      <c r="B4" s="23" t="s">
-        <v>43</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>44</v>
+        <v>418</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H4" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="23" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="23" t="s">
         <v>46</v>
-      </c>
-      <c r="I4" s="23" t="s">
-        <v>47</v>
-      </c>
-      <c r="J4" s="23" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>395</v>
+        <v>382</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>335</v>
+        <v>322</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H5" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" s="23" t="s">
         <v>50</v>
-      </c>
-      <c r="I5" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="J5" s="23" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>55</v>
+        <v>419</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>396</v>
+        <v>420</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>330</v>
+        <v>317</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>312</v>
+        <v>299</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>397</v>
+        <v>383</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>398</v>
+        <v>384</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="216" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>399</v>
+        <v>385</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>325</v>
+        <v>312</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>400</v>
+        <v>386</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>336</v>
+        <v>323</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="144" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>361</v>
+        <v>348</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="H14" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="I14" s="23" t="s">
+        <v>97</v>
+      </c>
+      <c r="J14" s="23" t="s">
         <v>98</v>
-      </c>
-      <c r="H14" s="23" t="s">
-        <v>99</v>
-      </c>
-      <c r="I14" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="J14" s="23" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>401</v>
+        <v>387</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>362</v>
+        <v>349</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>108</v>
+        <v>421</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C17" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>402</v>
+        <v>388</v>
       </c>
       <c r="E17" s="23" t="s">
-        <v>403</v>
+        <v>389</v>
       </c>
       <c r="F17" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C17,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G17" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I17" s="23" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C18" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>404</v>
+        <v>390</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>363</v>
+        <v>350</v>
       </c>
       <c r="F18" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C18,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G18" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="I18" s="23" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C19" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>123</v>
+        <v>422</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F19" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C19,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G19" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="I19" s="23" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C20" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>405</v>
+        <v>391</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F20" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C20,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G20" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I20" s="23" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="C21" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>406</v>
+        <v>392</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="F21" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C21,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G21" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="I21" s="23" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C22" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>137</v>
+        <v>423</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="F22" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C22,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G22" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="I22" s="23" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C23" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>364</v>
+        <v>351</v>
       </c>
       <c r="F23" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C23,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G23" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="I23" s="23" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -3438,529 +3438,529 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C2" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>349</v>
+        <v>336</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>350</v>
+        <v>337</v>
       </c>
       <c r="F2" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C2,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I2" s="23" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="J2" s="23" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>357</v>
+        <v>344</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>358</v>
+        <v>345</v>
       </c>
       <c r="F3" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C3,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0</v>
       </c>
       <c r="G3" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I3" s="23" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="J3" s="23" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C4" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>407</v>
+        <v>393</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>408</v>
+        <v>394</v>
       </c>
       <c r="F4" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C4,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G4" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I4" s="23" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="J4" s="23" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F5" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C5,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C6" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>409</v>
+        <v>395</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>299</v>
+        <v>286</v>
       </c>
       <c r="F6" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C6,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H6" s="23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="I6" s="23" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>359</v>
+        <v>346</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>360</v>
+        <v>347</v>
       </c>
       <c r="F7" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C7,Resumen!$B$36:$B$38,0)),0)</f>
         <v>0.5</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H7" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C8" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>355</v>
+        <v>342</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>356</v>
+        <v>343</v>
       </c>
       <c r="F8" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C8,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H8" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I8" s="23" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F9" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C9,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I9" s="23" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C10" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>353</v>
+        <v>340</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>354</v>
+        <v>341</v>
       </c>
       <c r="F10" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C10,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H10" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I10" s="23" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C11" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>410</v>
+        <v>396</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>331</v>
+        <v>318</v>
       </c>
       <c r="F11" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C11,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G11" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I11" s="23" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C12" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>411</v>
+        <v>397</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>412</v>
+        <v>398</v>
       </c>
       <c r="F12" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C12,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G12" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H12" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I12" s="23" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F13" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C13,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G13" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I13" s="23" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="C14" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>413</v>
+        <v>399</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F14" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C14,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G14" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I14" s="23" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C15" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>414</v>
+        <v>400</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="F15" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C15,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I15" s="23" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="72" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>12</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>352</v>
+        <v>339</v>
       </c>
       <c r="F16" s="25">
         <f>IFERROR(INDEX(Resumen!$C$36:$C$38,MATCH(C16,Resumen!$B$36:$B$38,0)),0)</f>
         <v>1</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I16" s="23" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -4005,7 +4005,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B1" s="6" t="s">
         <v>9</v>
@@ -4014,40 +4014,40 @@
         <v>16</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="H1" s="6" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B2" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>384</v>
+        <v>371</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G2" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A2,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A2,RNF!$A$2:$A$100,0)))</f>
@@ -4060,23 +4060,23 @@
     </row>
     <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B3" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>385</v>
+        <v>372</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>386</v>
+        <v>373</v>
       </c>
       <c r="F3" s="24" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G3" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A3,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A3,RNF!$A$2:$A$100,0)))</f>
@@ -4089,23 +4089,23 @@
     </row>
     <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B4" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
         <v>Parcial</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>387</v>
+        <v>374</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>388</v>
+        <v>375</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>389</v>
+        <v>376</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="G4" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A4,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A4,RNF!$A$2:$A$100,0)))</f>
@@ -4118,23 +4118,23 @@
     </row>
     <row r="5" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B5" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>390</v>
+        <v>377</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>391</v>
+        <v>378</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>392</v>
+        <v>379</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="G5" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A5,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A5,RNF!$A$2:$A$100,0)))</f>
@@ -4147,23 +4147,23 @@
     </row>
     <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B6" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G6" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A6,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A6,RNF!$A$2:$A$100,0)))</f>
@@ -4176,23 +4176,23 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B7" s="24" t="str">
         <f>IFERROR(INDEX(RF!$C$2:$C$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$C$2:$C$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
         <v>Pendiente</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="G7" s="25">
         <f>1-IFERROR(INDEX(RF!$F$2:$F$100,MATCH($A7,RF!$A$2:$A$100,0)),INDEX(RNF!$F$2:$F$100,MATCH($A7,RNF!$A$2:$A$100,0)))</f>
@@ -4205,7 +4205,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>305</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -4265,1180 +4265,1180 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="22" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>315</v>
+        <v>302</v>
       </c>
       <c r="E2" s="23" t="s">
-        <v>316</v>
+        <v>303</v>
       </c>
       <c r="F2" s="28" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="22" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B3" s="23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" s="23" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>317</v>
+        <v>304</v>
       </c>
       <c r="E3" s="23" t="s">
-        <v>318</v>
+        <v>305</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="22" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C4" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>415</v>
+        <v>401</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>348</v>
+        <v>335</v>
       </c>
       <c r="F4" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="22" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>320</v>
+        <v>307</v>
       </c>
       <c r="F5" s="28" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="22" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C6" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>232</v>
+        <v>424</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>233</v>
-      </c>
-      <c r="F6" s="23" t="s">
-        <v>225</v>
+        <v>226</v>
+      </c>
+      <c r="F6" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="22" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>235</v>
+        <v>425</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>236</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>225</v>
+        <v>228</v>
+      </c>
+      <c r="F7" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="22" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C8" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>307</v>
+        <v>294</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="F8" s="28" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="22" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C9" s="23" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>343</v>
+        <v>330</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>344</v>
+        <v>331</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>242</v>
+        <v>426</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>243</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>225</v>
+        <v>234</v>
+      </c>
+      <c r="F10" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G10" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>246</v>
+        <v>427</v>
       </c>
       <c r="E11" s="23" t="s">
-        <v>247</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>225</v>
+        <v>237</v>
+      </c>
+      <c r="F11" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G11" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>416</v>
+        <v>428</v>
       </c>
       <c r="E12" s="23" t="s">
-        <v>332</v>
+        <v>319</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G12" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C13" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>321</v>
+        <v>308</v>
       </c>
       <c r="E13" s="23" t="s">
-        <v>322</v>
+        <v>309</v>
       </c>
       <c r="F13" s="28" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G13" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>417</v>
+        <v>402</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>365</v>
+        <v>352</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="22" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C15" s="23" t="s">
-        <v>367</v>
+        <v>354</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>368</v>
+        <v>355</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>369</v>
+        <v>356</v>
       </c>
       <c r="F15" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="22" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>326</v>
+        <v>313</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>327</v>
+        <v>314</v>
       </c>
       <c r="F16" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B17" s="23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C17" s="23" t="s">
+        <v>232</v>
+      </c>
+      <c r="D17" s="23" t="s">
         <v>240</v>
       </c>
-      <c r="D17" s="23" t="s">
-        <v>250</v>
-      </c>
       <c r="E17" s="23" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="22" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>419</v>
+        <v>404</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>345</v>
+        <v>332</v>
       </c>
       <c r="F18" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="22" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="E19" s="23" t="s">
-        <v>254</v>
-      </c>
-      <c r="F19" s="23" t="s">
-        <v>225</v>
+        <v>244</v>
+      </c>
+      <c r="F19" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" s="22" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>338</v>
+        <v>325</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>339</v>
+        <v>326</v>
       </c>
       <c r="F20" s="27" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="22" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C21" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>420</v>
+        <v>405</v>
       </c>
       <c r="E21" s="23" t="s">
-        <v>341</v>
+        <v>328</v>
       </c>
       <c r="F21" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="22" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>421</v>
+        <v>406</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>342</v>
+        <v>329</v>
       </c>
       <c r="F22" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="22" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C23" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>258</v>
+        <v>429</v>
       </c>
       <c r="E23" s="23" t="s">
-        <v>259</v>
-      </c>
-      <c r="F23" s="23" t="s">
-        <v>225</v>
+        <v>248</v>
+      </c>
+      <c r="F23" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="22" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="E24" s="23" t="s">
-        <v>263</v>
-      </c>
-      <c r="F24" s="23" t="s">
-        <v>225</v>
+        <v>252</v>
+      </c>
+      <c r="F24" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="22" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="E25" s="23" t="s">
-        <v>266</v>
-      </c>
-      <c r="F25" s="23" t="s">
-        <v>225</v>
+        <v>255</v>
+      </c>
+      <c r="F25" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A26" s="22" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B26" s="23" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>422</v>
+        <v>407</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="F26" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="22" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="B27" s="23" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C27" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>423</v>
+        <v>408</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="F27" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="22" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="B28" s="23" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>424</v>
+        <v>409</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="F28" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="22" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B29" s="23" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C29" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>273</v>
+        <v>430</v>
       </c>
       <c r="E29" s="23" t="s">
-        <v>274</v>
-      </c>
-      <c r="F29" s="23" t="s">
-        <v>225</v>
+        <v>262</v>
+      </c>
+      <c r="F29" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="22" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B30" s="23" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>425</v>
+        <v>410</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="F30" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="22" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>426</v>
+        <v>411</v>
       </c>
       <c r="E31" s="23" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="F31" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A32" s="22" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>277</v>
+        <v>431</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>278</v>
-      </c>
-      <c r="F32" s="23" t="s">
-        <v>225</v>
+        <v>265</v>
+      </c>
+      <c r="F32" s="28" t="s">
+        <v>353</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="22" t="s">
-        <v>279</v>
+        <v>266</v>
       </c>
       <c r="B33" s="23" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C33" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>323</v>
+        <v>310</v>
       </c>
       <c r="E33" s="23" t="s">
-        <v>324</v>
+        <v>311</v>
       </c>
       <c r="F33" s="27" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A34" s="22" t="s">
-        <v>280</v>
+        <v>267</v>
       </c>
       <c r="B34" s="23" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C34" s="23" t="s">
-        <v>281</v>
+        <v>268</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>308</v>
+        <v>295</v>
       </c>
       <c r="E34" s="23" t="s">
-        <v>309</v>
+        <v>296</v>
       </c>
       <c r="F34" s="27" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="22" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C35" s="23" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>370</v>
+        <v>357</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>371</v>
+        <v>358</v>
       </c>
       <c r="F35" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A36" s="22" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B36" s="23" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C36" s="23" t="s">
-        <v>372</v>
+        <v>359</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>373</v>
+        <v>360</v>
       </c>
       <c r="E36" s="23" t="s">
-        <v>374</v>
+        <v>361</v>
       </c>
       <c r="F36" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A37" s="22" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B37" s="23" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C37" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>427</v>
+        <v>412</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>282</v>
+        <v>269</v>
       </c>
       <c r="F37" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="22" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B38" s="23" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C38" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>283</v>
+        <v>270</v>
       </c>
       <c r="E38" s="23" t="s">
-        <v>284</v>
+        <v>271</v>
       </c>
       <c r="F38" s="23" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="22" t="s">
-        <v>285</v>
+        <v>272</v>
       </c>
       <c r="B39" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C39" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>428</v>
+        <v>413</v>
       </c>
       <c r="E39" s="23" t="s">
-        <v>301</v>
+        <v>288</v>
       </c>
       <c r="F39" s="27" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G39" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A40" s="22" t="s">
-        <v>286</v>
+        <v>273</v>
       </c>
       <c r="B40" s="23" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C40" s="23" t="s">
-        <v>302</v>
+        <v>289</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>303</v>
+        <v>290</v>
       </c>
       <c r="E40" s="23" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
       <c r="F40" s="27" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
       <c r="G40" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A41" s="22" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B41" s="23" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C41" s="23" t="s">
-        <v>375</v>
+        <v>362</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>376</v>
+        <v>363</v>
       </c>
       <c r="E41" s="23" t="s">
-        <v>377</v>
+        <v>364</v>
       </c>
       <c r="F41" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
-        <v>287</v>
+        <v>274</v>
       </c>
       <c r="B42" s="23" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C42" s="23" t="s">
-        <v>288</v>
+        <v>275</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>346</v>
+        <v>333</v>
       </c>
       <c r="E42" s="23" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
       <c r="F42" s="28" t="s">
-        <v>340</v>
+        <v>327</v>
       </c>
       <c r="G42" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
-        <v>289</v>
+        <v>276</v>
       </c>
       <c r="B43" s="23" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C43" s="23" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>378</v>
+        <v>365</v>
       </c>
       <c r="E43" s="23" t="s">
-        <v>379</v>
+        <v>366</v>
       </c>
       <c r="F43" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G43" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="B44" s="23" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="C44" s="23" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>290</v>
+        <v>277</v>
       </c>
       <c r="E44" s="23" t="s">
-        <v>291</v>
+        <v>278</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A45" s="22" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="C45" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>380</v>
+        <v>367</v>
       </c>
       <c r="E45" s="23" t="s">
-        <v>381</v>
+        <v>368</v>
       </c>
       <c r="F45" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A46" s="22" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B46" s="23" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="C46" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>429</v>
+        <v>414</v>
       </c>
       <c r="E46" s="23" t="s">
-        <v>333</v>
+        <v>320</v>
       </c>
       <c r="F46" s="27" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A47" s="22" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C47" s="23" t="s">
-        <v>292</v>
+        <v>279</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>430</v>
+        <v>415</v>
       </c>
       <c r="E47" s="23" t="s">
-        <v>293</v>
+        <v>280</v>
       </c>
       <c r="F47" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A48" s="22" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="B48" s="23" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="C48" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>294</v>
+        <v>281</v>
       </c>
       <c r="E48" s="23" t="s">
-        <v>295</v>
+        <v>282</v>
       </c>
       <c r="F48" s="23" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="22" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B49" s="23" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="C49" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>431</v>
+        <v>416</v>
       </c>
       <c r="E49" s="23" t="s">
-        <v>296</v>
+        <v>283</v>
       </c>
       <c r="F49" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A50" s="22" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C50" s="23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>432</v>
+        <v>417</v>
       </c>
       <c r="E50" s="23" t="s">
-        <v>297</v>
+        <v>284</v>
       </c>
       <c r="F50" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="22" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B51" s="23" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C51" s="23" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>382</v>
+        <v>369</v>
       </c>
       <c r="E51" s="23" t="s">
-        <v>383</v>
+        <v>370</v>
       </c>
       <c r="F51" s="28" t="s">
-        <v>366</v>
+        <v>353</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="17" t="s">
-        <v>298</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>